<commit_message>
docs: collapse legacy map details by default
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -2350,6 +2350,7 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25"/>
     <row r="4" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
@@ -2472,7 +2473,7 @@
       <c r="M7" s="17"/>
       <c r="N7" s="17"/>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="8" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A8" s="18"/>
       <c r="B8" s="19" t="s">
         <v>31</v>
@@ -2502,7 +2503,7 @@
       <c r="M8" s="18"/>
       <c r="N8" s="18"/>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="9" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A9" s="18"/>
       <c r="B9" s="19" t="s">
         <v>38</v>
@@ -2532,7 +2533,7 @@
       <c r="M9" s="18"/>
       <c r="N9" s="18"/>
     </row>
-    <row r="10" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="10" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A10" s="18"/>
       <c r="B10" s="19" t="s">
         <v>44</v>
@@ -2562,7 +2563,7 @@
       <c r="M10" s="18"/>
       <c r="N10" s="18"/>
     </row>
-    <row r="11" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="11" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A11" s="18"/>
       <c r="B11" s="19" t="s">
         <v>49</v>
@@ -2592,7 +2593,7 @@
       <c r="M11" s="18"/>
       <c r="N11" s="18"/>
     </row>
-    <row r="12" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="12" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A12" s="18"/>
       <c r="B12" s="19" t="s">
         <v>54</v>
@@ -2622,7 +2623,7 @@
       <c r="M12" s="18"/>
       <c r="N12" s="18"/>
     </row>
-    <row r="13" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="13" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A13" s="18"/>
       <c r="B13" s="19" t="s">
         <v>59</v>
@@ -2652,7 +2653,7 @@
       <c r="M13" s="18"/>
       <c r="N13" s="18"/>
     </row>
-    <row r="14" ht="48" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="14" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A14" s="18"/>
       <c r="B14" s="19" t="s">
         <v>64</v>
@@ -2682,7 +2683,7 @@
       <c r="M14" s="18"/>
       <c r="N14" s="18"/>
     </row>
-    <row r="15" ht="48" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="15" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A15" s="18"/>
       <c r="B15" s="19" t="s">
         <v>69</v>
@@ -2712,7 +2713,7 @@
       <c r="M15" s="18"/>
       <c r="N15" s="18"/>
     </row>
-    <row r="16" ht="48" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="16" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A16" s="19"/>
       <c r="B16" s="19" t="s">
         <v>73</v>
@@ -2742,7 +2743,7 @@
       <c r="M16" s="19"/>
       <c r="N16" s="19"/>
     </row>
-    <row r="17" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="17" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A17" s="18"/>
       <c r="B17" s="19" t="s">
         <v>77</v>
@@ -2772,7 +2773,7 @@
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="18" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A18" s="18"/>
       <c r="B18" s="19" t="s">
         <v>82</v>
@@ -2826,7 +2827,7 @@
       <c r="M19" s="17"/>
       <c r="N19" s="17"/>
     </row>
-    <row r="20" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="20" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A20" s="18"/>
       <c r="B20" s="19" t="s">
         <v>90</v>
@@ -2856,7 +2857,7 @@
       <c r="M20" s="19"/>
       <c r="N20" s="18"/>
     </row>
-    <row r="21" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="21" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A21" s="18"/>
       <c r="B21" s="19" t="s">
         <v>95</v>
@@ -2886,7 +2887,7 @@
       <c r="M21" s="18"/>
       <c r="N21" s="18"/>
     </row>
-    <row r="22" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="22" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A22" s="18"/>
       <c r="B22" s="19" t="s">
         <v>100</v>
@@ -2916,7 +2917,7 @@
       <c r="M22" s="19"/>
       <c r="N22" s="18"/>
     </row>
-    <row r="23" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="23" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A23" s="18"/>
       <c r="B23" s="19" t="s">
         <v>105</v>
@@ -2946,7 +2947,7 @@
       <c r="M23" s="18"/>
       <c r="N23" s="18"/>
     </row>
-    <row r="24" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="24" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A24" s="18"/>
       <c r="B24" s="19" t="s">
         <v>110</v>
@@ -2976,7 +2977,7 @@
       <c r="M24" s="18"/>
       <c r="N24" s="18"/>
     </row>
-    <row r="25" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="25" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A25" s="19"/>
       <c r="B25" s="19" t="s">
         <v>116</v>
@@ -3030,7 +3031,7 @@
       <c r="M26" s="17"/>
       <c r="N26" s="17"/>
     </row>
-    <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="27" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A27" s="18"/>
       <c r="B27" s="19" t="s">
         <v>123</v>
@@ -3060,7 +3061,7 @@
       <c r="M27" s="18"/>
       <c r="N27" s="18"/>
     </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="28" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A28" s="18"/>
       <c r="B28" s="19" t="s">
         <v>128</v>
@@ -3090,7 +3091,7 @@
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
     </row>
-    <row r="29" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="29" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A29" s="18"/>
       <c r="B29" s="19" t="s">
         <v>133</v>
@@ -3120,7 +3121,7 @@
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
     </row>
-    <row r="30" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="30" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A30" s="18"/>
       <c r="B30" s="19" t="s">
         <v>138</v>
@@ -3150,7 +3151,7 @@
       <c r="M30" s="18"/>
       <c r="N30" s="18"/>
     </row>
-    <row r="31" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="31" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A31" s="18"/>
       <c r="B31" s="19" t="s">
         <v>143</v>
@@ -3180,7 +3181,7 @@
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
     </row>
-    <row r="32" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="32" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A32" s="19"/>
       <c r="B32" s="19" t="s">
         <v>148</v>
@@ -3210,7 +3211,7 @@
       <c r="M32" s="19"/>
       <c r="N32" s="19"/>
     </row>
-    <row r="33" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="33" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A33" s="18"/>
       <c r="B33" s="19" t="s">
         <v>153</v>
@@ -3240,7 +3241,7 @@
       <c r="M33" s="19"/>
       <c r="N33" s="18"/>
     </row>
-    <row r="34" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="34" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A34" s="18"/>
       <c r="B34" s="19" t="s">
         <v>158</v>
@@ -3270,7 +3271,7 @@
       <c r="M34" s="19"/>
       <c r="N34" s="18"/>
     </row>
-    <row r="35" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="35" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A35" s="18"/>
       <c r="B35" s="19" t="s">
         <v>163</v>
@@ -3300,7 +3301,7 @@
       <c r="M35" s="19"/>
       <c r="N35" s="18"/>
     </row>
-    <row r="36" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="36" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A36" s="18"/>
       <c r="B36" s="19" t="s">
         <v>168</v>
@@ -3330,7 +3331,7 @@
       <c r="M36" s="19"/>
       <c r="N36" s="18"/>
     </row>
-    <row r="37" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="37" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A37" s="19"/>
       <c r="B37" s="19" t="s">
         <v>173</v>
@@ -3384,7 +3385,7 @@
       <c r="M38" s="17"/>
       <c r="N38" s="17"/>
     </row>
-    <row r="39" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="39" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A39" s="18"/>
       <c r="B39" s="19" t="s">
         <v>180</v>
@@ -3414,7 +3415,7 @@
       <c r="M39" s="19"/>
       <c r="N39" s="18"/>
     </row>
-    <row r="40" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="40" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A40" s="18"/>
       <c r="B40" s="19" t="s">
         <v>185</v>
@@ -3444,7 +3445,7 @@
       <c r="M40" s="19"/>
       <c r="N40" s="18"/>
     </row>
-    <row r="41" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="41" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A41" s="18"/>
       <c r="B41" s="19" t="s">
         <v>190</v>
@@ -3474,7 +3475,7 @@
       <c r="M41" s="19"/>
       <c r="N41" s="18"/>
     </row>
-    <row r="42" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="42" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A42" s="18"/>
       <c r="B42" s="19" t="s">
         <v>195</v>
@@ -3504,7 +3505,7 @@
       <c r="M42" s="19"/>
       <c r="N42" s="18"/>
     </row>
-    <row r="43" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="43" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A43" s="19"/>
       <c r="B43" s="19" t="s">
         <v>200</v>
@@ -3534,7 +3535,7 @@
       <c r="M43" s="19"/>
       <c r="N43" s="19"/>
     </row>
-    <row r="44" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="44" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A44" s="18"/>
       <c r="B44" s="19" t="s">
         <v>205</v>
@@ -3564,7 +3565,7 @@
       <c r="M44" s="18"/>
       <c r="N44" s="18"/>
     </row>
-    <row r="45" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="45" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A45" s="18"/>
       <c r="B45" s="19" t="s">
         <v>210</v>
@@ -3594,7 +3595,7 @@
       <c r="M45" s="18"/>
       <c r="N45" s="18"/>
     </row>
-    <row r="46" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="46" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A46" s="18"/>
       <c r="B46" s="19" t="s">
         <v>215</v>
@@ -3648,7 +3649,7 @@
       <c r="M47" s="17"/>
       <c r="N47" s="17"/>
     </row>
-    <row r="48" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="48" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A48" s="18"/>
       <c r="B48" s="19" t="s">
         <v>222</v>
@@ -3678,7 +3679,7 @@
       <c r="M48" s="18"/>
       <c r="N48" s="18"/>
     </row>
-    <row r="49" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="49" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A49" s="18"/>
       <c r="B49" s="19" t="s">
         <v>227</v>
@@ -3708,7 +3709,7 @@
       <c r="M49" s="18"/>
       <c r="N49" s="18"/>
     </row>
-    <row r="50" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="50" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A50" s="18"/>
       <c r="B50" s="19" t="s">
         <v>232</v>
@@ -3738,7 +3739,7 @@
       <c r="M50" s="18"/>
       <c r="N50" s="18"/>
     </row>
-    <row r="51" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="51" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A51" s="18"/>
       <c r="B51" s="19" t="s">
         <v>237</v>
@@ -3768,7 +3769,7 @@
       <c r="M51" s="18"/>
       <c r="N51" s="18"/>
     </row>
-    <row r="52" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="52" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A52" s="19"/>
       <c r="B52" s="19" t="s">
         <v>242</v>
@@ -3798,7 +3799,7 @@
       <c r="M52" s="19"/>
       <c r="N52" s="19"/>
     </row>
-    <row r="53" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="53" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A53" s="18"/>
       <c r="B53" s="19" t="s">
         <v>247</v>
@@ -3828,7 +3829,7 @@
       <c r="M53" s="18"/>
       <c r="N53" s="18"/>
     </row>
-    <row r="54" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="54" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A54" s="18"/>
       <c r="B54" s="19" t="s">
         <v>252</v>
@@ -3858,7 +3859,7 @@
       <c r="M54" s="18"/>
       <c r="N54" s="18"/>
     </row>
-    <row r="55" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="55" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A55" s="18"/>
       <c r="B55" s="19" t="s">
         <v>257</v>
@@ -3888,7 +3889,7 @@
       <c r="M55" s="18"/>
       <c r="N55" s="18"/>
     </row>
-    <row r="56" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="56" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A56" s="18"/>
       <c r="B56" s="19" t="s">
         <v>262</v>
@@ -3942,7 +3943,7 @@
       <c r="M57" s="17"/>
       <c r="N57" s="17"/>
     </row>
-    <row r="58" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="58" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A58" s="18"/>
       <c r="B58" s="19" t="s">
         <v>269</v>
@@ -3972,7 +3973,7 @@
       <c r="M58" s="18"/>
       <c r="N58" s="18"/>
     </row>
-    <row r="59" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="59" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A59" s="18"/>
       <c r="B59" s="19" t="s">
         <v>274</v>
@@ -4002,7 +4003,7 @@
       <c r="M59" s="18"/>
       <c r="N59" s="18"/>
     </row>
-    <row r="60" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="60" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A60" s="18"/>
       <c r="B60" s="19" t="s">
         <v>279</v>
@@ -4032,7 +4033,7 @@
       <c r="M60" s="18"/>
       <c r="N60" s="18"/>
     </row>
-    <row r="61" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="61" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A61" s="18"/>
       <c r="B61" s="19" t="s">
         <v>284</v>
@@ -4062,7 +4063,7 @@
       <c r="M61" s="18"/>
       <c r="N61" s="18"/>
     </row>
-    <row r="62" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="62" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A62" s="18"/>
       <c r="B62" s="19" t="s">
         <v>289</v>
@@ -4092,7 +4093,7 @@
       <c r="M62" s="18"/>
       <c r="N62" s="18"/>
     </row>
-    <row r="63" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="63" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A63" s="19"/>
       <c r="B63" s="19" t="s">
         <v>294</v>
@@ -4122,7 +4123,7 @@
       <c r="M63" s="19"/>
       <c r="N63" s="19"/>
     </row>
-    <row r="64" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="64" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A64" s="18"/>
       <c r="B64" s="19" t="s">
         <v>299</v>
@@ -4152,7 +4153,7 @@
       <c r="M64" s="18"/>
       <c r="N64" s="18"/>
     </row>
-    <row r="65" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="65" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A65" s="18"/>
       <c r="B65" s="19" t="s">
         <v>304</v>
@@ -4182,7 +4183,7 @@
       <c r="M65" s="18"/>
       <c r="N65" s="18"/>
     </row>
-    <row r="66" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="66" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A66" s="18"/>
       <c r="B66" s="19" t="s">
         <v>309</v>
@@ -4212,7 +4213,7 @@
       <c r="M66" s="18"/>
       <c r="N66" s="18"/>
     </row>
-    <row r="67" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="67" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A67" s="18"/>
       <c r="B67" s="19" t="s">
         <v>314</v>
@@ -4242,7 +4243,7 @@
       <c r="M67" s="18"/>
       <c r="N67" s="18"/>
     </row>
-    <row r="68" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="68" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A68" s="19"/>
       <c r="B68" s="19" t="s">
         <v>319</v>
@@ -4272,7 +4273,7 @@
       <c r="M68" s="19"/>
       <c r="N68" s="19"/>
     </row>
-    <row r="69" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="69" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A69" s="18"/>
       <c r="B69" s="19" t="s">
         <v>324</v>
@@ -4302,7 +4303,7 @@
       <c r="M69" s="18"/>
       <c r="N69" s="18"/>
     </row>
-    <row r="70" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="70" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A70" s="18"/>
       <c r="B70" s="19" t="s">
         <v>329</v>
@@ -4332,7 +4333,7 @@
       <c r="M70" s="19"/>
       <c r="N70" s="18"/>
     </row>
-    <row r="71" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="71" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A71" s="19"/>
       <c r="B71" s="19" t="s">
         <v>334</v>
@@ -4386,7 +4387,7 @@
       <c r="M72" s="17"/>
       <c r="N72" s="17"/>
     </row>
-    <row r="73" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="73" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A73" s="18"/>
       <c r="B73" s="19" t="s">
         <v>341</v>
@@ -4416,7 +4417,7 @@
       <c r="M73" s="18"/>
       <c r="N73" s="18"/>
     </row>
-    <row r="74" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="74" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A74" s="19"/>
       <c r="B74" s="19" t="s">
         <v>346</v>
@@ -4446,7 +4447,7 @@
       <c r="M74" s="19"/>
       <c r="N74" s="19"/>
     </row>
-    <row r="75" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="75" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A75" s="18"/>
       <c r="B75" s="19" t="s">
         <v>351</v>
@@ -4476,7 +4477,7 @@
       <c r="M75" s="19"/>
       <c r="N75" s="18"/>
     </row>
-    <row r="76" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="76" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A76" s="18"/>
       <c r="B76" s="19" t="s">
         <v>356</v>
@@ -4506,7 +4507,7 @@
       <c r="M76" s="18"/>
       <c r="N76" s="18"/>
     </row>
-    <row r="77" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="77" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A77" s="19"/>
       <c r="B77" s="19" t="s">
         <v>361</v>
@@ -4536,7 +4537,7 @@
       <c r="M77" s="19"/>
       <c r="N77" s="19"/>
     </row>
-    <row r="78" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="78" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A78" s="18"/>
       <c r="B78" s="19" t="s">
         <v>367</v>
@@ -4590,7 +4591,7 @@
       <c r="M79" s="17"/>
       <c r="N79" s="17"/>
     </row>
-    <row r="80" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="80" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A80" s="18"/>
       <c r="B80" s="19" t="s">
         <v>374</v>
@@ -4620,7 +4621,7 @@
       <c r="M80" s="18"/>
       <c r="N80" s="18"/>
     </row>
-    <row r="81" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="81" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A81" s="19"/>
       <c r="B81" s="19" t="s">
         <v>379</v>
@@ -4650,7 +4651,7 @@
       <c r="M81" s="19"/>
       <c r="N81" s="19"/>
     </row>
-    <row r="82" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="82" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A82" s="18"/>
       <c r="B82" s="19" t="s">
         <v>384</v>
@@ -4680,7 +4681,7 @@
       <c r="M82" s="18"/>
       <c r="N82" s="18"/>
     </row>
-    <row r="83" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="83" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="18"/>
       <c r="B83" s="19" t="s">
         <v>389</v>
@@ -4710,7 +4711,7 @@
       <c r="M83" s="18"/>
       <c r="N83" s="18"/>
     </row>
-    <row r="84" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="84" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="19"/>
       <c r="B84" s="19" t="s">
         <v>394</v>
@@ -4740,7 +4741,7 @@
       <c r="M84" s="19"/>
       <c r="N84" s="19"/>
     </row>
-    <row r="85" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="85" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
         <v>399</v>
@@ -4770,7 +4771,7 @@
       <c r="M85" s="18"/>
       <c r="N85" s="18"/>
     </row>
-    <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="86" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A86" s="19"/>
       <c r="B86" s="19" t="s">
         <v>403</v>
@@ -4800,7 +4801,7 @@
       <c r="M86" s="19"/>
       <c r="N86" s="19"/>
     </row>
-    <row r="87" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="87" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
         <v>407</v>
@@ -4830,7 +4831,7 @@
       <c r="M87" s="18"/>
       <c r="N87" s="18"/>
     </row>
-    <row r="88" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="88" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
         <v>412</v>
@@ -4860,7 +4861,7 @@
       <c r="M88" s="18"/>
       <c r="N88" s="18"/>
     </row>
-    <row r="89" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="89" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
         <v>417</v>
@@ -4890,7 +4891,7 @@
       <c r="M89" s="18"/>
       <c r="N89" s="18"/>
     </row>
-    <row r="90" ht="60" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="90" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
         <v>422</v>
@@ -4944,7 +4945,7 @@
       <c r="M91" s="17"/>
       <c r="N91" s="17"/>
     </row>
-    <row r="92" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="92" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
         <v>429</v>
@@ -4974,7 +4975,7 @@
       <c r="M92" s="18"/>
       <c r="N92" s="18"/>
     </row>
-    <row r="93" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="93" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="19"/>
       <c r="B93" s="19" t="s">
         <v>434</v>
@@ -5004,7 +5005,7 @@
       <c r="M93" s="19"/>
       <c r="N93" s="19"/>
     </row>
-    <row r="94" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="94" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="19"/>
       <c r="B94" s="19" t="s">
         <v>439</v>
@@ -5034,7 +5035,7 @@
       <c r="M94" s="19"/>
       <c r="N94" s="19"/>
     </row>
-    <row r="95" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="95" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
         <v>444</v>
@@ -5064,7 +5065,7 @@
       <c r="M95" s="18"/>
       <c r="N95" s="18"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="96" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
         <v>449</v>
@@ -5094,7 +5095,7 @@
       <c r="M96" s="18"/>
       <c r="N96" s="18"/>
     </row>
-    <row r="97" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="97" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
         <v>454</v>
@@ -5124,7 +5125,7 @@
       <c r="M97" s="18"/>
       <c r="N97" s="18"/>
     </row>
-    <row r="98" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="98" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
         <v>459</v>
@@ -5154,7 +5155,7 @@
       <c r="M98" s="18"/>
       <c r="N98" s="18"/>
     </row>
-    <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="99" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A99" s="18"/>
       <c r="B99" s="19" t="s">
         <v>464</v>
@@ -5208,7 +5209,7 @@
       <c r="M100" s="17"/>
       <c r="N100" s="17"/>
     </row>
-    <row r="101" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="101" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="19"/>
       <c r="B101" s="19" t="s">
         <v>471</v>
@@ -5238,7 +5239,7 @@
       <c r="M101" s="19"/>
       <c r="N101" s="19"/>
     </row>
-    <row r="102" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="102" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
         <v>476</v>
@@ -5268,7 +5269,7 @@
       <c r="M102" s="18"/>
       <c r="N102" s="18"/>
     </row>
-    <row r="103" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="103" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
         <v>481</v>
@@ -5298,7 +5299,7 @@
       <c r="M103" s="18"/>
       <c r="N103" s="18"/>
     </row>
-    <row r="104" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="104" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
         <v>486</v>
@@ -5328,7 +5329,7 @@
       <c r="M104" s="18"/>
       <c r="N104" s="18"/>
     </row>
-    <row r="105" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="105" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="19"/>
       <c r="B105" s="19" t="s">
         <v>491</v>
@@ -5358,7 +5359,7 @@
       <c r="M105" s="19"/>
       <c r="N105" s="19"/>
     </row>
-    <row r="106" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="106" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
         <v>496</v>
@@ -5388,7 +5389,7 @@
       <c r="M106" s="18"/>
       <c r="N106" s="18"/>
     </row>
-    <row r="107" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="107" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
         <v>501</v>
@@ -5442,7 +5443,7 @@
       <c r="M108" s="17"/>
       <c r="N108" s="17"/>
     </row>
-    <row r="109" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="109" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
         <v>508</v>
@@ -5472,7 +5473,7 @@
       <c r="M109" s="18"/>
       <c r="N109" s="18"/>
     </row>
-    <row r="110" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="110" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
         <v>513</v>
@@ -5502,7 +5503,7 @@
       <c r="M110" s="18"/>
       <c r="N110" s="18"/>
     </row>
-    <row r="111" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="111" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
         <v>518</v>
@@ -5532,7 +5533,7 @@
       <c r="M111" s="18"/>
       <c r="N111" s="18"/>
     </row>
-    <row r="112" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="112" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
         <v>523</v>
@@ -5562,7 +5563,7 @@
       <c r="M112" s="18"/>
       <c r="N112" s="18"/>
     </row>
-    <row r="113" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="113" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
         <v>528</v>
@@ -5592,7 +5593,7 @@
       <c r="M113" s="18"/>
       <c r="N113" s="18"/>
     </row>
-    <row r="114" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="114" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
         <v>533</v>
@@ -5622,7 +5623,7 @@
       <c r="M114" s="18"/>
       <c r="N114" s="18"/>
     </row>
-    <row r="115" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="115" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
         <v>538</v>
@@ -5676,7 +5677,7 @@
       <c r="M116" s="17"/>
       <c r="N116" s="17"/>
     </row>
-    <row r="117" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="117" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="20"/>
       <c r="B117" s="20" t="s">
         <v>545</v>
@@ -5706,7 +5707,7 @@
       <c r="M117" s="20"/>
       <c r="N117" s="20"/>
     </row>
-    <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="118" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A118" s="20"/>
       <c r="B118" s="20" t="s">
         <v>550</v>
@@ -5736,7 +5737,7 @@
       <c r="M118" s="20"/>
       <c r="N118" s="20"/>
     </row>
-    <row r="119" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="119" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="20"/>
       <c r="B119" s="20" t="s">
         <v>555</v>
@@ -5766,7 +5767,7 @@
       <c r="M119" s="20"/>
       <c r="N119" s="20"/>
     </row>
-    <row r="120" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="120" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="20"/>
       <c r="B120" s="20" t="s">
         <v>560</v>
@@ -5796,7 +5797,7 @@
       <c r="M120" s="20"/>
       <c r="N120" s="20"/>
     </row>
-    <row r="121" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="121" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="20"/>
       <c r="B121" s="20" t="s">
         <v>565</v>
@@ -5826,7 +5827,7 @@
       <c r="M121" s="20"/>
       <c r="N121" s="20"/>
     </row>
-    <row r="122" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="122" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="20"/>
       <c r="B122" s="20" t="s">
         <v>570</v>
@@ -5856,7 +5857,7 @@
       <c r="M122" s="20"/>
       <c r="N122" s="20"/>
     </row>
-    <row r="123" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="123" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="20"/>
       <c r="B123" s="20" t="s">
         <v>575</v>
@@ -5886,7 +5887,7 @@
       <c r="M123" s="20"/>
       <c r="N123" s="20"/>
     </row>
-    <row r="124" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="124" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="20"/>
       <c r="B124" s="20" t="s">
         <v>580</v>
@@ -5916,7 +5917,7 @@
       <c r="M124" s="20"/>
       <c r="N124" s="20"/>
     </row>
-    <row r="125" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="125" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="20"/>
       <c r="B125" s="20" t="s">
         <v>585</v>
@@ -5946,7 +5947,7 @@
       <c r="M125" s="20"/>
       <c r="N125" s="20"/>
     </row>
-    <row r="126" ht="60" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="126" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="20"/>
       <c r="B126" s="20" t="s">
         <v>590</v>
@@ -5976,7 +5977,7 @@
       <c r="M126" s="20"/>
       <c r="N126" s="20"/>
     </row>
-    <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="127" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A127" s="20"/>
       <c r="B127" s="20" t="s">
         <v>595</v>
@@ -6006,7 +6007,7 @@
       <c r="M127" s="20"/>
       <c r="N127" s="20"/>
     </row>
-    <row r="128" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="128" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="20"/>
       <c r="B128" s="20" t="s">
         <v>600</v>

</xml_diff>

<commit_message>
docs: correct stage 1 parity map findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="648">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -160,6 +160,21 @@
     <t>legacy/src/base/cics/cobol/BNKMENU.cbl input-processing paragraphs; BNK1*.cbl VALID-DATA-SW</t>
   </si>
   <si>
+    <t>CICS operator enters an invalid menu choice</t>
+  </si>
+  <si>
+    <t>Reject a menu value other than 1-7 or A without dispatching a banking transaction.</t>
+  </si>
+  <si>
+    <t>A typed menu value follows a different validation branch from unsupported 3270 attention keys.</t>
+  </si>
+  <si>
+    <t>You must enter a valid value (1-7 or A). is shown and the menu is redisplayed without dispatch.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:363-378</t>
+  </si>
+  <si>
     <t>Web operator opens the control panel</t>
   </si>
   <si>
@@ -259,22 +274,37 @@
     <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:24-25,180-215</t>
   </si>
   <si>
-    <t>IMS logout update fails</t>
+    <t>IMS logout customer retrieval fails</t>
   </si>
   <si>
     <t>Operational path</t>
   </si>
   <si>
-    <t>Report inability to persist logout state.</t>
-  </si>
-  <si>
-    <t>A storage failure is not presented as a successful logout.</t>
+    <t>Report inability to retrieve the customer before changing logout state.</t>
+  </si>
+  <si>
+    <t>A failed IMS customer lookup prevents the logout update from being attempted.</t>
   </si>
   <si>
     <t>FAILED UPDATE FOR LOGOFF is returned.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:24-25,190-215</t>
+    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:180-202</t>
+  </si>
+  <si>
+    <t>IMS logout replacement fails but reports success</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly replace the observed false-success response when the IMS REPL call fails.</t>
+  </si>
+  <si>
+    <t>IBLOGOUT initially sets a failure message for a failed replacement, then overwrites it unconditionally.</t>
+  </si>
+  <si>
+    <t>LOGOFF SUCCESSFUL is returned even though the logout status replacement failed; this is a security and data-consistency deviation.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:203-212</t>
   </si>
   <si>
     <t>UF-002</t>
@@ -352,13 +382,13 @@
     <t>The UI contains name search, but the API client explicitly declares it unsupported.</t>
   </si>
   <si>
-    <t>Feature Not Implemented is shown instead of fabricated results.</t>
+    <t>An inline notification titled Error shows the unsupported-operation message; no fabricated results are displayed.</t>
   </si>
   <si>
     <t>Partial</t>
   </si>
   <si>
-    <t>legacy/src/frontend/customer-details.html:141-153,207-221; js/api.js:193-194</t>
+    <t>legacy/src/frontend/customer-details.html:207-229; legacy/src/frontend/js/api.js:193-194</t>
   </si>
   <si>
     <t>Web customer lookup returns no record</t>
@@ -628,19 +658,19 @@
     <t>legacy/src/base/ims/cobol/IBACSUM.cbl:101,186-265</t>
   </si>
   <si>
-    <t>IMS applies the old-account rule</t>
-  </si>
-  <si>
-    <t>Return zero balance for legacy customer IDs below 16.</t>
-  </si>
-  <si>
-    <t>The IMS implementation contains a compatibility rule for old accounts.</t>
-  </si>
-  <si>
-    <t>Affected account summaries expose zero rather than the stored balance.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/IBACSUM.cbl:267 onward</t>
+    <t>IMS old-account zero-balance rule is dormant</t>
+  </si>
+  <si>
+    <t>Return stored account balances because the old-customer compatibility routine is not invoked by the active summary path.</t>
+  </si>
+  <si>
+    <t>A zero-balance helper exists for customer IDs below 16, but its only call is commented out.</t>
+  </si>
+  <si>
+    <t>The active account-summary path returns the stored balance; no zero-balance override is executed.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/IBACSUM.cbl:221-224,269-274</t>
   </si>
   <si>
     <t>Web operator browses customer accounts</t>
@@ -925,34 +955,64 @@
     <t>legacy/src/base/ims/cobol/IBTRAN.cbl:31-32,302-422</t>
   </si>
   <si>
+    <t>IMS transaction uses mismatched customer and account identifiers</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly close the observed authorization gap where account ownership is not validated.</t>
+  </si>
+  <si>
+    <t>IBTRAN mutates the account selected by account ID, then independently builds the response portfolio from the supplied customer ID.</t>
+  </si>
+  <si>
+    <t>An existing account can be mutated while the returned summary belongs to another supplied customer; this is a security and data-integrity deviation.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:299-367,386-430; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BcustomerId%7D%2F%7BaccountId%7D%2Fdeposit/post/request.yaml</t>
+  </si>
+  <si>
     <t>IMS transaction history is persisted</t>
   </si>
   <si>
-    <t>Store the cash transaction in IMS history or, when Java is primed, in DB2 history.</t>
-  </si>
-  <si>
-    <t>The runtime can use either legacy history path.</t>
-  </si>
-  <si>
-    <t>History receives transaction ID, type, amount, account, and resulting balance.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:314-367,454-554; TransactionService.java:140</t>
-  </si>
-  <si>
-    <t>Web operator deposits to a selected account</t>
-  </si>
-  <si>
-    <t>Find customer accounts, select one, and submit a positive deposit with sort code and optional description.</t>
-  </si>
-  <si>
-    <t>The web channel supports deposits for CICS and IMS.</t>
-  </si>
-  <si>
-    <t>A success message shows deposited amount and resulting balance.</t>
-  </si>
-  <si>
-    <t>legacy/src/frontend/account-deposit.html:202-380; js/api.js:297-334</t>
+    <t>Attempt DB2 transaction-history persistence through Java, then insert IMS history, then replace the account record.</t>
+  </si>
+  <si>
+    <t>The active transaction path dual-writes history in a fixed order rather than choosing one interchangeable store.</t>
+  </si>
+  <si>
+    <t>DB2 history is attempted first, IMS history is inserted next, and the account is replaced last; failures can expose partial-write risk according to the coded status handling.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:326-367,454-554; legacy/src/base/ims/java/src/main/java/nazare/jmp/service/TransactionService.java:140</t>
+  </si>
+  <si>
+    <t>Web operator deposits to a selected CICS account</t>
+  </si>
+  <si>
+    <t>Find a CICS customer account, select it, and submit a positive deposit with sort code and optional description.</t>
+  </si>
+  <si>
+    <t>The CICS deposit succeeds, but its response uses scalar balance fields while the page expects an array for display.</t>
+  </si>
+  <si>
+    <t>A success notification shows the deposited amount and New balance: $N/A despite the successful balance update.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/account-deposit.html:202-380; legacy/src/frontend/js/api.js:297-334; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Fdeposit/post/response_201.yaml</t>
+  </si>
+  <si>
+    <t>Web operator deposits to a selected IMS account</t>
+  </si>
+  <si>
+    <t>Find an IMS customer account, select it, and submit a positive deposit.</t>
+  </si>
+  <si>
+    <t>The IMS response contains portfolio arrays that match the page's balance-selection branch.</t>
+  </si>
+  <si>
+    <t>A success notification shows the deposited amount and the selected account's resulting balance.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/account-deposit.html:202-380; legacy/src/frontend/js/api.js:297-334; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BcustomerId%7D%2F%7BaccountId%7D%2Fdeposit/post/response_201.yaml</t>
   </si>
   <si>
     <t>Web deposit validation or backend fails</t>
@@ -1030,6 +1090,45 @@
     <t>legacy/src/base/ims/cobol/IBTRAN.cbl:338-348</t>
   </si>
   <si>
+    <t>Direct IMS negative deposit reverses transaction direction</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly reject the direct IMS message behavior that accepts a negative deposit amount.</t>
+  </si>
+  <si>
+    <t>IBTRAN converts the signed value without a positive-amount check; OpenAPI/web validation is a separate boundary.</t>
+  </si>
+  <si>
+    <t>A negative deposit subtracts its absolute value and advances transaction/history processing.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:294-367</t>
+  </si>
+  <si>
+    <t>Direct IMS negative withdrawal reverses transaction direction</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly reject the direct IMS message behavior that accepts a negative withdrawal amount.</t>
+  </si>
+  <si>
+    <t>IBTRAN subtracts the signed value without a positive-amount check; OpenAPI/web validation is a separate boundary.</t>
+  </si>
+  <si>
+    <t>A negative withdrawal adds its absolute value and advances transaction/history processing.</t>
+  </si>
+  <si>
+    <t>Direct IMS zero-value transaction writes history</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly reject the direct IMS message behavior that accepts a zero amount.</t>
+  </si>
+  <si>
+    <t>The balance arithmetic has no effect, but the transaction ID and history/last-transaction path still advance.</t>
+  </si>
+  <si>
+    <t>The balance remains unchanged while transaction history and last-transaction processing run.</t>
+  </si>
+  <si>
     <t>UF-007</t>
   </si>
   <si>
@@ -1441,19 +1540,49 @@
     <t>legacy/src/api/src/main/api/openapi.yaml:25,616-635; auth.bankofz.example.com is a placeholder endpoint</t>
   </si>
   <si>
-    <t>API maps legacy account types</t>
-  </si>
-  <si>
-    <t>Translate legacy account types into API product categories.</t>
-  </si>
-  <si>
-    <t>CICS/IMS values are normalized for API consumers.</t>
-  </si>
-  <si>
-    <t>ISA maps to SAVINGS, MORTGAGE to LOAN, and remaining mapped values fall back to CURRENT.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/operations response.yaml account-type mapping expressions</t>
+    <t>CICS single-account API normalizes account type</t>
+  </si>
+  <si>
+    <t>Translate the CICS single-account response into API product categories.</t>
+  </si>
+  <si>
+    <t>Only the single-account CICS mapping applies the documented normalization.</t>
+  </si>
+  <si>
+    <t>ISA maps to SAVINGS, MORTGAGE maps to LOAN, and all other values map to CURRENT.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D/get/response_200.yaml:10-15</t>
+  </si>
+  <si>
+    <t>CICS account-list API passes raw account types</t>
+  </si>
+  <si>
+    <t>Expose the route-specific CICS customer-account list mapping without assuming single-account normalization.</t>
+  </si>
+  <si>
+    <t>The list mapping passes the legacy account type directly to API consumers.</t>
+  </si>
+  <si>
+    <t>Raw CICS account type values are returned by the customer account-list route.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_200.yaml:16-20</t>
+  </si>
+  <si>
+    <t>IMS account API emits schema-invalid CHECKING type</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly correct the route-specific IMS mapping for current/checking accounts.</t>
+  </si>
+  <si>
+    <t>IMS mappings convert type c to CHECKING even though the OpenAPI Account.accountType enum omits CHECKING.</t>
+  </si>
+  <si>
+    <t>IMS current/checking accounts are emitted as CHECKING, creating a response-contract deviation.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Fims%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_200.yaml:16-20; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BaccountId%7D/get/response_200.yaml:11-15; legacy/src/api/src/main/api/openapi.yaml</t>
   </si>
   <si>
     <t>Web server serves the static UI</t>
@@ -1832,7 +1961,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1887,6 +2016,17 @@
     <font>
       <color rgb="FF000000"/>
       <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -2029,7 +2169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2082,6 +2222,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2296,7 +2442,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N128"/>
+  <dimension ref="A1:N137"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2350,7 +2496,6 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25"/>
     <row r="4" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
@@ -2569,7 +2714,7 @@
         <v>49</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>50</v>
@@ -2629,7 +2774,7 @@
         <v>59</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D13" s="18" t="s">
         <v>60</v>
@@ -2659,7 +2804,7 @@
         <v>64</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="18" t="s">
         <v>65</v>
@@ -2689,7 +2834,7 @@
         <v>69</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D15" s="18" t="s">
         <v>70</v>
@@ -2704,7 +2849,7 @@
         <v>36</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I15" s="18"/>
       <c r="J15" s="18"/>
@@ -2716,25 +2861,25 @@
     <row r="16" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A16" s="19"/>
       <c r="B16" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>39</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G16" s="19" t="s">
         <v>36</v>
       </c>
       <c r="H16" s="19" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I16" s="19"/>
       <c r="J16" s="19"/>
@@ -2746,25 +2891,25 @@
     <row r="17" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A17" s="18"/>
       <c r="B17" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G17" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="I17" s="18"/>
       <c r="J17" s="18"/>
@@ -2779,22 +2924,22 @@
         <v>82</v>
       </c>
       <c r="C18" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="F18" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="G18" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" s="18" t="s">
         <v>86</v>
-      </c>
-      <c r="G18" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="18" t="s">
-        <v>87</v>
       </c>
       <c r="I18" s="18"/>
       <c r="J18" s="18"/>
@@ -2803,23 +2948,29 @@
       <c r="M18" s="18"/>
       <c r="N18" s="18"/>
     </row>
-    <row r="19" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="s">
+    <row r="19" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="D19" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
+      <c r="E19" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="17" t="s">
+        <v>92</v>
+      </c>
       <c r="I19" s="17"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
@@ -2830,25 +2981,25 @@
     <row r="20" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A20" s="18"/>
       <c r="B20" s="19" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G20" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="I20" s="18"/>
       <c r="J20" s="18"/>
@@ -2857,29 +3008,23 @@
       <c r="M20" s="19"/>
       <c r="N20" s="18"/>
     </row>
-    <row r="21" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A21" s="18"/>
+    <row r="21" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
+        <v>98</v>
+      </c>
       <c r="B21" s="19" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H21" s="18" t="s">
-        <v>99</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
       <c r="I21" s="18"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
@@ -2923,7 +3068,7 @@
         <v>105</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D23" s="18" t="s">
         <v>106</v>
@@ -2953,7 +3098,7 @@
         <v>110</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>111</v>
@@ -2965,10 +3110,10 @@
         <v>113</v>
       </c>
       <c r="G24" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="18" t="s">
         <v>114</v>
-      </c>
-      <c r="H24" s="18" t="s">
-        <v>115</v>
       </c>
       <c r="I24" s="18"/>
       <c r="J24" s="18"/>
@@ -2980,25 +3125,25 @@
     <row r="25" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A25" s="19"/>
       <c r="B25" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D25" s="19" t="s">
+      <c r="E25" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="F25" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="G25" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="19" t="s">
         <v>119</v>
-      </c>
-      <c r="G25" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="19" t="s">
-        <v>120</v>
       </c>
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
@@ -3007,23 +3152,29 @@
       <c r="M25" s="19"/>
       <c r="N25" s="19"/>
     </row>
-    <row r="26" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="17" t="s">
+    <row r="26" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A26" s="17"/>
+      <c r="B26" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="E26" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="C26" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
+      <c r="F26" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>125</v>
+      </c>
       <c r="I26" s="17"/>
       <c r="J26" s="17"/>
       <c r="K26" s="17"/>
@@ -3034,25 +3185,25 @@
     <row r="27" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A27" s="18"/>
       <c r="B27" s="19" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G27" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I27" s="18"/>
       <c r="J27" s="18"/>
@@ -3061,29 +3212,23 @@
       <c r="M27" s="18"/>
       <c r="N27" s="18"/>
     </row>
-    <row r="28" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A28" s="18"/>
+    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
+        <v>131</v>
+      </c>
       <c r="B28" s="19" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="E28" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="F28" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="G28" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="18" t="s">
-        <v>132</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
       <c r="I28" s="18"/>
       <c r="J28" s="18"/>
       <c r="K28" s="18"/>
@@ -3097,7 +3242,7 @@
         <v>133</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="D29" s="18" t="s">
         <v>134</v>
@@ -3157,7 +3302,7 @@
         <v>143</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D31" s="18" t="s">
         <v>144</v>
@@ -3187,7 +3332,7 @@
         <v>148</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D32" s="19" t="s">
         <v>149</v>
@@ -3217,7 +3362,7 @@
         <v>153</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D33" s="18" t="s">
         <v>154</v>
@@ -3277,7 +3422,7 @@
         <v>163</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D35" s="18" t="s">
         <v>164</v>
@@ -3349,7 +3494,7 @@
         <v>176</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="H37" s="19" t="s">
         <v>177</v>
@@ -3361,23 +3506,29 @@
       <c r="M37" s="19"/>
       <c r="N37" s="19"/>
     </row>
-    <row r="38" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="17" t="s">
+    <row r="38" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A38" s="17"/>
+      <c r="B38" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="C38" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D38" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="C38" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D38" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="17"/>
+      <c r="E38" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H38" s="17" t="s">
+        <v>182</v>
+      </c>
       <c r="I38" s="17"/>
       <c r="J38" s="17"/>
       <c r="K38" s="17"/>
@@ -3388,25 +3539,25 @@
     <row r="39" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A39" s="18"/>
       <c r="B39" s="19" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F39" s="18" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="I39" s="18"/>
       <c r="J39" s="18"/>
@@ -3415,29 +3566,23 @@
       <c r="M39" s="19"/>
       <c r="N39" s="18"/>
     </row>
-    <row r="40" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A40" s="18"/>
+    <row r="40" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" s="18" t="s">
+        <v>188</v>
+      </c>
       <c r="B40" s="19" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="E40" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="F40" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="G40" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H40" s="18" t="s">
-        <v>189</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
       <c r="I40" s="18"/>
       <c r="J40" s="18"/>
       <c r="K40" s="18"/>
@@ -3601,7 +3746,7 @@
         <v>215</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D46" s="18" t="s">
         <v>216</v>
@@ -3613,7 +3758,7 @@
         <v>218</v>
       </c>
       <c r="G46" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H46" s="18" t="s">
         <v>219</v>
@@ -3625,23 +3770,29 @@
       <c r="M46" s="18"/>
       <c r="N46" s="18"/>
     </row>
-    <row r="47" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A47" s="17" t="s">
+    <row r="47" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A47" s="17"/>
+      <c r="B47" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="C47" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D47" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="C47" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D47" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
+      <c r="E47" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="F47" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="G47" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" s="17" t="s">
+        <v>224</v>
+      </c>
       <c r="I47" s="17"/>
       <c r="J47" s="17"/>
       <c r="K47" s="17"/>
@@ -3652,25 +3803,25 @@
     <row r="48" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A48" s="18"/>
       <c r="B48" s="19" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C48" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D48" s="18" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E48" s="18" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F48" s="18" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G48" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
@@ -3679,29 +3830,23 @@
       <c r="M48" s="18"/>
       <c r="N48" s="18"/>
     </row>
-    <row r="49" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A49" s="18"/>
+    <row r="49" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="18" t="s">
+        <v>230</v>
+      </c>
       <c r="B49" s="19" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="E49" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="F49" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="G49" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H49" s="18" t="s">
-        <v>231</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
       <c r="I49" s="18"/>
       <c r="J49" s="18"/>
       <c r="K49" s="18"/>
@@ -3715,7 +3860,7 @@
         <v>232</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="D50" s="18" t="s">
         <v>233</v>
@@ -3757,7 +3902,7 @@
         <v>240</v>
       </c>
       <c r="G51" s="18" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="H51" s="18" t="s">
         <v>241</v>
@@ -3775,7 +3920,7 @@
         <v>242</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>243</v>
@@ -3817,7 +3962,7 @@
         <v>250</v>
       </c>
       <c r="G53" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H53" s="18" t="s">
         <v>251</v>
@@ -3835,7 +3980,7 @@
         <v>252</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D54" s="18" t="s">
         <v>253</v>
@@ -3847,7 +3992,7 @@
         <v>255</v>
       </c>
       <c r="G54" s="18" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="H54" s="18" t="s">
         <v>256</v>
@@ -3865,7 +4010,7 @@
         <v>257</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D55" s="18" t="s">
         <v>258</v>
@@ -3907,7 +4052,7 @@
         <v>265</v>
       </c>
       <c r="G56" s="18" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="H56" s="18" t="s">
         <v>266</v>
@@ -3919,23 +4064,29 @@
       <c r="M56" s="18"/>
       <c r="N56" s="18"/>
     </row>
-    <row r="57" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A57" s="17" t="s">
+    <row r="57" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A57" s="17"/>
+      <c r="B57" s="17" t="s">
         <v>267</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="C57" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D57" s="17" t="s">
         <v>268</v>
       </c>
-      <c r="C57" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D57" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
+      <c r="E57" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="F57" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="G57" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="17" t="s">
+        <v>271</v>
+      </c>
       <c r="I57" s="17"/>
       <c r="J57" s="17"/>
       <c r="K57" s="17"/>
@@ -3946,25 +4097,25 @@
     <row r="58" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A58" s="18"/>
       <c r="B58" s="19" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C58" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D58" s="18" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E58" s="18" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F58" s="18" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G58" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="I58" s="18"/>
       <c r="J58" s="18"/>
@@ -3973,29 +4124,23 @@
       <c r="M58" s="18"/>
       <c r="N58" s="18"/>
     </row>
-    <row r="59" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A59" s="18"/>
+    <row r="59" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" s="18" t="s">
+        <v>277</v>
+      </c>
       <c r="B59" s="19" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C59" s="18" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D59" s="18" t="s">
-        <v>275</v>
-      </c>
-      <c r="E59" s="18" t="s">
-        <v>276</v>
-      </c>
-      <c r="F59" s="18" t="s">
-        <v>277</v>
-      </c>
-      <c r="G59" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H59" s="18" t="s">
-        <v>278</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
       <c r="I59" s="18"/>
       <c r="J59" s="18"/>
       <c r="K59" s="18"/>
@@ -4009,7 +4154,7 @@
         <v>279</v>
       </c>
       <c r="C60" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D60" s="18" t="s">
         <v>280</v>
@@ -4039,7 +4184,7 @@
         <v>284</v>
       </c>
       <c r="C61" s="18" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="D61" s="18" t="s">
         <v>285</v>
@@ -4069,7 +4214,7 @@
         <v>289</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D62" s="18" t="s">
         <v>290</v>
@@ -4099,7 +4244,7 @@
         <v>294</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D63" s="19" t="s">
         <v>295</v>
@@ -4129,7 +4274,7 @@
         <v>299</v>
       </c>
       <c r="C64" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D64" s="18" t="s">
         <v>300</v>
@@ -4159,7 +4304,7 @@
         <v>304</v>
       </c>
       <c r="C65" s="18" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="D65" s="18" t="s">
         <v>305</v>
@@ -4189,7 +4334,7 @@
         <v>309</v>
       </c>
       <c r="C66" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D66" s="18" t="s">
         <v>310</v>
@@ -4249,7 +4394,7 @@
         <v>319</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D68" s="19" t="s">
         <v>320</v>
@@ -4279,7 +4424,7 @@
         <v>324</v>
       </c>
       <c r="C69" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D69" s="18" t="s">
         <v>325</v>
@@ -4309,7 +4454,7 @@
         <v>329</v>
       </c>
       <c r="C70" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D70" s="18" t="s">
         <v>330</v>
@@ -4363,23 +4508,29 @@
       <c r="M71" s="19"/>
       <c r="N71" s="19"/>
     </row>
-    <row r="72" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A72" s="17" t="s">
+    <row r="72" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A72" s="17"/>
+      <c r="B72" s="17" t="s">
         <v>339</v>
       </c>
-      <c r="B72" s="17" t="s">
+      <c r="C72" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D72" s="17" t="s">
         <v>340</v>
       </c>
-      <c r="C72" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D72" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E72" s="17"/>
-      <c r="F72" s="17"/>
-      <c r="G72" s="17"/>
-      <c r="H72" s="17"/>
+      <c r="E72" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="F72" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="G72" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H72" s="17" t="s">
+        <v>343</v>
+      </c>
       <c r="I72" s="17"/>
       <c r="J72" s="17"/>
       <c r="K72" s="17"/>
@@ -4390,25 +4541,25 @@
     <row r="73" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A73" s="18"/>
       <c r="B73" s="19" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E73" s="18" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="F73" s="18" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="G73" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="I73" s="18"/>
       <c r="J73" s="18"/>
@@ -4420,25 +4571,25 @@
     <row r="74" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A74" s="19"/>
       <c r="B74" s="19" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C74" s="19" t="s">
         <v>39</v>
       </c>
       <c r="D74" s="19" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="E74" s="19" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="F74" s="19" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="G74" s="19" t="s">
         <v>36</v>
       </c>
       <c r="H74" s="19" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="I74" s="19"/>
       <c r="J74" s="19"/>
@@ -4450,25 +4601,25 @@
     <row r="75" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A75" s="18"/>
       <c r="B75" s="19" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C75" s="18" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E75" s="18" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F75" s="18" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G75" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="I75" s="18"/>
       <c r="J75" s="18"/>
@@ -4480,25 +4631,25 @@
     <row r="76" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A76" s="18"/>
       <c r="B76" s="19" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C76" s="18" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="D76" s="18" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E76" s="18" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F76" s="18" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="G76" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H76" s="18" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="I76" s="18"/>
       <c r="J76" s="18"/>
@@ -4510,25 +4661,25 @@
     <row r="77" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A77" s="19"/>
       <c r="B77" s="19" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="C77" s="19" t="s">
         <v>39</v>
       </c>
       <c r="D77" s="19" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E77" s="19" t="s">
+        <v>366</v>
+      </c>
+      <c r="F77" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="G77" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="H77" s="19" t="s">
         <v>363</v>
-      </c>
-      <c r="F77" s="19" t="s">
-        <v>364</v>
-      </c>
-      <c r="G77" s="19" t="s">
-        <v>365</v>
-      </c>
-      <c r="H77" s="19" t="s">
-        <v>366</v>
       </c>
       <c r="I77" s="19"/>
       <c r="J77" s="19"/>
@@ -4540,25 +4691,25 @@
     <row r="78" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A78" s="18"/>
       <c r="B78" s="19" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C78" s="18" t="s">
         <v>39</v>
       </c>
       <c r="D78" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E78" s="18" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F78" s="18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G78" s="18" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="H78" s="18" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="I78" s="18"/>
       <c r="J78" s="18"/>
@@ -4627,7 +4778,7 @@
         <v>379</v>
       </c>
       <c r="C81" s="19" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D81" s="19" t="s">
         <v>380</v>
@@ -4657,7 +4808,7 @@
         <v>384</v>
       </c>
       <c r="C82" s="18" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D82" s="18" t="s">
         <v>385</v>
@@ -4687,7 +4838,7 @@
         <v>389</v>
       </c>
       <c r="C83" s="18" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D83" s="18" t="s">
         <v>390</v>
@@ -4729,10 +4880,10 @@
         <v>397</v>
       </c>
       <c r="G84" s="19" t="s">
-        <v>114</v>
+        <v>398</v>
       </c>
       <c r="H84" s="19" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I84" s="19"/>
       <c r="J84" s="19"/>
@@ -4744,25 +4895,25 @@
     <row r="85" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C85" s="18" t="s">
         <v>39</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E85" s="18" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F85" s="18" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="G85" s="18" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="H85" s="18" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="I85" s="18"/>
       <c r="J85" s="18"/>
@@ -4771,29 +4922,23 @@
       <c r="M85" s="18"/>
       <c r="N85" s="18"/>
     </row>
-    <row r="86" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A86" s="19"/>
+    <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86" s="19" t="s">
+        <v>405</v>
+      </c>
       <c r="B86" s="19" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="C86" s="19" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D86" s="19" t="s">
-        <v>404</v>
-      </c>
-      <c r="E86" s="19" t="s">
-        <v>405</v>
-      </c>
-      <c r="F86" s="19" t="s">
-        <v>397</v>
-      </c>
-      <c r="G86" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="H86" s="19" t="s">
-        <v>406</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E86" s="19"/>
+      <c r="F86" s="19"/>
+      <c r="G86" s="19"/>
+      <c r="H86" s="19"/>
       <c r="I86" s="19"/>
       <c r="J86" s="19"/>
       <c r="K86" s="19"/>
@@ -4837,7 +4982,7 @@
         <v>412</v>
       </c>
       <c r="C88" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D88" s="18" t="s">
         <v>413</v>
@@ -4921,23 +5066,29 @@
       <c r="M90" s="18"/>
       <c r="N90" s="18"/>
     </row>
-    <row r="91" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A91" s="17" t="s">
+    <row r="91" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A91" s="17"/>
+      <c r="B91" s="17" t="s">
         <v>427</v>
       </c>
-      <c r="B91" s="17" t="s">
+      <c r="C91" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D91" s="17" t="s">
         <v>428</v>
       </c>
-      <c r="C91" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D91" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E91" s="17"/>
-      <c r="F91" s="17"/>
-      <c r="G91" s="17"/>
-      <c r="H91" s="17"/>
+      <c r="E91" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F91" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="G91" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="H91" s="17" t="s">
+        <v>431</v>
+      </c>
       <c r="I91" s="17"/>
       <c r="J91" s="17"/>
       <c r="K91" s="17"/>
@@ -4948,25 +5099,25 @@
     <row r="92" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="C92" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D92" s="18" t="s">
+        <v>433</v>
+      </c>
+      <c r="E92" s="18" t="s">
+        <v>434</v>
+      </c>
+      <c r="F92" s="18" t="s">
         <v>430</v>
       </c>
-      <c r="E92" s="18" t="s">
-        <v>431</v>
-      </c>
-      <c r="F92" s="18" t="s">
-        <v>432</v>
-      </c>
       <c r="G92" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H92" s="18" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="I92" s="18"/>
       <c r="J92" s="18"/>
@@ -4978,25 +5129,25 @@
     <row r="93" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="19"/>
       <c r="B93" s="19" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C93" s="19" t="s">
         <v>39</v>
       </c>
       <c r="D93" s="19" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E93" s="19" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="F93" s="19" t="s">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="G93" s="19" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H93" s="19" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="I93" s="19"/>
       <c r="J93" s="19"/>
@@ -5008,25 +5159,25 @@
     <row r="94" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="19"/>
       <c r="B94" s="19" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C94" s="19" t="s">
         <v>32</v>
       </c>
       <c r="D94" s="19" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="E94" s="19" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F94" s="19" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G94" s="19" t="s">
         <v>36</v>
       </c>
       <c r="H94" s="19" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I94" s="19"/>
       <c r="J94" s="19"/>
@@ -5038,25 +5189,25 @@
     <row r="95" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C95" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D95" s="18" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E95" s="18" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F95" s="18" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G95" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H95" s="18" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I95" s="18"/>
       <c r="J95" s="18"/>
@@ -5068,25 +5219,25 @@
     <row r="96" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C96" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D96" s="18" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E96" s="18" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F96" s="18" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G96" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H96" s="18" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="I96" s="18"/>
       <c r="J96" s="18"/>
@@ -5098,25 +5249,25 @@
     <row r="97" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C97" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D97" s="18" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E97" s="18" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F97" s="18" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G97" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H97" s="18" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="I97" s="18"/>
       <c r="J97" s="18"/>
@@ -5125,29 +5276,23 @@
       <c r="M97" s="18"/>
       <c r="N97" s="18"/>
     </row>
-    <row r="98" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A98" s="18"/>
+    <row r="98" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98" s="18" t="s">
+        <v>460</v>
+      </c>
       <c r="B98" s="19" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="C98" s="18" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="D98" s="18" t="s">
-        <v>460</v>
-      </c>
-      <c r="E98" s="18" t="s">
-        <v>461</v>
-      </c>
-      <c r="F98" s="18" t="s">
-        <v>462</v>
-      </c>
-      <c r="G98" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H98" s="18" t="s">
-        <v>463</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E98" s="18"/>
+      <c r="F98" s="18"/>
+      <c r="G98" s="18"/>
+      <c r="H98" s="18"/>
       <c r="I98" s="18"/>
       <c r="J98" s="18"/>
       <c r="K98" s="18"/>
@@ -5158,25 +5303,25 @@
     <row r="99" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A99" s="18"/>
       <c r="B99" s="19" t="s">
+        <v>462</v>
+      </c>
+      <c r="C99" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D99" s="18" t="s">
+        <v>463</v>
+      </c>
+      <c r="E99" s="18" t="s">
         <v>464</v>
       </c>
-      <c r="C99" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="D99" s="18" t="s">
+      <c r="F99" s="18" t="s">
         <v>465</v>
       </c>
-      <c r="E99" s="18" t="s">
+      <c r="G99" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H99" s="18" t="s">
         <v>466</v>
-      </c>
-      <c r="F99" s="18" t="s">
-        <v>467</v>
-      </c>
-      <c r="G99" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H99" s="18" t="s">
-        <v>468</v>
       </c>
       <c r="I99" s="18"/>
       <c r="J99" s="18"/>
@@ -5185,23 +5330,29 @@
       <c r="M99" s="18"/>
       <c r="N99" s="18"/>
     </row>
-    <row r="100" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A100" s="17" t="s">
+    <row r="100" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A100" s="17"/>
+      <c r="B100" s="17" t="s">
+        <v>467</v>
+      </c>
+      <c r="C100" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D100" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="E100" s="17" t="s">
         <v>469</v>
       </c>
-      <c r="B100" s="17" t="s">
+      <c r="F100" s="17" t="s">
         <v>470</v>
       </c>
-      <c r="C100" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D100" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E100" s="17"/>
-      <c r="F100" s="17"/>
-      <c r="G100" s="17"/>
-      <c r="H100" s="17"/>
+      <c r="G100" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H100" s="17" t="s">
+        <v>471</v>
+      </c>
       <c r="I100" s="17"/>
       <c r="J100" s="17"/>
       <c r="K100" s="17"/>
@@ -5212,25 +5363,25 @@
     <row r="101" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="19"/>
       <c r="B101" s="19" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C101" s="19" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D101" s="19" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E101" s="19" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F101" s="19" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G101" s="19" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="H101" s="19" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I101" s="19"/>
       <c r="J101" s="19"/>
@@ -5242,25 +5393,25 @@
     <row r="102" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C102" s="18" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="D102" s="18" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E102" s="18" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F102" s="18" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G102" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H102" s="18" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I102" s="18"/>
       <c r="J102" s="18"/>
@@ -5272,25 +5423,25 @@
     <row r="103" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C103" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E103" s="18" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F103" s="18" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="G103" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H103" s="18" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="I103" s="18"/>
       <c r="J103" s="18"/>
@@ -5302,25 +5453,25 @@
     <row r="104" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D104" s="18" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E104" s="18" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F104" s="18" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="G104" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H104" s="18" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="I104" s="18"/>
       <c r="J104" s="18"/>
@@ -5332,25 +5483,25 @@
     <row r="105" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="19"/>
       <c r="B105" s="19" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C105" s="19" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D105" s="19" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E105" s="19" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F105" s="19" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="G105" s="19" t="s">
         <v>36</v>
       </c>
       <c r="H105" s="19" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="I105" s="19"/>
       <c r="J105" s="19"/>
@@ -5362,25 +5513,25 @@
     <row r="106" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C106" s="18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D106" s="18" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E106" s="18" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F106" s="18" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G106" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H106" s="18" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="I106" s="18"/>
       <c r="J106" s="18"/>
@@ -5389,29 +5540,23 @@
       <c r="M106" s="18"/>
       <c r="N106" s="18"/>
     </row>
-    <row r="107" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A107" s="18"/>
+    <row r="107" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A107" s="18" t="s">
+        <v>502</v>
+      </c>
       <c r="B107" s="19" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="C107" s="18" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="D107" s="18" t="s">
-        <v>502</v>
-      </c>
-      <c r="E107" s="18" t="s">
-        <v>503</v>
-      </c>
-      <c r="F107" s="18" t="s">
-        <v>504</v>
-      </c>
-      <c r="G107" s="18" t="s">
-        <v>365</v>
-      </c>
-      <c r="H107" s="18" t="s">
-        <v>505</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E107" s="18"/>
+      <c r="F107" s="18"/>
+      <c r="G107" s="18"/>
+      <c r="H107" s="18"/>
       <c r="I107" s="18"/>
       <c r="J107" s="18"/>
       <c r="K107" s="18"/>
@@ -5419,23 +5564,29 @@
       <c r="M107" s="18"/>
       <c r="N107" s="18"/>
     </row>
-    <row r="108" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A108" s="17" t="s">
+    <row r="108" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A108" s="17"/>
+      <c r="B108" s="17" t="s">
+        <v>504</v>
+      </c>
+      <c r="C108" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D108" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="E108" s="17" t="s">
         <v>506</v>
       </c>
-      <c r="B108" s="17" t="s">
+      <c r="F108" s="17" t="s">
         <v>507</v>
       </c>
-      <c r="C108" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D108" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E108" s="17"/>
-      <c r="F108" s="17"/>
-      <c r="G108" s="17"/>
-      <c r="H108" s="17"/>
+      <c r="G108" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="H108" s="17" t="s">
+        <v>508</v>
+      </c>
       <c r="I108" s="17"/>
       <c r="J108" s="17"/>
       <c r="K108" s="17"/>
@@ -5446,25 +5597,25 @@
     <row r="109" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C109" s="18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D109" s="18" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E109" s="18" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F109" s="18" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="G109" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H109" s="18" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="I109" s="18"/>
       <c r="J109" s="18"/>
@@ -5476,25 +5627,25 @@
     <row r="110" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C110" s="18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D110" s="18" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E110" s="18" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F110" s="18" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G110" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="18" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="I110" s="18"/>
       <c r="J110" s="18"/>
@@ -5506,25 +5657,25 @@
     <row r="111" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C111" s="18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D111" s="18" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E111" s="18" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F111" s="18" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="G111" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="18" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="I111" s="18"/>
       <c r="J111" s="18"/>
@@ -5536,25 +5687,25 @@
     <row r="112" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C112" s="18" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="D112" s="18" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E112" s="18" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F112" s="18" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G112" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H112" s="18" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="I112" s="18"/>
       <c r="J112" s="18"/>
@@ -5566,25 +5717,25 @@
     <row r="113" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C113" s="18" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="D113" s="18" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E113" s="18" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F113" s="18" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G113" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="18" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="I113" s="18"/>
       <c r="J113" s="18"/>
@@ -5596,25 +5747,25 @@
     <row r="114" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="C114" s="18" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="D114" s="18" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E114" s="18" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F114" s="18" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="G114" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="18" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="I114" s="18"/>
       <c r="J114" s="18"/>
@@ -5626,25 +5777,25 @@
     <row r="115" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C115" s="18" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D115" s="18" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E115" s="18" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F115" s="18" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="G115" s="18" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="18" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="I115" s="18"/>
       <c r="J115" s="18"/>
@@ -5653,23 +5804,29 @@
       <c r="M115" s="18"/>
       <c r="N115" s="18"/>
     </row>
-    <row r="116" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A116" s="17" t="s">
-        <v>543</v>
-      </c>
+    <row r="116" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A116" s="17"/>
       <c r="B116" s="17" t="s">
         <v>544</v>
       </c>
       <c r="C116" s="17" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="D116" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E116" s="17"/>
-      <c r="F116" s="17"/>
-      <c r="G116" s="17"/>
-      <c r="H116" s="17"/>
+        <v>545</v>
+      </c>
+      <c r="E116" s="17" t="s">
+        <v>546</v>
+      </c>
+      <c r="F116" s="17" t="s">
+        <v>547</v>
+      </c>
+      <c r="G116" s="17" t="s">
+        <v>398</v>
+      </c>
+      <c r="H116" s="17" t="s">
+        <v>548</v>
+      </c>
       <c r="I116" s="17"/>
       <c r="J116" s="17"/>
       <c r="K116" s="17"/>
@@ -5677,29 +5834,23 @@
       <c r="M116" s="17"/>
       <c r="N116" s="17"/>
     </row>
-    <row r="117" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A117" s="20"/>
+    <row r="117" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A117" s="20" t="s">
+        <v>549</v>
+      </c>
       <c r="B117" s="20" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="C117" s="20" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>546</v>
-      </c>
-      <c r="E117" s="20" t="s">
-        <v>547</v>
-      </c>
-      <c r="F117" s="20" t="s">
-        <v>548</v>
-      </c>
-      <c r="G117" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H117" s="20" t="s">
-        <v>549</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E117" s="20"/>
+      <c r="F117" s="20"/>
+      <c r="G117" s="20"/>
+      <c r="H117" s="20"/>
       <c r="I117" s="20"/>
       <c r="J117" s="20"/>
       <c r="K117" s="20"/>
@@ -5710,25 +5861,25 @@
     <row r="118" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A118" s="20"/>
       <c r="B118" s="20" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C118" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D118" s="20" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="E118" s="20" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="F118" s="20" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="G118" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H118" s="20" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="I118" s="20"/>
       <c r="J118" s="20"/>
@@ -5740,25 +5891,25 @@
     <row r="119" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="20"/>
       <c r="B119" s="20" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C119" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D119" s="20" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E119" s="20" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F119" s="20" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="G119" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="20" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="I119" s="20"/>
       <c r="J119" s="20"/>
@@ -5770,25 +5921,25 @@
     <row r="120" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="20"/>
       <c r="B120" s="20" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C120" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D120" s="20" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E120" s="20" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F120" s="20" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="G120" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="20" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="I120" s="20"/>
       <c r="J120" s="20"/>
@@ -5800,25 +5951,25 @@
     <row r="121" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="20"/>
       <c r="B121" s="20" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C121" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D121" s="20" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="E121" s="20" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="F121" s="20" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="G121" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="20" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="I121" s="20"/>
       <c r="J121" s="20"/>
@@ -5830,25 +5981,25 @@
     <row r="122" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="20"/>
       <c r="B122" s="20" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C122" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D122" s="20" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E122" s="20" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="F122" s="20" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="G122" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="20" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="I122" s="20"/>
       <c r="J122" s="20"/>
@@ -5860,25 +6011,25 @@
     <row r="123" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="20"/>
       <c r="B123" s="20" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C123" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D123" s="20" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E123" s="20" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="F123" s="20" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G123" s="20" t="s">
-        <v>114</v>
+        <v>36</v>
       </c>
       <c r="H123" s="20" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="I123" s="20"/>
       <c r="J123" s="20"/>
@@ -5890,25 +6041,25 @@
     <row r="124" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="20"/>
       <c r="B124" s="20" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C124" s="20" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D124" s="20" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F124" s="20" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="G124" s="20" t="s">
-        <v>365</v>
+        <v>36</v>
       </c>
       <c r="H124" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I124" s="20"/>
       <c r="J124" s="20"/>
@@ -5917,29 +6068,23 @@
       <c r="M124" s="20"/>
       <c r="N124" s="20"/>
     </row>
-    <row r="125" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A125" s="20"/>
+    <row r="125" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A125" s="20" t="s">
+        <v>586</v>
+      </c>
       <c r="B125" s="20" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="C125" s="20" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="D125" s="20" t="s">
-        <v>586</v>
-      </c>
-      <c r="E125" s="20" t="s">
-        <v>587</v>
-      </c>
-      <c r="F125" s="20" t="s">
-        <v>588</v>
-      </c>
-      <c r="G125" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H125" s="20" t="s">
-        <v>589</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E125" s="20"/>
+      <c r="F125" s="20"/>
+      <c r="G125" s="20"/>
+      <c r="H125" s="20"/>
       <c r="I125" s="20"/>
       <c r="J125" s="20"/>
       <c r="K125" s="20"/>
@@ -5950,25 +6095,25 @@
     <row r="126" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="20"/>
       <c r="B126" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="C126" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D126" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="E126" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="C126" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="D126" s="20" t="s">
+      <c r="F126" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="E126" s="20" t="s">
+      <c r="G126" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H126" s="20" t="s">
         <v>592</v>
-      </c>
-      <c r="F126" s="20" t="s">
-        <v>593</v>
-      </c>
-      <c r="G126" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H126" s="20" t="s">
-        <v>594</v>
       </c>
       <c r="I126" s="20"/>
       <c r="J126" s="20"/>
@@ -5980,25 +6125,25 @@
     <row r="127" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A127" s="20"/>
       <c r="B127" s="20" t="s">
+        <v>593</v>
+      </c>
+      <c r="C127" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D127" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="E127" s="20" t="s">
         <v>595</v>
       </c>
-      <c r="C127" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="D127" s="20" t="s">
+      <c r="F127" s="20" t="s">
         <v>596</v>
       </c>
-      <c r="E127" s="20" t="s">
+      <c r="G127" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H127" s="20" t="s">
         <v>597</v>
-      </c>
-      <c r="F127" s="20" t="s">
-        <v>598</v>
-      </c>
-      <c r="G127" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H127" s="20" t="s">
-        <v>599</v>
       </c>
       <c r="I127" s="20"/>
       <c r="J127" s="20"/>
@@ -6010,25 +6155,25 @@
     <row r="128" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="20"/>
       <c r="B128" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="C128" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D128" s="20" t="s">
+        <v>599</v>
+      </c>
+      <c r="E128" s="20" t="s">
         <v>600</v>
       </c>
-      <c r="C128" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="D128" s="20" t="s">
+      <c r="F128" s="20" t="s">
         <v>601</v>
       </c>
-      <c r="E128" s="20" t="s">
+      <c r="G128" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H128" s="20" t="s">
         <v>602</v>
-      </c>
-      <c r="F128" s="20" t="s">
-        <v>603</v>
-      </c>
-      <c r="G128" s="20" t="s">
-        <v>365</v>
-      </c>
-      <c r="H128" s="20" t="s">
-        <v>604</v>
       </c>
       <c r="I128" s="20"/>
       <c r="J128" s="20"/>
@@ -6036,6 +6181,276 @@
       <c r="L128" s="20"/>
       <c r="M128" s="20"/>
       <c r="N128" s="20"/>
+    </row>
+    <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A129" s="21"/>
+      <c r="B129" s="22" t="s">
+        <v>603</v>
+      </c>
+      <c r="C129" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D129" s="21" t="s">
+        <v>604</v>
+      </c>
+      <c r="E129" s="21" t="s">
+        <v>605</v>
+      </c>
+      <c r="F129" s="21" t="s">
+        <v>606</v>
+      </c>
+      <c r="G129" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H129" s="21" t="s">
+        <v>607</v>
+      </c>
+      <c r="I129" s="21"/>
+      <c r="J129" s="21"/>
+      <c r="K129" s="21"/>
+      <c r="L129" s="21"/>
+      <c r="M129" s="21"/>
+      <c r="N129" s="21"/>
+    </row>
+    <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A130" s="21"/>
+      <c r="B130" s="22" t="s">
+        <v>608</v>
+      </c>
+      <c r="C130" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D130" s="21" t="s">
+        <v>609</v>
+      </c>
+      <c r="E130" s="21" t="s">
+        <v>610</v>
+      </c>
+      <c r="F130" s="21" t="s">
+        <v>611</v>
+      </c>
+      <c r="G130" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H130" s="21" t="s">
+        <v>612</v>
+      </c>
+      <c r="I130" s="21"/>
+      <c r="J130" s="21"/>
+      <c r="K130" s="21"/>
+      <c r="L130" s="21"/>
+      <c r="M130" s="21"/>
+      <c r="N130" s="21"/>
+    </row>
+    <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A131" s="21"/>
+      <c r="B131" s="22" t="s">
+        <v>613</v>
+      </c>
+      <c r="C131" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D131" s="21" t="s">
+        <v>614</v>
+      </c>
+      <c r="E131" s="21" t="s">
+        <v>615</v>
+      </c>
+      <c r="F131" s="21" t="s">
+        <v>616</v>
+      </c>
+      <c r="G131" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H131" s="21" t="s">
+        <v>617</v>
+      </c>
+      <c r="I131" s="21"/>
+      <c r="J131" s="21"/>
+      <c r="K131" s="21"/>
+      <c r="L131" s="21"/>
+      <c r="M131" s="21"/>
+      <c r="N131" s="21"/>
+    </row>
+    <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A132" s="21"/>
+      <c r="B132" s="22" t="s">
+        <v>618</v>
+      </c>
+      <c r="C132" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D132" s="21" t="s">
+        <v>619</v>
+      </c>
+      <c r="E132" s="21" t="s">
+        <v>620</v>
+      </c>
+      <c r="F132" s="21" t="s">
+        <v>621</v>
+      </c>
+      <c r="G132" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="H132" s="21" t="s">
+        <v>622</v>
+      </c>
+      <c r="I132" s="21"/>
+      <c r="J132" s="21"/>
+      <c r="K132" s="21"/>
+      <c r="L132" s="21"/>
+      <c r="M132" s="21"/>
+      <c r="N132" s="21"/>
+    </row>
+    <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A133" s="21"/>
+      <c r="B133" s="22" t="s">
+        <v>623</v>
+      </c>
+      <c r="C133" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D133" s="21" t="s">
+        <v>624</v>
+      </c>
+      <c r="E133" s="21" t="s">
+        <v>625</v>
+      </c>
+      <c r="F133" s="21" t="s">
+        <v>626</v>
+      </c>
+      <c r="G133" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="H133" s="21" t="s">
+        <v>627</v>
+      </c>
+      <c r="I133" s="21"/>
+      <c r="J133" s="21"/>
+      <c r="K133" s="21"/>
+      <c r="L133" s="21"/>
+      <c r="M133" s="21"/>
+      <c r="N133" s="21"/>
+    </row>
+    <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A134" s="21"/>
+      <c r="B134" s="22" t="s">
+        <v>628</v>
+      </c>
+      <c r="C134" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D134" s="21" t="s">
+        <v>629</v>
+      </c>
+      <c r="E134" s="21" t="s">
+        <v>630</v>
+      </c>
+      <c r="F134" s="21" t="s">
+        <v>631</v>
+      </c>
+      <c r="G134" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H134" s="21" t="s">
+        <v>632</v>
+      </c>
+      <c r="I134" s="21"/>
+      <c r="J134" s="21"/>
+      <c r="K134" s="21"/>
+      <c r="L134" s="21"/>
+      <c r="M134" s="21"/>
+      <c r="N134" s="21"/>
+    </row>
+    <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A135" s="21"/>
+      <c r="B135" s="22" t="s">
+        <v>633</v>
+      </c>
+      <c r="C135" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D135" s="21" t="s">
+        <v>634</v>
+      </c>
+      <c r="E135" s="21" t="s">
+        <v>635</v>
+      </c>
+      <c r="F135" s="21" t="s">
+        <v>636</v>
+      </c>
+      <c r="G135" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H135" s="21" t="s">
+        <v>637</v>
+      </c>
+      <c r="I135" s="21"/>
+      <c r="J135" s="21"/>
+      <c r="K135" s="21"/>
+      <c r="L135" s="21"/>
+      <c r="M135" s="21"/>
+      <c r="N135" s="21"/>
+    </row>
+    <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A136" s="21"/>
+      <c r="B136" s="22" t="s">
+        <v>638</v>
+      </c>
+      <c r="C136" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D136" s="21" t="s">
+        <v>639</v>
+      </c>
+      <c r="E136" s="21" t="s">
+        <v>640</v>
+      </c>
+      <c r="F136" s="21" t="s">
+        <v>641</v>
+      </c>
+      <c r="G136" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H136" s="21" t="s">
+        <v>642</v>
+      </c>
+      <c r="I136" s="21"/>
+      <c r="J136" s="21"/>
+      <c r="K136" s="21"/>
+      <c r="L136" s="21"/>
+      <c r="M136" s="21"/>
+      <c r="N136" s="21"/>
+    </row>
+    <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A137" s="21"/>
+      <c r="B137" s="22" t="s">
+        <v>643</v>
+      </c>
+      <c r="C137" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D137" s="21" t="s">
+        <v>644</v>
+      </c>
+      <c r="E137" s="21" t="s">
+        <v>645</v>
+      </c>
+      <c r="F137" s="21" t="s">
+        <v>646</v>
+      </c>
+      <c r="G137" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="H137" s="21" t="s">
+        <v>647</v>
+      </c>
+      <c r="I137" s="21"/>
+      <c r="J137" s="21"/>
+      <c r="K137" s="21"/>
+      <c r="L137" s="21"/>
+      <c r="M137" s="21"/>
+      <c r="N137" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
docs: correct stage 2 pass 003 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="678">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1756,6 +1756,21 @@
     <t>legacy/src/base/ims/cobol/LOADTSTA.cbl</t>
   </si>
   <si>
+    <t>Operator stages IMS reference data without loading it</t>
+  </si>
+  <si>
+    <t>Stage ACCTYPE, CUSTTYPE, TSTATTYP, and TTYPE inputs without claiming that the supplied population flow loads them.</t>
+  </si>
+  <si>
+    <t>The setup script creates datasets for four IMS reference-data files but submits loaders only for the five application datasets.</t>
+  </si>
+  <si>
+    <t>Reference inputs are staged, but no active loader job in the supplied population flow inserts them; this is a partial deployment surface.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/setup/populate-ims-tables.sh:27-52; legacy/src/base/ims/LoadData/ACCTYPE.data; legacy/src/base/ims/LoadData/CUSTTYPE.data; legacy/src/base/ims/LoadData/TSTATTYP.data; legacy/src/base/ims/LoadData/TTYPE.data</t>
+  </si>
+  <si>
     <t>Operator prepares DB2 structures and access</t>
   </si>
   <si>
@@ -1822,6 +1837,21 @@
     <t>legacy/.setup/zconfig/bank-of-z-definitions.yaml:788-1156</t>
   </si>
   <si>
+    <t>Deployment enables INQACCTY without an implementation</t>
+  </si>
+  <si>
+    <t>Record the enabled CICS program definition without inventing account-type inquiry behavior.</t>
+  </si>
+  <si>
+    <t>The resource model enables INQACCTY, but the repository contains no matching executable source or transaction binding.</t>
+  </si>
+  <si>
+    <t>INQACCTY is a partial deployment surface and cannot be executed from the supplied application artifacts.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/zconfig/bank-of-z-definitions.yaml:520-529; no INQACCTY implementation exists under legacy/src</t>
+  </si>
+  <si>
     <t>Operator deploys IMS transactions</t>
   </si>
   <si>
@@ -1900,16 +1930,16 @@
     <t>Operator deploys the frontend as a Liberty WAR on z/OS</t>
   </si>
   <si>
-    <t>Package the dependency-free frontend as a WAR and deploy it to a dedicated Liberty server on z/OS.</t>
-  </si>
-  <si>
-    <t>The Node server is not the only legacy frontend deployment channel.</t>
-  </si>
-  <si>
-    <t>FEBANKZ serves the WAR on port 9081 and proxies API traffic to z/OS Connect under its configured server identity.</t>
-  </si>
-  <si>
-    <t>legacy/.setup/build/groovy/VanillaFrontend.groovy:13-20,96-197; legacy/.setup/setup/setup-frontend-server.sh:7-13,85-90,117-146</t>
+    <t>Package the dependency-free frontend as a static WAR and deploy it to a dedicated Liberty server on z/OS.</t>
+  </si>
+  <si>
+    <t>The WAR excludes the Node proxy server; browser code calls z/OS Connect directly on port 9080.</t>
+  </si>
+  <si>
+    <t>FEBANKZ serves static frontend assets on port 9081, while z/OS Connect permits that browser origin through CORS.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/build/groovy/VanillaFrontend.groovy:124-135; legacy/.setup/setup/setup-frontend-server.sh:68-102; legacy/src/frontend/config.js:14-20; legacy/.setup/setup/setup-zosconnect-server.sh:139-157</t>
   </si>
   <si>
     <t>Operator provisions IMS runtime datasets and metadata</t>
@@ -1940,6 +1970,66 @@
   </si>
   <si>
     <t>legacy/.setup/jcl/cics/plt-create.j2:21-29; legacy/.setup/jcl/cics/tcpip-create.j2; legacy/.setup/setup/setup-cics-region.sh:164-172</t>
+  </si>
+  <si>
+    <t>Operator builds and packages Bank of Z with DBB</t>
+  </si>
+  <si>
+    <t>Run full, impact, or preview DBB builds and package native, API, frontend, configuration, and IMS Java outputs.</t>
+  </si>
+  <si>
+    <t>The pipeline validates DBB status and produces build lists, logs, and deployable packages for the selected scope.</t>
+  </si>
+  <si>
+    <t>DBB reports success/failure and publishes the generated build/package evidence; runtime execution remains environment-dependent.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/pipeline-common.sh:128-247; legacy/.setup/tasks/task-dbb-build.sh; legacy/dbb-app.yaml:276-370</t>
+  </si>
+  <si>
+    <t>Operator runs Z Code Scan</t>
+  </si>
+  <si>
+    <t>Generate a preview build list and submit the selected source set to Z Code Scan.</t>
+  </si>
+  <si>
+    <t>Static analysis is an explicit pipeline operation with published results rather than an implicit build side effect.</t>
+  </si>
+  <si>
+    <t>The scan task publishes its result/evidence or fails visibly when prerequisites or scanning fail.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/pipeline-common.sh:25-98; legacy/.setup/tasks/task-zcodescan-static-scan.sh</t>
+  </si>
+  <si>
+    <t>Operator deploys build outputs with Wazi Deploy</t>
+  </si>
+  <si>
+    <t>Generate and execute a deployment plan for native modules, maps, DBRM/JCL, IMS DBD/PSB, WAR/JAR, and configuration artifacts.</t>
+  </si>
+  <si>
+    <t>Deployment includes DB2 binding, CICS/IMS activation, application/config refresh, and evidence publication.</t>
+  </si>
+  <si>
+    <t>Wazi Deploy reports the plan and result; deployed runtime behavior remains unverified without the IBM environment.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/tasks/task-wazi-deploy.sh; legacy/.setup/deploy/deployment-method.yml:304-501</t>
+  </si>
+  <si>
+    <t>Operator provisions and refreshes native z/OS Connect</t>
+  </si>
+  <si>
+    <t>Create/start the native z/OS Connect server and install its CICS, IMS, API, credential, and CORS configuration.</t>
+  </si>
+  <si>
+    <t>The native server is provisioned separately from the local Designer container and can be refreshed by deployment automation.</t>
+  </si>
+  <si>
+    <t>The configured server and applications are started or refreshed, with setup/deployment failures visible to the operator.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/setup/setup-zosconnect-server.sh:31-167; legacy/.setup/deploy/deployment-method.yml:304-501</t>
   </si>
   <si>
     <t>IBM MQ is documented but not evidenced in runtime banking code</t>
@@ -2442,7 +2532,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N137"/>
+  <dimension ref="A1:N143"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6056,7 +6146,7 @@
         <v>584</v>
       </c>
       <c r="G124" s="20" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H124" s="20" t="s">
         <v>585</v>
@@ -6068,23 +6158,29 @@
       <c r="M124" s="20"/>
       <c r="N124" s="20"/>
     </row>
-    <row r="125" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A125" s="20" t="s">
+    <row r="125" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A125" s="20"/>
+      <c r="B125" s="20" t="s">
         <v>586</v>
       </c>
-      <c r="B125" s="20" t="s">
+      <c r="C125" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D125" s="20" t="s">
         <v>587</v>
       </c>
-      <c r="C125" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D125" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E125" s="20"/>
-      <c r="F125" s="20"/>
-      <c r="G125" s="20"/>
-      <c r="H125" s="20"/>
+      <c r="E125" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="F125" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="G125" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H125" s="20" t="s">
+        <v>590</v>
+      </c>
       <c r="I125" s="20"/>
       <c r="J125" s="20"/>
       <c r="K125" s="20"/>
@@ -6092,29 +6188,23 @@
       <c r="M125" s="20"/>
       <c r="N125" s="20"/>
     </row>
-    <row r="126" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A126" s="20"/>
+    <row r="126" ht="60" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A126" s="20" t="s">
+        <v>591</v>
+      </c>
       <c r="B126" s="20" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="C126" s="20" t="s">
-        <v>88</v>
+        <v>29</v>
       </c>
       <c r="D126" s="20" t="s">
-        <v>589</v>
-      </c>
-      <c r="E126" s="20" t="s">
-        <v>590</v>
-      </c>
-      <c r="F126" s="20" t="s">
-        <v>591</v>
-      </c>
-      <c r="G126" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H126" s="20" t="s">
-        <v>592</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E126" s="20"/>
+      <c r="F126" s="20"/>
+      <c r="G126" s="20"/>
+      <c r="H126" s="20"/>
       <c r="I126" s="20"/>
       <c r="J126" s="20"/>
       <c r="K126" s="20"/>
@@ -6230,7 +6320,7 @@
         <v>611</v>
       </c>
       <c r="G130" s="21" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H130" s="21" t="s">
         <v>612</v>
@@ -6290,7 +6380,7 @@
         <v>621</v>
       </c>
       <c r="G132" s="21" t="s">
-        <v>124</v>
+        <v>36</v>
       </c>
       <c r="H132" s="21" t="s">
         <v>622</v>
@@ -6308,7 +6398,7 @@
         <v>623</v>
       </c>
       <c r="C133" s="21" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D133" s="21" t="s">
         <v>624</v>
@@ -6320,7 +6410,7 @@
         <v>626</v>
       </c>
       <c r="G133" s="21" t="s">
-        <v>398</v>
+        <v>36</v>
       </c>
       <c r="H133" s="21" t="s">
         <v>627</v>
@@ -6350,7 +6440,7 @@
         <v>631</v>
       </c>
       <c r="G134" s="21" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H134" s="21" t="s">
         <v>632</v>
@@ -6368,7 +6458,7 @@
         <v>633</v>
       </c>
       <c r="C135" s="21" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="D135" s="21" t="s">
         <v>634</v>
@@ -6380,7 +6470,7 @@
         <v>636</v>
       </c>
       <c r="G135" s="21" t="s">
-        <v>36</v>
+        <v>398</v>
       </c>
       <c r="H135" s="21" t="s">
         <v>637</v>
@@ -6428,7 +6518,7 @@
         <v>643</v>
       </c>
       <c r="C137" s="21" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D137" s="21" t="s">
         <v>644</v>
@@ -6440,7 +6530,7 @@
         <v>646</v>
       </c>
       <c r="G137" s="21" t="s">
-        <v>398</v>
+        <v>36</v>
       </c>
       <c r="H137" s="21" t="s">
         <v>647</v>
@@ -6451,6 +6541,186 @@
       <c r="L137" s="21"/>
       <c r="M137" s="21"/>
       <c r="N137" s="21"/>
+    </row>
+    <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A138" s="21"/>
+      <c r="B138" s="22" t="s">
+        <v>648</v>
+      </c>
+      <c r="C138" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D138" s="21" t="s">
+        <v>649</v>
+      </c>
+      <c r="E138" s="21" t="s">
+        <v>650</v>
+      </c>
+      <c r="F138" s="21" t="s">
+        <v>651</v>
+      </c>
+      <c r="G138" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H138" s="21" t="s">
+        <v>652</v>
+      </c>
+      <c r="I138" s="21"/>
+      <c r="J138" s="21"/>
+      <c r="K138" s="21"/>
+      <c r="L138" s="21"/>
+      <c r="M138" s="21"/>
+      <c r="N138" s="21"/>
+    </row>
+    <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A139" s="21"/>
+      <c r="B139" s="22" t="s">
+        <v>653</v>
+      </c>
+      <c r="C139" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D139" s="21" t="s">
+        <v>654</v>
+      </c>
+      <c r="E139" s="21" t="s">
+        <v>655</v>
+      </c>
+      <c r="F139" s="21" t="s">
+        <v>656</v>
+      </c>
+      <c r="G139" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H139" s="21" t="s">
+        <v>657</v>
+      </c>
+      <c r="I139" s="21"/>
+      <c r="J139" s="21"/>
+      <c r="K139" s="21"/>
+      <c r="L139" s="21"/>
+      <c r="M139" s="21"/>
+      <c r="N139" s="21"/>
+    </row>
+    <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A140" s="21"/>
+      <c r="B140" s="22" t="s">
+        <v>658</v>
+      </c>
+      <c r="C140" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D140" s="21" t="s">
+        <v>659</v>
+      </c>
+      <c r="E140" s="21" t="s">
+        <v>660</v>
+      </c>
+      <c r="F140" s="21" t="s">
+        <v>661</v>
+      </c>
+      <c r="G140" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H140" s="21" t="s">
+        <v>662</v>
+      </c>
+      <c r="I140" s="21"/>
+      <c r="J140" s="21"/>
+      <c r="K140" s="21"/>
+      <c r="L140" s="21"/>
+      <c r="M140" s="21"/>
+      <c r="N140" s="21"/>
+    </row>
+    <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A141" s="21"/>
+      <c r="B141" s="22" t="s">
+        <v>663</v>
+      </c>
+      <c r="C141" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D141" s="21" t="s">
+        <v>664</v>
+      </c>
+      <c r="E141" s="21" t="s">
+        <v>665</v>
+      </c>
+      <c r="F141" s="21" t="s">
+        <v>666</v>
+      </c>
+      <c r="G141" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H141" s="21" t="s">
+        <v>667</v>
+      </c>
+      <c r="I141" s="21"/>
+      <c r="J141" s="21"/>
+      <c r="K141" s="21"/>
+      <c r="L141" s="21"/>
+      <c r="M141" s="21"/>
+      <c r="N141" s="21"/>
+    </row>
+    <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A142" s="21"/>
+      <c r="B142" s="22" t="s">
+        <v>668</v>
+      </c>
+      <c r="C142" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D142" s="21" t="s">
+        <v>669</v>
+      </c>
+      <c r="E142" s="21" t="s">
+        <v>670</v>
+      </c>
+      <c r="F142" s="21" t="s">
+        <v>671</v>
+      </c>
+      <c r="G142" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H142" s="21" t="s">
+        <v>672</v>
+      </c>
+      <c r="I142" s="21"/>
+      <c r="J142" s="21"/>
+      <c r="K142" s="21"/>
+      <c r="L142" s="21"/>
+      <c r="M142" s="21"/>
+      <c r="N142" s="21"/>
+    </row>
+    <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A143" s="21"/>
+      <c r="B143" s="22" t="s">
+        <v>673</v>
+      </c>
+      <c r="C143" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D143" s="21" t="s">
+        <v>674</v>
+      </c>
+      <c r="E143" s="21" t="s">
+        <v>675</v>
+      </c>
+      <c r="F143" s="21" t="s">
+        <v>676</v>
+      </c>
+      <c r="G143" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="H143" s="21" t="s">
+        <v>677</v>
+      </c>
+      <c r="I143" s="21"/>
+      <c r="J143" s="21"/>
+      <c r="K143" s="21"/>
+      <c r="L143" s="21"/>
+      <c r="M143" s="21"/>
+      <c r="N143" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
docs: correct stage 2 pass 004 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="718">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1243,7 +1243,7 @@
     <t>REST clients can access the core CICS customer programs.</t>
   </si>
   <si>
-    <t>GET/PUT customer calls map to INQCUST and UPDCUST assets.</t>
+    <t>GET and PUT success mappings reach INQCUST/UPDCUST, but the PUT 401/403 response selections reference missing generated files.</t>
   </si>
   <si>
     <t>legacy/src/api/src/main/api/openapi.yaml:275-345; operations ...customers...; zosAssets/INQCUST and UPDCUST</t>
@@ -1258,7 +1258,7 @@
     <t>REST clients can inspect the CICS account portfolio.</t>
   </si>
   <si>
-    <t>Mapped operations return account and balance schemas.</t>
+    <t>Success mappings return account/balance schemas, but three selected 400 response files are absent.</t>
   </si>
   <si>
     <t>legacy/src/api/src/main/api/openapi.yaml:346-478; zosAssets/INQACCCU and INQACC</t>
@@ -1357,12 +1357,27 @@
     <t>External consumers need stable error classes.</t>
   </si>
   <si>
-    <t>The contract exposes 400, 401, 403, 404, and 500 responses as applicable.</t>
+    <t>The contract declares standard failures, but five bound and three unbound response selections reference missing generated YAML artifacts.</t>
   </si>
   <si>
     <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema</t>
   </si>
   <si>
+    <t>Generated API mappings select missing response files</t>
+  </si>
+  <si>
+    <t>Record generated response selections whose referenced sibling YAML artifacts are absent.</t>
+  </si>
+  <si>
+    <t>Five missing files affect bound CICS account/customer operations; three more occur in already-unbound account/transaction routes.</t>
+  </si>
+  <si>
+    <t>Those selected error/fallback responses are not deployable from the supplied artifacts and must not be treated as complete API behavior.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Fbalances/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D/put/response_mapping.yaml:8-10</t>
+  </si>
+  <si>
     <t>External client creates a CICS customer</t>
   </si>
   <si>
@@ -1912,6 +1927,21 @@
     <t>legacy/src/base/ims/java/src/main/java/nazare/jmp/controller/IMSBankHistory.java trust manager/hostname verifier</t>
   </si>
   <si>
+    <t>History diagnostic client queries fixed account 1501</t>
+  </si>
+  <si>
+    <t>Run the standalone DB2 history diagnostic without confusing it with parameterized IBGHIST behavior.</t>
+  </si>
+  <si>
+    <t>The Java main reads DB2 connection properties, queries every IMSBANK.HISTORY column for hard-coded account 1501, prints rows, and commits the read transaction.</t>
+  </si>
+  <si>
+    <t>A fixed-account diagnostic dump is printed or a connection/query error is surfaced; this is a partial operator utility, not a customer history API.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/java/src/main/java/nazare/jmp/controller/IMSBankHistory.java:61-109</t>
+  </si>
+  <si>
     <t>Team attempts a standalone local run</t>
   </si>
   <si>
@@ -1972,6 +2002,36 @@
     <t>legacy/.setup/jcl/cics/plt-create.j2:21-29; legacy/.setup/jcl/cics/tcpip-create.j2; legacy/.setup/setup/setup-cics-region.sh:164-172</t>
   </si>
   <si>
+    <t>Operator orchestrates remote Bank of Z setup</t>
+  </si>
+  <si>
+    <t>Initialize or preserve a remote USS workspace, validate it, configure the environment, and run ordered full-system installation.</t>
+  </si>
+  <si>
+    <t>Local and remote wrappers coordinate middleware/application setup, build/deploy, and DB2/IMS population.</t>
+  </si>
+  <si>
+    <t>The operator sees preserve/recreate choices and ordered setup results; actual execution remains unverified without the IBM environment.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/setup-local.sh:22-50; legacy/.setup/setup-remote.sh:24-68; legacy/.setup/setup-common.sh:466-590</t>
+  </si>
+  <si>
+    <t>Operator validates the IBM installation prerequisites</t>
+  </si>
+  <si>
+    <t>Check minimum DBB, ZOAU, zconfig, and Wazi Deploy installations before setup.</t>
+  </si>
+  <si>
+    <t>The installation validator gives one explicit readiness result instead of allowing a later opaque failure.</t>
+  </si>
+  <si>
+    <t>A pass/fail summary is printed and a failed prerequisite produces a failing exit status.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/setup/validate-install.sh:73-253</t>
+  </si>
+  <si>
     <t>Operator builds and packages Bank of Z with DBB</t>
   </si>
   <si>
@@ -2030,6 +2090,66 @@
   </si>
   <si>
     <t>legacy/.setup/setup/setup-zosconnect-server.sh:31-167; legacy/.setup/deploy/deployment-method.yml:304-501</t>
+  </si>
+  <si>
+    <t>Developer runs pre-commit secret detection</t>
+  </si>
+  <si>
+    <t>Scan committed content with IBM detect-secrets and fail on unaudited findings.</t>
+  </si>
+  <si>
+    <t>Secret scanning is an executable repository gate rather than narrative guidance.</t>
+  </si>
+  <si>
+    <t>The hook passes with the audited baseline or fails visibly for unapproved findings.</t>
+  </si>
+  <si>
+    <t>legacy/.pre-commit-config.yaml:14-21</t>
+  </si>
+  <si>
+    <t>Developer downloads and installs configured VSIX tools</t>
+  </si>
+  <si>
+    <t>Download the configured extension set and install discovered VSIX packages into VS Code or Bob IDE.</t>
+  </si>
+  <si>
+    <t>The repository supplies observable setup wrappers for developer tooling.</t>
+  </si>
+  <si>
+    <t>Each package reports success/failure and the command exits unsuccessfully when prerequisites or installation fail.</t>
+  </si>
+  <si>
+    <t>legacy/scripts/download-vsix.js:176-238; legacy/scripts/install-vscode-vsix.js:133-227; legacy/scripts/install-bobide-vsix.js:132-225</t>
+  </si>
+  <si>
+    <t>Developer connects zOpenDebug to a parked session</t>
+  </si>
+  <si>
+    <t>Expose the configured zOpenDebug launch connection for Bank of Z native debugging.</t>
+  </si>
+  <si>
+    <t>A developer can attach the IDE to the declared parked debug session when its external service is available.</t>
+  </si>
+  <si>
+    <t>The IDE attempts the configured connection; runtime availability remains environment-dependent.</t>
+  </si>
+  <si>
+    <t>legacy/.vscode/launch.json:6-15</t>
+  </si>
+  <si>
+    <t>Documentation operator regenerates the site TOC</t>
+  </si>
+  <si>
+    <t>Regenerate documentation navigation from Markdown metadata.</t>
+  </si>
+  <si>
+    <t>The deployable documentation site has an executable navigation-generation workflow.</t>
+  </si>
+  <si>
+    <t>The script rewrites the TOC from discovered metadata or fails visibly on invalid input.</t>
+  </si>
+  <si>
+    <t>legacy/docs/scripts/generate_toc_from_md.py:42-102</t>
   </si>
   <si>
     <t>IBM MQ is documented but not evidenced in runtime banking code</t>
@@ -2532,7 +2652,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N143"/>
+  <dimension ref="A1:N151"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5054,7 +5174,7 @@
         <v>410</v>
       </c>
       <c r="G87" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H87" s="18" t="s">
         <v>411</v>
@@ -5084,7 +5204,7 @@
         <v>415</v>
       </c>
       <c r="G88" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H88" s="18" t="s">
         <v>416</v>
@@ -5294,7 +5414,7 @@
         <v>448</v>
       </c>
       <c r="G95" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H95" s="18" t="s">
         <v>449</v>
@@ -5312,7 +5432,7 @@
         <v>450</v>
       </c>
       <c r="C96" s="18" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D96" s="18" t="s">
         <v>451</v>
@@ -5324,7 +5444,7 @@
         <v>453</v>
       </c>
       <c r="G96" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H96" s="18" t="s">
         <v>454</v>
@@ -5366,23 +5486,29 @@
       <c r="M97" s="18"/>
       <c r="N97" s="18"/>
     </row>
-    <row r="98" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A98" s="18" t="s">
+    <row r="98" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A98" s="18"/>
+      <c r="B98" s="19" t="s">
         <v>460</v>
       </c>
-      <c r="B98" s="19" t="s">
+      <c r="C98" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D98" s="18" t="s">
         <v>461</v>
       </c>
-      <c r="C98" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D98" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="E98" s="18"/>
-      <c r="F98" s="18"/>
-      <c r="G98" s="18"/>
-      <c r="H98" s="18"/>
+      <c r="E98" s="18" t="s">
+        <v>462</v>
+      </c>
+      <c r="F98" s="18" t="s">
+        <v>463</v>
+      </c>
+      <c r="G98" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H98" s="18" t="s">
+        <v>464</v>
+      </c>
       <c r="I98" s="18"/>
       <c r="J98" s="18"/>
       <c r="K98" s="18"/>
@@ -5390,29 +5516,23 @@
       <c r="M98" s="18"/>
       <c r="N98" s="18"/>
     </row>
-    <row r="99" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A99" s="18"/>
+    <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" s="18" t="s">
+        <v>465</v>
+      </c>
       <c r="B99" s="19" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="C99" s="18" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D99" s="18" t="s">
-        <v>463</v>
-      </c>
-      <c r="E99" s="18" t="s">
-        <v>464</v>
-      </c>
-      <c r="F99" s="18" t="s">
-        <v>465</v>
-      </c>
-      <c r="G99" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="H99" s="18" t="s">
-        <v>466</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E99" s="18"/>
+      <c r="F99" s="18"/>
+      <c r="G99" s="18"/>
+      <c r="H99" s="18"/>
       <c r="I99" s="18"/>
       <c r="J99" s="18"/>
       <c r="K99" s="18"/>
@@ -5426,7 +5546,7 @@
         <v>467</v>
       </c>
       <c r="C100" s="17" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D100" s="17" t="s">
         <v>468</v>
@@ -5456,7 +5576,7 @@
         <v>472</v>
       </c>
       <c r="C101" s="19" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D101" s="19" t="s">
         <v>473</v>
@@ -5516,7 +5636,7 @@
         <v>482</v>
       </c>
       <c r="C103" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D103" s="18" t="s">
         <v>483</v>
@@ -5546,7 +5666,7 @@
         <v>487</v>
       </c>
       <c r="C104" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D104" s="18" t="s">
         <v>488</v>
@@ -5576,7 +5696,7 @@
         <v>492</v>
       </c>
       <c r="C105" s="19" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="D105" s="19" t="s">
         <v>493</v>
@@ -5630,23 +5750,29 @@
       <c r="M106" s="18"/>
       <c r="N106" s="18"/>
     </row>
-    <row r="107" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A107" s="18" t="s">
+    <row r="107" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A107" s="18"/>
+      <c r="B107" s="19" t="s">
         <v>502</v>
       </c>
-      <c r="B107" s="19" t="s">
+      <c r="C107" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="D107" s="18" t="s">
         <v>503</v>
       </c>
-      <c r="C107" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D107" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="E107" s="18"/>
-      <c r="F107" s="18"/>
-      <c r="G107" s="18"/>
-      <c r="H107" s="18"/>
+      <c r="E107" s="18" t="s">
+        <v>504</v>
+      </c>
+      <c r="F107" s="18" t="s">
+        <v>505</v>
+      </c>
+      <c r="G107" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H107" s="18" t="s">
+        <v>506</v>
+      </c>
       <c r="I107" s="18"/>
       <c r="J107" s="18"/>
       <c r="K107" s="18"/>
@@ -5654,29 +5780,23 @@
       <c r="M107" s="18"/>
       <c r="N107" s="18"/>
     </row>
-    <row r="108" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A108" s="17"/>
+    <row r="108" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A108" s="17" t="s">
+        <v>507</v>
+      </c>
       <c r="B108" s="17" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C108" s="17" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D108" s="17" t="s">
-        <v>505</v>
-      </c>
-      <c r="E108" s="17" t="s">
-        <v>506</v>
-      </c>
-      <c r="F108" s="17" t="s">
-        <v>507</v>
-      </c>
-      <c r="G108" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="H108" s="17" t="s">
-        <v>508</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E108" s="17"/>
+      <c r="F108" s="17"/>
+      <c r="G108" s="17"/>
+      <c r="H108" s="17"/>
       <c r="I108" s="17"/>
       <c r="J108" s="17"/>
       <c r="K108" s="17"/>
@@ -5690,7 +5810,7 @@
         <v>509</v>
       </c>
       <c r="C109" s="18" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="D109" s="18" t="s">
         <v>510</v>
@@ -5702,7 +5822,7 @@
         <v>512</v>
       </c>
       <c r="G109" s="18" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H109" s="18" t="s">
         <v>513</v>
@@ -5780,7 +5900,7 @@
         <v>524</v>
       </c>
       <c r="C112" s="18" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D112" s="18" t="s">
         <v>525</v>
@@ -5840,7 +5960,7 @@
         <v>534</v>
       </c>
       <c r="C114" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D114" s="18" t="s">
         <v>535</v>
@@ -5870,7 +5990,7 @@
         <v>539</v>
       </c>
       <c r="C115" s="18" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="D115" s="18" t="s">
         <v>540</v>
@@ -5912,7 +6032,7 @@
         <v>547</v>
       </c>
       <c r="G116" s="17" t="s">
-        <v>398</v>
+        <v>36</v>
       </c>
       <c r="H116" s="17" t="s">
         <v>548</v>
@@ -5924,23 +6044,29 @@
       <c r="M116" s="17"/>
       <c r="N116" s="17"/>
     </row>
-    <row r="117" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A117" s="20" t="s">
+    <row r="117" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A117" s="20"/>
+      <c r="B117" s="20" t="s">
         <v>549</v>
       </c>
-      <c r="B117" s="20" t="s">
+      <c r="C117" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D117" s="20" t="s">
         <v>550</v>
       </c>
-      <c r="C117" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D117" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E117" s="20"/>
-      <c r="F117" s="20"/>
-      <c r="G117" s="20"/>
-      <c r="H117" s="20"/>
+      <c r="E117" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="F117" s="20" t="s">
+        <v>552</v>
+      </c>
+      <c r="G117" s="20" t="s">
+        <v>398</v>
+      </c>
+      <c r="H117" s="20" t="s">
+        <v>553</v>
+      </c>
       <c r="I117" s="20"/>
       <c r="J117" s="20"/>
       <c r="K117" s="20"/>
@@ -5948,29 +6074,23 @@
       <c r="M117" s="20"/>
       <c r="N117" s="20"/>
     </row>
-    <row r="118" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A118" s="20"/>
+    <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A118" s="20" t="s">
+        <v>554</v>
+      </c>
       <c r="B118" s="20" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="C118" s="20" t="s">
-        <v>88</v>
+        <v>29</v>
       </c>
       <c r="D118" s="20" t="s">
-        <v>552</v>
-      </c>
-      <c r="E118" s="20" t="s">
-        <v>553</v>
-      </c>
-      <c r="F118" s="20" t="s">
-        <v>554</v>
-      </c>
-      <c r="G118" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H118" s="20" t="s">
-        <v>555</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E118" s="20"/>
+      <c r="F118" s="20"/>
+      <c r="G118" s="20"/>
+      <c r="H118" s="20"/>
       <c r="I118" s="20"/>
       <c r="J118" s="20"/>
       <c r="K118" s="20"/>
@@ -6146,7 +6266,7 @@
         <v>584</v>
       </c>
       <c r="G124" s="20" t="s">
-        <v>124</v>
+        <v>36</v>
       </c>
       <c r="H124" s="20" t="s">
         <v>585</v>
@@ -6176,7 +6296,7 @@
         <v>589</v>
       </c>
       <c r="G125" s="20" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H125" s="20" t="s">
         <v>590</v>
@@ -6188,23 +6308,29 @@
       <c r="M125" s="20"/>
       <c r="N125" s="20"/>
     </row>
-    <row r="126" ht="60" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A126" s="20" t="s">
+    <row r="126" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A126" s="20"/>
+      <c r="B126" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="B126" s="20" t="s">
+      <c r="C126" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D126" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="C126" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D126" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="E126" s="20"/>
-      <c r="F126" s="20"/>
-      <c r="G126" s="20"/>
-      <c r="H126" s="20"/>
+      <c r="E126" s="20" t="s">
+        <v>593</v>
+      </c>
+      <c r="F126" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="G126" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H126" s="20" t="s">
+        <v>595</v>
+      </c>
       <c r="I126" s="20"/>
       <c r="J126" s="20"/>
       <c r="K126" s="20"/>
@@ -6212,29 +6338,23 @@
       <c r="M126" s="20"/>
       <c r="N126" s="20"/>
     </row>
-    <row r="127" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A127" s="20"/>
+    <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A127" s="20" t="s">
+        <v>596</v>
+      </c>
       <c r="B127" s="20" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="C127" s="20" t="s">
-        <v>88</v>
+        <v>29</v>
       </c>
       <c r="D127" s="20" t="s">
-        <v>594</v>
-      </c>
-      <c r="E127" s="20" t="s">
-        <v>595</v>
-      </c>
-      <c r="F127" s="20" t="s">
-        <v>596</v>
-      </c>
-      <c r="G127" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H127" s="20" t="s">
-        <v>597</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E127" s="20"/>
+      <c r="F127" s="20"/>
+      <c r="G127" s="20"/>
+      <c r="H127" s="20"/>
       <c r="I127" s="20"/>
       <c r="J127" s="20"/>
       <c r="K127" s="20"/>
@@ -6320,7 +6440,7 @@
         <v>611</v>
       </c>
       <c r="G130" s="21" t="s">
-        <v>124</v>
+        <v>36</v>
       </c>
       <c r="H130" s="21" t="s">
         <v>612</v>
@@ -6350,7 +6470,7 @@
         <v>616</v>
       </c>
       <c r="G131" s="21" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H131" s="21" t="s">
         <v>617</v>
@@ -6440,7 +6560,7 @@
         <v>631</v>
       </c>
       <c r="G134" s="21" t="s">
-        <v>124</v>
+        <v>36</v>
       </c>
       <c r="H134" s="21" t="s">
         <v>632</v>
@@ -6458,7 +6578,7 @@
         <v>633</v>
       </c>
       <c r="C135" s="21" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D135" s="21" t="s">
         <v>634</v>
@@ -6470,7 +6590,7 @@
         <v>636</v>
       </c>
       <c r="G135" s="21" t="s">
-        <v>398</v>
+        <v>124</v>
       </c>
       <c r="H135" s="21" t="s">
         <v>637</v>
@@ -6500,7 +6620,7 @@
         <v>641</v>
       </c>
       <c r="G136" s="21" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H136" s="21" t="s">
         <v>642</v>
@@ -6518,7 +6638,7 @@
         <v>643</v>
       </c>
       <c r="C137" s="21" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="D137" s="21" t="s">
         <v>644</v>
@@ -6530,7 +6650,7 @@
         <v>646</v>
       </c>
       <c r="G137" s="21" t="s">
-        <v>36</v>
+        <v>398</v>
       </c>
       <c r="H137" s="21" t="s">
         <v>647</v>
@@ -6698,7 +6818,7 @@
         <v>673</v>
       </c>
       <c r="C143" s="21" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D143" s="21" t="s">
         <v>674</v>
@@ -6710,7 +6830,7 @@
         <v>676</v>
       </c>
       <c r="G143" s="21" t="s">
-        <v>398</v>
+        <v>36</v>
       </c>
       <c r="H143" s="21" t="s">
         <v>677</v>
@@ -6721,6 +6841,246 @@
       <c r="L143" s="21"/>
       <c r="M143" s="21"/>
       <c r="N143" s="21"/>
+    </row>
+    <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A144" s="21"/>
+      <c r="B144" s="22" t="s">
+        <v>678</v>
+      </c>
+      <c r="C144" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D144" s="21" t="s">
+        <v>679</v>
+      </c>
+      <c r="E144" s="21" t="s">
+        <v>680</v>
+      </c>
+      <c r="F144" s="21" t="s">
+        <v>681</v>
+      </c>
+      <c r="G144" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H144" s="21" t="s">
+        <v>682</v>
+      </c>
+      <c r="I144" s="21"/>
+      <c r="J144" s="21"/>
+      <c r="K144" s="21"/>
+      <c r="L144" s="21"/>
+      <c r="M144" s="21"/>
+      <c r="N144" s="21"/>
+    </row>
+    <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A145" s="21"/>
+      <c r="B145" s="22" t="s">
+        <v>683</v>
+      </c>
+      <c r="C145" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D145" s="21" t="s">
+        <v>684</v>
+      </c>
+      <c r="E145" s="21" t="s">
+        <v>685</v>
+      </c>
+      <c r="F145" s="21" t="s">
+        <v>686</v>
+      </c>
+      <c r="G145" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H145" s="21" t="s">
+        <v>687</v>
+      </c>
+      <c r="I145" s="21"/>
+      <c r="J145" s="21"/>
+      <c r="K145" s="21"/>
+      <c r="L145" s="21"/>
+      <c r="M145" s="21"/>
+      <c r="N145" s="21"/>
+    </row>
+    <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A146" s="21"/>
+      <c r="B146" s="22" t="s">
+        <v>688</v>
+      </c>
+      <c r="C146" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D146" s="21" t="s">
+        <v>689</v>
+      </c>
+      <c r="E146" s="21" t="s">
+        <v>690</v>
+      </c>
+      <c r="F146" s="21" t="s">
+        <v>691</v>
+      </c>
+      <c r="G146" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H146" s="21" t="s">
+        <v>692</v>
+      </c>
+      <c r="I146" s="21"/>
+      <c r="J146" s="21"/>
+      <c r="K146" s="21"/>
+      <c r="L146" s="21"/>
+      <c r="M146" s="21"/>
+      <c r="N146" s="21"/>
+    </row>
+    <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A147" s="21"/>
+      <c r="B147" s="22" t="s">
+        <v>693</v>
+      </c>
+      <c r="C147" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D147" s="21" t="s">
+        <v>694</v>
+      </c>
+      <c r="E147" s="21" t="s">
+        <v>695</v>
+      </c>
+      <c r="F147" s="21" t="s">
+        <v>696</v>
+      </c>
+      <c r="G147" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H147" s="21" t="s">
+        <v>697</v>
+      </c>
+      <c r="I147" s="21"/>
+      <c r="J147" s="21"/>
+      <c r="K147" s="21"/>
+      <c r="L147" s="21"/>
+      <c r="M147" s="21"/>
+      <c r="N147" s="21"/>
+    </row>
+    <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A148" s="21"/>
+      <c r="B148" s="22" t="s">
+        <v>698</v>
+      </c>
+      <c r="C148" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D148" s="21" t="s">
+        <v>699</v>
+      </c>
+      <c r="E148" s="21" t="s">
+        <v>700</v>
+      </c>
+      <c r="F148" s="21" t="s">
+        <v>701</v>
+      </c>
+      <c r="G148" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H148" s="21" t="s">
+        <v>702</v>
+      </c>
+      <c r="I148" s="21"/>
+      <c r="J148" s="21"/>
+      <c r="K148" s="21"/>
+      <c r="L148" s="21"/>
+      <c r="M148" s="21"/>
+      <c r="N148" s="21"/>
+    </row>
+    <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A149" s="21"/>
+      <c r="B149" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="C149" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D149" s="21" t="s">
+        <v>704</v>
+      </c>
+      <c r="E149" s="21" t="s">
+        <v>705</v>
+      </c>
+      <c r="F149" s="21" t="s">
+        <v>706</v>
+      </c>
+      <c r="G149" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H149" s="21" t="s">
+        <v>707</v>
+      </c>
+      <c r="I149" s="21"/>
+      <c r="J149" s="21"/>
+      <c r="K149" s="21"/>
+      <c r="L149" s="21"/>
+      <c r="M149" s="21"/>
+      <c r="N149" s="21"/>
+    </row>
+    <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A150" s="21"/>
+      <c r="B150" s="22" t="s">
+        <v>708</v>
+      </c>
+      <c r="C150" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D150" s="21" t="s">
+        <v>709</v>
+      </c>
+      <c r="E150" s="21" t="s">
+        <v>710</v>
+      </c>
+      <c r="F150" s="21" t="s">
+        <v>711</v>
+      </c>
+      <c r="G150" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H150" s="21" t="s">
+        <v>712</v>
+      </c>
+      <c r="I150" s="21"/>
+      <c r="J150" s="21"/>
+      <c r="K150" s="21"/>
+      <c r="L150" s="21"/>
+      <c r="M150" s="21"/>
+      <c r="N150" s="21"/>
+    </row>
+    <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A151" s="21"/>
+      <c r="B151" s="22" t="s">
+        <v>713</v>
+      </c>
+      <c r="C151" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D151" s="21" t="s">
+        <v>714</v>
+      </c>
+      <c r="E151" s="21" t="s">
+        <v>715</v>
+      </c>
+      <c r="F151" s="21" t="s">
+        <v>716</v>
+      </c>
+      <c r="G151" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="H151" s="21" t="s">
+        <v>717</v>
+      </c>
+      <c r="I151" s="21"/>
+      <c r="J151" s="21"/>
+      <c r="K151" s="21"/>
+      <c r="L151" s="21"/>
+      <c r="M151" s="21"/>
+      <c r="N151" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
docs: correct stage 2 pass 005 finding
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -2140,16 +2140,16 @@
     <t>Documentation operator regenerates the site TOC</t>
   </si>
   <si>
-    <t>Regenerate documentation navigation from Markdown metadata.</t>
-  </si>
-  <si>
-    <t>The deployable documentation site has an executable navigation-generation workflow.</t>
-  </si>
-  <si>
-    <t>The script rewrites the TOC from discovered metadata or fails visibly on invalid input.</t>
-  </si>
-  <si>
-    <t>legacy/docs/scripts/generate_toc_from_md.py:42-102</t>
+    <t>Record the supplied TOC generator as a non-runnable partial tool rather than claiming successful regeneration.</t>
+  </si>
+  <si>
+    <t>The Python file contains malformed syntax/indentation and defines generate_toc() without invoking it.</t>
+  </si>
+  <si>
+    <t>The supplied script does not successfully regenerate the TOC without repair; no successful operator result is code-proven.</t>
+  </si>
+  <si>
+    <t>legacy/docs/scripts/generate_toc_from_md.py:42-102; no executable generate_toc() invocation is present</t>
   </si>
   <si>
     <t>IBM MQ is documented but not evidenced in runtime banking code</t>
@@ -7040,7 +7040,7 @@
         <v>711</v>
       </c>
       <c r="G150" s="21" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="H150" s="21" t="s">
         <v>712</v>

</xml_diff>

<commit_message>
docs: correct stage 2 pass 006 finding
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="728">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -2150,6 +2150,36 @@
   </si>
   <si>
     <t>legacy/docs/scripts/generate_toc_from_md.py:42-102; no executable generate_toc() invocation is present</t>
+  </si>
+  <si>
+    <t>Zowe management connections bypass certificate verification</t>
+  </si>
+  <si>
+    <t>Treat the shared Zowe profile's disabled certificate verification as a legacy security deviation that must not become the target default.</t>
+  </si>
+  <si>
+    <t>Setup, pipeline, and debug tooling use an HTTPS profile with rejectUnauthorized set to false.</t>
+  </si>
+  <si>
+    <t>Management connections accept untrusted TLS certificates; the replacement requires verified TLS unless the owner approves a documented exception.</t>
+  </si>
+  <si>
+    <t>legacy/zowe.config.json:4-11</t>
+  </si>
+  <si>
+    <t>CICS management is provisioned without authentication or TLS</t>
+  </si>
+  <si>
+    <t>Treat disabled CMCI authentication/SSL and resource-security controls as legacy deployment deviations.</t>
+  </si>
+  <si>
+    <t>The applied CICS region configuration disables secure TCP/IP, CMCI authentication/SSL, and xtran/xcmd/xuser controls.</t>
+  </si>
+  <si>
+    <t>The supplied region exposes an unauthenticated non-TLS management channel and reduced resource checks; these settings must not be copied into the target.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/zconfig/cics-region.yaml:56-82; legacy/.setup/setup/setup-cics-region.sh:125-140</t>
   </si>
   <si>
     <t>IBM MQ is documented but not evidenced in runtime banking code</t>
@@ -2652,7 +2682,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N151"/>
+  <dimension ref="A1:N153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -7058,7 +7088,7 @@
         <v>713</v>
       </c>
       <c r="C151" s="21" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="D151" s="21" t="s">
         <v>714</v>
@@ -7070,7 +7100,7 @@
         <v>716</v>
       </c>
       <c r="G151" s="21" t="s">
-        <v>398</v>
+        <v>124</v>
       </c>
       <c r="H151" s="21" t="s">
         <v>717</v>
@@ -7081,6 +7111,66 @@
       <c r="L151" s="21"/>
       <c r="M151" s="21"/>
       <c r="N151" s="21"/>
+    </row>
+    <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A152" s="21"/>
+      <c r="B152" s="22" t="s">
+        <v>718</v>
+      </c>
+      <c r="C152" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D152" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="E152" s="21" t="s">
+        <v>720</v>
+      </c>
+      <c r="F152" s="21" t="s">
+        <v>721</v>
+      </c>
+      <c r="G152" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="H152" s="21" t="s">
+        <v>722</v>
+      </c>
+      <c r="I152" s="21"/>
+      <c r="J152" s="21"/>
+      <c r="K152" s="21"/>
+      <c r="L152" s="21"/>
+      <c r="M152" s="21"/>
+      <c r="N152" s="21"/>
+    </row>
+    <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+      <c r="A153" s="21"/>
+      <c r="B153" s="22" t="s">
+        <v>723</v>
+      </c>
+      <c r="C153" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D153" s="21" t="s">
+        <v>724</v>
+      </c>
+      <c r="E153" s="21" t="s">
+        <v>725</v>
+      </c>
+      <c r="F153" s="21" t="s">
+        <v>726</v>
+      </c>
+      <c r="G153" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="H153" s="21" t="s">
+        <v>727</v>
+      </c>
+      <c r="I153" s="21"/>
+      <c r="J153" s="21"/>
+      <c r="K153" s="21"/>
+      <c r="L153" s="21"/>
+      <c r="M153" s="21"/>
+      <c r="N153" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
feat: add traceable Stage 3 legacy simulation
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -124,7 +124,7 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:384-958; legacy/src/base/cics/bms/BNK1MAI.bms</t>
+    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:384-958; legacy/src/base/cics/bms/BNK1MAI.bms; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-menu; harness: simulation/test; basis: legacy/src/base/cics/cobol/BNKMENU.cbl:135-171,363-384,958; legacy/src/base/cics/bms/BNK1MAI.bms</t>
   </si>
   <si>
     <t>CICS operator exits or cancels</t>
@@ -142,7 +142,7 @@
     <t>The session ends or returns to the main menu without applying the pending action.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:135-171; BNK1*.cbl EIBAID handlers</t>
+    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:135-171; BNK1*.cbl EIBAID handlers; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-menu; harness: simulation/test; basis: legacy/src/base/cics/cobol/BNKMENU.cbl:135-171,363-384,958; legacy/src/base/cics/bms/BNK1MAI.bms</t>
   </si>
   <si>
     <t>CICS operator presses an unsupported key</t>
@@ -157,7 +157,7 @@
     <t>An explanatory message is shown and the screen is redisplayed.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNKMENU.cbl input-processing paragraphs; BNK1*.cbl VALID-DATA-SW</t>
+    <t>legacy/src/base/cics/cobol/BNKMENU.cbl input-processing paragraphs; BNK1*.cbl VALID-DATA-SW; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-menu; harness: simulation/test; basis: legacy/src/base/cics/cobol/BNKMENU.cbl:135-171,363-384,958; legacy/src/base/cics/bms/BNK1MAI.bms</t>
   </si>
   <si>
     <t>CICS operator enters an invalid menu choice</t>
@@ -172,7 +172,7 @@
     <t>You must enter a valid value (1-7 or A). is shown and the menu is redisplayed without dispatch.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:363-378</t>
+    <t>legacy/src/base/cics/cobol/BNKMENU.cbl:363-378; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-menu; harness: simulation/test; basis: legacy/src/base/cics/cobol/BNKMENU.cbl:135-171,363-384,958; legacy/src/base/cics/bms/BNK1MAI.bms</t>
   </si>
   <si>
     <t>Web operator opens the control panel</t>
@@ -232,7 +232,7 @@
     <t>LOGIN SUCCESSFUL is returned and login status/time are updated.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/pli/IBLOGIN.pli:202-342; legacy/src/base/ims/PSB/IBLOGIN.asm:13; legacy/.setup/deploy/ims_spoc.jcl.j2:72-73,91,96-97; IBLOGIN1.cbl is a non-deployed COBOL sibling</t>
+    <t>legacy/src/base/ims/pli/IBLOGIN.pli:202-342; legacy/src/base/ims/PSB/IBLOGIN.asm:13; legacy/.setup/deploy/ims_spoc.jcl.j2:72-73,91,96-97; IBLOGIN1.cbl is a non-deployed COBOL sibling; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-session; harness: simulation/test; basis: legacy/src/base/ims/pli/IBLOGIN.pli; legacy/src/base/ims/cobol/IBLOGOUT.cbl</t>
   </si>
   <si>
     <t>IMS customer is already logged in</t>
@@ -271,7 +271,7 @@
     <t>LOGOFF SUCCESSFUL is returned and the status is persisted.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:24-25,180-215</t>
+    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:24-25,180-215; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-session; harness: simulation/test; basis: legacy/src/base/ims/pli/IBLOGIN.pli; legacy/src/base/ims/cobol/IBLOGOUT.cbl</t>
   </si>
   <si>
     <t>IMS logout customer retrieval fails</t>
@@ -289,7 +289,7 @@
     <t>FAILED UPDATE FOR LOGOFF is returned.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:180-202</t>
+    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:180-202; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-session; harness: simulation/test; basis: legacy/src/base/ims/pli/IBLOGIN.pli; legacy/src/base/ims/cobol/IBLOGOUT.cbl</t>
   </si>
   <si>
     <t>IMS logout replacement fails but reports success</t>
@@ -304,7 +304,7 @@
     <t>LOGOFF SUCCESSFUL is returned even though the logout status replacement failed; this is a security and data-consistency deviation.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:203-212</t>
+    <t>legacy/src/base/ims/cobol/IBLOGOUT.cbl:203-212; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-session; harness: simulation/test; basis: legacy/src/base/ims/pli/IBLOGIN.pli; legacy/src/base/ims/cobol/IBLOGOUT.cbl</t>
   </si>
   <si>
     <t>UF-002</t>
@@ -862,7 +862,7 @@
     <t>Actual and available balances increase and the result is displayed.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNK1CRA.cbl; DBCRFUN.cbl; BNK1CDM.bms</t>
+    <t>legacy/src/base/cics/cobol/BNK1CRA.cbl; DBCRFUN.cbl; BNK1CDM.bms; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>CICS operator debits an account</t>
@@ -877,7 +877,7 @@
     <t>Actual and available balances decrease and the result is displayed.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNK1CRA.cbl; DBCRFUN.cbl</t>
+    <t>legacy/src/base/cics/cobol/BNK1CRA.cbl; DBCRFUN.cbl; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>CICS cash transaction validates input</t>
@@ -892,7 +892,7 @@
     <t>A validation/not-found message is shown and no balance change occurs.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNK1CRA.cbl:962-1148</t>
+    <t>legacy/src/base/cics/cobol/BNK1CRA.cbl:962-1148; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>CICS cash transaction is audited</t>
@@ -907,7 +907,7 @@
     <t>ACCOUNT and PROCTRAN are updated consistently or rolled back.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl ACCOUNT update and PROCTRAN insert</t>
+    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl ACCOUNT update and PROCTRAN insert; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>IMS customer deposits or withdraws</t>
@@ -922,7 +922,7 @@
     <t>Balance and last transaction ID update; account summary is returned.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:31-34,265-383</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:31-34,265-383; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>IMS transaction action is invalid</t>
@@ -937,7 +937,7 @@
     <t>INVALID ACCOUNT ACTION is returned.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:34,265-291</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:34,265-291; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>IMS account/customer is missing</t>
@@ -952,7 +952,7 @@
     <t>ACCOUNT DOES NOT EXIST or CUSTOMER DOES NOT EXIST is returned.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:31-32,302-422</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:31-32,302-422; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>IMS transaction uses mismatched customer and account identifiers</t>
@@ -967,7 +967,7 @@
     <t>An existing account can be mutated while the returned summary belongs to another supplied customer; this is a security and data-integrity deviation.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:299-367,386-430; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BcustomerId%7D%2F%7BaccountId%7D%2Fdeposit/post/request.yaml</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:299-367,386-430; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BcustomerId%7D%2F%7BaccountId%7D%2Fdeposit/post/request.yaml; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>IMS transaction history is persisted</t>
@@ -982,7 +982,7 @@
     <t>DB2 history is attempted first, IMS history is inserted next, and the account is replaced last; failures can expose partial-write risk according to the coded status handling.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:326-367,454-554; legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:140</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:326-367,454-554; legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:140; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>Web operator deposits to a selected CICS account</t>
@@ -1042,7 +1042,7 @@
     <t>The operation fails with code 3 (insufficient funds) and the balance is unchanged.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl:340-350</t>
+    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl:340-350; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>CICS payment rejects mortgage or loan cash activity</t>
@@ -1057,7 +1057,7 @@
     <t>The operation fails with code 4 and no balance mutation is performed.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl:320-376</t>
+    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl:320-376; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>CICS teller bypasses payment-only cash restrictions</t>
@@ -1072,7 +1072,7 @@
     <t>A teller request proceeds to the balance update without those two payment-only rejections.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl:320-376; facility type checks at 331-344 and 368-371</t>
+    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl:320-376; facility type checks at 331-344 and 368-371; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
   </si>
   <si>
     <t>IMS withdrawal can make the balance negative</t>
@@ -1087,7 +1087,7 @@
     <t>The requested amount is subtracted and the stored/history balance can become negative.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:338-348</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:338-348; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>Direct IMS negative deposit reverses transaction direction</t>
@@ -1102,7 +1102,7 @@
     <t>A negative deposit subtracts its absolute value and advances transaction/history processing.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:294-367</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:294-367; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
   </si>
   <si>
     <t>Direct IMS negative withdrawal reverses transaction direction</t>
@@ -1147,7 +1147,7 @@
     <t>Both resulting balances are displayed after success.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl; XFRFUN.cbl; BNK1TFM.bms</t>
+    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl; XFRFUN.cbl; BNK1TFM.bms; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
   </si>
   <si>
     <t>Transfer input is invalid</t>
@@ -1162,7 +1162,7 @@
     <t>An explanatory message is shown and balances remain unchanged.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl:988-1204; XFRFUN.cbl inquiry sections</t>
+    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl:988-1204; XFRFUN.cbl inquiry sections; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
   </si>
   <si>
     <t>Transfer updates both accounts atomically</t>
@@ -1177,7 +1177,7 @@
     <t>Both account updates commit, otherwise a CICS syncpoint rollback is performed.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:998-1450</t>
+    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:998-1450; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
   </si>
   <si>
     <t>Transfer writes transaction evidence</t>
@@ -1192,7 +1192,7 @@
     <t>PROCTRAN receives transfer type, amount, counterparty sort code/account, date, time, and reference.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:1563-1639</t>
+    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:1563-1639; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
   </si>
   <si>
     <t>Transfer overdraft behavior requires owner decision</t>
@@ -1210,7 +1210,7 @@
     <t>Inferred</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:10-22 explicitly states that no overdraft-limit checking is made</t>
+    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:10-22 explicitly states that no overdraft-limit checking is made; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
   </si>
   <si>
     <t>Bank-to-bank transfer screen is a non-deployed surface</t>
@@ -1246,7 +1246,7 @@
     <t>GET and PUT success mappings reach INQCUST/UPDCUST, but the PUT 401/403 response selections reference missing generated files.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:275-345; operations ...customers...; zosAssets/INQCUST and UPDCUST</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:275-345; operations ...customers...; zosAssets/INQCUST and UPDCUST; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>External client retrieves CICS accounts and balances</t>
@@ -1261,7 +1261,7 @@
     <t>Success mappings return account/balance schemas, but three selected 400 response files are absent.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:346-478; zosAssets/INQACCCU and INQACC</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:346-478; zosAssets/INQACCCU and INQACC; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>External client deposits to CICS</t>
@@ -1276,7 +1276,7 @@
     <t>The DBCRFUN-backed mapping returns the updated account/balance response.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:479-517,1025; zosAssets/DBCRFUN</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:479-517,1025; zosAssets/DBCRFUN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>External client uses IMS customer/account APIs</t>
@@ -1291,7 +1291,7 @@
     <t>Operations map to IBGCUDAT, IBSCUDAT, IBACSUM, and IBTRAN.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:31-245; zosAssets/IBGCUDAT,IBSCUDAT,IBACSUM,IBTRAN</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:31-245; zosAssets/IBGCUDAT,IBSCUDAT,IBACSUM,IBTRAN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>External client lists all accounts</t>
@@ -1306,7 +1306,7 @@
     <t>The contract exists; deployable mapping is absent.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:379-412; operations/%2Faccounts/get (no operation.yaml)</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:379-412; operations/%2Faccounts/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>External client lists account transactions</t>
@@ -1318,7 +1318,7 @@
     <t>OpenAPI and the JS client publish the route, but no z/OS operation mapping exists.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:518-579; js/api.js:260-279; operations/...transactions/get (no operation.yaml)</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:518-579; js/api.js:260-279; operations/...transactions/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>External client retrieves one transaction</t>
@@ -1330,7 +1330,7 @@
     <t>The route is published but has no operation mapping.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:580-615; js/api.js:286-292; operations/...transactionId/get (no operation.yaml)</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:580-615; js/api.js:286-292; operations/...transactionId/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>Java history service reads recent activity</t>
@@ -1360,7 +1360,7 @@
     <t>The contract declares standard failures, but five bound and three unbound response selections reference missing generated YAML artifacts.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>Generated API mappings select missing response files</t>
@@ -1390,7 +1390,7 @@
     <t>A successful response returns the created customer identity; mapped failures use the declared API responses.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:246-274; legacy/src/api/src/main/operations/%2Fcustomers/post/operation.yaml; legacy/src/api/src/main/zosAssets/CRECUST/zosAsset.yaml</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:246-274; legacy/src/api/src/main/operations/%2Fcustomers/post/operation.yaml; legacy/src/api/src/main/zosAssets/CRECUST/zosAsset.yaml; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
     <t>IMS client requests recent history through IBGHIST</t>
@@ -1426,7 +1426,7 @@
     <t>BNKSTMT processes matching accounts and writes formatted statements to SYSPRINT.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/jcl/BNKSTMT.jcl:1-22; pli/BNKSTMT.pli:18-27,187-205</t>
+    <t>legacy/src/base/batch/jcl/BNKSTMT.jcl:1-22; pli/BNKSTMT.pli:18-27,187-205; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement parameters are missing</t>
@@ -1441,7 +1441,7 @@
     <t>Default sort code 123456 and calculated/default statement period are used with diagnostic output.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:210-292</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:210-292; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement includes customer and account identity</t>
@@ -1456,7 +1456,7 @@
     <t>Customer and account information sections are printed.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:430-635</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:430-635; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement lists period transactions</t>
@@ -1471,7 +1471,7 @@
     <t>Each transaction includes date, time, type, reference, description, amount, and balance context.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:638-779</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:638-779; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement period has no transactions</t>
@@ -1486,7 +1486,7 @@
     <t>NO TRANSACTIONS FOR THIS PERIOD is printed.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:719-725</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:719-725; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement prints financial summary</t>
@@ -1501,7 +1501,7 @@
     <t>A statement summary is printed with all totals.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:782-859</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:782-859; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement paginates and closes</t>
@@ -1516,7 +1516,7 @@
     <t>Page headers and the closing footer are produced.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:519-560,862-905</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:519-560,862-905; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>Statement database operation fails</t>
@@ -1531,7 +1531,7 @@
     <t>SQLCODE diagnostics/warnings are written to SYSPRINT and processing follows the coded branch.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:328-389,475-502,670-704</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:328-389,475-502,670-704; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
   </si>
   <si>
     <t>UF-010</t>
@@ -1612,7 +1612,7 @@
     <t>Static files are returned and index.html redirects the browser to admin.html.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js:14-51; legacy/src/frontend/index.html redirects to admin.html</t>
+    <t>legacy/src/frontend/server.js:14-51; legacy/src/frontend/index.html redirects to admin.html; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
   </si>
   <si>
     <t>Web server proxies API traffic</t>
@@ -1627,7 +1627,7 @@
     <t>Requests and responses are streamed to/from API_BASE_URL.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js proxy paths; config.js base URL</t>
+    <t>legacy/src/frontend/server.js proxy paths; config.js base URL; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
   </si>
   <si>
     <t>Web static file is missing</t>
@@ -1642,7 +1642,7 @@
     <t>HTTP 404 is returned.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js missing-file branch</t>
+    <t>legacy/src/frontend/server.js missing-file branch; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
   </si>
   <si>
     <t>Web proxy target is unavailable</t>
@@ -1657,7 +1657,7 @@
     <t>HTTP 502 with JSON error information is returned.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js proxy error handler</t>
+    <t>legacy/src/frontend/server.js proxy error handler; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
   </si>
   <si>
     <t>Web control panel has no application authentication</t>
@@ -1672,7 +1672,7 @@
     <t>No application login challenge is presented; target access control requires explicit owner approval rather than silent inheritance.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js:1-111; legacy/src/frontend/admin.html:1-103; no authentication middleware or login page is present under legacy/src/frontend</t>
+    <t>legacy/src/frontend/server.js:1-111; legacy/src/frontend/admin.html:1-103; no authentication middleware or login page is present under legacy/src/frontend; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
   </si>
   <si>
     <t>UF-011</t>
@@ -2682,7 +2682,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N153"/>
+  <dimension ref="A1:O153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2700,7 +2700,7 @@
     <col min="14" max="14" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="M1"/>
       <c r="N1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2736,7 +2736,8 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="31.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2768,7 +2769,7 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>10</v>
       </c>
@@ -2790,7 +2791,7 @@
       <c r="M5" s="10"/>
       <c r="N5" s="11"/>
     </row>
-    <row r="6" ht="37.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" ht="37.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>13</v>
       </c>
@@ -2834,7 +2835,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>27</v>
       </c>
@@ -2858,7 +2859,7 @@
       <c r="M7" s="17"/>
       <c r="N7" s="17"/>
     </row>
-    <row r="8" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="8" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A8" s="18"/>
       <c r="B8" s="19" t="s">
         <v>31</v>
@@ -2888,7 +2889,7 @@
       <c r="M8" s="18"/>
       <c r="N8" s="18"/>
     </row>
-    <row r="9" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="9" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A9" s="18"/>
       <c r="B9" s="19" t="s">
         <v>38</v>
@@ -2918,7 +2919,7 @@
       <c r="M9" s="18"/>
       <c r="N9" s="18"/>
     </row>
-    <row r="10" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="10" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A10" s="18"/>
       <c r="B10" s="19" t="s">
         <v>44</v>
@@ -2948,7 +2949,7 @@
       <c r="M10" s="18"/>
       <c r="N10" s="18"/>
     </row>
-    <row r="11" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="11" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A11" s="18"/>
       <c r="B11" s="19" t="s">
         <v>49</v>
@@ -2978,7 +2979,7 @@
       <c r="M11" s="18"/>
       <c r="N11" s="18"/>
     </row>
-    <row r="12" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="12" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A12" s="18"/>
       <c r="B12" s="19" t="s">
         <v>54</v>
@@ -3008,7 +3009,7 @@
       <c r="M12" s="18"/>
       <c r="N12" s="18"/>
     </row>
-    <row r="13" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="13" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A13" s="18"/>
       <c r="B13" s="19" t="s">
         <v>59</v>
@@ -3038,7 +3039,7 @@
       <c r="M13" s="18"/>
       <c r="N13" s="18"/>
     </row>
-    <row r="14" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="14" ht="48" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A14" s="18"/>
       <c r="B14" s="19" t="s">
         <v>64</v>
@@ -3068,7 +3069,7 @@
       <c r="M14" s="18"/>
       <c r="N14" s="18"/>
     </row>
-    <row r="15" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="15" ht="48" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A15" s="18"/>
       <c r="B15" s="19" t="s">
         <v>69</v>
@@ -3098,7 +3099,7 @@
       <c r="M15" s="18"/>
       <c r="N15" s="18"/>
     </row>
-    <row r="16" ht="48" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="16" ht="48" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A16" s="19"/>
       <c r="B16" s="19" t="s">
         <v>74</v>
@@ -3128,7 +3129,7 @@
       <c r="M16" s="19"/>
       <c r="N16" s="19"/>
     </row>
-    <row r="17" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="17" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A17" s="18"/>
       <c r="B17" s="19" t="s">
         <v>78</v>
@@ -3158,7 +3159,7 @@
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
     </row>
-    <row r="18" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="18" ht="15" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A18" s="18"/>
       <c r="B18" s="19" t="s">
         <v>82</v>
@@ -3188,7 +3189,7 @@
       <c r="M18" s="18"/>
       <c r="N18" s="18"/>
     </row>
-    <row r="19" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="19" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A19" s="17"/>
       <c r="B19" s="17" t="s">
         <v>87</v>
@@ -3218,7 +3219,7 @@
       <c r="M19" s="17"/>
       <c r="N19" s="17"/>
     </row>
-    <row r="20" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="20" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A20" s="18"/>
       <c r="B20" s="19" t="s">
         <v>93</v>
@@ -3248,7 +3249,7 @@
       <c r="M20" s="19"/>
       <c r="N20" s="18"/>
     </row>
-    <row r="21" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
         <v>98</v>
       </c>
@@ -3272,7 +3273,7 @@
       <c r="M21" s="18"/>
       <c r="N21" s="18"/>
     </row>
-    <row r="22" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="22" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A22" s="18"/>
       <c r="B22" s="19" t="s">
         <v>100</v>
@@ -3302,7 +3303,7 @@
       <c r="M22" s="19"/>
       <c r="N22" s="18"/>
     </row>
-    <row r="23" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="23" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A23" s="18"/>
       <c r="B23" s="19" t="s">
         <v>105</v>
@@ -3332,7 +3333,7 @@
       <c r="M23" s="18"/>
       <c r="N23" s="18"/>
     </row>
-    <row r="24" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="24" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A24" s="18"/>
       <c r="B24" s="19" t="s">
         <v>110</v>
@@ -3362,7 +3363,7 @@
       <c r="M24" s="18"/>
       <c r="N24" s="18"/>
     </row>
-    <row r="25" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="25" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A25" s="19"/>
       <c r="B25" s="19" t="s">
         <v>115</v>
@@ -3392,7 +3393,7 @@
       <c r="M25" s="19"/>
       <c r="N25" s="19"/>
     </row>
-    <row r="26" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="26" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A26" s="17"/>
       <c r="B26" s="17" t="s">
         <v>120</v>
@@ -3422,7 +3423,7 @@
       <c r="M26" s="17"/>
       <c r="N26" s="17"/>
     </row>
-    <row r="27" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="27" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A27" s="18"/>
       <c r="B27" s="19" t="s">
         <v>126</v>
@@ -3452,7 +3453,7 @@
       <c r="M27" s="18"/>
       <c r="N27" s="18"/>
     </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
         <v>131</v>
       </c>
@@ -3476,7 +3477,7 @@
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
     </row>
-    <row r="29" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="29" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A29" s="18"/>
       <c r="B29" s="19" t="s">
         <v>133</v>
@@ -3506,7 +3507,7 @@
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
     </row>
-    <row r="30" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="30" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A30" s="18"/>
       <c r="B30" s="19" t="s">
         <v>138</v>
@@ -3536,7 +3537,7 @@
       <c r="M30" s="18"/>
       <c r="N30" s="18"/>
     </row>
-    <row r="31" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="31" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A31" s="18"/>
       <c r="B31" s="19" t="s">
         <v>143</v>
@@ -3566,7 +3567,7 @@
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
     </row>
-    <row r="32" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="32" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A32" s="19"/>
       <c r="B32" s="19" t="s">
         <v>148</v>
@@ -3596,7 +3597,7 @@
       <c r="M32" s="19"/>
       <c r="N32" s="19"/>
     </row>
-    <row r="33" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="33" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A33" s="18"/>
       <c r="B33" s="19" t="s">
         <v>153</v>
@@ -3626,7 +3627,7 @@
       <c r="M33" s="19"/>
       <c r="N33" s="18"/>
     </row>
-    <row r="34" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="34" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A34" s="18"/>
       <c r="B34" s="19" t="s">
         <v>158</v>
@@ -3656,7 +3657,7 @@
       <c r="M34" s="19"/>
       <c r="N34" s="18"/>
     </row>
-    <row r="35" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="35" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A35" s="18"/>
       <c r="B35" s="19" t="s">
         <v>163</v>
@@ -3686,7 +3687,7 @@
       <c r="M35" s="19"/>
       <c r="N35" s="18"/>
     </row>
-    <row r="36" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="36" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A36" s="18"/>
       <c r="B36" s="19" t="s">
         <v>168</v>
@@ -3716,7 +3717,7 @@
       <c r="M36" s="19"/>
       <c r="N36" s="18"/>
     </row>
-    <row r="37" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="37" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A37" s="19"/>
       <c r="B37" s="19" t="s">
         <v>173</v>
@@ -3746,7 +3747,7 @@
       <c r="M37" s="19"/>
       <c r="N37" s="19"/>
     </row>
-    <row r="38" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="38" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A38" s="17"/>
       <c r="B38" s="17" t="s">
         <v>178</v>
@@ -3776,7 +3777,7 @@
       <c r="M38" s="17"/>
       <c r="N38" s="17"/>
     </row>
-    <row r="39" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="39" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A39" s="18"/>
       <c r="B39" s="19" t="s">
         <v>183</v>
@@ -3806,7 +3807,7 @@
       <c r="M39" s="19"/>
       <c r="N39" s="18"/>
     </row>
-    <row r="40" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
         <v>188</v>
       </c>
@@ -3830,7 +3831,7 @@
       <c r="M40" s="19"/>
       <c r="N40" s="18"/>
     </row>
-    <row r="41" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="41" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A41" s="18"/>
       <c r="B41" s="19" t="s">
         <v>190</v>
@@ -3860,7 +3861,7 @@
       <c r="M41" s="19"/>
       <c r="N41" s="18"/>
     </row>
-    <row r="42" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="42" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A42" s="18"/>
       <c r="B42" s="19" t="s">
         <v>195</v>
@@ -3890,7 +3891,7 @@
       <c r="M42" s="19"/>
       <c r="N42" s="18"/>
     </row>
-    <row r="43" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="43" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A43" s="19"/>
       <c r="B43" s="19" t="s">
         <v>200</v>
@@ -3920,7 +3921,7 @@
       <c r="M43" s="19"/>
       <c r="N43" s="19"/>
     </row>
-    <row r="44" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="44" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A44" s="18"/>
       <c r="B44" s="19" t="s">
         <v>205</v>
@@ -3950,7 +3951,7 @@
       <c r="M44" s="18"/>
       <c r="N44" s="18"/>
     </row>
-    <row r="45" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="45" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A45" s="18"/>
       <c r="B45" s="19" t="s">
         <v>210</v>
@@ -3980,7 +3981,7 @@
       <c r="M45" s="18"/>
       <c r="N45" s="18"/>
     </row>
-    <row r="46" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="46" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A46" s="18"/>
       <c r="B46" s="19" t="s">
         <v>215</v>
@@ -4010,7 +4011,7 @@
       <c r="M46" s="18"/>
       <c r="N46" s="18"/>
     </row>
-    <row r="47" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="47" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A47" s="17"/>
       <c r="B47" s="17" t="s">
         <v>220</v>
@@ -4040,7 +4041,7 @@
       <c r="M47" s="17"/>
       <c r="N47" s="17"/>
     </row>
-    <row r="48" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="48" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A48" s="18"/>
       <c r="B48" s="19" t="s">
         <v>225</v>
@@ -4070,7 +4071,7 @@
       <c r="M48" s="18"/>
       <c r="N48" s="18"/>
     </row>
-    <row r="49" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" ht="36" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="18" t="s">
         <v>230</v>
       </c>
@@ -4094,7 +4095,7 @@
       <c r="M49" s="18"/>
       <c r="N49" s="18"/>
     </row>
-    <row r="50" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="50" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A50" s="18"/>
       <c r="B50" s="19" t="s">
         <v>232</v>
@@ -4124,7 +4125,7 @@
       <c r="M50" s="18"/>
       <c r="N50" s="18"/>
     </row>
-    <row r="51" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="51" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A51" s="18"/>
       <c r="B51" s="19" t="s">
         <v>237</v>
@@ -4154,7 +4155,7 @@
       <c r="M51" s="18"/>
       <c r="N51" s="18"/>
     </row>
-    <row r="52" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="52" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A52" s="19"/>
       <c r="B52" s="19" t="s">
         <v>242</v>
@@ -4184,7 +4185,7 @@
       <c r="M52" s="19"/>
       <c r="N52" s="19"/>
     </row>
-    <row r="53" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="53" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A53" s="18"/>
       <c r="B53" s="19" t="s">
         <v>247</v>
@@ -4214,7 +4215,7 @@
       <c r="M53" s="18"/>
       <c r="N53" s="18"/>
     </row>
-    <row r="54" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="54" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A54" s="18"/>
       <c r="B54" s="19" t="s">
         <v>252</v>
@@ -4244,7 +4245,7 @@
       <c r="M54" s="18"/>
       <c r="N54" s="18"/>
     </row>
-    <row r="55" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="55" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A55" s="18"/>
       <c r="B55" s="19" t="s">
         <v>257</v>
@@ -4274,7 +4275,7 @@
       <c r="M55" s="18"/>
       <c r="N55" s="18"/>
     </row>
-    <row r="56" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="56" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A56" s="18"/>
       <c r="B56" s="19" t="s">
         <v>262</v>
@@ -4304,7 +4305,7 @@
       <c r="M56" s="18"/>
       <c r="N56" s="18"/>
     </row>
-    <row r="57" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="57" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A57" s="17"/>
       <c r="B57" s="17" t="s">
         <v>267</v>
@@ -4334,7 +4335,7 @@
       <c r="M57" s="17"/>
       <c r="N57" s="17"/>
     </row>
-    <row r="58" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="58" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A58" s="18"/>
       <c r="B58" s="19" t="s">
         <v>272</v>
@@ -4364,7 +4365,7 @@
       <c r="M58" s="18"/>
       <c r="N58" s="18"/>
     </row>
-    <row r="59" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="18" t="s">
         <v>277</v>
       </c>
@@ -4388,7 +4389,7 @@
       <c r="M59" s="18"/>
       <c r="N59" s="18"/>
     </row>
-    <row r="60" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="60" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A60" s="18"/>
       <c r="B60" s="19" t="s">
         <v>279</v>
@@ -4418,7 +4419,7 @@
       <c r="M60" s="18"/>
       <c r="N60" s="18"/>
     </row>
-    <row r="61" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="61" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A61" s="18"/>
       <c r="B61" s="19" t="s">
         <v>284</v>
@@ -4448,7 +4449,7 @@
       <c r="M61" s="18"/>
       <c r="N61" s="18"/>
     </row>
-    <row r="62" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="62" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A62" s="18"/>
       <c r="B62" s="19" t="s">
         <v>289</v>
@@ -4478,7 +4479,7 @@
       <c r="M62" s="18"/>
       <c r="N62" s="18"/>
     </row>
-    <row r="63" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="63" ht="15" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A63" s="19"/>
       <c r="B63" s="19" t="s">
         <v>294</v>
@@ -4508,7 +4509,7 @@
       <c r="M63" s="19"/>
       <c r="N63" s="19"/>
     </row>
-    <row r="64" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="64" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A64" s="18"/>
       <c r="B64" s="19" t="s">
         <v>299</v>
@@ -4538,7 +4539,7 @@
       <c r="M64" s="18"/>
       <c r="N64" s="18"/>
     </row>
-    <row r="65" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="65" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A65" s="18"/>
       <c r="B65" s="19" t="s">
         <v>304</v>
@@ -4568,7 +4569,7 @@
       <c r="M65" s="18"/>
       <c r="N65" s="18"/>
     </row>
-    <row r="66" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="66" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A66" s="18"/>
       <c r="B66" s="19" t="s">
         <v>309</v>
@@ -4598,7 +4599,7 @@
       <c r="M66" s="18"/>
       <c r="N66" s="18"/>
     </row>
-    <row r="67" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="67" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A67" s="18"/>
       <c r="B67" s="19" t="s">
         <v>314</v>
@@ -4628,7 +4629,7 @@
       <c r="M67" s="18"/>
       <c r="N67" s="18"/>
     </row>
-    <row r="68" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="68" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A68" s="19"/>
       <c r="B68" s="19" t="s">
         <v>319</v>
@@ -4658,7 +4659,7 @@
       <c r="M68" s="19"/>
       <c r="N68" s="19"/>
     </row>
-    <row r="69" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="69" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A69" s="18"/>
       <c r="B69" s="19" t="s">
         <v>324</v>
@@ -4688,7 +4689,7 @@
       <c r="M69" s="18"/>
       <c r="N69" s="18"/>
     </row>
-    <row r="70" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="70" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A70" s="18"/>
       <c r="B70" s="19" t="s">
         <v>329</v>
@@ -4718,7 +4719,7 @@
       <c r="M70" s="19"/>
       <c r="N70" s="18"/>
     </row>
-    <row r="71" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="71" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A71" s="19"/>
       <c r="B71" s="19" t="s">
         <v>334</v>
@@ -4748,7 +4749,7 @@
       <c r="M71" s="19"/>
       <c r="N71" s="19"/>
     </row>
-    <row r="72" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="72" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A72" s="17"/>
       <c r="B72" s="17" t="s">
         <v>339</v>
@@ -4778,7 +4779,7 @@
       <c r="M72" s="17"/>
       <c r="N72" s="17"/>
     </row>
-    <row r="73" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="73" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A73" s="18"/>
       <c r="B73" s="19" t="s">
         <v>344</v>
@@ -4808,7 +4809,7 @@
       <c r="M73" s="18"/>
       <c r="N73" s="18"/>
     </row>
-    <row r="74" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="74" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A74" s="19"/>
       <c r="B74" s="19" t="s">
         <v>349</v>
@@ -4838,7 +4839,7 @@
       <c r="M74" s="19"/>
       <c r="N74" s="19"/>
     </row>
-    <row r="75" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="75" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A75" s="18"/>
       <c r="B75" s="19" t="s">
         <v>354</v>
@@ -4868,7 +4869,7 @@
       <c r="M75" s="19"/>
       <c r="N75" s="18"/>
     </row>
-    <row r="76" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="76" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A76" s="18"/>
       <c r="B76" s="19" t="s">
         <v>359</v>
@@ -4898,7 +4899,7 @@
       <c r="M76" s="18"/>
       <c r="N76" s="18"/>
     </row>
-    <row r="77" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="77" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A77" s="19"/>
       <c r="B77" s="19" t="s">
         <v>364</v>
@@ -4928,7 +4929,7 @@
       <c r="M77" s="19"/>
       <c r="N77" s="19"/>
     </row>
-    <row r="78" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="78" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A78" s="18"/>
       <c r="B78" s="19" t="s">
         <v>368</v>
@@ -4958,7 +4959,7 @@
       <c r="M78" s="18"/>
       <c r="N78" s="18"/>
     </row>
-    <row r="79" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
         <v>372</v>
       </c>
@@ -4982,7 +4983,7 @@
       <c r="M79" s="17"/>
       <c r="N79" s="17"/>
     </row>
-    <row r="80" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="80" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A80" s="18"/>
       <c r="B80" s="19" t="s">
         <v>374</v>
@@ -5012,7 +5013,7 @@
       <c r="M80" s="18"/>
       <c r="N80" s="18"/>
     </row>
-    <row r="81" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="81" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A81" s="19"/>
       <c r="B81" s="19" t="s">
         <v>379</v>
@@ -5042,7 +5043,7 @@
       <c r="M81" s="19"/>
       <c r="N81" s="19"/>
     </row>
-    <row r="82" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="82" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A82" s="18"/>
       <c r="B82" s="19" t="s">
         <v>384</v>
@@ -5072,7 +5073,7 @@
       <c r="M82" s="18"/>
       <c r="N82" s="18"/>
     </row>
-    <row r="83" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="83" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="18"/>
       <c r="B83" s="19" t="s">
         <v>389</v>
@@ -5102,7 +5103,7 @@
       <c r="M83" s="18"/>
       <c r="N83" s="18"/>
     </row>
-    <row r="84" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="84" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="19"/>
       <c r="B84" s="19" t="s">
         <v>394</v>
@@ -5132,7 +5133,7 @@
       <c r="M84" s="19"/>
       <c r="N84" s="19"/>
     </row>
-    <row r="85" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="85" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
         <v>400</v>
@@ -5162,7 +5163,7 @@
       <c r="M85" s="18"/>
       <c r="N85" s="18"/>
     </row>
-    <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" ht="36" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A86" s="19" t="s">
         <v>405</v>
       </c>
@@ -5186,7 +5187,7 @@
       <c r="M86" s="19"/>
       <c r="N86" s="19"/>
     </row>
-    <row r="87" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="87" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
         <v>407</v>
@@ -5216,7 +5217,7 @@
       <c r="M87" s="18"/>
       <c r="N87" s="18"/>
     </row>
-    <row r="88" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="88" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
         <v>412</v>
@@ -5246,7 +5247,7 @@
       <c r="M88" s="18"/>
       <c r="N88" s="18"/>
     </row>
-    <row r="89" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="89" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
         <v>417</v>
@@ -5276,7 +5277,7 @@
       <c r="M89" s="18"/>
       <c r="N89" s="18"/>
     </row>
-    <row r="90" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="90" ht="60" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
         <v>422</v>
@@ -5306,7 +5307,7 @@
       <c r="M90" s="18"/>
       <c r="N90" s="18"/>
     </row>
-    <row r="91" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="91" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="17"/>
       <c r="B91" s="17" t="s">
         <v>427</v>
@@ -5336,7 +5337,7 @@
       <c r="M91" s="17"/>
       <c r="N91" s="17"/>
     </row>
-    <row r="92" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="92" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
         <v>432</v>
@@ -5366,7 +5367,7 @@
       <c r="M92" s="18"/>
       <c r="N92" s="18"/>
     </row>
-    <row r="93" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="93" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="19"/>
       <c r="B93" s="19" t="s">
         <v>436</v>
@@ -5396,7 +5397,7 @@
       <c r="M93" s="19"/>
       <c r="N93" s="19"/>
     </row>
-    <row r="94" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="94" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="19"/>
       <c r="B94" s="19" t="s">
         <v>440</v>
@@ -5426,7 +5427,7 @@
       <c r="M94" s="19"/>
       <c r="N94" s="19"/>
     </row>
-    <row r="95" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="95" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
         <v>445</v>
@@ -5456,7 +5457,7 @@
       <c r="M95" s="18"/>
       <c r="N95" s="18"/>
     </row>
-    <row r="96" ht="15" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="96" ht="15" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
         <v>450</v>
@@ -5486,7 +5487,7 @@
       <c r="M96" s="18"/>
       <c r="N96" s="18"/>
     </row>
-    <row r="97" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="97" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
         <v>455</v>
@@ -5516,7 +5517,7 @@
       <c r="M97" s="18"/>
       <c r="N97" s="18"/>
     </row>
-    <row r="98" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="98" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
         <v>460</v>
@@ -5546,7 +5547,7 @@
       <c r="M98" s="18"/>
       <c r="N98" s="18"/>
     </row>
-    <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A99" s="18" t="s">
         <v>465</v>
       </c>
@@ -5570,7 +5571,7 @@
       <c r="M99" s="18"/>
       <c r="N99" s="18"/>
     </row>
-    <row r="100" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="100" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="17"/>
       <c r="B100" s="17" t="s">
         <v>467</v>
@@ -5600,7 +5601,7 @@
       <c r="M100" s="17"/>
       <c r="N100" s="17"/>
     </row>
-    <row r="101" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="101" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="19"/>
       <c r="B101" s="19" t="s">
         <v>472</v>
@@ -5630,7 +5631,7 @@
       <c r="M101" s="19"/>
       <c r="N101" s="19"/>
     </row>
-    <row r="102" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="102" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
         <v>477</v>
@@ -5660,7 +5661,7 @@
       <c r="M102" s="18"/>
       <c r="N102" s="18"/>
     </row>
-    <row r="103" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="103" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
         <v>482</v>
@@ -5690,7 +5691,7 @@
       <c r="M103" s="18"/>
       <c r="N103" s="18"/>
     </row>
-    <row r="104" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="104" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
         <v>487</v>
@@ -5720,7 +5721,7 @@
       <c r="M104" s="18"/>
       <c r="N104" s="18"/>
     </row>
-    <row r="105" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="105" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="19"/>
       <c r="B105" s="19" t="s">
         <v>492</v>
@@ -5750,7 +5751,7 @@
       <c r="M105" s="19"/>
       <c r="N105" s="19"/>
     </row>
-    <row r="106" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="106" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
         <v>497</v>
@@ -5780,7 +5781,7 @@
       <c r="M106" s="18"/>
       <c r="N106" s="18"/>
     </row>
-    <row r="107" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="107" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
         <v>502</v>
@@ -5810,7 +5811,7 @@
       <c r="M107" s="18"/>
       <c r="N107" s="18"/>
     </row>
-    <row r="108" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="108" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
         <v>507</v>
       </c>
@@ -5834,7 +5835,7 @@
       <c r="M108" s="17"/>
       <c r="N108" s="17"/>
     </row>
-    <row r="109" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="109" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
         <v>509</v>
@@ -5864,7 +5865,7 @@
       <c r="M109" s="18"/>
       <c r="N109" s="18"/>
     </row>
-    <row r="110" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="110" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
         <v>514</v>
@@ -5894,7 +5895,7 @@
       <c r="M110" s="18"/>
       <c r="N110" s="18"/>
     </row>
-    <row r="111" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="111" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
         <v>519</v>
@@ -5924,7 +5925,7 @@
       <c r="M111" s="18"/>
       <c r="N111" s="18"/>
     </row>
-    <row r="112" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="112" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
         <v>524</v>
@@ -5954,7 +5955,7 @@
       <c r="M112" s="18"/>
       <c r="N112" s="18"/>
     </row>
-    <row r="113" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="113" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
         <v>529</v>
@@ -5984,7 +5985,7 @@
       <c r="M113" s="18"/>
       <c r="N113" s="18"/>
     </row>
-    <row r="114" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="114" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
         <v>534</v>
@@ -6014,7 +6015,7 @@
       <c r="M114" s="18"/>
       <c r="N114" s="18"/>
     </row>
-    <row r="115" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="115" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
         <v>539</v>
@@ -6044,7 +6045,7 @@
       <c r="M115" s="18"/>
       <c r="N115" s="18"/>
     </row>
-    <row r="116" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="116" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="17"/>
       <c r="B116" s="17" t="s">
         <v>544</v>
@@ -6074,7 +6075,7 @@
       <c r="M116" s="17"/>
       <c r="N116" s="17"/>
     </row>
-    <row r="117" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="117" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="20"/>
       <c r="B117" s="20" t="s">
         <v>549</v>
@@ -6104,7 +6105,7 @@
       <c r="M117" s="20"/>
       <c r="N117" s="20"/>
     </row>
-    <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="118" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118" s="20" t="s">
         <v>554</v>
       </c>
@@ -6128,7 +6129,7 @@
       <c r="M118" s="20"/>
       <c r="N118" s="20"/>
     </row>
-    <row r="119" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="119" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="20"/>
       <c r="B119" s="20" t="s">
         <v>556</v>
@@ -6158,7 +6159,7 @@
       <c r="M119" s="20"/>
       <c r="N119" s="20"/>
     </row>
-    <row r="120" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="120" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="20"/>
       <c r="B120" s="20" t="s">
         <v>561</v>
@@ -6188,7 +6189,7 @@
       <c r="M120" s="20"/>
       <c r="N120" s="20"/>
     </row>
-    <row r="121" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="121" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="20"/>
       <c r="B121" s="20" t="s">
         <v>566</v>
@@ -6218,7 +6219,7 @@
       <c r="M121" s="20"/>
       <c r="N121" s="20"/>
     </row>
-    <row r="122" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="122" ht="24" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="20"/>
       <c r="B122" s="20" t="s">
         <v>571</v>
@@ -6248,7 +6249,7 @@
       <c r="M122" s="20"/>
       <c r="N122" s="20"/>
     </row>
-    <row r="123" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="123" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="20"/>
       <c r="B123" s="20" t="s">
         <v>576</v>
@@ -6278,7 +6279,7 @@
       <c r="M123" s="20"/>
       <c r="N123" s="20"/>
     </row>
-    <row r="124" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="124" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="20"/>
       <c r="B124" s="20" t="s">
         <v>581</v>
@@ -6308,7 +6309,7 @@
       <c r="M124" s="20"/>
       <c r="N124" s="20"/>
     </row>
-    <row r="125" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="125" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="20"/>
       <c r="B125" s="20" t="s">
         <v>586</v>
@@ -6338,7 +6339,7 @@
       <c r="M125" s="20"/>
       <c r="N125" s="20"/>
     </row>
-    <row r="126" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="126" ht="60" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="20"/>
       <c r="B126" s="20" t="s">
         <v>591</v>
@@ -6368,7 +6369,7 @@
       <c r="M126" s="20"/>
       <c r="N126" s="20"/>
     </row>
-    <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="127" ht="36" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A127" s="20" t="s">
         <v>596</v>
       </c>
@@ -6392,7 +6393,7 @@
       <c r="M127" s="20"/>
       <c r="N127" s="20"/>
     </row>
-    <row r="128" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="128" ht="36" customHeight="1" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="20"/>
       <c r="B128" s="20" t="s">
         <v>598</v>
@@ -6422,7 +6423,7 @@
       <c r="M128" s="20"/>
       <c r="N128" s="20"/>
     </row>
-    <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="129" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="21"/>
       <c r="B129" s="22" t="s">
         <v>603</v>
@@ -6452,7 +6453,7 @@
       <c r="M129" s="21"/>
       <c r="N129" s="21"/>
     </row>
-    <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="130" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="21"/>
       <c r="B130" s="22" t="s">
         <v>608</v>
@@ -6482,7 +6483,7 @@
       <c r="M130" s="21"/>
       <c r="N130" s="21"/>
     </row>
-    <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="131" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="21"/>
       <c r="B131" s="22" t="s">
         <v>613</v>
@@ -6512,7 +6513,7 @@
       <c r="M131" s="21"/>
       <c r="N131" s="21"/>
     </row>
-    <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="132" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="21"/>
       <c r="B132" s="22" t="s">
         <v>618</v>
@@ -6542,7 +6543,7 @@
       <c r="M132" s="21"/>
       <c r="N132" s="21"/>
     </row>
-    <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="133" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="21"/>
       <c r="B133" s="22" t="s">
         <v>623</v>
@@ -6572,7 +6573,7 @@
       <c r="M133" s="21"/>
       <c r="N133" s="21"/>
     </row>
-    <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="134" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="21"/>
       <c r="B134" s="22" t="s">
         <v>628</v>
@@ -6602,7 +6603,7 @@
       <c r="M134" s="21"/>
       <c r="N134" s="21"/>
     </row>
-    <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="135" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="21"/>
       <c r="B135" s="22" t="s">
         <v>633</v>
@@ -6632,7 +6633,7 @@
       <c r="M135" s="21"/>
       <c r="N135" s="21"/>
     </row>
-    <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="136" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="21"/>
       <c r="B136" s="22" t="s">
         <v>638</v>
@@ -6662,7 +6663,7 @@
       <c r="M136" s="21"/>
       <c r="N136" s="21"/>
     </row>
-    <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="137" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="21"/>
       <c r="B137" s="22" t="s">
         <v>643</v>
@@ -6692,7 +6693,7 @@
       <c r="M137" s="21"/>
       <c r="N137" s="21"/>
     </row>
-    <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="138" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="21"/>
       <c r="B138" s="22" t="s">
         <v>648</v>
@@ -6722,7 +6723,7 @@
       <c r="M138" s="21"/>
       <c r="N138" s="21"/>
     </row>
-    <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="139" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="21"/>
       <c r="B139" s="22" t="s">
         <v>653</v>
@@ -6752,7 +6753,7 @@
       <c r="M139" s="21"/>
       <c r="N139" s="21"/>
     </row>
-    <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="140" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="21"/>
       <c r="B140" s="22" t="s">
         <v>658</v>
@@ -6782,7 +6783,7 @@
       <c r="M140" s="21"/>
       <c r="N140" s="21"/>
     </row>
-    <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="141" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="21"/>
       <c r="B141" s="22" t="s">
         <v>663</v>
@@ -6812,7 +6813,7 @@
       <c r="M141" s="21"/>
       <c r="N141" s="21"/>
     </row>
-    <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="142" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="21"/>
       <c r="B142" s="22" t="s">
         <v>668</v>
@@ -6842,7 +6843,7 @@
       <c r="M142" s="21"/>
       <c r="N142" s="21"/>
     </row>
-    <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="143" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="21"/>
       <c r="B143" s="22" t="s">
         <v>673</v>
@@ -6872,7 +6873,7 @@
       <c r="M143" s="21"/>
       <c r="N143" s="21"/>
     </row>
-    <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="144" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="21"/>
       <c r="B144" s="22" t="s">
         <v>678</v>
@@ -6902,7 +6903,7 @@
       <c r="M144" s="21"/>
       <c r="N144" s="21"/>
     </row>
-    <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="145" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="21"/>
       <c r="B145" s="22" t="s">
         <v>683</v>
@@ -6932,7 +6933,7 @@
       <c r="M145" s="21"/>
       <c r="N145" s="21"/>
     </row>
-    <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="146" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="21"/>
       <c r="B146" s="22" t="s">
         <v>688</v>
@@ -6962,7 +6963,7 @@
       <c r="M146" s="21"/>
       <c r="N146" s="21"/>
     </row>
-    <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="147" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="21"/>
       <c r="B147" s="22" t="s">
         <v>693</v>
@@ -6992,7 +6993,7 @@
       <c r="M147" s="21"/>
       <c r="N147" s="21"/>
     </row>
-    <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="148" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="21"/>
       <c r="B148" s="22" t="s">
         <v>698</v>
@@ -7022,7 +7023,7 @@
       <c r="M148" s="21"/>
       <c r="N148" s="21"/>
     </row>
-    <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="149" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="21"/>
       <c r="B149" s="22" t="s">
         <v>703</v>
@@ -7052,7 +7053,7 @@
       <c r="M149" s="21"/>
       <c r="N149" s="21"/>
     </row>
-    <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="150" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="21"/>
       <c r="B150" s="22" t="s">
         <v>708</v>
@@ -7082,7 +7083,7 @@
       <c r="M150" s="21"/>
       <c r="N150" s="21"/>
     </row>
-    <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="151" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="21"/>
       <c r="B151" s="22" t="s">
         <v>713</v>
@@ -7112,7 +7113,7 @@
       <c r="M151" s="21"/>
       <c r="N151" s="21"/>
     </row>
-    <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="152" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="21"/>
       <c r="B152" s="22" t="s">
         <v>718</v>
@@ -7142,7 +7143,7 @@
       <c r="M152" s="21"/>
       <c r="N152" s="21"/>
     </row>
-    <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="153" hidden="1" spans="1:15" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="21"/>
       <c r="B153" s="22" t="s">
         <v>723</v>

</xml_diff>

<commit_message>
docs: enforce workbook format stability
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -2646,7 +2646,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -2683,8 +2683,8 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9C0006"/>
-      <sz val="10"/>
+      <color rgb="FF7F0000"/>
+      <sz val="11"/>
       <name val="Carlito"/>
     </font>
     <font>
@@ -2695,6 +2695,12 @@
     <font>
       <b/>
       <color rgb="FF000000"/>
+      <sz val="10"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF9C0006"/>
       <sz val="10"/>
       <name val="Carlito"/>
     </font>
@@ -3005,7 +3011,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3060,72 +3066,75 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3932,40 +3941,40 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17" t="s">
+      <c r="A19" s="20"/>
+      <c r="B19" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="17" t="s">
+      <c r="G19" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17" t="s">
+      <c r="I19" s="20"/>
+      <c r="J19" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M19" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N19" s="17" t="s">
+      <c r="K19" s="20"/>
+      <c r="L19" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M19" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N19" s="20" t="s">
         <v>40</v>
       </c>
     </row>
@@ -4008,28 +4017,28 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17"/>
     </row>
     <row r="22" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A22" s="18"/>
@@ -4176,38 +4185,38 @@
       </c>
     </row>
     <row r="26" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17" t="s">
+      <c r="A26" s="20"/>
+      <c r="B26" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M26" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N26" s="17" t="s">
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M26" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N26" s="20" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4248,28 +4257,28 @@
       </c>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="17"/>
+      <c r="M28" s="17"/>
+      <c r="N28" s="17"/>
     </row>
     <row r="29" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A29" s="18"/>
@@ -4600,38 +4609,38 @@
       </c>
     </row>
     <row r="38" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A38" s="17"/>
-      <c r="B38" s="17" t="s">
+      <c r="A38" s="20"/>
+      <c r="B38" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="C38" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="E38" s="17" t="s">
+      <c r="E38" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="F38" s="17" t="s">
+      <c r="F38" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="G38" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H38" s="17" t="s">
+      <c r="G38" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H38" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M38" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N38" s="17" t="s">
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
+      <c r="L38" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M38" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N38" s="20" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4674,28 +4683,28 @@
       </c>
     </row>
     <row r="40" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="18" t="s">
+      <c r="A40" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="B40" s="19" t="s">
+      <c r="B40" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D40" s="18" t="s">
+      <c r="D40" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
-      <c r="I40" s="18"/>
-      <c r="J40" s="18"/>
-      <c r="K40" s="18"/>
-      <c r="L40" s="18"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="18"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+      <c r="L40" s="17"/>
+      <c r="M40" s="17"/>
+      <c r="N40" s="17"/>
     </row>
     <row r="41" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A41" s="18"/>
@@ -4916,38 +4925,38 @@
       </c>
     </row>
     <row r="47" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A47" s="17"/>
-      <c r="B47" s="17" t="s">
+      <c r="A47" s="20"/>
+      <c r="B47" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="C47" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D47" s="17" t="s">
+      <c r="D47" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="E47" s="17" t="s">
+      <c r="E47" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="F47" s="17" t="s">
+      <c r="F47" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="G47" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H47" s="17" t="s">
+      <c r="G47" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" s="20" t="s">
         <v>234</v>
       </c>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M47" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N47" s="17" t="s">
+      <c r="I47" s="20"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
+      <c r="L47" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M47" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N47" s="20" t="s">
         <v>203</v>
       </c>
     </row>
@@ -4988,28 +4997,28 @@
       </c>
     </row>
     <row r="49" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="B49" s="19" t="s">
+      <c r="B49" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="C49" s="18" t="s">
+      <c r="C49" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D49" s="18" t="s">
+      <c r="D49" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E49" s="18"/>
-      <c r="F49" s="18"/>
-      <c r="G49" s="18"/>
-      <c r="H49" s="18"/>
-      <c r="I49" s="18"/>
-      <c r="J49" s="18"/>
-      <c r="K49" s="18"/>
-      <c r="L49" s="18"/>
-      <c r="M49" s="18"/>
-      <c r="N49" s="18"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="17"/>
+      <c r="L49" s="17"/>
+      <c r="M49" s="17"/>
+      <c r="N49" s="17"/>
     </row>
     <row r="50" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A50" s="18"/>
@@ -5268,38 +5277,38 @@
       </c>
     </row>
     <row r="57" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A57" s="17"/>
-      <c r="B57" s="17" t="s">
+      <c r="A57" s="20"/>
+      <c r="B57" s="20" t="s">
         <v>278</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D57" s="17" t="s">
+      <c r="D57" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="E57" s="17" t="s">
+      <c r="E57" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="F57" s="17" t="s">
+      <c r="F57" s="20" t="s">
         <v>281</v>
       </c>
-      <c r="G57" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H57" s="17" t="s">
+      <c r="G57" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="20" t="s">
         <v>282</v>
       </c>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M57" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N57" s="17" t="s">
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
+      <c r="L57" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M57" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N57" s="20" t="s">
         <v>203</v>
       </c>
     </row>
@@ -5342,28 +5351,28 @@
       </c>
     </row>
     <row r="59" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="17" t="s">
         <v>288</v>
       </c>
-      <c r="B59" s="19" t="s">
+      <c r="B59" s="17" t="s">
         <v>289</v>
       </c>
-      <c r="C59" s="18" t="s">
+      <c r="C59" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D59" s="18" t="s">
+      <c r="D59" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="18"/>
-      <c r="H59" s="18"/>
-      <c r="I59" s="18"/>
-      <c r="J59" s="18"/>
-      <c r="K59" s="18"/>
-      <c r="L59" s="18"/>
-      <c r="M59" s="18"/>
-      <c r="N59" s="18"/>
+      <c r="E59" s="17"/>
+      <c r="F59" s="17"/>
+      <c r="G59" s="17"/>
+      <c r="H59" s="17"/>
+      <c r="I59" s="17"/>
+      <c r="J59" s="17"/>
+      <c r="K59" s="17"/>
+      <c r="L59" s="17"/>
+      <c r="M59" s="17"/>
+      <c r="N59" s="17"/>
     </row>
     <row r="60" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A60" s="18"/>
@@ -5804,40 +5813,40 @@
       </c>
     </row>
     <row r="72" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A72" s="17"/>
-      <c r="B72" s="17" t="s">
+      <c r="A72" s="20"/>
+      <c r="B72" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="C72" s="17" t="s">
+      <c r="C72" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D72" s="17" t="s">
+      <c r="D72" s="20" t="s">
         <v>355</v>
       </c>
-      <c r="E72" s="17" t="s">
+      <c r="E72" s="20" t="s">
         <v>356</v>
       </c>
-      <c r="F72" s="17" t="s">
+      <c r="F72" s="20" t="s">
         <v>357</v>
       </c>
-      <c r="G72" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H72" s="17" t="s">
+      <c r="G72" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H72" s="20" t="s">
         <v>358</v>
       </c>
-      <c r="I72" s="17"/>
-      <c r="J72" s="17" t="s">
+      <c r="I72" s="20"/>
+      <c r="J72" s="20" t="s">
         <v>359</v>
       </c>
-      <c r="K72" s="17"/>
-      <c r="L72" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M72" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N72" s="17" t="s">
+      <c r="K72" s="20"/>
+      <c r="L72" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M72" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N72" s="20" t="s">
         <v>295</v>
       </c>
     </row>
@@ -6314,28 +6323,28 @@
       </c>
     </row>
     <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A86" s="19" t="s">
+      <c r="A86" s="17" t="s">
         <v>424</v>
       </c>
-      <c r="B86" s="19" t="s">
+      <c r="B86" s="17" t="s">
         <v>425</v>
       </c>
-      <c r="C86" s="19" t="s">
+      <c r="C86" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D86" s="19" t="s">
+      <c r="D86" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E86" s="19"/>
-      <c r="F86" s="19"/>
-      <c r="G86" s="19"/>
-      <c r="H86" s="19"/>
-      <c r="I86" s="19"/>
-      <c r="J86" s="19"/>
-      <c r="K86" s="19"/>
-      <c r="L86" s="19"/>
-      <c r="M86" s="19"/>
-      <c r="N86" s="19"/>
+      <c r="E86" s="17"/>
+      <c r="F86" s="17"/>
+      <c r="G86" s="17"/>
+      <c r="H86" s="17"/>
+      <c r="I86" s="17"/>
+      <c r="J86" s="17"/>
+      <c r="K86" s="17"/>
+      <c r="L86" s="17"/>
+      <c r="M86" s="17"/>
+      <c r="N86" s="17"/>
     </row>
     <row r="87" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
@@ -6482,40 +6491,40 @@
       </c>
     </row>
     <row r="91" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A91" s="17"/>
-      <c r="B91" s="17" t="s">
+      <c r="A91" s="20"/>
+      <c r="B91" s="20" t="s">
         <v>446</v>
       </c>
-      <c r="C91" s="17" t="s">
+      <c r="C91" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D91" s="17" t="s">
+      <c r="D91" s="20" t="s">
         <v>447</v>
       </c>
-      <c r="E91" s="17" t="s">
+      <c r="E91" s="20" t="s">
         <v>448</v>
       </c>
-      <c r="F91" s="17" t="s">
+      <c r="F91" s="20" t="s">
         <v>449</v>
       </c>
-      <c r="G91" s="17" t="s">
+      <c r="G91" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="H91" s="17" t="s">
+      <c r="H91" s="20" t="s">
         <v>450</v>
       </c>
-      <c r="I91" s="17"/>
-      <c r="J91" s="17" t="s">
+      <c r="I91" s="20"/>
+      <c r="J91" s="20" t="s">
         <v>451</v>
       </c>
-      <c r="K91" s="17"/>
-      <c r="L91" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M91" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N91" s="17" t="s">
+      <c r="K91" s="20"/>
+      <c r="L91" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M91" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N91" s="20" t="s">
         <v>452</v>
       </c>
     </row>
@@ -6780,62 +6789,62 @@
       </c>
     </row>
     <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A99" s="18" t="s">
+      <c r="A99" s="17" t="s">
         <v>488</v>
       </c>
-      <c r="B99" s="19" t="s">
+      <c r="B99" s="17" t="s">
         <v>489</v>
       </c>
-      <c r="C99" s="18" t="s">
+      <c r="C99" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D99" s="18" t="s">
+      <c r="D99" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E99" s="18"/>
-      <c r="F99" s="18"/>
-      <c r="G99" s="18"/>
-      <c r="H99" s="18"/>
-      <c r="I99" s="18"/>
-      <c r="J99" s="18"/>
-      <c r="K99" s="18"/>
-      <c r="L99" s="18"/>
-      <c r="M99" s="18"/>
-      <c r="N99" s="18"/>
+      <c r="E99" s="17"/>
+      <c r="F99" s="17"/>
+      <c r="G99" s="17"/>
+      <c r="H99" s="17"/>
+      <c r="I99" s="17"/>
+      <c r="J99" s="17"/>
+      <c r="K99" s="17"/>
+      <c r="L99" s="17"/>
+      <c r="M99" s="17"/>
+      <c r="N99" s="17"/>
     </row>
     <row r="100" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A100" s="17"/>
-      <c r="B100" s="17" t="s">
+      <c r="A100" s="20"/>
+      <c r="B100" s="20" t="s">
         <v>490</v>
       </c>
-      <c r="C100" s="17" t="s">
+      <c r="C100" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D100" s="17" t="s">
+      <c r="D100" s="20" t="s">
         <v>491</v>
       </c>
-      <c r="E100" s="17" t="s">
+      <c r="E100" s="20" t="s">
         <v>492</v>
       </c>
-      <c r="F100" s="17" t="s">
+      <c r="F100" s="20" t="s">
         <v>493</v>
       </c>
-      <c r="G100" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H100" s="17" t="s">
+      <c r="G100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H100" s="20" t="s">
         <v>494</v>
       </c>
-      <c r="I100" s="17"/>
-      <c r="J100" s="17"/>
-      <c r="K100" s="17"/>
-      <c r="L100" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M100" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N100" s="17" t="s">
+      <c r="I100" s="20"/>
+      <c r="J100" s="20"/>
+      <c r="K100" s="20"/>
+      <c r="L100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M100" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N100" s="20" t="s">
         <v>495</v>
       </c>
     </row>
@@ -7382,1418 +7391,1418 @@
       </c>
     </row>
     <row r="116" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A116" s="17"/>
-      <c r="B116" s="17" t="s">
+      <c r="A116" s="20"/>
+      <c r="B116" s="20" t="s">
         <v>571</v>
       </c>
-      <c r="C116" s="17" t="s">
+      <c r="C116" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="D116" s="17" t="s">
+      <c r="D116" s="20" t="s">
         <v>572</v>
       </c>
-      <c r="E116" s="17" t="s">
+      <c r="E116" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="F116" s="17" t="s">
+      <c r="F116" s="20" t="s">
         <v>574</v>
       </c>
-      <c r="G116" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="H116" s="17" t="s">
+      <c r="G116" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H116" s="20" t="s">
         <v>575</v>
       </c>
-      <c r="I116" s="17"/>
-      <c r="J116" s="17" t="s">
+      <c r="I116" s="20"/>
+      <c r="J116" s="20" t="s">
         <v>560</v>
       </c>
-      <c r="K116" s="17"/>
-      <c r="L116" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M116" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="N116" s="17" t="s">
+      <c r="K116" s="20"/>
+      <c r="L116" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M116" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N116" s="20" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="117" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A117" s="20"/>
-      <c r="B117" s="20" t="s">
+      <c r="A117" s="21"/>
+      <c r="B117" s="21" t="s">
         <v>576</v>
       </c>
-      <c r="C117" s="20" t="s">
+      <c r="C117" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D117" s="20" t="s">
+      <c r="D117" s="21" t="s">
         <v>577</v>
       </c>
-      <c r="E117" s="20" t="s">
+      <c r="E117" s="21" t="s">
         <v>578</v>
       </c>
-      <c r="F117" s="20" t="s">
+      <c r="F117" s="21" t="s">
         <v>579</v>
       </c>
-      <c r="G117" s="20" t="s">
+      <c r="G117" s="21" t="s">
         <v>415</v>
       </c>
-      <c r="H117" s="20" t="s">
+      <c r="H117" s="21" t="s">
         <v>580</v>
       </c>
-      <c r="I117" s="20"/>
-      <c r="J117" s="20" t="s">
+      <c r="I117" s="21"/>
+      <c r="J117" s="21" t="s">
         <v>560</v>
       </c>
-      <c r="K117" s="20"/>
-      <c r="L117" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M117" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N117" s="20" t="s">
+      <c r="K117" s="21"/>
+      <c r="L117" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M117" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N117" s="21" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A118" s="20" t="s">
+      <c r="A118" s="17" t="s">
         <v>581</v>
       </c>
-      <c r="B118" s="20" t="s">
+      <c r="B118" s="17" t="s">
         <v>582</v>
       </c>
-      <c r="C118" s="20" t="s">
+      <c r="C118" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D118" s="20" t="s">
+      <c r="D118" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E118" s="20"/>
-      <c r="F118" s="20"/>
-      <c r="G118" s="20"/>
-      <c r="H118" s="20"/>
-      <c r="I118" s="20"/>
-      <c r="J118" s="20"/>
-      <c r="K118" s="20"/>
-      <c r="L118" s="20"/>
-      <c r="M118" s="20"/>
-      <c r="N118" s="20"/>
+      <c r="E118" s="17"/>
+      <c r="F118" s="17"/>
+      <c r="G118" s="17"/>
+      <c r="H118" s="17"/>
+      <c r="I118" s="17"/>
+      <c r="J118" s="17"/>
+      <c r="K118" s="17"/>
+      <c r="L118" s="17"/>
+      <c r="M118" s="17"/>
+      <c r="N118" s="17"/>
     </row>
     <row r="119" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A119" s="20"/>
-      <c r="B119" s="20" t="s">
+      <c r="A119" s="21"/>
+      <c r="B119" s="21" t="s">
         <v>583</v>
       </c>
-      <c r="C119" s="20" t="s">
+      <c r="C119" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D119" s="20" t="s">
+      <c r="D119" s="21" t="s">
         <v>584</v>
       </c>
-      <c r="E119" s="20" t="s">
+      <c r="E119" s="21" t="s">
         <v>585</v>
       </c>
-      <c r="F119" s="20" t="s">
+      <c r="F119" s="21" t="s">
         <v>586</v>
       </c>
-      <c r="G119" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H119" s="20" t="s">
+      <c r="G119" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H119" s="21" t="s">
         <v>587</v>
       </c>
-      <c r="I119" s="20"/>
-      <c r="J119" s="20" t="s">
+      <c r="I119" s="21"/>
+      <c r="J119" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K119" s="20"/>
-      <c r="L119" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M119" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N119" s="20" t="s">
+      <c r="K119" s="21"/>
+      <c r="L119" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M119" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N119" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="120" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A120" s="20"/>
-      <c r="B120" s="20" t="s">
+      <c r="A120" s="21"/>
+      <c r="B120" s="21" t="s">
         <v>590</v>
       </c>
-      <c r="C120" s="20" t="s">
+      <c r="C120" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D120" s="20" t="s">
+      <c r="D120" s="21" t="s">
         <v>591</v>
       </c>
-      <c r="E120" s="20" t="s">
+      <c r="E120" s="21" t="s">
         <v>592</v>
       </c>
-      <c r="F120" s="20" t="s">
+      <c r="F120" s="21" t="s">
         <v>593</v>
       </c>
-      <c r="G120" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H120" s="20" t="s">
+      <c r="G120" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H120" s="21" t="s">
         <v>594</v>
       </c>
-      <c r="I120" s="20"/>
-      <c r="J120" s="20" t="s">
+      <c r="I120" s="21"/>
+      <c r="J120" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K120" s="20"/>
-      <c r="L120" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M120" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N120" s="20" t="s">
+      <c r="K120" s="21"/>
+      <c r="L120" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M120" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N120" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="121" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A121" s="20"/>
-      <c r="B121" s="20" t="s">
+      <c r="A121" s="21"/>
+      <c r="B121" s="21" t="s">
         <v>595</v>
       </c>
-      <c r="C121" s="20" t="s">
+      <c r="C121" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D121" s="20" t="s">
+      <c r="D121" s="21" t="s">
         <v>596</v>
       </c>
-      <c r="E121" s="20" t="s">
+      <c r="E121" s="21" t="s">
         <v>597</v>
       </c>
-      <c r="F121" s="20" t="s">
+      <c r="F121" s="21" t="s">
         <v>598</v>
       </c>
-      <c r="G121" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H121" s="20" t="s">
+      <c r="G121" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H121" s="21" t="s">
         <v>599</v>
       </c>
-      <c r="I121" s="20"/>
-      <c r="J121" s="20" t="s">
+      <c r="I121" s="21"/>
+      <c r="J121" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K121" s="20"/>
-      <c r="L121" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M121" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N121" s="20" t="s">
+      <c r="K121" s="21"/>
+      <c r="L121" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M121" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N121" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="122" ht="24" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A122" s="20"/>
-      <c r="B122" s="20" t="s">
+      <c r="A122" s="21"/>
+      <c r="B122" s="21" t="s">
         <v>600</v>
       </c>
-      <c r="C122" s="20" t="s">
+      <c r="C122" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D122" s="20" t="s">
+      <c r="D122" s="21" t="s">
         <v>601</v>
       </c>
-      <c r="E122" s="20" t="s">
+      <c r="E122" s="21" t="s">
         <v>602</v>
       </c>
-      <c r="F122" s="20" t="s">
+      <c r="F122" s="21" t="s">
         <v>603</v>
       </c>
-      <c r="G122" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H122" s="20" t="s">
+      <c r="G122" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H122" s="21" t="s">
         <v>604</v>
       </c>
-      <c r="I122" s="20"/>
-      <c r="J122" s="20" t="s">
+      <c r="I122" s="21"/>
+      <c r="J122" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K122" s="20"/>
-      <c r="L122" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M122" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N122" s="20" t="s">
+      <c r="K122" s="21"/>
+      <c r="L122" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M122" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N122" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="123" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A123" s="20"/>
-      <c r="B123" s="20" t="s">
+      <c r="A123" s="21"/>
+      <c r="B123" s="21" t="s">
         <v>605</v>
       </c>
-      <c r="C123" s="20" t="s">
+      <c r="C123" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D123" s="20" t="s">
+      <c r="D123" s="21" t="s">
         <v>606</v>
       </c>
-      <c r="E123" s="20" t="s">
+      <c r="E123" s="21" t="s">
         <v>607</v>
       </c>
-      <c r="F123" s="20" t="s">
+      <c r="F123" s="21" t="s">
         <v>608</v>
       </c>
-      <c r="G123" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H123" s="20" t="s">
+      <c r="G123" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H123" s="21" t="s">
         <v>609</v>
       </c>
-      <c r="I123" s="20"/>
-      <c r="J123" s="20" t="s">
+      <c r="I123" s="21"/>
+      <c r="J123" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K123" s="20"/>
-      <c r="L123" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M123" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N123" s="20" t="s">
+      <c r="K123" s="21"/>
+      <c r="L123" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M123" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N123" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="124" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A124" s="20"/>
-      <c r="B124" s="20" t="s">
+      <c r="A124" s="21"/>
+      <c r="B124" s="21" t="s">
         <v>610</v>
       </c>
-      <c r="C124" s="20" t="s">
+      <c r="C124" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D124" s="20" t="s">
+      <c r="D124" s="21" t="s">
         <v>611</v>
       </c>
-      <c r="E124" s="20" t="s">
+      <c r="E124" s="21" t="s">
         <v>612</v>
       </c>
-      <c r="F124" s="20" t="s">
+      <c r="F124" s="21" t="s">
         <v>613</v>
       </c>
-      <c r="G124" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H124" s="20" t="s">
+      <c r="G124" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H124" s="21" t="s">
         <v>614</v>
       </c>
-      <c r="I124" s="20"/>
-      <c r="J124" s="20" t="s">
+      <c r="I124" s="21"/>
+      <c r="J124" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K124" s="20"/>
-      <c r="L124" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M124" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N124" s="20" t="s">
+      <c r="K124" s="21"/>
+      <c r="L124" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M124" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N124" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="125" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A125" s="20"/>
-      <c r="B125" s="20" t="s">
+      <c r="A125" s="21"/>
+      <c r="B125" s="21" t="s">
         <v>615</v>
       </c>
-      <c r="C125" s="20" t="s">
+      <c r="C125" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D125" s="20" t="s">
+      <c r="D125" s="21" t="s">
         <v>616</v>
       </c>
-      <c r="E125" s="20" t="s">
+      <c r="E125" s="21" t="s">
         <v>617</v>
       </c>
-      <c r="F125" s="20" t="s">
+      <c r="F125" s="21" t="s">
         <v>618</v>
       </c>
-      <c r="G125" s="20" t="s">
+      <c r="G125" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="H125" s="20" t="s">
+      <c r="H125" s="21" t="s">
         <v>619</v>
       </c>
-      <c r="I125" s="20"/>
-      <c r="J125" s="20" t="s">
+      <c r="I125" s="21"/>
+      <c r="J125" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K125" s="20"/>
-      <c r="L125" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M125" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N125" s="20" t="s">
+      <c r="K125" s="21"/>
+      <c r="L125" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M125" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N125" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="126" ht="60" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A126" s="20"/>
-      <c r="B126" s="20" t="s">
+      <c r="A126" s="21"/>
+      <c r="B126" s="21" t="s">
         <v>620</v>
       </c>
-      <c r="C126" s="20" t="s">
+      <c r="C126" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D126" s="20" t="s">
+      <c r="D126" s="21" t="s">
         <v>621</v>
       </c>
-      <c r="E126" s="20" t="s">
+      <c r="E126" s="21" t="s">
         <v>622</v>
       </c>
-      <c r="F126" s="20" t="s">
+      <c r="F126" s="21" t="s">
         <v>623</v>
       </c>
-      <c r="G126" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H126" s="20" t="s">
+      <c r="G126" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H126" s="21" t="s">
         <v>624</v>
       </c>
-      <c r="I126" s="20"/>
-      <c r="J126" s="20" t="s">
+      <c r="I126" s="21"/>
+      <c r="J126" s="21" t="s">
         <v>588</v>
       </c>
-      <c r="K126" s="20"/>
-      <c r="L126" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M126" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N126" s="20" t="s">
+      <c r="K126" s="21"/>
+      <c r="L126" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M126" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N126" s="21" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A127" s="20" t="s">
+      <c r="A127" s="17" t="s">
         <v>625</v>
       </c>
-      <c r="B127" s="20" t="s">
+      <c r="B127" s="17" t="s">
         <v>626</v>
       </c>
-      <c r="C127" s="20" t="s">
+      <c r="C127" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="D127" s="20" t="s">
+      <c r="D127" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E127" s="20"/>
-      <c r="F127" s="20"/>
-      <c r="G127" s="20"/>
-      <c r="H127" s="20"/>
-      <c r="I127" s="20"/>
-      <c r="J127" s="20"/>
-      <c r="K127" s="20"/>
-      <c r="L127" s="20"/>
-      <c r="M127" s="20"/>
-      <c r="N127" s="20"/>
+      <c r="E127" s="17"/>
+      <c r="F127" s="17"/>
+      <c r="G127" s="17"/>
+      <c r="H127" s="17"/>
+      <c r="I127" s="17"/>
+      <c r="J127" s="17"/>
+      <c r="K127" s="17"/>
+      <c r="L127" s="17"/>
+      <c r="M127" s="17"/>
+      <c r="N127" s="17"/>
     </row>
     <row r="128" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A128" s="20"/>
-      <c r="B128" s="20" t="s">
+      <c r="A128" s="21"/>
+      <c r="B128" s="21" t="s">
         <v>627</v>
       </c>
-      <c r="C128" s="20" t="s">
+      <c r="C128" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D128" s="20" t="s">
+      <c r="D128" s="21" t="s">
         <v>628</v>
       </c>
-      <c r="E128" s="20" t="s">
+      <c r="E128" s="21" t="s">
         <v>629</v>
       </c>
-      <c r="F128" s="20" t="s">
+      <c r="F128" s="21" t="s">
         <v>630</v>
       </c>
-      <c r="G128" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H128" s="20" t="s">
+      <c r="G128" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H128" s="21" t="s">
         <v>631</v>
       </c>
-      <c r="I128" s="20"/>
-      <c r="J128" s="20" t="s">
+      <c r="I128" s="21"/>
+      <c r="J128" s="21" t="s">
         <v>632</v>
       </c>
-      <c r="K128" s="20"/>
-      <c r="L128" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="M128" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="N128" s="20" t="s">
+      <c r="K128" s="21"/>
+      <c r="L128" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M128" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N128" s="21" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A129" s="21"/>
-      <c r="B129" s="22" t="s">
+      <c r="A129" s="22"/>
+      <c r="B129" s="23" t="s">
         <v>634</v>
       </c>
-      <c r="C129" s="21" t="s">
+      <c r="C129" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D129" s="21" t="s">
+      <c r="D129" s="22" t="s">
         <v>635</v>
       </c>
-      <c r="E129" s="21" t="s">
+      <c r="E129" s="22" t="s">
         <v>636</v>
       </c>
-      <c r="F129" s="21" t="s">
+      <c r="F129" s="22" t="s">
         <v>637</v>
       </c>
-      <c r="G129" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H129" s="21" t="s">
+      <c r="G129" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H129" s="22" t="s">
         <v>638</v>
       </c>
-      <c r="I129" s="21"/>
-      <c r="J129" s="21" t="s">
+      <c r="I129" s="22"/>
+      <c r="J129" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K129" s="21"/>
-      <c r="L129" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M129" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N129" s="21" t="s">
+      <c r="K129" s="22"/>
+      <c r="L129" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M129" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N129" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A130" s="21"/>
-      <c r="B130" s="22" t="s">
+      <c r="A130" s="22"/>
+      <c r="B130" s="23" t="s">
         <v>639</v>
       </c>
-      <c r="C130" s="21" t="s">
+      <c r="C130" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D130" s="21" t="s">
+      <c r="D130" s="22" t="s">
         <v>640</v>
       </c>
-      <c r="E130" s="21" t="s">
+      <c r="E130" s="22" t="s">
         <v>641</v>
       </c>
-      <c r="F130" s="21" t="s">
+      <c r="F130" s="22" t="s">
         <v>642</v>
       </c>
-      <c r="G130" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H130" s="21" t="s">
+      <c r="G130" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H130" s="22" t="s">
         <v>643</v>
       </c>
-      <c r="I130" s="21"/>
-      <c r="J130" s="21" t="s">
+      <c r="I130" s="22"/>
+      <c r="J130" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K130" s="21"/>
-      <c r="L130" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M130" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N130" s="21" t="s">
+      <c r="K130" s="22"/>
+      <c r="L130" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M130" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N130" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A131" s="21"/>
-      <c r="B131" s="22" t="s">
+      <c r="A131" s="22"/>
+      <c r="B131" s="23" t="s">
         <v>644</v>
       </c>
-      <c r="C131" s="21" t="s">
+      <c r="C131" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D131" s="21" t="s">
+      <c r="D131" s="22" t="s">
         <v>645</v>
       </c>
-      <c r="E131" s="21" t="s">
+      <c r="E131" s="22" t="s">
         <v>646</v>
       </c>
-      <c r="F131" s="21" t="s">
+      <c r="F131" s="22" t="s">
         <v>647</v>
       </c>
-      <c r="G131" s="21" t="s">
+      <c r="G131" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H131" s="21" t="s">
+      <c r="H131" s="22" t="s">
         <v>648</v>
       </c>
-      <c r="I131" s="21"/>
-      <c r="J131" s="21" t="s">
+      <c r="I131" s="22"/>
+      <c r="J131" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K131" s="21"/>
-      <c r="L131" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M131" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N131" s="21" t="s">
+      <c r="K131" s="22"/>
+      <c r="L131" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M131" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N131" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A132" s="21"/>
-      <c r="B132" s="22" t="s">
+      <c r="A132" s="22"/>
+      <c r="B132" s="23" t="s">
         <v>649</v>
       </c>
-      <c r="C132" s="21" t="s">
+      <c r="C132" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D132" s="21" t="s">
+      <c r="D132" s="22" t="s">
         <v>650</v>
       </c>
-      <c r="E132" s="21" t="s">
+      <c r="E132" s="22" t="s">
         <v>651</v>
       </c>
-      <c r="F132" s="21" t="s">
+      <c r="F132" s="22" t="s">
         <v>652</v>
       </c>
-      <c r="G132" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H132" s="21" t="s">
+      <c r="G132" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H132" s="22" t="s">
         <v>653</v>
       </c>
-      <c r="I132" s="21"/>
-      <c r="J132" s="21" t="s">
+      <c r="I132" s="22"/>
+      <c r="J132" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K132" s="21"/>
-      <c r="L132" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M132" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N132" s="21" t="s">
+      <c r="K132" s="22"/>
+      <c r="L132" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M132" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N132" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A133" s="21"/>
-      <c r="B133" s="22" t="s">
+      <c r="A133" s="22"/>
+      <c r="B133" s="23" t="s">
         <v>654</v>
       </c>
-      <c r="C133" s="21" t="s">
+      <c r="C133" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D133" s="21" t="s">
+      <c r="D133" s="22" t="s">
         <v>655</v>
       </c>
-      <c r="E133" s="21" t="s">
+      <c r="E133" s="22" t="s">
         <v>656</v>
       </c>
-      <c r="F133" s="21" t="s">
+      <c r="F133" s="22" t="s">
         <v>657</v>
       </c>
-      <c r="G133" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H133" s="21" t="s">
+      <c r="G133" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H133" s="22" t="s">
         <v>658</v>
       </c>
-      <c r="I133" s="21"/>
-      <c r="J133" s="21" t="s">
+      <c r="I133" s="22"/>
+      <c r="J133" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K133" s="21"/>
-      <c r="L133" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M133" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N133" s="21" t="s">
+      <c r="K133" s="22"/>
+      <c r="L133" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M133" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N133" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A134" s="21"/>
-      <c r="B134" s="22" t="s">
+      <c r="A134" s="22"/>
+      <c r="B134" s="23" t="s">
         <v>659</v>
       </c>
-      <c r="C134" s="21" t="s">
+      <c r="C134" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D134" s="21" t="s">
+      <c r="D134" s="22" t="s">
         <v>660</v>
       </c>
-      <c r="E134" s="21" t="s">
+      <c r="E134" s="22" t="s">
         <v>661</v>
       </c>
-      <c r="F134" s="21" t="s">
+      <c r="F134" s="22" t="s">
         <v>662</v>
       </c>
-      <c r="G134" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H134" s="21" t="s">
+      <c r="G134" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H134" s="22" t="s">
         <v>663</v>
       </c>
-      <c r="I134" s="21"/>
-      <c r="J134" s="21" t="s">
+      <c r="I134" s="22"/>
+      <c r="J134" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K134" s="21"/>
-      <c r="L134" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M134" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N134" s="21" t="s">
+      <c r="K134" s="22"/>
+      <c r="L134" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M134" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N134" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A135" s="21"/>
-      <c r="B135" s="22" t="s">
+      <c r="A135" s="22"/>
+      <c r="B135" s="23" t="s">
         <v>664</v>
       </c>
-      <c r="C135" s="21" t="s">
+      <c r="C135" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D135" s="21" t="s">
+      <c r="D135" s="22" t="s">
         <v>665</v>
       </c>
-      <c r="E135" s="21" t="s">
+      <c r="E135" s="22" t="s">
         <v>666</v>
       </c>
-      <c r="F135" s="21" t="s">
+      <c r="F135" s="22" t="s">
         <v>667</v>
       </c>
-      <c r="G135" s="21" t="s">
+      <c r="G135" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H135" s="21" t="s">
+      <c r="H135" s="22" t="s">
         <v>668</v>
       </c>
-      <c r="I135" s="21"/>
-      <c r="J135" s="21" t="s">
+      <c r="I135" s="22"/>
+      <c r="J135" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K135" s="21"/>
-      <c r="L135" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M135" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N135" s="21" t="s">
+      <c r="K135" s="22"/>
+      <c r="L135" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M135" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N135" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A136" s="21"/>
-      <c r="B136" s="22" t="s">
+      <c r="A136" s="22"/>
+      <c r="B136" s="23" t="s">
         <v>669</v>
       </c>
-      <c r="C136" s="21" t="s">
+      <c r="C136" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D136" s="21" t="s">
+      <c r="D136" s="22" t="s">
         <v>670</v>
       </c>
-      <c r="E136" s="21" t="s">
+      <c r="E136" s="22" t="s">
         <v>671</v>
       </c>
-      <c r="F136" s="21" t="s">
+      <c r="F136" s="22" t="s">
         <v>672</v>
       </c>
-      <c r="G136" s="21" t="s">
+      <c r="G136" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H136" s="21" t="s">
+      <c r="H136" s="22" t="s">
         <v>673</v>
       </c>
-      <c r="I136" s="21"/>
-      <c r="J136" s="21" t="s">
+      <c r="I136" s="22"/>
+      <c r="J136" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K136" s="21"/>
-      <c r="L136" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M136" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N136" s="21" t="s">
+      <c r="K136" s="22"/>
+      <c r="L136" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M136" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N136" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A137" s="21"/>
-      <c r="B137" s="22" t="s">
+      <c r="A137" s="22"/>
+      <c r="B137" s="23" t="s">
         <v>674</v>
       </c>
-      <c r="C137" s="21" t="s">
+      <c r="C137" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D137" s="21" t="s">
+      <c r="D137" s="22" t="s">
         <v>675</v>
       </c>
-      <c r="E137" s="21" t="s">
+      <c r="E137" s="22" t="s">
         <v>676</v>
       </c>
-      <c r="F137" s="21" t="s">
+      <c r="F137" s="22" t="s">
         <v>677</v>
       </c>
-      <c r="G137" s="21" t="s">
+      <c r="G137" s="22" t="s">
         <v>415</v>
       </c>
-      <c r="H137" s="21" t="s">
+      <c r="H137" s="22" t="s">
         <v>678</v>
       </c>
-      <c r="I137" s="21"/>
-      <c r="J137" s="21" t="s">
+      <c r="I137" s="22"/>
+      <c r="J137" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K137" s="21"/>
-      <c r="L137" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M137" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N137" s="21" t="s">
+      <c r="K137" s="22"/>
+      <c r="L137" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M137" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N137" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A138" s="21"/>
-      <c r="B138" s="22" t="s">
+      <c r="A138" s="22"/>
+      <c r="B138" s="23" t="s">
         <v>679</v>
       </c>
-      <c r="C138" s="21" t="s">
+      <c r="C138" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D138" s="21" t="s">
+      <c r="D138" s="22" t="s">
         <v>680</v>
       </c>
-      <c r="E138" s="21" t="s">
+      <c r="E138" s="22" t="s">
         <v>681</v>
       </c>
-      <c r="F138" s="21" t="s">
+      <c r="F138" s="22" t="s">
         <v>682</v>
       </c>
-      <c r="G138" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H138" s="21" t="s">
+      <c r="G138" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H138" s="22" t="s">
         <v>683</v>
       </c>
-      <c r="I138" s="21"/>
-      <c r="J138" s="21" t="s">
+      <c r="I138" s="22"/>
+      <c r="J138" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K138" s="21"/>
-      <c r="L138" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M138" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N138" s="21" t="s">
+      <c r="K138" s="22"/>
+      <c r="L138" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M138" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N138" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A139" s="21"/>
-      <c r="B139" s="22" t="s">
+      <c r="A139" s="22"/>
+      <c r="B139" s="23" t="s">
         <v>684</v>
       </c>
-      <c r="C139" s="21" t="s">
+      <c r="C139" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D139" s="21" t="s">
+      <c r="D139" s="22" t="s">
         <v>685</v>
       </c>
-      <c r="E139" s="21" t="s">
+      <c r="E139" s="22" t="s">
         <v>686</v>
       </c>
-      <c r="F139" s="21" t="s">
+      <c r="F139" s="22" t="s">
         <v>687</v>
       </c>
-      <c r="G139" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H139" s="21" t="s">
+      <c r="G139" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H139" s="22" t="s">
         <v>688</v>
       </c>
-      <c r="I139" s="21"/>
-      <c r="J139" s="21" t="s">
+      <c r="I139" s="22"/>
+      <c r="J139" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K139" s="21"/>
-      <c r="L139" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M139" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N139" s="21" t="s">
+      <c r="K139" s="22"/>
+      <c r="L139" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M139" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N139" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A140" s="21"/>
-      <c r="B140" s="22" t="s">
+      <c r="A140" s="22"/>
+      <c r="B140" s="23" t="s">
         <v>689</v>
       </c>
-      <c r="C140" s="21" t="s">
+      <c r="C140" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D140" s="21" t="s">
+      <c r="D140" s="22" t="s">
         <v>690</v>
       </c>
-      <c r="E140" s="21" t="s">
+      <c r="E140" s="22" t="s">
         <v>691</v>
       </c>
-      <c r="F140" s="21" t="s">
+      <c r="F140" s="22" t="s">
         <v>692</v>
       </c>
-      <c r="G140" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H140" s="21" t="s">
+      <c r="G140" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H140" s="22" t="s">
         <v>693</v>
       </c>
-      <c r="I140" s="21"/>
-      <c r="J140" s="21" t="s">
+      <c r="I140" s="22"/>
+      <c r="J140" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K140" s="21"/>
-      <c r="L140" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M140" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N140" s="21" t="s">
+      <c r="K140" s="22"/>
+      <c r="L140" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M140" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N140" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A141" s="21"/>
-      <c r="B141" s="22" t="s">
+      <c r="A141" s="22"/>
+      <c r="B141" s="23" t="s">
         <v>694</v>
       </c>
-      <c r="C141" s="21" t="s">
+      <c r="C141" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D141" s="21" t="s">
+      <c r="D141" s="22" t="s">
         <v>695</v>
       </c>
-      <c r="E141" s="21" t="s">
+      <c r="E141" s="22" t="s">
         <v>696</v>
       </c>
-      <c r="F141" s="21" t="s">
+      <c r="F141" s="22" t="s">
         <v>697</v>
       </c>
-      <c r="G141" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H141" s="21" t="s">
+      <c r="G141" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H141" s="22" t="s">
         <v>698</v>
       </c>
-      <c r="I141" s="21"/>
-      <c r="J141" s="21" t="s">
+      <c r="I141" s="22"/>
+      <c r="J141" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K141" s="21"/>
-      <c r="L141" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M141" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N141" s="21" t="s">
+      <c r="K141" s="22"/>
+      <c r="L141" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M141" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N141" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A142" s="21"/>
-      <c r="B142" s="22" t="s">
+      <c r="A142" s="22"/>
+      <c r="B142" s="23" t="s">
         <v>699</v>
       </c>
-      <c r="C142" s="21" t="s">
+      <c r="C142" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D142" s="21" t="s">
+      <c r="D142" s="22" t="s">
         <v>700</v>
       </c>
-      <c r="E142" s="21" t="s">
+      <c r="E142" s="22" t="s">
         <v>701</v>
       </c>
-      <c r="F142" s="21" t="s">
+      <c r="F142" s="22" t="s">
         <v>702</v>
       </c>
-      <c r="G142" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H142" s="21" t="s">
+      <c r="G142" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H142" s="22" t="s">
         <v>703</v>
       </c>
-      <c r="I142" s="21"/>
-      <c r="J142" s="21" t="s">
+      <c r="I142" s="22"/>
+      <c r="J142" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K142" s="21"/>
-      <c r="L142" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M142" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N142" s="21" t="s">
+      <c r="K142" s="22"/>
+      <c r="L142" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M142" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N142" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A143" s="21"/>
-      <c r="B143" s="22" t="s">
+      <c r="A143" s="22"/>
+      <c r="B143" s="23" t="s">
         <v>704</v>
       </c>
-      <c r="C143" s="21" t="s">
+      <c r="C143" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D143" s="21" t="s">
+      <c r="D143" s="22" t="s">
         <v>705</v>
       </c>
-      <c r="E143" s="21" t="s">
+      <c r="E143" s="22" t="s">
         <v>706</v>
       </c>
-      <c r="F143" s="21" t="s">
+      <c r="F143" s="22" t="s">
         <v>707</v>
       </c>
-      <c r="G143" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H143" s="21" t="s">
+      <c r="G143" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H143" s="22" t="s">
         <v>708</v>
       </c>
-      <c r="I143" s="21"/>
-      <c r="J143" s="21" t="s">
+      <c r="I143" s="22"/>
+      <c r="J143" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K143" s="21"/>
-      <c r="L143" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M143" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N143" s="21" t="s">
+      <c r="K143" s="22"/>
+      <c r="L143" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M143" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N143" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A144" s="21"/>
-      <c r="B144" s="22" t="s">
+      <c r="A144" s="22"/>
+      <c r="B144" s="23" t="s">
         <v>709</v>
       </c>
-      <c r="C144" s="21" t="s">
+      <c r="C144" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D144" s="21" t="s">
+      <c r="D144" s="22" t="s">
         <v>710</v>
       </c>
-      <c r="E144" s="21" t="s">
+      <c r="E144" s="22" t="s">
         <v>711</v>
       </c>
-      <c r="F144" s="21" t="s">
+      <c r="F144" s="22" t="s">
         <v>712</v>
       </c>
-      <c r="G144" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H144" s="21" t="s">
+      <c r="G144" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H144" s="22" t="s">
         <v>713</v>
       </c>
-      <c r="I144" s="21"/>
-      <c r="J144" s="21" t="s">
+      <c r="I144" s="22"/>
+      <c r="J144" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K144" s="21"/>
-      <c r="L144" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M144" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N144" s="21" t="s">
+      <c r="K144" s="22"/>
+      <c r="L144" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M144" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N144" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A145" s="21"/>
-      <c r="B145" s="22" t="s">
+      <c r="A145" s="22"/>
+      <c r="B145" s="23" t="s">
         <v>714</v>
       </c>
-      <c r="C145" s="21" t="s">
+      <c r="C145" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D145" s="21" t="s">
+      <c r="D145" s="22" t="s">
         <v>715</v>
       </c>
-      <c r="E145" s="21" t="s">
+      <c r="E145" s="22" t="s">
         <v>716</v>
       </c>
-      <c r="F145" s="21" t="s">
+      <c r="F145" s="22" t="s">
         <v>717</v>
       </c>
-      <c r="G145" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H145" s="21" t="s">
+      <c r="G145" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H145" s="22" t="s">
         <v>718</v>
       </c>
-      <c r="I145" s="21"/>
-      <c r="J145" s="21" t="s">
+      <c r="I145" s="22"/>
+      <c r="J145" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K145" s="21"/>
-      <c r="L145" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M145" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N145" s="21" t="s">
+      <c r="K145" s="22"/>
+      <c r="L145" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M145" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N145" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A146" s="21"/>
-      <c r="B146" s="22" t="s">
+      <c r="A146" s="22"/>
+      <c r="B146" s="23" t="s">
         <v>719</v>
       </c>
-      <c r="C146" s="21" t="s">
+      <c r="C146" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D146" s="21" t="s">
+      <c r="D146" s="22" t="s">
         <v>720</v>
       </c>
-      <c r="E146" s="21" t="s">
+      <c r="E146" s="22" t="s">
         <v>721</v>
       </c>
-      <c r="F146" s="21" t="s">
+      <c r="F146" s="22" t="s">
         <v>722</v>
       </c>
-      <c r="G146" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H146" s="21" t="s">
+      <c r="G146" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H146" s="22" t="s">
         <v>723</v>
       </c>
-      <c r="I146" s="21"/>
-      <c r="J146" s="21" t="s">
+      <c r="I146" s="22"/>
+      <c r="J146" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K146" s="21"/>
-      <c r="L146" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M146" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N146" s="21" t="s">
+      <c r="K146" s="22"/>
+      <c r="L146" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M146" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N146" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A147" s="21"/>
-      <c r="B147" s="22" t="s">
+      <c r="A147" s="22"/>
+      <c r="B147" s="23" t="s">
         <v>724</v>
       </c>
-      <c r="C147" s="21" t="s">
+      <c r="C147" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D147" s="21" t="s">
+      <c r="D147" s="22" t="s">
         <v>725</v>
       </c>
-      <c r="E147" s="21" t="s">
+      <c r="E147" s="22" t="s">
         <v>726</v>
       </c>
-      <c r="F147" s="21" t="s">
+      <c r="F147" s="22" t="s">
         <v>727</v>
       </c>
-      <c r="G147" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H147" s="21" t="s">
+      <c r="G147" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H147" s="22" t="s">
         <v>728</v>
       </c>
-      <c r="I147" s="21"/>
-      <c r="J147" s="21" t="s">
+      <c r="I147" s="22"/>
+      <c r="J147" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K147" s="21"/>
-      <c r="L147" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M147" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N147" s="21" t="s">
+      <c r="K147" s="22"/>
+      <c r="L147" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M147" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N147" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A148" s="21"/>
-      <c r="B148" s="22" t="s">
+      <c r="A148" s="22"/>
+      <c r="B148" s="23" t="s">
         <v>729</v>
       </c>
-      <c r="C148" s="21" t="s">
+      <c r="C148" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D148" s="21" t="s">
+      <c r="D148" s="22" t="s">
         <v>730</v>
       </c>
-      <c r="E148" s="21" t="s">
+      <c r="E148" s="22" t="s">
         <v>731</v>
       </c>
-      <c r="F148" s="21" t="s">
+      <c r="F148" s="22" t="s">
         <v>732</v>
       </c>
-      <c r="G148" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H148" s="21" t="s">
+      <c r="G148" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H148" s="22" t="s">
         <v>733</v>
       </c>
-      <c r="I148" s="21"/>
-      <c r="J148" s="21" t="s">
+      <c r="I148" s="22"/>
+      <c r="J148" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K148" s="21"/>
-      <c r="L148" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M148" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N148" s="21" t="s">
+      <c r="K148" s="22"/>
+      <c r="L148" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M148" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N148" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A149" s="21"/>
-      <c r="B149" s="22" t="s">
+      <c r="A149" s="22"/>
+      <c r="B149" s="23" t="s">
         <v>734</v>
       </c>
-      <c r="C149" s="21" t="s">
+      <c r="C149" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D149" s="21" t="s">
+      <c r="D149" s="22" t="s">
         <v>735</v>
       </c>
-      <c r="E149" s="21" t="s">
+      <c r="E149" s="22" t="s">
         <v>736</v>
       </c>
-      <c r="F149" s="21" t="s">
+      <c r="F149" s="22" t="s">
         <v>737</v>
       </c>
-      <c r="G149" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H149" s="21" t="s">
+      <c r="G149" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="H149" s="22" t="s">
         <v>738</v>
       </c>
-      <c r="I149" s="21"/>
-      <c r="J149" s="21" t="s">
+      <c r="I149" s="22"/>
+      <c r="J149" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K149" s="21"/>
-      <c r="L149" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M149" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N149" s="21" t="s">
+      <c r="K149" s="22"/>
+      <c r="L149" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M149" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N149" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A150" s="21"/>
-      <c r="B150" s="22" t="s">
+      <c r="A150" s="22"/>
+      <c r="B150" s="23" t="s">
         <v>739</v>
       </c>
-      <c r="C150" s="21" t="s">
+      <c r="C150" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D150" s="21" t="s">
+      <c r="D150" s="22" t="s">
         <v>740</v>
       </c>
-      <c r="E150" s="21" t="s">
+      <c r="E150" s="22" t="s">
         <v>741</v>
       </c>
-      <c r="F150" s="21" t="s">
+      <c r="F150" s="22" t="s">
         <v>742</v>
       </c>
-      <c r="G150" s="21" t="s">
+      <c r="G150" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H150" s="21" t="s">
+      <c r="H150" s="22" t="s">
         <v>743</v>
       </c>
-      <c r="I150" s="21"/>
-      <c r="J150" s="21" t="s">
+      <c r="I150" s="22"/>
+      <c r="J150" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K150" s="21"/>
-      <c r="L150" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M150" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N150" s="21" t="s">
+      <c r="K150" s="22"/>
+      <c r="L150" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M150" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N150" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A151" s="21"/>
-      <c r="B151" s="22" t="s">
+      <c r="A151" s="22"/>
+      <c r="B151" s="23" t="s">
         <v>744</v>
       </c>
-      <c r="C151" s="21" t="s">
+      <c r="C151" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D151" s="21" t="s">
+      <c r="D151" s="22" t="s">
         <v>745</v>
       </c>
-      <c r="E151" s="21" t="s">
+      <c r="E151" s="22" t="s">
         <v>746</v>
       </c>
-      <c r="F151" s="21" t="s">
+      <c r="F151" s="22" t="s">
         <v>747</v>
       </c>
-      <c r="G151" s="21" t="s">
+      <c r="G151" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H151" s="21" t="s">
+      <c r="H151" s="22" t="s">
         <v>748</v>
       </c>
-      <c r="I151" s="21"/>
-      <c r="J151" s="21" t="s">
+      <c r="I151" s="22"/>
+      <c r="J151" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K151" s="21"/>
-      <c r="L151" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M151" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N151" s="21" t="s">
+      <c r="K151" s="22"/>
+      <c r="L151" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M151" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N151" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A152" s="21"/>
-      <c r="B152" s="22" t="s">
+      <c r="A152" s="22"/>
+      <c r="B152" s="23" t="s">
         <v>749</v>
       </c>
-      <c r="C152" s="21" t="s">
+      <c r="C152" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D152" s="21" t="s">
+      <c r="D152" s="22" t="s">
         <v>750</v>
       </c>
-      <c r="E152" s="21" t="s">
+      <c r="E152" s="22" t="s">
         <v>751</v>
       </c>
-      <c r="F152" s="21" t="s">
+      <c r="F152" s="22" t="s">
         <v>752</v>
       </c>
-      <c r="G152" s="21" t="s">
+      <c r="G152" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="H152" s="21" t="s">
+      <c r="H152" s="22" t="s">
         <v>753</v>
       </c>
-      <c r="I152" s="21"/>
-      <c r="J152" s="21" t="s">
+      <c r="I152" s="22"/>
+      <c r="J152" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K152" s="21"/>
-      <c r="L152" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M152" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N152" s="21" t="s">
+      <c r="K152" s="22"/>
+      <c r="L152" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M152" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N152" s="22" t="s">
         <v>633</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A153" s="21"/>
-      <c r="B153" s="22" t="s">
+      <c r="A153" s="22"/>
+      <c r="B153" s="23" t="s">
         <v>754</v>
       </c>
-      <c r="C153" s="21" t="s">
+      <c r="C153" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D153" s="21" t="s">
+      <c r="D153" s="22" t="s">
         <v>755</v>
       </c>
-      <c r="E153" s="21" t="s">
+      <c r="E153" s="22" t="s">
         <v>756</v>
       </c>
-      <c r="F153" s="21" t="s">
+      <c r="F153" s="22" t="s">
         <v>757</v>
       </c>
-      <c r="G153" s="21" t="s">
+      <c r="G153" s="22" t="s">
         <v>415</v>
       </c>
-      <c r="H153" s="21" t="s">
+      <c r="H153" s="22" t="s">
         <v>758</v>
       </c>
-      <c r="I153" s="21"/>
-      <c r="J153" s="21" t="s">
+      <c r="I153" s="22"/>
+      <c r="J153" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="K153" s="21"/>
-      <c r="L153" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M153" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N153" s="21" t="s">
+      <c r="K153" s="22"/>
+      <c r="L153" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M153" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N153" s="22" t="s">
         <v>633</v>
       </c>
     </row>
@@ -8826,697 +8835,697 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>759</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>760</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>762</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>763</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>764</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>765</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="I1" s="26" t="s">
         <v>766</v>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
         <v>767</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="28" t="s">
         <v>768</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="28" t="s">
         <v>769</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="28" t="s">
         <v>770</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="28" t="s">
         <v>771</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="28" t="s">
         <v>772</v>
       </c>
-      <c r="G2" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" s="28" t="s">
+      <c r="G2" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="29" t="s">
         <v>773</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>774</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>775</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="31" t="s">
         <v>776</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E3" s="30" t="s">
+      <c r="E3" s="31" t="s">
         <v>777</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="31" t="s">
         <v>778</v>
       </c>
-      <c r="G3" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="31" t="s">
+      <c r="G3" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="32" t="s">
         <v>779</v>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="30" t="s">
         <v>780</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>781</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>782</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>783</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>784</v>
       </c>
-      <c r="G4" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="31" t="s">
+      <c r="G4" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="32" t="s">
         <v>785</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="30" t="s">
         <v>786</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="31" t="s">
         <v>787</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="31" t="s">
         <v>788</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="31" t="s">
         <v>789</v>
       </c>
-      <c r="F5" s="30" t="s">
+      <c r="F5" s="31" t="s">
         <v>790</v>
       </c>
-      <c r="G5" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="31" t="s">
+      <c r="G5" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="32" t="s">
         <v>791</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="30" t="s">
         <v>792</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="31" t="s">
         <v>388</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="31" t="s">
         <v>793</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="31" t="s">
         <v>794</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="31" t="s">
         <v>795</v>
       </c>
-      <c r="G6" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="31" t="s">
+      <c r="G6" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="32" t="s">
         <v>796</v>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="30" t="s">
         <v>797</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="31" t="s">
         <v>424</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="31" t="s">
         <v>798</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="31" t="s">
         <v>799</v>
       </c>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="31" t="s">
         <v>800</v>
       </c>
-      <c r="G7" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="31" t="s">
+      <c r="G7" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="32" t="s">
         <v>801</v>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="30" t="s">
         <v>802</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="31" t="s">
         <v>488</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="31" t="s">
         <v>803</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="E8" s="31" t="s">
         <v>804</v>
       </c>
-      <c r="F8" s="30" t="s">
+      <c r="F8" s="31" t="s">
         <v>805</v>
       </c>
-      <c r="G8" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I8" s="31" t="s">
+      <c r="G8" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="32" t="s">
         <v>806</v>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="30" t="s">
         <v>807</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="31" t="s">
         <v>581</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="31" t="s">
         <v>808</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="31" t="s">
         <v>770</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="31" t="s">
         <v>809</v>
       </c>
-      <c r="F9" s="30" t="s">
+      <c r="F9" s="31" t="s">
         <v>810</v>
       </c>
-      <c r="G9" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="31" t="s">
+      <c r="G9" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="32" t="s">
         <v>811</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="33" t="s">
         <v>812</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="34" t="s">
         <v>625</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="34" t="s">
         <v>813</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="34" t="s">
         <v>770</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="34" t="s">
         <v>814</v>
       </c>
-      <c r="F10" s="33" t="s">
+      <c r="F10" s="34" t="s">
         <v>815</v>
       </c>
-      <c r="G10" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="34" t="s">
+      <c r="G10" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="35" t="s">
         <v>816</v>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="35" t="s">
+      <c r="A11" s="36" t="s">
         <v>817</v>
       </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="36" t="s">
+      <c r="B11" s="37"/>
+      <c r="C11" s="37" t="s">
         <v>818</v>
       </c>
-      <c r="D11" s="36" t="s">
+      <c r="D11" s="37" t="s">
         <v>819</v>
       </c>
-      <c r="E11" s="36" t="s">
+      <c r="E11" s="37" t="s">
         <v>820</v>
       </c>
-      <c r="F11" s="36" t="s">
+      <c r="F11" s="37" t="s">
         <v>821</v>
       </c>
-      <c r="G11" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I11" s="37" t="s">
+      <c r="G11" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" s="38" t="s">
         <v>822</v>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="39" t="s">
         <v>823</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39" t="s">
+      <c r="B12" s="40"/>
+      <c r="C12" s="40" t="s">
         <v>824</v>
       </c>
-      <c r="D12" s="39" t="s">
+      <c r="D12" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="40" t="s">
         <v>825</v>
       </c>
-      <c r="G12" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H12" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I12" s="40" t="s">
+      <c r="G12" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="41" t="s">
         <v>826</v>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="39" t="s">
         <v>827</v>
       </c>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39" t="s">
+      <c r="B13" s="40"/>
+      <c r="C13" s="40" t="s">
         <v>828</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D13" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="40" t="s">
         <v>829</v>
       </c>
-      <c r="G13" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H13" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I13" s="40" t="s">
+      <c r="G13" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H13" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" s="41" t="s">
         <v>830</v>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="38" t="s">
+      <c r="A14" s="39" t="s">
         <v>831</v>
       </c>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39" t="s">
+      <c r="B14" s="40"/>
+      <c r="C14" s="40" t="s">
         <v>832</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F14" s="39" t="s">
+      <c r="F14" s="40" t="s">
         <v>833</v>
       </c>
-      <c r="G14" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="40" t="s">
+      <c r="G14" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="41" t="s">
         <v>834</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="39" t="s">
         <v>835</v>
       </c>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39" t="s">
+      <c r="B15" s="40"/>
+      <c r="C15" s="40" t="s">
         <v>836</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E15" s="39" t="s">
+      <c r="E15" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F15" s="39" t="s">
+      <c r="F15" s="40" t="s">
         <v>837</v>
       </c>
-      <c r="G15" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I15" s="40" t="s">
+      <c r="G15" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I15" s="41" t="s">
         <v>838</v>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="39" t="s">
         <v>839</v>
       </c>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39" t="s">
+      <c r="B16" s="40"/>
+      <c r="C16" s="40" t="s">
         <v>840</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E16" s="39" t="s">
+      <c r="E16" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F16" s="39" t="s">
+      <c r="F16" s="40" t="s">
         <v>841</v>
       </c>
-      <c r="G16" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I16" s="40" t="s">
+      <c r="G16" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="41" t="s">
         <v>842</v>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="39" t="s">
         <v>843</v>
       </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39" t="s">
+      <c r="B17" s="40"/>
+      <c r="C17" s="40" t="s">
         <v>844</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E17" s="39" t="s">
+      <c r="E17" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F17" s="39" t="s">
+      <c r="F17" s="40" t="s">
         <v>845</v>
       </c>
-      <c r="G17" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H17" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I17" s="40" t="s">
+      <c r="G17" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="41" t="s">
         <v>846</v>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="39" t="s">
         <v>847</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39" t="s">
+      <c r="B18" s="40"/>
+      <c r="C18" s="40" t="s">
         <v>848</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E18" s="39" t="s">
+      <c r="E18" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="F18" s="40" t="s">
         <v>849</v>
       </c>
-      <c r="G18" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I18" s="40" t="s">
+      <c r="G18" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" s="41" t="s">
         <v>850</v>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="39" t="s">
         <v>851</v>
       </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39" t="s">
+      <c r="B19" s="40"/>
+      <c r="C19" s="40" t="s">
         <v>852</v>
       </c>
-      <c r="D19" s="39" t="s">
+      <c r="D19" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="E19" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F19" s="39" t="s">
+      <c r="F19" s="40" t="s">
         <v>853</v>
       </c>
-      <c r="G19" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I19" s="40" t="s">
+      <c r="G19" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19" s="41" t="s">
         <v>854</v>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="39" t="s">
         <v>855</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39" t="s">
+      <c r="B20" s="40"/>
+      <c r="C20" s="40" t="s">
         <v>856</v>
       </c>
-      <c r="D20" s="39" t="s">
+      <c r="D20" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E20" s="39" t="s">
+      <c r="E20" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F20" s="39" t="s">
+      <c r="F20" s="40" t="s">
         <v>857</v>
       </c>
-      <c r="G20" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H20" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I20" s="40" t="s">
+      <c r="G20" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I20" s="41" t="s">
         <v>858</v>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="39" t="s">
         <v>859</v>
       </c>
-      <c r="B21" s="39"/>
-      <c r="C21" s="39" t="s">
+      <c r="B21" s="40"/>
+      <c r="C21" s="40" t="s">
         <v>860</v>
       </c>
-      <c r="D21" s="39" t="s">
+      <c r="D21" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E21" s="39" t="s">
+      <c r="E21" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F21" s="39" t="s">
+      <c r="F21" s="40" t="s">
         <v>861</v>
       </c>
-      <c r="G21" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H21" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I21" s="40" t="s">
+      <c r="G21" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="41" t="s">
         <v>862</v>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="39" t="s">
         <v>863</v>
       </c>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39" t="s">
+      <c r="B22" s="40"/>
+      <c r="C22" s="40" t="s">
         <v>803</v>
       </c>
-      <c r="D22" s="39" t="s">
+      <c r="D22" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E22" s="39" t="s">
+      <c r="E22" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F22" s="39" t="s">
+      <c r="F22" s="40" t="s">
         <v>864</v>
       </c>
-      <c r="G22" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H22" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I22" s="40" t="s">
+      <c r="G22" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H22" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="41" t="s">
         <v>865</v>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="39" t="s">
         <v>866</v>
       </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39" t="s">
+      <c r="B23" s="40"/>
+      <c r="C23" s="40" t="s">
         <v>808</v>
       </c>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E23" s="39" t="s">
+      <c r="E23" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F23" s="39" t="s">
+      <c r="F23" s="40" t="s">
         <v>867</v>
       </c>
-      <c r="G23" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H23" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I23" s="40" t="s">
+      <c r="G23" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H23" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="41" t="s">
         <v>868</v>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="38" t="s">
+      <c r="A24" s="39" t="s">
         <v>869</v>
       </c>
-      <c r="B24" s="39"/>
-      <c r="C24" s="39" t="s">
+      <c r="B24" s="40"/>
+      <c r="C24" s="40" t="s">
         <v>870</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="40" t="s">
         <v>819</v>
       </c>
-      <c r="E24" s="39" t="s">
+      <c r="E24" s="40" t="s">
         <v>820</v>
       </c>
-      <c r="F24" s="39" t="s">
+      <c r="F24" s="40" t="s">
         <v>871</v>
       </c>
-      <c r="G24" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H24" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I24" s="40" t="s">
+      <c r="G24" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" s="41" t="s">
         <v>872</v>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="42" t="s">
         <v>873</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42" t="s">
+      <c r="B25" s="43"/>
+      <c r="C25" s="43" t="s">
         <v>813</v>
       </c>
-      <c r="D25" s="42" t="s">
+      <c r="D25" s="43" t="s">
         <v>819</v>
       </c>
-      <c r="E25" s="42" t="s">
+      <c r="E25" s="43" t="s">
         <v>820</v>
       </c>
-      <c r="F25" s="42" t="s">
+      <c r="F25" s="43" t="s">
         <v>874</v>
       </c>
-      <c r="G25" s="42" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="42" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="43" t="s">
+      <c r="G25" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="44" t="s">
         <v>875</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: correct Stage 6 Pass 006 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1800" uniqueCount="938">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1802" uniqueCount="939">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1119,6 +1119,9 @@
     <t>legacy/src/frontend/account-deposit.html:314-392; openapi.yaml:1025; DepositRequest schema; Runtime: static-only</t>
   </si>
   <si>
+    <t>Decision D-020: target derives the sort code from account/bank configuration instead of trusting request input.</t>
+  </si>
+  <si>
     <t>CICS payment debit is rejected for insufficient funds</t>
   </si>
   <si>
@@ -1446,7 +1449,7 @@
     <t>The route is published but has no operation mapping.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:580-615; js/api.js:286-292; operations/...transactionId/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml:580-615; js/api.js:286-292; operations/...transactionId/get (no operation.yaml); Runtime: static-only</t>
   </si>
   <si>
     <t>Java history service reads recent activity</t>
@@ -1476,7 +1479,7 @@
     <t>The contract declares standard failures, but five bound and three unbound response selections reference missing generated YAML artifacts.</t>
   </si>
   <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+    <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema; Runtime: static-only</t>
   </si>
   <si>
     <t>Deviation D-008: target Problem Details replace missing generated response files.</t>
@@ -1581,7 +1584,7 @@
     <t>Customer and account information sections are printed.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:430-635; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:430-635; Runtime: static-only</t>
   </si>
   <si>
     <t>Statement lists period transactions</t>
@@ -1596,7 +1599,7 @@
     <t>Each transaction includes date, time, type, reference, description, and amount; balances appear in the statement summary.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:638-779; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:638-779; Runtime: static-only</t>
   </si>
   <si>
     <t>Statement period has no transactions</t>
@@ -1626,7 +1629,7 @@
     <t>A statement summary is printed with all totals.</t>
   </si>
   <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:782-859; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:782-859; Runtime: static-only</t>
   </si>
   <si>
     <t>Statement paginates and closes</t>
@@ -2433,7 +2436,7 @@
     <t>UF-004, UF-005, UF-008, UF-010</t>
   </si>
   <si>
-    <t>41-58,88,110-112</t>
+    <t>41-48,50-58,88,110-112</t>
   </si>
   <si>
     <t>Account business behavior is mapped; target is absent.</t>
@@ -6003,7 +6006,9 @@
         <v>366</v>
       </c>
       <c r="I71" s="21"/>
-      <c r="J71" s="21"/>
+      <c r="J71" s="21" t="s">
+        <v>367</v>
+      </c>
       <c r="K71" s="21"/>
       <c r="L71" s="21" t="s">
         <v>36</v>
@@ -6018,29 +6023,29 @@
     <row r="72" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A72" s="22"/>
       <c r="B72" s="22" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C72" s="22" t="s">
         <v>42</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E72" s="23" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F72" s="23" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G72" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H72" s="23" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I72" s="23"/>
       <c r="J72" s="23" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K72" s="23"/>
       <c r="L72" s="23" t="s">
@@ -6056,29 +6061,29 @@
     <row r="73" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A73" s="18"/>
       <c r="B73" s="19" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C73" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D73" s="20" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E73" s="20" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F73" s="20" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G73" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H73" s="20" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="I73" s="20"/>
       <c r="J73" s="20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K73" s="20"/>
       <c r="L73" s="20" t="s">
@@ -6094,29 +6099,29 @@
     <row r="74" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A74" s="19"/>
       <c r="B74" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C74" s="19" t="s">
         <v>42</v>
       </c>
       <c r="D74" s="21" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E74" s="21" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F74" s="21" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G74" s="21" t="s">
         <v>36</v>
       </c>
       <c r="H74" s="21" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I74" s="21"/>
       <c r="J74" s="21" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K74" s="21"/>
       <c r="L74" s="21" t="s">
@@ -6132,29 +6137,29 @@
     <row r="75" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A75" s="18"/>
       <c r="B75" s="19" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C75" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D75" s="20" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E75" s="20" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G75" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H75" s="20" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="I75" s="20"/>
       <c r="J75" s="20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K75" s="20"/>
       <c r="L75" s="20" t="s">
@@ -6170,29 +6175,29 @@
     <row r="76" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A76" s="18"/>
       <c r="B76" s="19" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C76" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D76" s="20" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F76" s="20" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G76" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H76" s="20" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="I76" s="20"/>
       <c r="J76" s="20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K76" s="20"/>
       <c r="L76" s="20" t="s">
@@ -6208,29 +6213,29 @@
     <row r="77" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A77" s="19"/>
       <c r="B77" s="19" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C77" s="19" t="s">
         <v>42</v>
       </c>
       <c r="D77" s="21" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E77" s="21" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F77" s="21" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G77" s="21" t="s">
         <v>36</v>
       </c>
       <c r="H77" s="21" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="I77" s="21"/>
       <c r="J77" s="21" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K77" s="21"/>
       <c r="L77" s="21" t="s">
@@ -6246,29 +6251,29 @@
     <row r="78" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A78" s="18"/>
       <c r="B78" s="19" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C78" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="20" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E78" s="20" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F78" s="20" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G78" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H78" s="20" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="I78" s="20"/>
       <c r="J78" s="20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K78" s="20"/>
       <c r="L78" s="20" t="s">
@@ -6283,10 +6288,10 @@
     </row>
     <row r="79" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C79" s="17" t="s">
         <v>29</v>
@@ -6308,29 +6313,29 @@
     <row r="80" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A80" s="18"/>
       <c r="B80" s="19" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C80" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D80" s="20" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E80" s="20" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F80" s="20" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G80" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H80" s="20" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="I80" s="20"/>
       <c r="J80" s="20" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K80" s="20"/>
       <c r="L80" s="20" t="s">
@@ -6340,31 +6345,31 @@
         <v>39</v>
       </c>
       <c r="N80" s="20" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="81" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A81" s="19"/>
       <c r="B81" s="19" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C81" s="19" t="s">
         <v>42</v>
       </c>
       <c r="D81" s="21" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E81" s="21" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F81" s="21" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G81" s="21" t="s">
         <v>36</v>
       </c>
       <c r="H81" s="21" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="I81" s="21"/>
       <c r="J81" s="21"/>
@@ -6376,31 +6381,31 @@
         <v>39</v>
       </c>
       <c r="N81" s="21" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="82" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A82" s="18"/>
       <c r="B82" s="19" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C82" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E82" s="20" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F82" s="20" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G82" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H82" s="20" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="I82" s="20"/>
       <c r="J82" s="20"/>
@@ -6412,31 +6417,31 @@
         <v>39</v>
       </c>
       <c r="N82" s="20" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="83" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="18"/>
       <c r="B83" s="19" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C83" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D83" s="20" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E83" s="20" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F83" s="20" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G83" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H83" s="20" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I83" s="20"/>
       <c r="J83" s="20"/>
@@ -6448,35 +6453,35 @@
         <v>39</v>
       </c>
       <c r="N83" s="20" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="84" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="19"/>
       <c r="B84" s="19" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C84" s="19" t="s">
         <v>42</v>
       </c>
       <c r="D84" s="21" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E84" s="21" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F84" s="21" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G84" s="21" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H84" s="21" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I84" s="21"/>
       <c r="J84" s="21" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K84" s="21"/>
       <c r="L84" s="21" t="s">
@@ -6486,35 +6491,35 @@
         <v>39</v>
       </c>
       <c r="N84" s="21" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="85" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C85" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D85" s="20" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E85" s="20" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F85" s="20" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G85" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H85" s="20" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I85" s="20"/>
       <c r="J85" s="20" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K85" s="20"/>
       <c r="L85" s="20" t="s">
@@ -6524,15 +6529,15 @@
         <v>39</v>
       </c>
       <c r="N85" s="20" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B86" s="17" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C86" s="17" t="s">
         <v>29</v>
@@ -6554,25 +6559,25 @@
     <row r="87" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C87" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D87" s="20" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E87" s="20" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F87" s="20" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G87" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H87" s="20" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I87" s="20"/>
       <c r="J87" s="20"/>
@@ -6590,29 +6595,29 @@
     <row r="88" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C88" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E88" s="20" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F88" s="20" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G88" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H88" s="20" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I88" s="20"/>
       <c r="J88" s="20" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K88" s="20"/>
       <c r="L88" s="20" t="s">
@@ -6628,28 +6633,30 @@
     <row r="89" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C89" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F89" s="20" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G89" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H89" s="20" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I89" s="20"/>
-      <c r="J89" s="20"/>
+      <c r="J89" s="20" t="s">
+        <v>367</v>
+      </c>
       <c r="K89" s="20"/>
       <c r="L89" s="20" t="s">
         <v>36</v>
@@ -6664,25 +6671,25 @@
     <row r="90" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C90" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D90" s="20" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E90" s="20" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F90" s="20" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G90" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H90" s="20" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I90" s="20"/>
       <c r="J90" s="20"/>
@@ -6700,29 +6707,29 @@
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="22"/>
       <c r="B91" s="22" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C91" s="22" t="s">
         <v>42</v>
       </c>
       <c r="D91" s="23" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E91" s="23" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F91" s="23" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G91" s="23" t="s">
         <v>132</v>
       </c>
       <c r="H91" s="23" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="I91" s="23"/>
       <c r="J91" s="23" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K91" s="23"/>
       <c r="L91" s="23" t="s">
@@ -6732,35 +6739,35 @@
         <v>39</v>
       </c>
       <c r="N91" s="23" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="92" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C92" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D92" s="20" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F92" s="20" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G92" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H92" s="20" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="I92" s="20"/>
       <c r="J92" s="20" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K92" s="20"/>
       <c r="L92" s="20" t="s">
@@ -6770,35 +6777,35 @@
         <v>39</v>
       </c>
       <c r="N92" s="20" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="19"/>
       <c r="B93" s="19" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C93" s="19" t="s">
         <v>42</v>
       </c>
       <c r="D93" s="21" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E93" s="21" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F93" s="21" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G93" s="21" t="s">
         <v>132</v>
       </c>
       <c r="H93" s="21" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="I93" s="21"/>
       <c r="J93" s="21" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K93" s="21"/>
       <c r="L93" s="21" t="s">
@@ -6808,31 +6815,31 @@
         <v>39</v>
       </c>
       <c r="N93" s="21" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="19"/>
       <c r="B94" s="19" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C94" s="19" t="s">
         <v>32</v>
       </c>
       <c r="D94" s="21" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E94" s="21" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F94" s="21" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G94" s="21" t="s">
         <v>36</v>
       </c>
       <c r="H94" s="21" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="I94" s="21"/>
       <c r="J94" s="21"/>
@@ -6844,35 +6851,35 @@
         <v>39</v>
       </c>
       <c r="N94" s="21" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C95" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D95" s="20" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E95" s="20" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F95" s="20" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G95" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H95" s="20" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="I95" s="20"/>
       <c r="J95" s="20" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K95" s="20"/>
       <c r="L95" s="20" t="s">
@@ -6882,35 +6889,35 @@
         <v>39</v>
       </c>
       <c r="N95" s="20" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="96" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D96" s="20" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E96" s="20" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F96" s="20" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G96" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H96" s="20" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="I96" s="20"/>
       <c r="J96" s="20" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K96" s="20"/>
       <c r="L96" s="20" t="s">
@@ -6920,31 +6927,31 @@
         <v>39</v>
       </c>
       <c r="N96" s="20" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="97" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C97" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D97" s="20" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E97" s="20" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F97" s="20" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="G97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H97" s="20" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="I97" s="20"/>
       <c r="J97" s="20"/>
@@ -6962,25 +6969,25 @@
     <row r="98" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C98" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D98" s="20" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E98" s="20" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F98" s="20" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="G98" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H98" s="20" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="I98" s="20"/>
       <c r="J98" s="20"/>
@@ -6992,15 +6999,15 @@
         <v>39</v>
       </c>
       <c r="N98" s="20" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B99" s="17" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C99" s="17" t="s">
         <v>29</v>
@@ -7022,29 +7029,29 @@
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="22"/>
       <c r="B100" s="22" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C100" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D100" s="23" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E100" s="23" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F100" s="23" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G100" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H100" s="23" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="I100" s="23"/>
       <c r="J100" s="23" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K100" s="23"/>
       <c r="L100" s="23" t="s">
@@ -7054,35 +7061,35 @@
         <v>39</v>
       </c>
       <c r="N100" s="23" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="19"/>
       <c r="B101" s="19" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C101" s="19" t="s">
         <v>42</v>
       </c>
       <c r="D101" s="21" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E101" s="21" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F101" s="21" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="G101" s="21" t="s">
         <v>36</v>
       </c>
       <c r="H101" s="21" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="I101" s="21"/>
       <c r="J101" s="21" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K101" s="21"/>
       <c r="L101" s="21" t="s">
@@ -7092,35 +7099,35 @@
         <v>39</v>
       </c>
       <c r="N101" s="21" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D102" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E102" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F102" s="20" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G102" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H102" s="20" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="I102" s="20"/>
       <c r="J102" s="20" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K102" s="20"/>
       <c r="L102" s="20" t="s">
@@ -7130,35 +7137,35 @@
         <v>39</v>
       </c>
       <c r="N102" s="20" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C103" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D103" s="20" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E103" s="20" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F103" s="20" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="G103" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H103" s="20" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="I103" s="20"/>
       <c r="J103" s="20" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K103" s="20"/>
       <c r="L103" s="20" t="s">
@@ -7168,35 +7175,35 @@
         <v>39</v>
       </c>
       <c r="N103" s="20" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D104" s="20" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E104" s="20" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F104" s="20" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="G104" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H104" s="20" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="I104" s="20"/>
       <c r="J104" s="20" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K104" s="20"/>
       <c r="L104" s="20" t="s">
@@ -7206,35 +7213,35 @@
         <v>39</v>
       </c>
       <c r="N104" s="20" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="19"/>
       <c r="B105" s="19" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C105" s="19" t="s">
         <v>32</v>
       </c>
       <c r="D105" s="21" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E105" s="21" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F105" s="21" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G105" s="21" t="s">
         <v>36</v>
       </c>
       <c r="H105" s="21" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="I105" s="21"/>
       <c r="J105" s="21" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K105" s="21"/>
       <c r="L105" s="21" t="s">
@@ -7244,35 +7251,35 @@
         <v>39</v>
       </c>
       <c r="N105" s="21" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C106" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D106" s="20" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E106" s="20" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F106" s="20" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="G106" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H106" s="20" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="I106" s="20"/>
       <c r="J106" s="20" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K106" s="20"/>
       <c r="L106" s="20" t="s">
@@ -7282,35 +7289,35 @@
         <v>39</v>
       </c>
       <c r="N106" s="20" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C107" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D107" s="20" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E107" s="20" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F107" s="20" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G107" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H107" s="20" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="I107" s="20"/>
       <c r="J107" s="20" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="K107" s="20"/>
       <c r="L107" s="20" t="s">
@@ -7320,15 +7327,15 @@
         <v>39</v>
       </c>
       <c r="N107" s="20" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="108" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B108" s="17" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C108" s="17" t="s">
         <v>29</v>
@@ -7350,29 +7357,29 @@
     <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C109" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E109" s="20" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F109" s="20" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="I109" s="20"/>
       <c r="J109" s="20" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K109" s="20"/>
       <c r="L109" s="20" t="s">
@@ -7388,29 +7395,29 @@
     <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C110" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F110" s="20" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="G110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="I110" s="20"/>
       <c r="J110" s="20" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="K110" s="20"/>
       <c r="L110" s="20" t="s">
@@ -7426,29 +7433,29 @@
     <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C111" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D111" s="20" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E111" s="20" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="F111" s="20" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="G111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="I111" s="20"/>
       <c r="J111" s="20" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="K111" s="20"/>
       <c r="L111" s="20" t="s">
@@ -7464,29 +7471,29 @@
     <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C112" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="F112" s="20" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="G112" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="I112" s="20"/>
       <c r="J112" s="20" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="K112" s="20"/>
       <c r="L112" s="20" t="s">
@@ -7502,29 +7509,29 @@
     <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C113" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="I113" s="20"/>
       <c r="J113" s="20" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="K113" s="20"/>
       <c r="L113" s="20" t="s">
@@ -7540,29 +7547,29 @@
     <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C114" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D114" s="20" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E114" s="20" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="F114" s="20" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="G114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="20" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="I114" s="20"/>
       <c r="J114" s="20" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="K114" s="20"/>
       <c r="L114" s="20" t="s">
@@ -7578,29 +7585,29 @@
     <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C115" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D115" s="20" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F115" s="20" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="G115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="20" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="I115" s="20"/>
       <c r="J115" s="20" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="K115" s="20"/>
       <c r="L115" s="20" t="s">
@@ -7616,29 +7623,29 @@
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="22"/>
       <c r="B116" s="22" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C116" s="22" t="s">
         <v>95</v>
       </c>
       <c r="D116" s="23" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E116" s="23" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F116" s="23" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="G116" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H116" s="23" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="I116" s="23"/>
       <c r="J116" s="23" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="K116" s="23"/>
       <c r="L116" s="23" t="s">
@@ -7654,29 +7661,29 @@
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
       <c r="B117" s="18" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="C117" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="E117" s="20" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G117" s="20" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="I117" s="20"/>
       <c r="J117" s="20" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="K117" s="20"/>
       <c r="L117" s="20" t="s">
@@ -7691,10 +7698,10 @@
     </row>
     <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="17" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B118" s="17" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C118" s="17" t="s">
         <v>29</v>
@@ -7716,29 +7723,29 @@
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="18" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D119" s="20" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E119" s="20" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F119" s="20" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="G119" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="20" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="I119" s="20"/>
       <c r="J119" s="20" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="K119" s="20"/>
       <c r="L119" s="20" t="s">
@@ -7748,35 +7755,35 @@
         <v>39</v>
       </c>
       <c r="N119" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="18" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D120" s="20" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E120" s="20" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F120" s="20" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G120" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="20" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="I120" s="20"/>
       <c r="J120" s="20" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="K120" s="20"/>
       <c r="L120" s="20" t="s">
@@ -7786,35 +7793,35 @@
         <v>39</v>
       </c>
       <c r="N120" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
       <c r="B121" s="18" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="C121" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D121" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E121" s="20" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="F121" s="20" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="G121" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="20" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="I121" s="20"/>
       <c r="J121" s="20" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="K121" s="20"/>
       <c r="L121" s="20" t="s">
@@ -7824,35 +7831,35 @@
         <v>39</v>
       </c>
       <c r="N121" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="18" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D122" s="20" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E122" s="20" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F122" s="20" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="G122" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="20" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="I122" s="20"/>
       <c r="J122" s="20" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="K122" s="20"/>
       <c r="L122" s="20" t="s">
@@ -7862,35 +7869,35 @@
         <v>39</v>
       </c>
       <c r="N122" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="18" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D123" s="20" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E123" s="20" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="F123" s="20" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="G123" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H123" s="20" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I123" s="20"/>
       <c r="J123" s="20" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="K123" s="20"/>
       <c r="L123" s="20" t="s">
@@ -7900,35 +7907,35 @@
         <v>39</v>
       </c>
       <c r="N123" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="18" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D124" s="20" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F124" s="20" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="G124" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H124" s="20" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="I124" s="20"/>
       <c r="J124" s="20" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="K124" s="20"/>
       <c r="L124" s="20" t="s">
@@ -7938,35 +7945,35 @@
         <v>39</v>
       </c>
       <c r="N124" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="18" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D125" s="20" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E125" s="20" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F125" s="20" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G125" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H125" s="20" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="I125" s="20"/>
       <c r="J125" s="20" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="K125" s="20"/>
       <c r="L125" s="20" t="s">
@@ -7976,35 +7983,35 @@
         <v>39</v>
       </c>
       <c r="N125" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="18" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D126" s="20" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E126" s="20" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="F126" s="20" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="G126" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="20" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="I126" s="20"/>
       <c r="J126" s="20" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="K126" s="20"/>
       <c r="L126" s="20" t="s">
@@ -8014,15 +8021,15 @@
         <v>39</v>
       </c>
       <c r="N126" s="20" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="17" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B127" s="17" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C127" s="17" t="s">
         <v>29</v>
@@ -8044,29 +8051,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="18" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D128" s="20" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E128" s="20" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="F128" s="20" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G128" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="20" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="I128" s="20"/>
       <c r="J128" s="20" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K128" s="20"/>
       <c r="L128" s="20" t="s">
@@ -8076,35 +8083,35 @@
         <v>39</v>
       </c>
       <c r="N128" s="20" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="24"/>
       <c r="B129" s="25" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C129" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D129" s="26" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E129" s="26" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="F129" s="26" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G129" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="26" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="I129" s="26"/>
       <c r="J129" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K129" s="26"/>
       <c r="L129" s="26" t="s">
@@ -8114,35 +8121,35 @@
         <v>39</v>
       </c>
       <c r="N129" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="24"/>
       <c r="B130" s="25" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C130" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D130" s="26" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E130" s="26" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F130" s="26" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="G130" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="26" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="I130" s="26"/>
       <c r="J130" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K130" s="26"/>
       <c r="L130" s="26" t="s">
@@ -8152,35 +8159,35 @@
         <v>39</v>
       </c>
       <c r="N130" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="24"/>
       <c r="B131" s="25" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C131" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D131" s="26" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E131" s="26" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="F131" s="26" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="G131" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H131" s="26" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="I131" s="26"/>
       <c r="J131" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K131" s="26"/>
       <c r="L131" s="26" t="s">
@@ -8190,35 +8197,35 @@
         <v>39</v>
       </c>
       <c r="N131" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="24"/>
       <c r="B132" s="25" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C132" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D132" s="26" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E132" s="26" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F132" s="26" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G132" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="26" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="I132" s="26"/>
       <c r="J132" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K132" s="26"/>
       <c r="L132" s="26" t="s">
@@ -8228,35 +8235,35 @@
         <v>39</v>
       </c>
       <c r="N132" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="24"/>
       <c r="B133" s="25" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C133" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D133" s="26" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E133" s="26" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="F133" s="26" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="G133" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H133" s="26" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="I133" s="26"/>
       <c r="J133" s="26" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="K133" s="26"/>
       <c r="L133" s="26" t="s">
@@ -8266,35 +8273,35 @@
         <v>39</v>
       </c>
       <c r="N133" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="24"/>
       <c r="B134" s="25" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C134" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D134" s="26" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="E134" s="26" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="F134" s="26" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="G134" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="26" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="I134" s="26"/>
       <c r="J134" s="26" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="K134" s="26"/>
       <c r="L134" s="26" t="s">
@@ -8304,35 +8311,35 @@
         <v>39</v>
       </c>
       <c r="N134" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="24"/>
       <c r="B135" s="25" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C135" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D135" s="26" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E135" s="26" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F135" s="26" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="G135" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H135" s="26" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="I135" s="26"/>
       <c r="J135" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K135" s="26"/>
       <c r="L135" s="26" t="s">
@@ -8342,35 +8349,35 @@
         <v>39</v>
       </c>
       <c r="N135" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="24"/>
       <c r="B136" s="25" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C136" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D136" s="26" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E136" s="26" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="F136" s="26" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G136" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H136" s="26" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="I136" s="26"/>
       <c r="J136" s="26" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="K136" s="26"/>
       <c r="L136" s="26" t="s">
@@ -8380,35 +8387,35 @@
         <v>39</v>
       </c>
       <c r="N136" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="24"/>
       <c r="B137" s="25" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C137" s="24" t="s">
         <v>42</v>
       </c>
       <c r="D137" s="26" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="E137" s="26" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F137" s="26" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="G137" s="26" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H137" s="26" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="I137" s="26"/>
       <c r="J137" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K137" s="26"/>
       <c r="L137" s="26" t="s">
@@ -8418,35 +8425,35 @@
         <v>39</v>
       </c>
       <c r="N137" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="24"/>
       <c r="B138" s="25" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C138" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D138" s="26" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="E138" s="26" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F138" s="26" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="G138" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="26" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="I138" s="26"/>
       <c r="J138" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K138" s="26"/>
       <c r="L138" s="26" t="s">
@@ -8456,35 +8463,35 @@
         <v>39</v>
       </c>
       <c r="N138" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="24"/>
       <c r="B139" s="25" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C139" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D139" s="26" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E139" s="26" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F139" s="26" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="G139" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="26" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="I139" s="26"/>
       <c r="J139" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K139" s="26"/>
       <c r="L139" s="26" t="s">
@@ -8494,35 +8501,35 @@
         <v>39</v>
       </c>
       <c r="N139" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="24"/>
       <c r="B140" s="25" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C140" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D140" s="26" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="E140" s="26" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="F140" s="26" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="G140" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="26" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="I140" s="26"/>
       <c r="J140" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K140" s="26"/>
       <c r="L140" s="26" t="s">
@@ -8532,35 +8539,35 @@
         <v>39</v>
       </c>
       <c r="N140" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="24"/>
       <c r="B141" s="25" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C141" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D141" s="26" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E141" s="26" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F141" s="26" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="G141" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="26" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="I141" s="26"/>
       <c r="J141" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K141" s="26"/>
       <c r="L141" s="26" t="s">
@@ -8570,35 +8577,35 @@
         <v>39</v>
       </c>
       <c r="N141" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="24"/>
       <c r="B142" s="25" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C142" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D142" s="26" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="E142" s="26" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="F142" s="26" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="G142" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="26" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="I142" s="26"/>
       <c r="J142" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K142" s="26"/>
       <c r="L142" s="26" t="s">
@@ -8608,35 +8615,35 @@
         <v>39</v>
       </c>
       <c r="N142" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="24"/>
       <c r="B143" s="25" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="C143" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D143" s="26" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="E143" s="26" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="F143" s="26" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="G143" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="26" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="I143" s="26"/>
       <c r="J143" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K143" s="26"/>
       <c r="L143" s="26" t="s">
@@ -8646,35 +8653,35 @@
         <v>39</v>
       </c>
       <c r="N143" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="24"/>
       <c r="B144" s="25" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C144" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D144" s="26" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E144" s="26" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="F144" s="26" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="G144" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H144" s="26" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="I144" s="26"/>
       <c r="J144" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K144" s="26"/>
       <c r="L144" s="26" t="s">
@@ -8684,35 +8691,35 @@
         <v>39</v>
       </c>
       <c r="N144" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="24"/>
       <c r="B145" s="25" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C145" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D145" s="26" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E145" s="26" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="F145" s="26" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="G145" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="26" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="I145" s="26"/>
       <c r="J145" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K145" s="26"/>
       <c r="L145" s="26" t="s">
@@ -8722,35 +8729,35 @@
         <v>39</v>
       </c>
       <c r="N145" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="24"/>
       <c r="B146" s="25" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C146" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D146" s="26" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="E146" s="26" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="F146" s="26" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="G146" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="26" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="I146" s="26"/>
       <c r="J146" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K146" s="26"/>
       <c r="L146" s="26" t="s">
@@ -8760,35 +8767,35 @@
         <v>39</v>
       </c>
       <c r="N146" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="24"/>
       <c r="B147" s="25" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C147" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D147" s="26" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="E147" s="26" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="F147" s="26" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="G147" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="26" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="I147" s="26"/>
       <c r="J147" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K147" s="26"/>
       <c r="L147" s="26" t="s">
@@ -8798,35 +8805,35 @@
         <v>39</v>
       </c>
       <c r="N147" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="24"/>
       <c r="B148" s="25" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C148" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D148" s="26" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="E148" s="26" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="F148" s="26" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="G148" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="26" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="I148" s="26"/>
       <c r="J148" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K148" s="26"/>
       <c r="L148" s="26" t="s">
@@ -8836,35 +8843,35 @@
         <v>39</v>
       </c>
       <c r="N148" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="24"/>
       <c r="B149" s="25" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C149" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D149" s="26" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="E149" s="26" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="F149" s="26" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="G149" s="26" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="26" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="I149" s="26"/>
       <c r="J149" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K149" s="26"/>
       <c r="L149" s="26" t="s">
@@ -8874,35 +8881,35 @@
         <v>39</v>
       </c>
       <c r="N149" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="24"/>
       <c r="B150" s="25" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="C150" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D150" s="26" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="E150" s="26" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="F150" s="26" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="G150" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H150" s="26" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="I150" s="26"/>
       <c r="J150" s="26" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="K150" s="26"/>
       <c r="L150" s="26" t="s">
@@ -8912,35 +8919,35 @@
         <v>39</v>
       </c>
       <c r="N150" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="24"/>
       <c r="B151" s="25" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C151" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D151" s="26" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="E151" s="26" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="F151" s="26" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="G151" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H151" s="26" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="I151" s="26"/>
       <c r="J151" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K151" s="26"/>
       <c r="L151" s="26" t="s">
@@ -8950,35 +8957,35 @@
         <v>39</v>
       </c>
       <c r="N151" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="24"/>
       <c r="B152" s="25" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="C152" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D152" s="26" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="E152" s="26" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="F152" s="26" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="G152" s="26" t="s">
         <v>132</v>
       </c>
       <c r="H152" s="26" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="I152" s="26"/>
       <c r="J152" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K152" s="26"/>
       <c r="L152" s="26" t="s">
@@ -8988,35 +8995,35 @@
         <v>39</v>
       </c>
       <c r="N152" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="24"/>
       <c r="B153" s="25" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="C153" s="24" t="s">
         <v>42</v>
       </c>
       <c r="D153" s="26" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="E153" s="26" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="F153" s="26" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="G153" s="26" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H153" s="26" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="I153" s="26"/>
       <c r="J153" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K153" s="26"/>
       <c r="L153" s="26" t="s">
@@ -9026,7 +9033,7 @@
         <v>39</v>
       </c>
       <c r="N153" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>
@@ -9059,51 +9066,51 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="C1" s="28" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="D1" s="28" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="E1" s="28" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="F1" s="28" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="G1" s="28" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="28" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C2" s="31" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="D2" s="31" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E2" s="31" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="F2" s="31" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="G2" s="31" t="s">
         <v>36</v>
@@ -9112,27 +9119,27 @@
         <v>39</v>
       </c>
       <c r="I2" s="32" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E3" s="34" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="F3" s="34" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="G3" s="34" t="s">
         <v>36</v>
@@ -9141,27 +9148,27 @@
         <v>39</v>
       </c>
       <c r="I3" s="35" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E4" s="34" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="G4" s="34" t="s">
         <v>36</v>
@@ -9170,27 +9177,27 @@
         <v>39</v>
       </c>
       <c r="I4" s="35" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="D5" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E5" s="34" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="F5" s="34" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="G5" s="34" t="s">
         <v>36</v>
@@ -9199,27 +9206,27 @@
         <v>39</v>
       </c>
       <c r="I5" s="35" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="D6" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E6" s="34" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="F6" s="34" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="G6" s="34" t="s">
         <v>36</v>
@@ -9228,27 +9235,27 @@
         <v>39</v>
       </c>
       <c r="I6" s="35" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B7" s="34" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E7" s="34" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="F7" s="34" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="G7" s="34" t="s">
         <v>36</v>
@@ -9257,27 +9264,27 @@
         <v>39</v>
       </c>
       <c r="I7" s="35" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E8" s="34" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="F8" s="34" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="G8" s="34" t="s">
         <v>36</v>
@@ -9286,27 +9293,27 @@
         <v>39</v>
       </c>
       <c r="I8" s="35" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="F9" s="34" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="G9" s="34" t="s">
         <v>36</v>
@@ -9315,27 +9322,27 @@
         <v>39</v>
       </c>
       <c r="I9" s="35" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="36" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="G10" s="37" t="s">
         <v>36</v>
@@ -9344,25 +9351,25 @@
         <v>39</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="39" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="B11" s="40"/>
       <c r="C11" s="40" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E11" s="40" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F11" s="40" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="G11" s="40" t="s">
         <v>36</v>
@@ -9371,25 +9378,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="41" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="42" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B12" s="43"/>
       <c r="C12" s="43" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="D12" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F12" s="43" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="G12" s="43" t="s">
         <v>36</v>
@@ -9398,25 +9405,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="44" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B13" s="43"/>
       <c r="C13" s="43" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="D13" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F13" s="43" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="G13" s="43" t="s">
         <v>36</v>
@@ -9425,25 +9432,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="44" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="42" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="B14" s="43"/>
       <c r="C14" s="43" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="D14" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F14" s="43" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="G14" s="43" t="s">
         <v>36</v>
@@ -9452,25 +9459,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="44" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="42" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="B15" s="43"/>
       <c r="C15" s="43" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="D15" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E15" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F15" s="43" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="G15" s="43" t="s">
         <v>36</v>
@@ -9479,25 +9486,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="44" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="42" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="B16" s="43"/>
       <c r="C16" s="43" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D16" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E16" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F16" s="43" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="G16" s="43" t="s">
         <v>36</v>
@@ -9506,25 +9513,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="44" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="42" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="B17" s="43"/>
       <c r="C17" s="43" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="D17" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E17" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F17" s="43" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="G17" s="43" t="s">
         <v>36</v>
@@ -9533,25 +9540,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="44" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="42" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="B18" s="43"/>
       <c r="C18" s="43" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="D18" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E18" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F18" s="43" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="G18" s="43" t="s">
         <v>36</v>
@@ -9560,25 +9567,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="44" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="42" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B19" s="43"/>
       <c r="C19" s="43" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="D19" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E19" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F19" s="43" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="G19" s="43" t="s">
         <v>36</v>
@@ -9587,25 +9594,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="44" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="42" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B20" s="43"/>
       <c r="C20" s="43" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="D20" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E20" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F20" s="43" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="G20" s="43" t="s">
         <v>36</v>
@@ -9614,25 +9621,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="44" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="42" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="B21" s="43"/>
       <c r="C21" s="43" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="D21" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E21" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F21" s="43" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="G21" s="43" t="s">
         <v>36</v>
@@ -9641,25 +9648,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="44" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="42" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="43" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="D22" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E22" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F22" s="43" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="G22" s="43" t="s">
         <v>36</v>
@@ -9668,25 +9675,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="44" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="42" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="B23" s="43"/>
       <c r="C23" s="43" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="D23" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E23" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F23" s="43" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="G23" s="43" t="s">
         <v>36</v>
@@ -9695,25 +9702,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="44" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="42" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="B24" s="43"/>
       <c r="C24" s="43" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="D24" s="43" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E24" s="43" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F24" s="43" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="G24" s="43" t="s">
         <v>36</v>
@@ -9722,25 +9729,25 @@
         <v>36</v>
       </c>
       <c r="I24" s="44" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="45" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="B25" s="46"/>
       <c r="C25" s="46" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="D25" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E25" s="46" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F25" s="46" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="G25" s="46" t="s">
         <v>36</v>
@@ -9749,25 +9756,25 @@
         <v>36</v>
       </c>
       <c r="I25" s="47" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="45" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="B26" s="46"/>
       <c r="C26" s="46" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E26" s="46" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="F26" s="46" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="G26" s="46" t="s">
         <v>36</v>
@@ -9776,25 +9783,25 @@
         <v>36</v>
       </c>
       <c r="I26" s="47" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="45" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="B27" s="46"/>
       <c r="C27" s="46" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="D27" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E27" s="46" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="F27" s="46" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="G27" s="46" t="s">
         <v>36</v>
@@ -9803,25 +9810,25 @@
         <v>36</v>
       </c>
       <c r="I27" s="47" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="45" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B28" s="46"/>
       <c r="C28" s="46" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="D28" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E28" s="46" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="F28" s="46" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="G28" s="46" t="s">
         <v>36</v>
@@ -9830,25 +9837,25 @@
         <v>36</v>
       </c>
       <c r="I28" s="47" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="45" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B29" s="46"/>
       <c r="C29" s="46" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="D29" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E29" s="46" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="F29" s="46" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="G29" s="46" t="s">
         <v>36</v>
@@ -9857,25 +9864,25 @@
         <v>36</v>
       </c>
       <c r="I29" s="47" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="45" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E30" s="46" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="F30" s="46" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="G30" s="46" t="s">
         <v>36</v>
@@ -9884,25 +9891,25 @@
         <v>36</v>
       </c>
       <c r="I30" s="47" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="45" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B31" s="46"/>
       <c r="C31" s="46" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="D31" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E31" s="46" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="F31" s="46" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="G31" s="46" t="s">
         <v>36</v>
@@ -9911,25 +9918,25 @@
         <v>36</v>
       </c>
       <c r="I31" s="47" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="45" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="B32" s="46"/>
       <c r="C32" s="46" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="D32" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E32" s="46" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="F32" s="46" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="G32" s="46" t="s">
         <v>36</v>
@@ -9938,25 +9945,25 @@
         <v>36</v>
       </c>
       <c r="I32" s="47" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="45" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="B33" s="46"/>
       <c r="C33" s="46" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="D33" s="46" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="E33" s="46" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="F33" s="46" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="G33" s="46" t="s">
         <v>36</v>
@@ -9965,7 +9972,7 @@
         <v>36</v>
       </c>
       <c r="I33" s="47" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: correct Stage 6 Pass 007 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -2839,7 +2839,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -2888,12 +2888,6 @@
     <font>
       <b/>
       <color rgb="FF000000"/>
-      <sz val="10"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF9C0006"/>
       <sz val="10"/>
       <name val="Carlito"/>
     </font>
@@ -3182,7 +3176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3228,31 +3222,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4125,40 +4104,40 @@
       </c>
     </row>
     <row r="19" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22" t="s">
+      <c r="A19" s="19"/>
+      <c r="B19" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="G19" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="23" t="s">
+      <c r="G19" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23" t="s">
+      <c r="I19" s="21"/>
+      <c r="J19" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M19" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N19" s="23" t="s">
+      <c r="K19" s="21"/>
+      <c r="L19" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M19" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N19" s="21" t="s">
         <v>40</v>
       </c>
     </row>
@@ -4369,40 +4348,40 @@
       </c>
     </row>
     <row r="26" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A26" s="22"/>
-      <c r="B26" s="22" t="s">
+      <c r="A26" s="19"/>
+      <c r="B26" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="D26" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="E26" s="23" t="s">
+      <c r="E26" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="F26" s="23" t="s">
+      <c r="F26" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="G26" s="23" t="s">
+      <c r="G26" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="H26" s="23" t="s">
+      <c r="H26" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23" t="s">
+      <c r="I26" s="21"/>
+      <c r="J26" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="K26" s="23"/>
-      <c r="L26" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M26" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N26" s="23" t="s">
+      <c r="K26" s="21"/>
+      <c r="L26" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M26" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N26" s="21" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4799,40 +4778,40 @@
       </c>
     </row>
     <row r="38" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A38" s="22"/>
-      <c r="B38" s="22" t="s">
+      <c r="A38" s="19"/>
+      <c r="B38" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="C38" s="22" t="s">
+      <c r="C38" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D38" s="23" t="s">
+      <c r="D38" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E38" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="F38" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="G38" s="23" t="s">
+      <c r="G38" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="H38" s="23" t="s">
+      <c r="H38" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="I38" s="23"/>
-      <c r="J38" s="23" t="s">
+      <c r="I38" s="21"/>
+      <c r="J38" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="K38" s="23"/>
-      <c r="L38" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M38" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N38" s="23" t="s">
+      <c r="K38" s="21"/>
+      <c r="L38" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M38" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N38" s="21" t="s">
         <v>112</v>
       </c>
     </row>
@@ -5121,38 +5100,38 @@
       </c>
     </row>
     <row r="47" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A47" s="22"/>
-      <c r="B47" s="22" t="s">
+      <c r="A47" s="19"/>
+      <c r="B47" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="C47" s="22" t="s">
+      <c r="C47" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D47" s="23" t="s">
+      <c r="D47" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="E47" s="23" t="s">
+      <c r="E47" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F47" s="23" t="s">
+      <c r="F47" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="G47" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H47" s="23" t="s">
+      <c r="G47" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="I47" s="23"/>
-      <c r="J47" s="23"/>
-      <c r="K47" s="23"/>
-      <c r="L47" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M47" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N47" s="23" t="s">
+      <c r="I47" s="21"/>
+      <c r="J47" s="21"/>
+      <c r="K47" s="21"/>
+      <c r="L47" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M47" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N47" s="21" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5481,40 +5460,40 @@
       </c>
     </row>
     <row r="57" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A57" s="22"/>
-      <c r="B57" s="22" t="s">
+      <c r="A57" s="19"/>
+      <c r="B57" s="19" t="s">
         <v>290</v>
       </c>
-      <c r="C57" s="22" t="s">
+      <c r="C57" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D57" s="23" t="s">
+      <c r="D57" s="21" t="s">
         <v>291</v>
       </c>
-      <c r="E57" s="23" t="s">
+      <c r="E57" s="21" t="s">
         <v>292</v>
       </c>
-      <c r="F57" s="23" t="s">
+      <c r="F57" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="G57" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H57" s="23" t="s">
+      <c r="G57" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="I57" s="23"/>
-      <c r="J57" s="23" t="s">
+      <c r="I57" s="21"/>
+      <c r="J57" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="K57" s="23"/>
-      <c r="L57" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M57" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N57" s="23" t="s">
+      <c r="K57" s="21"/>
+      <c r="L57" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M57" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N57" s="21" t="s">
         <v>209</v>
       </c>
     </row>
@@ -6021,40 +6000,40 @@
       </c>
     </row>
     <row r="72" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A72" s="22"/>
-      <c r="B72" s="22" t="s">
+      <c r="A72" s="19"/>
+      <c r="B72" s="19" t="s">
         <v>368</v>
       </c>
-      <c r="C72" s="22" t="s">
+      <c r="C72" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="D72" s="23" t="s">
+      <c r="D72" s="21" t="s">
         <v>369</v>
       </c>
-      <c r="E72" s="23" t="s">
+      <c r="E72" s="21" t="s">
         <v>370</v>
       </c>
-      <c r="F72" s="23" t="s">
+      <c r="F72" s="21" t="s">
         <v>371</v>
       </c>
-      <c r="G72" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H72" s="23" t="s">
+      <c r="G72" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H72" s="21" t="s">
         <v>372</v>
       </c>
-      <c r="I72" s="23"/>
-      <c r="J72" s="23" t="s">
+      <c r="I72" s="21"/>
+      <c r="J72" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="K72" s="23"/>
-      <c r="L72" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M72" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N72" s="23" t="s">
+      <c r="K72" s="21"/>
+      <c r="L72" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M72" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N72" s="21" t="s">
         <v>308</v>
       </c>
     </row>
@@ -6705,40 +6684,40 @@
       </c>
     </row>
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A91" s="22"/>
-      <c r="B91" s="22" t="s">
+      <c r="A91" s="19"/>
+      <c r="B91" s="19" t="s">
         <v>462</v>
       </c>
-      <c r="C91" s="22" t="s">
+      <c r="C91" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="D91" s="23" t="s">
+      <c r="D91" s="21" t="s">
         <v>463</v>
       </c>
-      <c r="E91" s="23" t="s">
+      <c r="E91" s="21" t="s">
         <v>464</v>
       </c>
-      <c r="F91" s="23" t="s">
+      <c r="F91" s="21" t="s">
         <v>465</v>
       </c>
-      <c r="G91" s="23" t="s">
+      <c r="G91" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="H91" s="23" t="s">
+      <c r="H91" s="21" t="s">
         <v>466</v>
       </c>
-      <c r="I91" s="23"/>
-      <c r="J91" s="23" t="s">
+      <c r="I91" s="21"/>
+      <c r="J91" s="21" t="s">
         <v>467</v>
       </c>
-      <c r="K91" s="23"/>
-      <c r="L91" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M91" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N91" s="23" t="s">
+      <c r="K91" s="21"/>
+      <c r="L91" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M91" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N91" s="21" t="s">
         <v>468</v>
       </c>
     </row>
@@ -7027,40 +7006,40 @@
       <c r="N99" s="17"/>
     </row>
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A100" s="22"/>
-      <c r="B100" s="22" t="s">
+      <c r="A100" s="19"/>
+      <c r="B100" s="19" t="s">
         <v>506</v>
       </c>
-      <c r="C100" s="22" t="s">
+      <c r="C100" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D100" s="23" t="s">
+      <c r="D100" s="21" t="s">
         <v>507</v>
       </c>
-      <c r="E100" s="23" t="s">
+      <c r="E100" s="21" t="s">
         <v>508</v>
       </c>
-      <c r="F100" s="23" t="s">
+      <c r="F100" s="21" t="s">
         <v>509</v>
       </c>
-      <c r="G100" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H100" s="23" t="s">
+      <c r="G100" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H100" s="21" t="s">
         <v>510</v>
       </c>
-      <c r="I100" s="23"/>
-      <c r="J100" s="23" t="s">
+      <c r="I100" s="21"/>
+      <c r="J100" s="21" t="s">
         <v>511</v>
       </c>
-      <c r="K100" s="23"/>
-      <c r="L100" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M100" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N100" s="23" t="s">
+      <c r="K100" s="21"/>
+      <c r="L100" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M100" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N100" s="21" t="s">
         <v>512</v>
       </c>
     </row>
@@ -7621,40 +7600,40 @@
       </c>
     </row>
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A116" s="22"/>
-      <c r="B116" s="22" t="s">
+      <c r="A116" s="19"/>
+      <c r="B116" s="19" t="s">
         <v>588</v>
       </c>
-      <c r="C116" s="22" t="s">
+      <c r="C116" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="D116" s="23" t="s">
+      <c r="D116" s="21" t="s">
         <v>589</v>
       </c>
-      <c r="E116" s="23" t="s">
+      <c r="E116" s="21" t="s">
         <v>590</v>
       </c>
-      <c r="F116" s="23" t="s">
+      <c r="F116" s="21" t="s">
         <v>591</v>
       </c>
-      <c r="G116" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="H116" s="23" t="s">
+      <c r="G116" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="H116" s="21" t="s">
         <v>592</v>
       </c>
-      <c r="I116" s="23"/>
-      <c r="J116" s="23" t="s">
+      <c r="I116" s="21"/>
+      <c r="J116" s="21" t="s">
         <v>577</v>
       </c>
-      <c r="K116" s="23"/>
-      <c r="L116" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M116" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="N116" s="23" t="s">
+      <c r="K116" s="21"/>
+      <c r="L116" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="M116" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="N116" s="21" t="s">
         <v>40</v>
       </c>
     </row>
@@ -8087,952 +8066,952 @@
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A129" s="24"/>
-      <c r="B129" s="25" t="s">
+      <c r="A129" s="18"/>
+      <c r="B129" s="19" t="s">
         <v>654</v>
       </c>
-      <c r="C129" s="24" t="s">
+      <c r="C129" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D129" s="26" t="s">
+      <c r="D129" s="20" t="s">
         <v>655</v>
       </c>
-      <c r="E129" s="26" t="s">
+      <c r="E129" s="20" t="s">
         <v>656</v>
       </c>
-      <c r="F129" s="26" t="s">
+      <c r="F129" s="20" t="s">
         <v>657</v>
       </c>
-      <c r="G129" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H129" s="26" t="s">
+      <c r="G129" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H129" s="20" t="s">
         <v>658</v>
       </c>
-      <c r="I129" s="26"/>
-      <c r="J129" s="26" t="s">
+      <c r="I129" s="20"/>
+      <c r="J129" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K129" s="26"/>
-      <c r="L129" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M129" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N129" s="26" t="s">
+      <c r="K129" s="20"/>
+      <c r="L129" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M129" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N129" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A130" s="24"/>
-      <c r="B130" s="25" t="s">
+      <c r="A130" s="18"/>
+      <c r="B130" s="19" t="s">
         <v>659</v>
       </c>
-      <c r="C130" s="24" t="s">
+      <c r="C130" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D130" s="26" t="s">
+      <c r="D130" s="20" t="s">
         <v>660</v>
       </c>
-      <c r="E130" s="26" t="s">
+      <c r="E130" s="20" t="s">
         <v>661</v>
       </c>
-      <c r="F130" s="26" t="s">
+      <c r="F130" s="20" t="s">
         <v>662</v>
       </c>
-      <c r="G130" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H130" s="26" t="s">
+      <c r="G130" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H130" s="20" t="s">
         <v>663</v>
       </c>
-      <c r="I130" s="26"/>
-      <c r="J130" s="26" t="s">
+      <c r="I130" s="20"/>
+      <c r="J130" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K130" s="26"/>
-      <c r="L130" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M130" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N130" s="26" t="s">
+      <c r="K130" s="20"/>
+      <c r="L130" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M130" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N130" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A131" s="24"/>
-      <c r="B131" s="25" t="s">
+      <c r="A131" s="18"/>
+      <c r="B131" s="19" t="s">
         <v>664</v>
       </c>
-      <c r="C131" s="24" t="s">
+      <c r="C131" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D131" s="26" t="s">
+      <c r="D131" s="20" t="s">
         <v>665</v>
       </c>
-      <c r="E131" s="26" t="s">
+      <c r="E131" s="20" t="s">
         <v>666</v>
       </c>
-      <c r="F131" s="26" t="s">
+      <c r="F131" s="20" t="s">
         <v>667</v>
       </c>
-      <c r="G131" s="26" t="s">
+      <c r="G131" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H131" s="26" t="s">
+      <c r="H131" s="20" t="s">
         <v>668</v>
       </c>
-      <c r="I131" s="26"/>
-      <c r="J131" s="26" t="s">
+      <c r="I131" s="20"/>
+      <c r="J131" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K131" s="26"/>
-      <c r="L131" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M131" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N131" s="26" t="s">
+      <c r="K131" s="20"/>
+      <c r="L131" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M131" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N131" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A132" s="24"/>
-      <c r="B132" s="25" t="s">
+      <c r="A132" s="18"/>
+      <c r="B132" s="19" t="s">
         <v>669</v>
       </c>
-      <c r="C132" s="24" t="s">
+      <c r="C132" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D132" s="26" t="s">
+      <c r="D132" s="20" t="s">
         <v>670</v>
       </c>
-      <c r="E132" s="26" t="s">
+      <c r="E132" s="20" t="s">
         <v>671</v>
       </c>
-      <c r="F132" s="26" t="s">
+      <c r="F132" s="20" t="s">
         <v>672</v>
       </c>
-      <c r="G132" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H132" s="26" t="s">
+      <c r="G132" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H132" s="20" t="s">
         <v>673</v>
       </c>
-      <c r="I132" s="26"/>
-      <c r="J132" s="26" t="s">
+      <c r="I132" s="20"/>
+      <c r="J132" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K132" s="26"/>
-      <c r="L132" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M132" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N132" s="26" t="s">
+      <c r="K132" s="20"/>
+      <c r="L132" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M132" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N132" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A133" s="24"/>
-      <c r="B133" s="25" t="s">
+      <c r="A133" s="18"/>
+      <c r="B133" s="19" t="s">
         <v>674</v>
       </c>
-      <c r="C133" s="24" t="s">
+      <c r="C133" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D133" s="26" t="s">
+      <c r="D133" s="20" t="s">
         <v>675</v>
       </c>
-      <c r="E133" s="26" t="s">
+      <c r="E133" s="20" t="s">
         <v>676</v>
       </c>
-      <c r="F133" s="26" t="s">
+      <c r="F133" s="20" t="s">
         <v>677</v>
       </c>
-      <c r="G133" s="26" t="s">
+      <c r="G133" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H133" s="26" t="s">
+      <c r="H133" s="20" t="s">
         <v>678</v>
       </c>
-      <c r="I133" s="26"/>
-      <c r="J133" s="26" t="s">
+      <c r="I133" s="20"/>
+      <c r="J133" s="20" t="s">
         <v>679</v>
       </c>
-      <c r="K133" s="26"/>
-      <c r="L133" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M133" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N133" s="26" t="s">
+      <c r="K133" s="20"/>
+      <c r="L133" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M133" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N133" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A134" s="24"/>
-      <c r="B134" s="25" t="s">
+      <c r="A134" s="18"/>
+      <c r="B134" s="19" t="s">
         <v>680</v>
       </c>
-      <c r="C134" s="24" t="s">
+      <c r="C134" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D134" s="26" t="s">
+      <c r="D134" s="20" t="s">
         <v>681</v>
       </c>
-      <c r="E134" s="26" t="s">
+      <c r="E134" s="20" t="s">
         <v>682</v>
       </c>
-      <c r="F134" s="26" t="s">
+      <c r="F134" s="20" t="s">
         <v>683</v>
       </c>
-      <c r="G134" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H134" s="26" t="s">
+      <c r="G134" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H134" s="20" t="s">
         <v>684</v>
       </c>
-      <c r="I134" s="26"/>
-      <c r="J134" s="26" t="s">
+      <c r="I134" s="20"/>
+      <c r="J134" s="20" t="s">
         <v>685</v>
       </c>
-      <c r="K134" s="26"/>
-      <c r="L134" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M134" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N134" s="26" t="s">
+      <c r="K134" s="20"/>
+      <c r="L134" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M134" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N134" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A135" s="24"/>
-      <c r="B135" s="25" t="s">
+      <c r="A135" s="18"/>
+      <c r="B135" s="19" t="s">
         <v>686</v>
       </c>
-      <c r="C135" s="24" t="s">
+      <c r="C135" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D135" s="26" t="s">
+      <c r="D135" s="20" t="s">
         <v>687</v>
       </c>
-      <c r="E135" s="26" t="s">
+      <c r="E135" s="20" t="s">
         <v>688</v>
       </c>
-      <c r="F135" s="26" t="s">
+      <c r="F135" s="20" t="s">
         <v>689</v>
       </c>
-      <c r="G135" s="26" t="s">
+      <c r="G135" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H135" s="26" t="s">
+      <c r="H135" s="20" t="s">
         <v>690</v>
       </c>
-      <c r="I135" s="26"/>
-      <c r="J135" s="26" t="s">
+      <c r="I135" s="20"/>
+      <c r="J135" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K135" s="26"/>
-      <c r="L135" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M135" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N135" s="26" t="s">
+      <c r="K135" s="20"/>
+      <c r="L135" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M135" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N135" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A136" s="24"/>
-      <c r="B136" s="25" t="s">
+      <c r="A136" s="18"/>
+      <c r="B136" s="19" t="s">
         <v>691</v>
       </c>
-      <c r="C136" s="24" t="s">
+      <c r="C136" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D136" s="26" t="s">
+      <c r="D136" s="20" t="s">
         <v>692</v>
       </c>
-      <c r="E136" s="26" t="s">
+      <c r="E136" s="20" t="s">
         <v>693</v>
       </c>
-      <c r="F136" s="26" t="s">
+      <c r="F136" s="20" t="s">
         <v>694</v>
       </c>
-      <c r="G136" s="26" t="s">
+      <c r="G136" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H136" s="26" t="s">
+      <c r="H136" s="20" t="s">
         <v>695</v>
       </c>
-      <c r="I136" s="26"/>
-      <c r="J136" s="26" t="s">
+      <c r="I136" s="20"/>
+      <c r="J136" s="20" t="s">
         <v>696</v>
       </c>
-      <c r="K136" s="26"/>
-      <c r="L136" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M136" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N136" s="26" t="s">
+      <c r="K136" s="20"/>
+      <c r="L136" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M136" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N136" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A137" s="24"/>
-      <c r="B137" s="25" t="s">
+      <c r="A137" s="18"/>
+      <c r="B137" s="19" t="s">
         <v>697</v>
       </c>
-      <c r="C137" s="24" t="s">
+      <c r="C137" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D137" s="26" t="s">
+      <c r="D137" s="20" t="s">
         <v>698</v>
       </c>
-      <c r="E137" s="26" t="s">
+      <c r="E137" s="20" t="s">
         <v>699</v>
       </c>
-      <c r="F137" s="26" t="s">
+      <c r="F137" s="20" t="s">
         <v>700</v>
       </c>
-      <c r="G137" s="26" t="s">
+      <c r="G137" s="20" t="s">
         <v>430</v>
       </c>
-      <c r="H137" s="26" t="s">
+      <c r="H137" s="20" t="s">
         <v>701</v>
       </c>
-      <c r="I137" s="26"/>
-      <c r="J137" s="26" t="s">
+      <c r="I137" s="20"/>
+      <c r="J137" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K137" s="26"/>
-      <c r="L137" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M137" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N137" s="26" t="s">
+      <c r="K137" s="20"/>
+      <c r="L137" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M137" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N137" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A138" s="24"/>
-      <c r="B138" s="25" t="s">
+      <c r="A138" s="18"/>
+      <c r="B138" s="19" t="s">
         <v>702</v>
       </c>
-      <c r="C138" s="24" t="s">
+      <c r="C138" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D138" s="26" t="s">
+      <c r="D138" s="20" t="s">
         <v>703</v>
       </c>
-      <c r="E138" s="26" t="s">
+      <c r="E138" s="20" t="s">
         <v>704</v>
       </c>
-      <c r="F138" s="26" t="s">
+      <c r="F138" s="20" t="s">
         <v>705</v>
       </c>
-      <c r="G138" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H138" s="26" t="s">
+      <c r="G138" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H138" s="20" t="s">
         <v>706</v>
       </c>
-      <c r="I138" s="26"/>
-      <c r="J138" s="26" t="s">
+      <c r="I138" s="20"/>
+      <c r="J138" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K138" s="26"/>
-      <c r="L138" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M138" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N138" s="26" t="s">
+      <c r="K138" s="20"/>
+      <c r="L138" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M138" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N138" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A139" s="24"/>
-      <c r="B139" s="25" t="s">
+      <c r="A139" s="18"/>
+      <c r="B139" s="19" t="s">
         <v>707</v>
       </c>
-      <c r="C139" s="24" t="s">
+      <c r="C139" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D139" s="26" t="s">
+      <c r="D139" s="20" t="s">
         <v>708</v>
       </c>
-      <c r="E139" s="26" t="s">
+      <c r="E139" s="20" t="s">
         <v>709</v>
       </c>
-      <c r="F139" s="26" t="s">
+      <c r="F139" s="20" t="s">
         <v>710</v>
       </c>
-      <c r="G139" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H139" s="26" t="s">
+      <c r="G139" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H139" s="20" t="s">
         <v>711</v>
       </c>
-      <c r="I139" s="26"/>
-      <c r="J139" s="26" t="s">
+      <c r="I139" s="20"/>
+      <c r="J139" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K139" s="26"/>
-      <c r="L139" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M139" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N139" s="26" t="s">
+      <c r="K139" s="20"/>
+      <c r="L139" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M139" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N139" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A140" s="24"/>
-      <c r="B140" s="25" t="s">
+      <c r="A140" s="18"/>
+      <c r="B140" s="19" t="s">
         <v>712</v>
       </c>
-      <c r="C140" s="24" t="s">
+      <c r="C140" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D140" s="26" t="s">
+      <c r="D140" s="20" t="s">
         <v>713</v>
       </c>
-      <c r="E140" s="26" t="s">
+      <c r="E140" s="20" t="s">
         <v>714</v>
       </c>
-      <c r="F140" s="26" t="s">
+      <c r="F140" s="20" t="s">
         <v>715</v>
       </c>
-      <c r="G140" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H140" s="26" t="s">
+      <c r="G140" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H140" s="20" t="s">
         <v>716</v>
       </c>
-      <c r="I140" s="26"/>
-      <c r="J140" s="26" t="s">
+      <c r="I140" s="20"/>
+      <c r="J140" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K140" s="26"/>
-      <c r="L140" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M140" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N140" s="26" t="s">
+      <c r="K140" s="20"/>
+      <c r="L140" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M140" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N140" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A141" s="24"/>
-      <c r="B141" s="25" t="s">
+      <c r="A141" s="18"/>
+      <c r="B141" s="19" t="s">
         <v>717</v>
       </c>
-      <c r="C141" s="24" t="s">
+      <c r="C141" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D141" s="26" t="s">
+      <c r="D141" s="20" t="s">
         <v>718</v>
       </c>
-      <c r="E141" s="26" t="s">
+      <c r="E141" s="20" t="s">
         <v>719</v>
       </c>
-      <c r="F141" s="26" t="s">
+      <c r="F141" s="20" t="s">
         <v>720</v>
       </c>
-      <c r="G141" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H141" s="26" t="s">
+      <c r="G141" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H141" s="20" t="s">
         <v>721</v>
       </c>
-      <c r="I141" s="26"/>
-      <c r="J141" s="26" t="s">
+      <c r="I141" s="20"/>
+      <c r="J141" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K141" s="26"/>
-      <c r="L141" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M141" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N141" s="26" t="s">
+      <c r="K141" s="20"/>
+      <c r="L141" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M141" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N141" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A142" s="24"/>
-      <c r="B142" s="25" t="s">
+      <c r="A142" s="18"/>
+      <c r="B142" s="19" t="s">
         <v>722</v>
       </c>
-      <c r="C142" s="24" t="s">
+      <c r="C142" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D142" s="26" t="s">
+      <c r="D142" s="20" t="s">
         <v>723</v>
       </c>
-      <c r="E142" s="26" t="s">
+      <c r="E142" s="20" t="s">
         <v>724</v>
       </c>
-      <c r="F142" s="26" t="s">
+      <c r="F142" s="20" t="s">
         <v>725</v>
       </c>
-      <c r="G142" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H142" s="26" t="s">
+      <c r="G142" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H142" s="20" t="s">
         <v>726</v>
       </c>
-      <c r="I142" s="26"/>
-      <c r="J142" s="26" t="s">
+      <c r="I142" s="20"/>
+      <c r="J142" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K142" s="26"/>
-      <c r="L142" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M142" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N142" s="26" t="s">
+      <c r="K142" s="20"/>
+      <c r="L142" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M142" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N142" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A143" s="24"/>
-      <c r="B143" s="25" t="s">
+      <c r="A143" s="18"/>
+      <c r="B143" s="19" t="s">
         <v>727</v>
       </c>
-      <c r="C143" s="24" t="s">
+      <c r="C143" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D143" s="26" t="s">
+      <c r="D143" s="20" t="s">
         <v>728</v>
       </c>
-      <c r="E143" s="26" t="s">
+      <c r="E143" s="20" t="s">
         <v>729</v>
       </c>
-      <c r="F143" s="26" t="s">
+      <c r="F143" s="20" t="s">
         <v>730</v>
       </c>
-      <c r="G143" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H143" s="26" t="s">
+      <c r="G143" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H143" s="20" t="s">
         <v>731</v>
       </c>
-      <c r="I143" s="26"/>
-      <c r="J143" s="26" t="s">
+      <c r="I143" s="20"/>
+      <c r="J143" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K143" s="26"/>
-      <c r="L143" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M143" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N143" s="26" t="s">
+      <c r="K143" s="20"/>
+      <c r="L143" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M143" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N143" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A144" s="24"/>
-      <c r="B144" s="25" t="s">
+      <c r="A144" s="18"/>
+      <c r="B144" s="19" t="s">
         <v>732</v>
       </c>
-      <c r="C144" s="24" t="s">
+      <c r="C144" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D144" s="26" t="s">
+      <c r="D144" s="20" t="s">
         <v>733</v>
       </c>
-      <c r="E144" s="26" t="s">
+      <c r="E144" s="20" t="s">
         <v>734</v>
       </c>
-      <c r="F144" s="26" t="s">
+      <c r="F144" s="20" t="s">
         <v>735</v>
       </c>
-      <c r="G144" s="26" t="s">
+      <c r="G144" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H144" s="26" t="s">
+      <c r="H144" s="20" t="s">
         <v>736</v>
       </c>
-      <c r="I144" s="26"/>
-      <c r="J144" s="26" t="s">
+      <c r="I144" s="20"/>
+      <c r="J144" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K144" s="26"/>
-      <c r="L144" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M144" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N144" s="26" t="s">
+      <c r="K144" s="20"/>
+      <c r="L144" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M144" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N144" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A145" s="24"/>
-      <c r="B145" s="25" t="s">
+      <c r="A145" s="18"/>
+      <c r="B145" s="19" t="s">
         <v>737</v>
       </c>
-      <c r="C145" s="24" t="s">
+      <c r="C145" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D145" s="26" t="s">
+      <c r="D145" s="20" t="s">
         <v>738</v>
       </c>
-      <c r="E145" s="26" t="s">
+      <c r="E145" s="20" t="s">
         <v>739</v>
       </c>
-      <c r="F145" s="26" t="s">
+      <c r="F145" s="20" t="s">
         <v>740</v>
       </c>
-      <c r="G145" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H145" s="26" t="s">
+      <c r="G145" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H145" s="20" t="s">
         <v>741</v>
       </c>
-      <c r="I145" s="26"/>
-      <c r="J145" s="26" t="s">
+      <c r="I145" s="20"/>
+      <c r="J145" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K145" s="26"/>
-      <c r="L145" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M145" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N145" s="26" t="s">
+      <c r="K145" s="20"/>
+      <c r="L145" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M145" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N145" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A146" s="24"/>
-      <c r="B146" s="25" t="s">
+      <c r="A146" s="18"/>
+      <c r="B146" s="19" t="s">
         <v>742</v>
       </c>
-      <c r="C146" s="24" t="s">
+      <c r="C146" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D146" s="26" t="s">
+      <c r="D146" s="20" t="s">
         <v>743</v>
       </c>
-      <c r="E146" s="26" t="s">
+      <c r="E146" s="20" t="s">
         <v>744</v>
       </c>
-      <c r="F146" s="26" t="s">
+      <c r="F146" s="20" t="s">
         <v>745</v>
       </c>
-      <c r="G146" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H146" s="26" t="s">
+      <c r="G146" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H146" s="20" t="s">
         <v>746</v>
       </c>
-      <c r="I146" s="26"/>
-      <c r="J146" s="26" t="s">
+      <c r="I146" s="20"/>
+      <c r="J146" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K146" s="26"/>
-      <c r="L146" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M146" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N146" s="26" t="s">
+      <c r="K146" s="20"/>
+      <c r="L146" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M146" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N146" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A147" s="24"/>
-      <c r="B147" s="25" t="s">
+      <c r="A147" s="18"/>
+      <c r="B147" s="19" t="s">
         <v>747</v>
       </c>
-      <c r="C147" s="24" t="s">
+      <c r="C147" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D147" s="26" t="s">
+      <c r="D147" s="20" t="s">
         <v>748</v>
       </c>
-      <c r="E147" s="26" t="s">
+      <c r="E147" s="20" t="s">
         <v>749</v>
       </c>
-      <c r="F147" s="26" t="s">
+      <c r="F147" s="20" t="s">
         <v>750</v>
       </c>
-      <c r="G147" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H147" s="26" t="s">
+      <c r="G147" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H147" s="20" t="s">
         <v>751</v>
       </c>
-      <c r="I147" s="26"/>
-      <c r="J147" s="26" t="s">
+      <c r="I147" s="20"/>
+      <c r="J147" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K147" s="26"/>
-      <c r="L147" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M147" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N147" s="26" t="s">
+      <c r="K147" s="20"/>
+      <c r="L147" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M147" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N147" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A148" s="24"/>
-      <c r="B148" s="25" t="s">
+      <c r="A148" s="18"/>
+      <c r="B148" s="19" t="s">
         <v>752</v>
       </c>
-      <c r="C148" s="24" t="s">
+      <c r="C148" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D148" s="26" t="s">
+      <c r="D148" s="20" t="s">
         <v>753</v>
       </c>
-      <c r="E148" s="26" t="s">
+      <c r="E148" s="20" t="s">
         <v>754</v>
       </c>
-      <c r="F148" s="26" t="s">
+      <c r="F148" s="20" t="s">
         <v>755</v>
       </c>
-      <c r="G148" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H148" s="26" t="s">
+      <c r="G148" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H148" s="20" t="s">
         <v>756</v>
       </c>
-      <c r="I148" s="26"/>
-      <c r="J148" s="26" t="s">
+      <c r="I148" s="20"/>
+      <c r="J148" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K148" s="26"/>
-      <c r="L148" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M148" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N148" s="26" t="s">
+      <c r="K148" s="20"/>
+      <c r="L148" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M148" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N148" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A149" s="24"/>
-      <c r="B149" s="25" t="s">
+      <c r="A149" s="18"/>
+      <c r="B149" s="19" t="s">
         <v>757</v>
       </c>
-      <c r="C149" s="24" t="s">
+      <c r="C149" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D149" s="26" t="s">
+      <c r="D149" s="20" t="s">
         <v>758</v>
       </c>
-      <c r="E149" s="26" t="s">
+      <c r="E149" s="20" t="s">
         <v>759</v>
       </c>
-      <c r="F149" s="26" t="s">
+      <c r="F149" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="G149" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H149" s="26" t="s">
+      <c r="G149" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H149" s="20" t="s">
         <v>761</v>
       </c>
-      <c r="I149" s="26"/>
-      <c r="J149" s="26" t="s">
+      <c r="I149" s="20"/>
+      <c r="J149" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K149" s="26"/>
-      <c r="L149" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M149" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N149" s="26" t="s">
+      <c r="K149" s="20"/>
+      <c r="L149" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M149" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N149" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A150" s="24"/>
-      <c r="B150" s="25" t="s">
+      <c r="A150" s="18"/>
+      <c r="B150" s="19" t="s">
         <v>762</v>
       </c>
-      <c r="C150" s="24" t="s">
+      <c r="C150" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D150" s="26" t="s">
+      <c r="D150" s="20" t="s">
         <v>763</v>
       </c>
-      <c r="E150" s="26" t="s">
+      <c r="E150" s="20" t="s">
         <v>764</v>
       </c>
-      <c r="F150" s="26" t="s">
+      <c r="F150" s="20" t="s">
         <v>765</v>
       </c>
-      <c r="G150" s="26" t="s">
+      <c r="G150" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H150" s="26" t="s">
+      <c r="H150" s="20" t="s">
         <v>766</v>
       </c>
-      <c r="I150" s="26"/>
-      <c r="J150" s="26" t="s">
+      <c r="I150" s="20"/>
+      <c r="J150" s="20" t="s">
         <v>767</v>
       </c>
-      <c r="K150" s="26"/>
-      <c r="L150" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M150" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N150" s="26" t="s">
+      <c r="K150" s="20"/>
+      <c r="L150" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M150" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N150" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A151" s="24"/>
-      <c r="B151" s="25" t="s">
+      <c r="A151" s="18"/>
+      <c r="B151" s="19" t="s">
         <v>768</v>
       </c>
-      <c r="C151" s="24" t="s">
+      <c r="C151" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D151" s="26" t="s">
+      <c r="D151" s="20" t="s">
         <v>769</v>
       </c>
-      <c r="E151" s="26" t="s">
+      <c r="E151" s="20" t="s">
         <v>770</v>
       </c>
-      <c r="F151" s="26" t="s">
+      <c r="F151" s="20" t="s">
         <v>771</v>
       </c>
-      <c r="G151" s="26" t="s">
+      <c r="G151" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H151" s="26" t="s">
+      <c r="H151" s="20" t="s">
         <v>772</v>
       </c>
-      <c r="I151" s="26"/>
-      <c r="J151" s="26" t="s">
+      <c r="I151" s="20"/>
+      <c r="J151" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K151" s="26"/>
-      <c r="L151" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M151" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N151" s="26" t="s">
+      <c r="K151" s="20"/>
+      <c r="L151" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M151" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N151" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A152" s="24"/>
-      <c r="B152" s="25" t="s">
+      <c r="A152" s="18"/>
+      <c r="B152" s="19" t="s">
         <v>773</v>
       </c>
-      <c r="C152" s="24" t="s">
+      <c r="C152" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D152" s="26" t="s">
+      <c r="D152" s="20" t="s">
         <v>774</v>
       </c>
-      <c r="E152" s="26" t="s">
+      <c r="E152" s="20" t="s">
         <v>775</v>
       </c>
-      <c r="F152" s="26" t="s">
+      <c r="F152" s="20" t="s">
         <v>776</v>
       </c>
-      <c r="G152" s="26" t="s">
+      <c r="G152" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H152" s="26" t="s">
+      <c r="H152" s="20" t="s">
         <v>777</v>
       </c>
-      <c r="I152" s="26"/>
-      <c r="J152" s="26" t="s">
+      <c r="I152" s="20"/>
+      <c r="J152" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K152" s="26"/>
-      <c r="L152" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M152" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N152" s="26" t="s">
+      <c r="K152" s="20"/>
+      <c r="L152" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M152" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N152" s="20" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A153" s="24"/>
-      <c r="B153" s="25" t="s">
+      <c r="A153" s="18"/>
+      <c r="B153" s="19" t="s">
         <v>778</v>
       </c>
-      <c r="C153" s="24" t="s">
+      <c r="C153" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D153" s="26" t="s">
+      <c r="D153" s="20" t="s">
         <v>779</v>
       </c>
-      <c r="E153" s="26" t="s">
+      <c r="E153" s="20" t="s">
         <v>780</v>
       </c>
-      <c r="F153" s="26" t="s">
+      <c r="F153" s="20" t="s">
         <v>781</v>
       </c>
-      <c r="G153" s="26" t="s">
+      <c r="G153" s="20" t="s">
         <v>430</v>
       </c>
-      <c r="H153" s="26" t="s">
+      <c r="H153" s="20" t="s">
         <v>782</v>
       </c>
-      <c r="I153" s="26"/>
-      <c r="J153" s="26" t="s">
+      <c r="I153" s="20"/>
+      <c r="J153" s="20" t="s">
         <v>652</v>
       </c>
-      <c r="K153" s="26"/>
-      <c r="L153" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="M153" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="N153" s="26" t="s">
+      <c r="K153" s="20"/>
+      <c r="L153" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M153" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N153" s="20" t="s">
         <v>653</v>
       </c>
     </row>
@@ -9065,913 +9044,913 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="22" t="s">
         <v>783</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="23" t="s">
         <v>784</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="23" t="s">
         <v>785</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="23" t="s">
         <v>786</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="23" t="s">
         <v>787</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="23" t="s">
         <v>788</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="23" t="s">
         <v>789</v>
       </c>
-      <c r="I1" s="29" t="s">
+      <c r="I1" s="24" t="s">
         <v>790</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="25" t="s">
         <v>791</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="26" t="s">
         <v>792</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="26" t="s">
         <v>793</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="26" t="s">
         <v>794</v>
       </c>
-      <c r="E2" s="31" t="s">
+      <c r="E2" s="26" t="s">
         <v>795</v>
       </c>
-      <c r="F2" s="31" t="s">
+      <c r="F2" s="26" t="s">
         <v>796</v>
       </c>
-      <c r="G2" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" s="32" t="s">
+      <c r="G2" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="27" t="s">
         <v>797</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="28" t="s">
         <v>798</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="29" t="s">
         <v>799</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="29" t="s">
         <v>800</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E3" s="34" t="s">
+      <c r="E3" s="29" t="s">
         <v>801</v>
       </c>
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="29" t="s">
         <v>802</v>
       </c>
-      <c r="G3" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="35" t="s">
+      <c r="G3" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="30" t="s">
         <v>803</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="28" t="s">
         <v>804</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>805</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="29" t="s">
         <v>806</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="29" t="s">
         <v>807</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="F4" s="29" t="s">
         <v>808</v>
       </c>
-      <c r="G4" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="35" t="s">
+      <c r="G4" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="30" t="s">
         <v>809</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="28" t="s">
         <v>810</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="29" t="s">
         <v>811</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="29" t="s">
         <v>812</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="29" t="s">
         <v>813</v>
       </c>
-      <c r="F5" s="34" t="s">
+      <c r="F5" s="29" t="s">
         <v>814</v>
       </c>
-      <c r="G5" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="35" t="s">
+      <c r="G5" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="30" t="s">
         <v>815</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="28" t="s">
         <v>816</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="29" t="s">
         <v>402</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="29" t="s">
         <v>817</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="29" t="s">
         <v>818</v>
       </c>
-      <c r="F6" s="34" t="s">
+      <c r="F6" s="29" t="s">
         <v>819</v>
       </c>
-      <c r="G6" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="35" t="s">
+      <c r="G6" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="30" t="s">
         <v>820</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="28" t="s">
         <v>821</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="29" t="s">
         <v>439</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="29" t="s">
         <v>822</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E7" s="34" t="s">
+      <c r="E7" s="29" t="s">
         <v>823</v>
       </c>
-      <c r="F7" s="34" t="s">
+      <c r="F7" s="29" t="s">
         <v>824</v>
       </c>
-      <c r="G7" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="35" t="s">
+      <c r="G7" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="30" t="s">
         <v>825</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="28" t="s">
         <v>826</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="29" t="s">
         <v>504</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="29" t="s">
         <v>827</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E8" s="34" t="s">
+      <c r="E8" s="29" t="s">
         <v>828</v>
       </c>
-      <c r="F8" s="34" t="s">
+      <c r="F8" s="29" t="s">
         <v>829</v>
       </c>
-      <c r="G8" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I8" s="35" t="s">
+      <c r="G8" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="30" t="s">
         <v>830</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="28" t="s">
         <v>831</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="29" t="s">
         <v>598</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="29" t="s">
         <v>832</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="29" t="s">
         <v>794</v>
       </c>
-      <c r="E9" s="34" t="s">
+      <c r="E9" s="29" t="s">
         <v>833</v>
       </c>
-      <c r="F9" s="34" t="s">
+      <c r="F9" s="29" t="s">
         <v>834</v>
       </c>
-      <c r="G9" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="35" t="s">
+      <c r="G9" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="30" t="s">
         <v>835</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="31" t="s">
         <v>836</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="32" t="s">
         <v>645</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="32" t="s">
         <v>837</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="32" t="s">
         <v>794</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="32" t="s">
         <v>838</v>
       </c>
-      <c r="F10" s="37" t="s">
+      <c r="F10" s="32" t="s">
         <v>839</v>
       </c>
-      <c r="G10" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="38" t="s">
+      <c r="G10" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="33" t="s">
         <v>840</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="34" t="s">
         <v>841</v>
       </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="40" t="s">
+      <c r="B11" s="35"/>
+      <c r="C11" s="35" t="s">
         <v>842</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="35" t="s">
         <v>843</v>
       </c>
-      <c r="E11" s="40" t="s">
+      <c r="E11" s="35" t="s">
         <v>844</v>
       </c>
-      <c r="F11" s="40" t="s">
+      <c r="F11" s="35" t="s">
         <v>845</v>
       </c>
-      <c r="G11" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="I11" s="41" t="s">
+      <c r="G11" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" s="36" t="s">
         <v>846</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="37" t="s">
         <v>847</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43" t="s">
+      <c r="B12" s="38"/>
+      <c r="C12" s="38" t="s">
         <v>848</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E12" s="43" t="s">
+      <c r="E12" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F12" s="43" t="s">
+      <c r="F12" s="38" t="s">
         <v>849</v>
       </c>
-      <c r="G12" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H12" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I12" s="44" t="s">
+      <c r="G12" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="39" t="s">
         <v>850</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="37" t="s">
         <v>851</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43" t="s">
+      <c r="B13" s="38"/>
+      <c r="C13" s="38" t="s">
         <v>852</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E13" s="43" t="s">
+      <c r="E13" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F13" s="43" t="s">
+      <c r="F13" s="38" t="s">
         <v>853</v>
       </c>
-      <c r="G13" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H13" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I13" s="44" t="s">
+      <c r="G13" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H13" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" s="39" t="s">
         <v>854</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="42" t="s">
+      <c r="A14" s="37" t="s">
         <v>855</v>
       </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="43" t="s">
+      <c r="B14" s="38"/>
+      <c r="C14" s="38" t="s">
         <v>856</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E14" s="43" t="s">
+      <c r="E14" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F14" s="43" t="s">
+      <c r="F14" s="38" t="s">
         <v>857</v>
       </c>
-      <c r="G14" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="44" t="s">
+      <c r="G14" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="39" t="s">
         <v>858</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="42" t="s">
+      <c r="A15" s="37" t="s">
         <v>859</v>
       </c>
-      <c r="B15" s="43"/>
-      <c r="C15" s="43" t="s">
+      <c r="B15" s="38"/>
+      <c r="C15" s="38" t="s">
         <v>860</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E15" s="43" t="s">
+      <c r="E15" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F15" s="43" t="s">
+      <c r="F15" s="38" t="s">
         <v>861</v>
       </c>
-      <c r="G15" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I15" s="44" t="s">
+      <c r="G15" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I15" s="39" t="s">
         <v>862</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="37" t="s">
         <v>863</v>
       </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43" t="s">
+      <c r="B16" s="38"/>
+      <c r="C16" s="38" t="s">
         <v>864</v>
       </c>
-      <c r="D16" s="43" t="s">
+      <c r="D16" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E16" s="43" t="s">
+      <c r="E16" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F16" s="43" t="s">
+      <c r="F16" s="38" t="s">
         <v>865</v>
       </c>
-      <c r="G16" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I16" s="44" t="s">
+      <c r="G16" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="39" t="s">
         <v>866</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="37" t="s">
         <v>867</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="43" t="s">
+      <c r="B17" s="38"/>
+      <c r="C17" s="38" t="s">
         <v>868</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="D17" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E17" s="43" t="s">
+      <c r="E17" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F17" s="43" t="s">
+      <c r="F17" s="38" t="s">
         <v>869</v>
       </c>
-      <c r="G17" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H17" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I17" s="44" t="s">
+      <c r="G17" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="39" t="s">
         <v>870</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="37" t="s">
         <v>871</v>
       </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43" t="s">
+      <c r="B18" s="38"/>
+      <c r="C18" s="38" t="s">
         <v>872</v>
       </c>
-      <c r="D18" s="43" t="s">
+      <c r="D18" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E18" s="43" t="s">
+      <c r="E18" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F18" s="43" t="s">
+      <c r="F18" s="38" t="s">
         <v>873</v>
       </c>
-      <c r="G18" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I18" s="44" t="s">
+      <c r="G18" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" s="39" t="s">
         <v>874</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="37" t="s">
         <v>875</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43" t="s">
+      <c r="B19" s="38"/>
+      <c r="C19" s="38" t="s">
         <v>876</v>
       </c>
-      <c r="D19" s="43" t="s">
+      <c r="D19" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E19" s="43" t="s">
+      <c r="E19" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F19" s="43" t="s">
+      <c r="F19" s="38" t="s">
         <v>877</v>
       </c>
-      <c r="G19" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I19" s="44" t="s">
+      <c r="G19" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19" s="39" t="s">
         <v>878</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="37" t="s">
         <v>879</v>
       </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43" t="s">
+      <c r="B20" s="38"/>
+      <c r="C20" s="38" t="s">
         <v>880</v>
       </c>
-      <c r="D20" s="43" t="s">
+      <c r="D20" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E20" s="43" t="s">
+      <c r="E20" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="F20" s="38" t="s">
         <v>881</v>
       </c>
-      <c r="G20" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H20" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I20" s="44" t="s">
+      <c r="G20" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I20" s="39" t="s">
         <v>882</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="37" t="s">
         <v>883</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43" t="s">
+      <c r="B21" s="38"/>
+      <c r="C21" s="38" t="s">
         <v>884</v>
       </c>
-      <c r="D21" s="43" t="s">
+      <c r="D21" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E21" s="43" t="s">
+      <c r="E21" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F21" s="43" t="s">
+      <c r="F21" s="38" t="s">
         <v>885</v>
       </c>
-      <c r="G21" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H21" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I21" s="44" t="s">
+      <c r="G21" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="39" t="s">
         <v>886</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="37" t="s">
         <v>887</v>
       </c>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43" t="s">
+      <c r="B22" s="38"/>
+      <c r="C22" s="38" t="s">
         <v>827</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E22" s="43" t="s">
+      <c r="E22" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F22" s="43" t="s">
+      <c r="F22" s="38" t="s">
         <v>888</v>
       </c>
-      <c r="G22" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H22" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I22" s="44" t="s">
+      <c r="G22" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H22" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="39" t="s">
         <v>889</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="37" t="s">
         <v>890</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="43" t="s">
+      <c r="B23" s="38"/>
+      <c r="C23" s="38" t="s">
         <v>832</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E23" s="43" t="s">
+      <c r="E23" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F23" s="43" t="s">
+      <c r="F23" s="38" t="s">
         <v>891</v>
       </c>
-      <c r="G23" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H23" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I23" s="44" t="s">
+      <c r="G23" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H23" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="39" t="s">
         <v>892</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="42" t="s">
+      <c r="A24" s="37" t="s">
         <v>893</v>
       </c>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43" t="s">
+      <c r="B24" s="38"/>
+      <c r="C24" s="38" t="s">
         <v>894</v>
       </c>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="38" t="s">
         <v>843</v>
       </c>
-      <c r="E24" s="43" t="s">
+      <c r="E24" s="38" t="s">
         <v>844</v>
       </c>
-      <c r="F24" s="43" t="s">
+      <c r="F24" s="38" t="s">
         <v>895</v>
       </c>
-      <c r="G24" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="H24" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="I24" s="44" t="s">
+      <c r="G24" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" s="39" t="s">
         <v>896</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="45" t="s">
+      <c r="A25" s="40" t="s">
         <v>897</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46" t="s">
+      <c r="B25" s="41"/>
+      <c r="C25" s="41" t="s">
         <v>837</v>
       </c>
-      <c r="D25" s="46" t="s">
+      <c r="D25" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E25" s="46" t="s">
+      <c r="E25" s="41" t="s">
         <v>844</v>
       </c>
-      <c r="F25" s="46" t="s">
+      <c r="F25" s="41" t="s">
         <v>898</v>
       </c>
-      <c r="G25" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="47" t="s">
+      <c r="G25" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="42" t="s">
         <v>899</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="45" t="s">
+      <c r="A26" s="40" t="s">
         <v>900</v>
       </c>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46" t="s">
+      <c r="B26" s="41"/>
+      <c r="C26" s="41" t="s">
         <v>901</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="D26" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E26" s="46" t="s">
+      <c r="E26" s="41" t="s">
         <v>902</v>
       </c>
-      <c r="F26" s="46" t="s">
+      <c r="F26" s="41" t="s">
         <v>903</v>
       </c>
-      <c r="G26" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I26" s="47" t="s">
+      <c r="G26" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="42" t="s">
         <v>904</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="45" t="s">
+      <c r="A27" s="40" t="s">
         <v>905</v>
       </c>
-      <c r="B27" s="46"/>
-      <c r="C27" s="46" t="s">
+      <c r="B27" s="41"/>
+      <c r="C27" s="41" t="s">
         <v>906</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E27" s="46" t="s">
+      <c r="E27" s="41" t="s">
         <v>907</v>
       </c>
-      <c r="F27" s="46" t="s">
+      <c r="F27" s="41" t="s">
         <v>908</v>
       </c>
-      <c r="G27" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H27" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I27" s="47" t="s">
+      <c r="G27" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H27" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="42" t="s">
         <v>909</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="45" t="s">
+      <c r="A28" s="40" t="s">
         <v>910</v>
       </c>
-      <c r="B28" s="46"/>
-      <c r="C28" s="46" t="s">
+      <c r="B28" s="41"/>
+      <c r="C28" s="41" t="s">
         <v>911</v>
       </c>
-      <c r="D28" s="46" t="s">
+      <c r="D28" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E28" s="46" t="s">
+      <c r="E28" s="41" t="s">
         <v>912</v>
       </c>
-      <c r="F28" s="46" t="s">
+      <c r="F28" s="41" t="s">
         <v>913</v>
       </c>
-      <c r="G28" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="47" t="s">
+      <c r="G28" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="42" t="s">
         <v>914</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="40" t="s">
         <v>915</v>
       </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46" t="s">
+      <c r="B29" s="41"/>
+      <c r="C29" s="41" t="s">
         <v>916</v>
       </c>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E29" s="46" t="s">
+      <c r="E29" s="41" t="s">
         <v>917</v>
       </c>
-      <c r="F29" s="46" t="s">
+      <c r="F29" s="41" t="s">
         <v>918</v>
       </c>
-      <c r="G29" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H29" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29" s="47" t="s">
+      <c r="G29" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="42" t="s">
         <v>919</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="40" t="s">
         <v>920</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46" t="s">
+      <c r="B30" s="41"/>
+      <c r="C30" s="41" t="s">
         <v>921</v>
       </c>
-      <c r="D30" s="46" t="s">
+      <c r="D30" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E30" s="46" t="s">
+      <c r="E30" s="41" t="s">
         <v>922</v>
       </c>
-      <c r="F30" s="46" t="s">
+      <c r="F30" s="41" t="s">
         <v>923</v>
       </c>
-      <c r="G30" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="47" t="s">
+      <c r="G30" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H30" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="42" t="s">
         <v>924</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="45" t="s">
+      <c r="A31" s="40" t="s">
         <v>925</v>
       </c>
-      <c r="B31" s="46"/>
-      <c r="C31" s="46" t="s">
+      <c r="B31" s="41"/>
+      <c r="C31" s="41" t="s">
         <v>832</v>
       </c>
-      <c r="D31" s="46" t="s">
+      <c r="D31" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E31" s="46" t="s">
+      <c r="E31" s="41" t="s">
         <v>926</v>
       </c>
-      <c r="F31" s="46" t="s">
+      <c r="F31" s="41" t="s">
         <v>927</v>
       </c>
-      <c r="G31" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H31" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I31" s="47" t="s">
+      <c r="G31" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H31" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="42" t="s">
         <v>928</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="45" t="s">
+      <c r="A32" s="40" t="s">
         <v>929</v>
       </c>
-      <c r="B32" s="46"/>
-      <c r="C32" s="46" t="s">
+      <c r="B32" s="41"/>
+      <c r="C32" s="41" t="s">
         <v>930</v>
       </c>
-      <c r="D32" s="46" t="s">
+      <c r="D32" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E32" s="46" t="s">
+      <c r="E32" s="41" t="s">
         <v>931</v>
       </c>
-      <c r="F32" s="46" t="s">
+      <c r="F32" s="41" t="s">
         <v>932</v>
       </c>
-      <c r="G32" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32" s="47" t="s">
+      <c r="G32" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" s="42" t="s">
         <v>933</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="45" t="s">
+      <c r="A33" s="40" t="s">
         <v>934</v>
       </c>
-      <c r="B33" s="46"/>
-      <c r="C33" s="46" t="s">
+      <c r="B33" s="41"/>
+      <c r="C33" s="41" t="s">
         <v>935</v>
       </c>
-      <c r="D33" s="46" t="s">
+      <c r="D33" s="41" t="s">
         <v>843</v>
       </c>
-      <c r="E33" s="46" t="s">
+      <c r="E33" s="41" t="s">
         <v>936</v>
       </c>
-      <c r="F33" s="46" t="s">
+      <c r="F33" s="41" t="s">
         <v>937</v>
       </c>
-      <c r="G33" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="H33" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="I33" s="47" t="s">
+      <c r="G33" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H33" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="42" t="s">
         <v>938</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: correct Stage 6 Pass 008 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -3176,7 +3176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3228,9 +3228,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3990,40 +3987,40 @@
       </c>
     </row>
     <row r="16" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A16" s="19"/>
+      <c r="A16" s="18"/>
       <c r="B16" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="F16" s="21" t="s">
+      <c r="F16" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="G16" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="21" t="s">
+      <c r="G16" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21" t="s">
+      <c r="I16" s="20"/>
+      <c r="J16" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M16" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N16" s="21" t="s">
+      <c r="K16" s="20"/>
+      <c r="L16" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M16" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N16" s="20" t="s">
         <v>40</v>
       </c>
     </row>
@@ -4104,40 +4101,40 @@
       </c>
     </row>
     <row r="19" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A19" s="19"/>
+      <c r="A19" s="18"/>
       <c r="B19" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="E19" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="F19" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G19" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="21" t="s">
+      <c r="G19" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21" t="s">
+      <c r="I19" s="20"/>
+      <c r="J19" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M19" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N19" s="21" t="s">
+      <c r="K19" s="20"/>
+      <c r="L19" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M19" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N19" s="20" t="s">
         <v>40</v>
       </c>
     </row>
@@ -4172,7 +4169,7 @@
       <c r="L20" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M20" s="21" t="s">
+      <c r="M20" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N20" s="20" t="s">
@@ -4232,7 +4229,7 @@
       <c r="L22" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M22" s="21" t="s">
+      <c r="M22" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N22" s="20" t="s">
@@ -4312,76 +4309,76 @@
       </c>
     </row>
     <row r="25" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="D25" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="E25" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="G25" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="21" t="s">
+      <c r="G25" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M25" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N25" s="21" t="s">
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M25" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N25" s="20" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="26" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="E26" s="21" t="s">
+      <c r="E26" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="F26" s="21" t="s">
+      <c r="F26" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="G26" s="21" t="s">
+      <c r="G26" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H26" s="21" t="s">
+      <c r="H26" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21" t="s">
+      <c r="I26" s="20"/>
+      <c r="J26" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M26" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N26" s="21" t="s">
+      <c r="K26" s="20"/>
+      <c r="L26" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M26" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N26" s="20" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4558,40 +4555,40 @@
       </c>
     </row>
     <row r="32" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A32" s="19"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D32" s="21" t="s">
+      <c r="D32" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="F32" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="G32" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="21" t="s">
+      <c r="G32" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21" t="s">
+      <c r="I32" s="20"/>
+      <c r="J32" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M32" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N32" s="21" t="s">
+      <c r="K32" s="20"/>
+      <c r="L32" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M32" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N32" s="20" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4626,7 +4623,7 @@
       <c r="L33" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M33" s="21" t="s">
+      <c r="M33" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N33" s="20" t="s">
@@ -4662,7 +4659,7 @@
       <c r="L34" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M34" s="21" t="s">
+      <c r="M34" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N34" s="20" t="s">
@@ -4698,7 +4695,7 @@
       <c r="L35" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M35" s="21" t="s">
+      <c r="M35" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N35" s="20" t="s">
@@ -4734,7 +4731,7 @@
       <c r="L36" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M36" s="21" t="s">
+      <c r="M36" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N36" s="20" t="s">
@@ -4742,76 +4739,76 @@
       </c>
     </row>
     <row r="37" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A37" s="19"/>
+      <c r="A37" s="18"/>
       <c r="B37" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="C37" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="E37" s="21" t="s">
+      <c r="E37" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="F37" s="21" t="s">
+      <c r="F37" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="G37" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H37" s="21" t="s">
+      <c r="G37" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H37" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="21"/>
-      <c r="L37" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M37" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N37" s="21" t="s">
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
+      <c r="L37" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M37" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N37" s="20" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="38" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A38" s="19"/>
+      <c r="A38" s="18"/>
       <c r="B38" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="C38" s="19" t="s">
+      <c r="C38" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="E38" s="21" t="s">
+      <c r="E38" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="F38" s="21" t="s">
+      <c r="F38" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="G38" s="21" t="s">
+      <c r="G38" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H38" s="21" t="s">
+      <c r="H38" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="I38" s="21"/>
-      <c r="J38" s="21" t="s">
+      <c r="I38" s="20"/>
+      <c r="J38" s="20" t="s">
         <v>195</v>
       </c>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M38" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N38" s="21" t="s">
+      <c r="K38" s="20"/>
+      <c r="L38" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M38" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N38" s="20" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4846,7 +4843,7 @@
       <c r="L39" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M39" s="21" t="s">
+      <c r="M39" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N39" s="20" t="s">
@@ -4906,7 +4903,7 @@
       <c r="L41" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M41" s="21" t="s">
+      <c r="M41" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N41" s="20" t="s">
@@ -4942,7 +4939,7 @@
       <c r="L42" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M42" s="21" t="s">
+      <c r="M42" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N42" s="20" t="s">
@@ -4950,40 +4947,40 @@
       </c>
     </row>
     <row r="43" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A43" s="19"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="C43" s="19" t="s">
+      <c r="C43" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D43" s="21" t="s">
+      <c r="D43" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="E43" s="21" t="s">
+      <c r="E43" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="F43" s="21" t="s">
+      <c r="F43" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="G43" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H43" s="21" t="s">
+      <c r="G43" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H43" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="I43" s="21"/>
-      <c r="J43" s="21" t="s">
+      <c r="I43" s="20"/>
+      <c r="J43" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="K43" s="21"/>
-      <c r="L43" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M43" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N43" s="21" t="s">
+      <c r="K43" s="20"/>
+      <c r="L43" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M43" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N43" s="20" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5100,38 +5097,38 @@
       </c>
     </row>
     <row r="47" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A47" s="19"/>
+      <c r="A47" s="18"/>
       <c r="B47" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="C47" s="19" t="s">
+      <c r="C47" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D47" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="E47" s="21" t="s">
+      <c r="E47" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="F47" s="21" t="s">
+      <c r="F47" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="G47" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H47" s="21" t="s">
+      <c r="G47" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="I47" s="21"/>
-      <c r="J47" s="21"/>
-      <c r="K47" s="21"/>
-      <c r="L47" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M47" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N47" s="21" t="s">
+      <c r="I47" s="20"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
+      <c r="L47" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M47" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N47" s="20" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5272,40 +5269,40 @@
       </c>
     </row>
     <row r="52" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A52" s="19"/>
+      <c r="A52" s="18"/>
       <c r="B52" s="19" t="s">
         <v>262</v>
       </c>
-      <c r="C52" s="19" t="s">
+      <c r="C52" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="D52" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="E52" s="21" t="s">
+      <c r="E52" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="F52" s="21" t="s">
+      <c r="F52" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="G52" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H52" s="21" t="s">
+      <c r="G52" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H52" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="I52" s="21"/>
-      <c r="J52" s="21" t="s">
+      <c r="I52" s="20"/>
+      <c r="J52" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="K52" s="21"/>
-      <c r="L52" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M52" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N52" s="21" t="s">
+      <c r="K52" s="20"/>
+      <c r="L52" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M52" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N52" s="20" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5460,40 +5457,40 @@
       </c>
     </row>
     <row r="57" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A57" s="19"/>
+      <c r="A57" s="18"/>
       <c r="B57" s="19" t="s">
         <v>290</v>
       </c>
-      <c r="C57" s="19" t="s">
+      <c r="C57" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="D57" s="20" t="s">
         <v>291</v>
       </c>
-      <c r="E57" s="21" t="s">
+      <c r="E57" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="F57" s="21" t="s">
+      <c r="F57" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="G57" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H57" s="21" t="s">
+      <c r="G57" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H57" s="20" t="s">
         <v>294</v>
       </c>
-      <c r="I57" s="21"/>
-      <c r="J57" s="21" t="s">
+      <c r="I57" s="20"/>
+      <c r="J57" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="K57" s="21"/>
-      <c r="L57" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M57" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N57" s="21" t="s">
+      <c r="K57" s="20"/>
+      <c r="L57" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M57" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N57" s="20" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5668,38 +5665,38 @@
       </c>
     </row>
     <row r="63" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A63" s="19"/>
+      <c r="A63" s="18"/>
       <c r="B63" s="19" t="s">
         <v>319</v>
       </c>
-      <c r="C63" s="19" t="s">
+      <c r="C63" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D63" s="21" t="s">
+      <c r="D63" s="20" t="s">
         <v>320</v>
       </c>
-      <c r="E63" s="21" t="s">
+      <c r="E63" s="20" t="s">
         <v>321</v>
       </c>
-      <c r="F63" s="21" t="s">
+      <c r="F63" s="20" t="s">
         <v>322</v>
       </c>
-      <c r="G63" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H63" s="21" t="s">
+      <c r="G63" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H63" s="20" t="s">
         <v>323</v>
       </c>
-      <c r="I63" s="21"/>
-      <c r="J63" s="21"/>
-      <c r="K63" s="21"/>
-      <c r="L63" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M63" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N63" s="21" t="s">
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
+      <c r="K63" s="20"/>
+      <c r="L63" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M63" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N63" s="20" t="s">
         <v>308</v>
       </c>
     </row>
@@ -5850,40 +5847,40 @@
       </c>
     </row>
     <row r="68" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A68" s="19"/>
+      <c r="A68" s="18"/>
       <c r="B68" s="19" t="s">
         <v>345</v>
       </c>
-      <c r="C68" s="19" t="s">
+      <c r="C68" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D68" s="21" t="s">
+      <c r="D68" s="20" t="s">
         <v>346</v>
       </c>
-      <c r="E68" s="21" t="s">
+      <c r="E68" s="20" t="s">
         <v>347</v>
       </c>
-      <c r="F68" s="21" t="s">
+      <c r="F68" s="20" t="s">
         <v>348</v>
       </c>
-      <c r="G68" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H68" s="21" t="s">
+      <c r="G68" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H68" s="20" t="s">
         <v>349</v>
       </c>
-      <c r="I68" s="21"/>
-      <c r="J68" s="21" t="s">
+      <c r="I68" s="20"/>
+      <c r="J68" s="20" t="s">
         <v>350</v>
       </c>
-      <c r="K68" s="21"/>
-      <c r="L68" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M68" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N68" s="21" t="s">
+      <c r="K68" s="20"/>
+      <c r="L68" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M68" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N68" s="20" t="s">
         <v>308</v>
       </c>
     </row>
@@ -5954,7 +5951,7 @@
       <c r="L70" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M70" s="21" t="s">
+      <c r="M70" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N70" s="20" t="s">
@@ -5962,78 +5959,78 @@
       </c>
     </row>
     <row r="71" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A71" s="19"/>
+      <c r="A71" s="18"/>
       <c r="B71" s="19" t="s">
         <v>362</v>
       </c>
-      <c r="C71" s="19" t="s">
+      <c r="C71" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D71" s="21" t="s">
+      <c r="D71" s="20" t="s">
         <v>363</v>
       </c>
-      <c r="E71" s="21" t="s">
+      <c r="E71" s="20" t="s">
         <v>364</v>
       </c>
-      <c r="F71" s="21" t="s">
+      <c r="F71" s="20" t="s">
         <v>365</v>
       </c>
-      <c r="G71" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H71" s="21" t="s">
+      <c r="G71" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H71" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="I71" s="21"/>
-      <c r="J71" s="21" t="s">
+      <c r="I71" s="20"/>
+      <c r="J71" s="20" t="s">
         <v>367</v>
       </c>
-      <c r="K71" s="21"/>
-      <c r="L71" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M71" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N71" s="21" t="s">
+      <c r="K71" s="20"/>
+      <c r="L71" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M71" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N71" s="20" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="72" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A72" s="19"/>
+      <c r="A72" s="18"/>
       <c r="B72" s="19" t="s">
         <v>368</v>
       </c>
-      <c r="C72" s="19" t="s">
+      <c r="C72" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D72" s="21" t="s">
+      <c r="D72" s="20" t="s">
         <v>369</v>
       </c>
-      <c r="E72" s="21" t="s">
+      <c r="E72" s="20" t="s">
         <v>370</v>
       </c>
-      <c r="F72" s="21" t="s">
+      <c r="F72" s="20" t="s">
         <v>371</v>
       </c>
-      <c r="G72" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H72" s="21" t="s">
+      <c r="G72" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H72" s="20" t="s">
         <v>372</v>
       </c>
-      <c r="I72" s="21"/>
-      <c r="J72" s="21" t="s">
+      <c r="I72" s="20"/>
+      <c r="J72" s="20" t="s">
         <v>373</v>
       </c>
-      <c r="K72" s="21"/>
-      <c r="L72" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M72" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N72" s="21" t="s">
+      <c r="K72" s="20"/>
+      <c r="L72" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M72" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N72" s="20" t="s">
         <v>308</v>
       </c>
     </row>
@@ -6076,40 +6073,40 @@
       </c>
     </row>
     <row r="74" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A74" s="19"/>
+      <c r="A74" s="18"/>
       <c r="B74" s="19" t="s">
         <v>379</v>
       </c>
-      <c r="C74" s="19" t="s">
+      <c r="C74" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D74" s="21" t="s">
+      <c r="D74" s="20" t="s">
         <v>380</v>
       </c>
-      <c r="E74" s="21" t="s">
+      <c r="E74" s="20" t="s">
         <v>381</v>
       </c>
-      <c r="F74" s="21" t="s">
+      <c r="F74" s="20" t="s">
         <v>382</v>
       </c>
-      <c r="G74" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H74" s="21" t="s">
+      <c r="G74" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H74" s="20" t="s">
         <v>383</v>
       </c>
-      <c r="I74" s="21"/>
-      <c r="J74" s="21" t="s">
+      <c r="I74" s="20"/>
+      <c r="J74" s="20" t="s">
         <v>373</v>
       </c>
-      <c r="K74" s="21"/>
-      <c r="L74" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M74" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N74" s="21" t="s">
+      <c r="K74" s="20"/>
+      <c r="L74" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M74" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N74" s="20" t="s">
         <v>308</v>
       </c>
     </row>
@@ -6144,7 +6141,7 @@
       <c r="L75" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M75" s="21" t="s">
+      <c r="M75" s="20" t="s">
         <v>39</v>
       </c>
       <c r="N75" s="20" t="s">
@@ -6190,40 +6187,40 @@
       </c>
     </row>
     <row r="77" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A77" s="19"/>
+      <c r="A77" s="18"/>
       <c r="B77" s="19" t="s">
         <v>394</v>
       </c>
-      <c r="C77" s="19" t="s">
+      <c r="C77" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D77" s="21" t="s">
+      <c r="D77" s="20" t="s">
         <v>395</v>
       </c>
-      <c r="E77" s="21" t="s">
+      <c r="E77" s="20" t="s">
         <v>396</v>
       </c>
-      <c r="F77" s="21" t="s">
+      <c r="F77" s="20" t="s">
         <v>397</v>
       </c>
-      <c r="G77" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H77" s="21" t="s">
+      <c r="G77" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H77" s="20" t="s">
         <v>393</v>
       </c>
-      <c r="I77" s="21"/>
-      <c r="J77" s="21" t="s">
+      <c r="I77" s="20"/>
+      <c r="J77" s="20" t="s">
         <v>373</v>
       </c>
-      <c r="K77" s="21"/>
-      <c r="L77" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M77" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N77" s="21" t="s">
+      <c r="K77" s="20"/>
+      <c r="L77" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M77" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N77" s="20" t="s">
         <v>308</v>
       </c>
     </row>
@@ -6328,38 +6325,38 @@
       </c>
     </row>
     <row r="81" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A81" s="19"/>
+      <c r="A81" s="18"/>
       <c r="B81" s="19" t="s">
         <v>411</v>
       </c>
-      <c r="C81" s="19" t="s">
+      <c r="C81" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D81" s="21" t="s">
+      <c r="D81" s="20" t="s">
         <v>412</v>
       </c>
-      <c r="E81" s="21" t="s">
+      <c r="E81" s="20" t="s">
         <v>413</v>
       </c>
-      <c r="F81" s="21" t="s">
+      <c r="F81" s="20" t="s">
         <v>414</v>
       </c>
-      <c r="G81" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H81" s="21" t="s">
+      <c r="G81" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H81" s="20" t="s">
         <v>415</v>
       </c>
-      <c r="I81" s="21"/>
-      <c r="J81" s="21"/>
-      <c r="K81" s="21"/>
-      <c r="L81" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M81" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N81" s="21" t="s">
+      <c r="I81" s="20"/>
+      <c r="J81" s="20"/>
+      <c r="K81" s="20"/>
+      <c r="L81" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M81" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N81" s="20" t="s">
         <v>410</v>
       </c>
     </row>
@@ -6436,40 +6433,40 @@
       </c>
     </row>
     <row r="84" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A84" s="19"/>
+      <c r="A84" s="18"/>
       <c r="B84" s="19" t="s">
         <v>426</v>
       </c>
-      <c r="C84" s="19" t="s">
+      <c r="C84" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D84" s="21" t="s">
+      <c r="D84" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="E84" s="21" t="s">
+      <c r="E84" s="20" t="s">
         <v>428</v>
       </c>
-      <c r="F84" s="21" t="s">
+      <c r="F84" s="20" t="s">
         <v>429</v>
       </c>
-      <c r="G84" s="21" t="s">
+      <c r="G84" s="20" t="s">
         <v>430</v>
       </c>
-      <c r="H84" s="21" t="s">
+      <c r="H84" s="20" t="s">
         <v>431</v>
       </c>
-      <c r="I84" s="21"/>
-      <c r="J84" s="21" t="s">
+      <c r="I84" s="20"/>
+      <c r="J84" s="20" t="s">
         <v>432</v>
       </c>
-      <c r="K84" s="21"/>
-      <c r="L84" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M84" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N84" s="21" t="s">
+      <c r="K84" s="20"/>
+      <c r="L84" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M84" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N84" s="20" t="s">
         <v>410</v>
       </c>
     </row>
@@ -6684,40 +6681,40 @@
       </c>
     </row>
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A91" s="19"/>
+      <c r="A91" s="18"/>
       <c r="B91" s="19" t="s">
         <v>462</v>
       </c>
-      <c r="C91" s="19" t="s">
+      <c r="C91" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D91" s="21" t="s">
+      <c r="D91" s="20" t="s">
         <v>463</v>
       </c>
-      <c r="E91" s="21" t="s">
+      <c r="E91" s="20" t="s">
         <v>464</v>
       </c>
-      <c r="F91" s="21" t="s">
+      <c r="F91" s="20" t="s">
         <v>465</v>
       </c>
-      <c r="G91" s="21" t="s">
+      <c r="G91" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H91" s="21" t="s">
+      <c r="H91" s="20" t="s">
         <v>466</v>
       </c>
-      <c r="I91" s="21"/>
-      <c r="J91" s="21" t="s">
+      <c r="I91" s="20"/>
+      <c r="J91" s="20" t="s">
         <v>467</v>
       </c>
-      <c r="K91" s="21"/>
-      <c r="L91" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M91" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N91" s="21" t="s">
+      <c r="K91" s="20"/>
+      <c r="L91" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M91" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N91" s="20" t="s">
         <v>468</v>
       </c>
     </row>
@@ -6760,76 +6757,76 @@
       </c>
     </row>
     <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A93" s="19"/>
+      <c r="A93" s="18"/>
       <c r="B93" s="19" t="s">
         <v>474</v>
       </c>
-      <c r="C93" s="19" t="s">
+      <c r="C93" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D93" s="21" t="s">
+      <c r="D93" s="20" t="s">
         <v>475</v>
       </c>
-      <c r="E93" s="21" t="s">
+      <c r="E93" s="20" t="s">
         <v>476</v>
       </c>
-      <c r="F93" s="21" t="s">
+      <c r="F93" s="20" t="s">
         <v>465</v>
       </c>
-      <c r="G93" s="21" t="s">
+      <c r="G93" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H93" s="21" t="s">
+      <c r="H93" s="20" t="s">
         <v>477</v>
       </c>
-      <c r="I93" s="21"/>
-      <c r="J93" s="21" t="s">
+      <c r="I93" s="20"/>
+      <c r="J93" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="K93" s="21"/>
-      <c r="L93" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M93" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N93" s="21" t="s">
+      <c r="K93" s="20"/>
+      <c r="L93" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M93" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N93" s="20" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A94" s="19"/>
+      <c r="A94" s="18"/>
       <c r="B94" s="19" t="s">
         <v>478</v>
       </c>
-      <c r="C94" s="19" t="s">
+      <c r="C94" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D94" s="21" t="s">
+      <c r="D94" s="20" t="s">
         <v>479</v>
       </c>
-      <c r="E94" s="21" t="s">
+      <c r="E94" s="20" t="s">
         <v>480</v>
       </c>
-      <c r="F94" s="21" t="s">
+      <c r="F94" s="20" t="s">
         <v>481</v>
       </c>
-      <c r="G94" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H94" s="21" t="s">
+      <c r="G94" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H94" s="20" t="s">
         <v>482</v>
       </c>
-      <c r="I94" s="21"/>
-      <c r="J94" s="21"/>
-      <c r="K94" s="21"/>
-      <c r="L94" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M94" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N94" s="21" t="s">
+      <c r="I94" s="20"/>
+      <c r="J94" s="20"/>
+      <c r="K94" s="20"/>
+      <c r="L94" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M94" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N94" s="20" t="s">
         <v>468</v>
       </c>
     </row>
@@ -7006,78 +7003,78 @@
       <c r="N99" s="17"/>
     </row>
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A100" s="19"/>
+      <c r="A100" s="18"/>
       <c r="B100" s="19" t="s">
         <v>506</v>
       </c>
-      <c r="C100" s="19" t="s">
+      <c r="C100" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D100" s="21" t="s">
+      <c r="D100" s="20" t="s">
         <v>507</v>
       </c>
-      <c r="E100" s="21" t="s">
+      <c r="E100" s="20" t="s">
         <v>508</v>
       </c>
-      <c r="F100" s="21" t="s">
+      <c r="F100" s="20" t="s">
         <v>509</v>
       </c>
-      <c r="G100" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H100" s="21" t="s">
+      <c r="G100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H100" s="20" t="s">
         <v>510</v>
       </c>
-      <c r="I100" s="21"/>
-      <c r="J100" s="21" t="s">
+      <c r="I100" s="20"/>
+      <c r="J100" s="20" t="s">
         <v>511</v>
       </c>
-      <c r="K100" s="21"/>
-      <c r="L100" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M100" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N100" s="21" t="s">
+      <c r="K100" s="20"/>
+      <c r="L100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M100" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N100" s="20" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A101" s="19"/>
+      <c r="A101" s="18"/>
       <c r="B101" s="19" t="s">
         <v>513</v>
       </c>
-      <c r="C101" s="19" t="s">
+      <c r="C101" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D101" s="21" t="s">
+      <c r="D101" s="20" t="s">
         <v>514</v>
       </c>
-      <c r="E101" s="21" t="s">
+      <c r="E101" s="20" t="s">
         <v>515</v>
       </c>
-      <c r="F101" s="21" t="s">
+      <c r="F101" s="20" t="s">
         <v>516</v>
       </c>
-      <c r="G101" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H101" s="21" t="s">
+      <c r="G101" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H101" s="20" t="s">
         <v>517</v>
       </c>
-      <c r="I101" s="21"/>
-      <c r="J101" s="21" t="s">
+      <c r="I101" s="20"/>
+      <c r="J101" s="20" t="s">
         <v>511</v>
       </c>
-      <c r="K101" s="21"/>
-      <c r="L101" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M101" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N101" s="21" t="s">
+      <c r="K101" s="20"/>
+      <c r="L101" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M101" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N101" s="20" t="s">
         <v>512</v>
       </c>
     </row>
@@ -7196,40 +7193,40 @@
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A105" s="19"/>
+      <c r="A105" s="18"/>
       <c r="B105" s="19" t="s">
         <v>533</v>
       </c>
-      <c r="C105" s="19" t="s">
+      <c r="C105" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D105" s="21" t="s">
+      <c r="D105" s="20" t="s">
         <v>534</v>
       </c>
-      <c r="E105" s="21" t="s">
+      <c r="E105" s="20" t="s">
         <v>535</v>
       </c>
-      <c r="F105" s="21" t="s">
+      <c r="F105" s="20" t="s">
         <v>536</v>
       </c>
-      <c r="G105" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H105" s="21" t="s">
+      <c r="G105" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H105" s="20" t="s">
         <v>537</v>
       </c>
-      <c r="I105" s="21"/>
-      <c r="J105" s="21" t="s">
+      <c r="I105" s="20"/>
+      <c r="J105" s="20" t="s">
         <v>511</v>
       </c>
-      <c r="K105" s="21"/>
-      <c r="L105" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M105" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N105" s="21" t="s">
+      <c r="K105" s="20"/>
+      <c r="L105" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M105" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N105" s="20" t="s">
         <v>512</v>
       </c>
     </row>
@@ -7600,46 +7597,46 @@
       </c>
     </row>
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
-      <c r="A116" s="19"/>
+      <c r="A116" s="18"/>
       <c r="B116" s="19" t="s">
         <v>588</v>
       </c>
-      <c r="C116" s="19" t="s">
+      <c r="C116" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D116" s="21" t="s">
+      <c r="D116" s="20" t="s">
         <v>589</v>
       </c>
-      <c r="E116" s="21" t="s">
+      <c r="E116" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="F116" s="21" t="s">
+      <c r="F116" s="20" t="s">
         <v>591</v>
       </c>
-      <c r="G116" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="H116" s="21" t="s">
+      <c r="G116" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H116" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="I116" s="21"/>
-      <c r="J116" s="21" t="s">
+      <c r="I116" s="20"/>
+      <c r="J116" s="20" t="s">
         <v>577</v>
       </c>
-      <c r="K116" s="21"/>
-      <c r="L116" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="M116" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="N116" s="21" t="s">
+      <c r="K116" s="20"/>
+      <c r="L116" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M116" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N116" s="20" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
-      <c r="B117" s="18" t="s">
+      <c r="B117" s="19" t="s">
         <v>593</v>
       </c>
       <c r="C117" s="18" t="s">
@@ -7701,7 +7698,7 @@
     </row>
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
-      <c r="B119" s="18" t="s">
+      <c r="B119" s="19" t="s">
         <v>600</v>
       </c>
       <c r="C119" s="18" t="s">
@@ -7739,7 +7736,7 @@
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
-      <c r="B120" s="18" t="s">
+      <c r="B120" s="19" t="s">
         <v>607</v>
       </c>
       <c r="C120" s="18" t="s">
@@ -7777,7 +7774,7 @@
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
-      <c r="B121" s="18" t="s">
+      <c r="B121" s="19" t="s">
         <v>613</v>
       </c>
       <c r="C121" s="18" t="s">
@@ -7815,7 +7812,7 @@
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
-      <c r="B122" s="18" t="s">
+      <c r="B122" s="19" t="s">
         <v>618</v>
       </c>
       <c r="C122" s="18" t="s">
@@ -7853,7 +7850,7 @@
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
-      <c r="B123" s="18" t="s">
+      <c r="B123" s="19" t="s">
         <v>623</v>
       </c>
       <c r="C123" s="18" t="s">
@@ -7891,7 +7888,7 @@
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
-      <c r="B124" s="18" t="s">
+      <c r="B124" s="19" t="s">
         <v>628</v>
       </c>
       <c r="C124" s="18" t="s">
@@ -7929,7 +7926,7 @@
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
-      <c r="B125" s="18" t="s">
+      <c r="B125" s="19" t="s">
         <v>634</v>
       </c>
       <c r="C125" s="18" t="s">
@@ -7967,7 +7964,7 @@
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
-      <c r="B126" s="18" t="s">
+      <c r="B126" s="19" t="s">
         <v>639</v>
       </c>
       <c r="C126" s="18" t="s">
@@ -8029,7 +8026,7 @@
     </row>
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
-      <c r="B128" s="18" t="s">
+      <c r="B128" s="19" t="s">
         <v>647</v>
       </c>
       <c r="C128" s="18" t="s">
@@ -9044,913 +9041,913 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>783</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="22" t="s">
         <v>784</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="22" t="s">
         <v>785</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="22" t="s">
         <v>786</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="22" t="s">
         <v>787</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="22" t="s">
         <v>788</v>
       </c>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="22" t="s">
         <v>789</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="23" t="s">
         <v>790</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>791</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="25" t="s">
         <v>792</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="25" t="s">
         <v>793</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="25" t="s">
         <v>794</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="25" t="s">
         <v>795</v>
       </c>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="25" t="s">
         <v>796</v>
       </c>
-      <c r="G2" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" s="27" t="s">
+      <c r="G2" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="26" t="s">
         <v>797</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="27" t="s">
         <v>798</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="28" t="s">
         <v>799</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="28" t="s">
         <v>800</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="D3" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="28" t="s">
         <v>801</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="F3" s="28" t="s">
         <v>802</v>
       </c>
-      <c r="G3" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="30" t="s">
+      <c r="G3" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="29" t="s">
         <v>803</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="27" t="s">
         <v>804</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="28" t="s">
         <v>805</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="28" t="s">
         <v>806</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="28" t="s">
         <v>807</v>
       </c>
-      <c r="F4" s="29" t="s">
+      <c r="F4" s="28" t="s">
         <v>808</v>
       </c>
-      <c r="G4" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="30" t="s">
+      <c r="G4" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="29" t="s">
         <v>809</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="27" t="s">
         <v>810</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="28" t="s">
         <v>811</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="28" t="s">
         <v>812</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="28" t="s">
         <v>813</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" s="28" t="s">
         <v>814</v>
       </c>
-      <c r="G5" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="30" t="s">
+      <c r="G5" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="29" t="s">
         <v>815</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="27" t="s">
         <v>816</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="28" t="s">
         <v>402</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="28" t="s">
         <v>817</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="28" t="s">
         <v>818</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="28" t="s">
         <v>819</v>
       </c>
-      <c r="G6" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" s="30" t="s">
+      <c r="G6" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="29" t="s">
         <v>820</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="27" t="s">
         <v>821</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="28" t="s">
         <v>439</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="28" t="s">
         <v>822</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="28" t="s">
         <v>823</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="F7" s="28" t="s">
         <v>824</v>
       </c>
-      <c r="G7" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="30" t="s">
+      <c r="G7" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="29" t="s">
         <v>825</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="27" t="s">
         <v>826</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="28" t="s">
         <v>504</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="28" t="s">
         <v>827</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="28" t="s">
         <v>828</v>
       </c>
-      <c r="F8" s="29" t="s">
+      <c r="F8" s="28" t="s">
         <v>829</v>
       </c>
-      <c r="G8" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I8" s="30" t="s">
+      <c r="G8" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="29" t="s">
         <v>830</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="27" t="s">
         <v>831</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="28" t="s">
         <v>598</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="28" t="s">
         <v>832</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="28" t="s">
         <v>794</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="28" t="s">
         <v>833</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="28" t="s">
         <v>834</v>
       </c>
-      <c r="G9" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="I9" s="30" t="s">
+      <c r="G9" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="29" t="s">
         <v>835</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="30" t="s">
         <v>836</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="31" t="s">
         <v>645</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="31" t="s">
         <v>837</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="31" t="s">
         <v>794</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="E10" s="31" t="s">
         <v>838</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="31" t="s">
         <v>839</v>
       </c>
-      <c r="G10" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="33" t="s">
+      <c r="G10" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="32" t="s">
         <v>840</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="33" t="s">
         <v>841</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35" t="s">
+      <c r="B11" s="34"/>
+      <c r="C11" s="34" t="s">
         <v>842</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="34" t="s">
         <v>843</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="34" t="s">
         <v>844</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="34" t="s">
         <v>845</v>
       </c>
-      <c r="G11" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="I11" s="36" t="s">
+      <c r="G11" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" s="35" t="s">
         <v>846</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="36" t="s">
         <v>847</v>
       </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38" t="s">
+      <c r="B12" s="37"/>
+      <c r="C12" s="37" t="s">
         <v>848</v>
       </c>
-      <c r="D12" s="38" t="s">
+      <c r="D12" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E12" s="38" t="s">
+      <c r="E12" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F12" s="38" t="s">
+      <c r="F12" s="37" t="s">
         <v>849</v>
       </c>
-      <c r="G12" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H12" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I12" s="39" t="s">
+      <c r="G12" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="38" t="s">
         <v>850</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="36" t="s">
         <v>851</v>
       </c>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38" t="s">
+      <c r="B13" s="37"/>
+      <c r="C13" s="37" t="s">
         <v>852</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E13" s="38" t="s">
+      <c r="E13" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F13" s="38" t="s">
+      <c r="F13" s="37" t="s">
         <v>853</v>
       </c>
-      <c r="G13" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H13" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I13" s="39" t="s">
+      <c r="G13" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H13" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" s="38" t="s">
         <v>854</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="36" t="s">
         <v>855</v>
       </c>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38" t="s">
+      <c r="B14" s="37"/>
+      <c r="C14" s="37" t="s">
         <v>856</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E14" s="38" t="s">
+      <c r="E14" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F14" s="38" t="s">
+      <c r="F14" s="37" t="s">
         <v>857</v>
       </c>
-      <c r="G14" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="39" t="s">
+      <c r="G14" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="38" t="s">
         <v>858</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="36" t="s">
         <v>859</v>
       </c>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38" t="s">
+      <c r="B15" s="37"/>
+      <c r="C15" s="37" t="s">
         <v>860</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E15" s="38" t="s">
+      <c r="E15" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F15" s="38" t="s">
+      <c r="F15" s="37" t="s">
         <v>861</v>
       </c>
-      <c r="G15" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I15" s="39" t="s">
+      <c r="G15" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I15" s="38" t="s">
         <v>862</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="36" t="s">
         <v>863</v>
       </c>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38" t="s">
+      <c r="B16" s="37"/>
+      <c r="C16" s="37" t="s">
         <v>864</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E16" s="38" t="s">
+      <c r="E16" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F16" s="38" t="s">
+      <c r="F16" s="37" t="s">
         <v>865</v>
       </c>
-      <c r="G16" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I16" s="39" t="s">
+      <c r="G16" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="38" t="s">
         <v>866</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="36" t="s">
         <v>867</v>
       </c>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38" t="s">
+      <c r="B17" s="37"/>
+      <c r="C17" s="37" t="s">
         <v>868</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F17" s="38" t="s">
+      <c r="F17" s="37" t="s">
         <v>869</v>
       </c>
-      <c r="G17" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H17" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I17" s="39" t="s">
+      <c r="G17" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="38" t="s">
         <v>870</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="36" t="s">
         <v>871</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38" t="s">
+      <c r="B18" s="37"/>
+      <c r="C18" s="37" t="s">
         <v>872</v>
       </c>
-      <c r="D18" s="38" t="s">
+      <c r="D18" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E18" s="38" t="s">
+      <c r="E18" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F18" s="38" t="s">
+      <c r="F18" s="37" t="s">
         <v>873</v>
       </c>
-      <c r="G18" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I18" s="39" t="s">
+      <c r="G18" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" s="38" t="s">
         <v>874</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="36" t="s">
         <v>875</v>
       </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38" t="s">
+      <c r="B19" s="37"/>
+      <c r="C19" s="37" t="s">
         <v>876</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E19" s="38" t="s">
+      <c r="E19" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F19" s="38" t="s">
+      <c r="F19" s="37" t="s">
         <v>877</v>
       </c>
-      <c r="G19" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I19" s="39" t="s">
+      <c r="G19" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19" s="38" t="s">
         <v>878</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="37" t="s">
+      <c r="A20" s="36" t="s">
         <v>879</v>
       </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38" t="s">
+      <c r="B20" s="37"/>
+      <c r="C20" s="37" t="s">
         <v>880</v>
       </c>
-      <c r="D20" s="38" t="s">
+      <c r="D20" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E20" s="38" t="s">
+      <c r="E20" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F20" s="38" t="s">
+      <c r="F20" s="37" t="s">
         <v>881</v>
       </c>
-      <c r="G20" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H20" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I20" s="39" t="s">
+      <c r="G20" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I20" s="38" t="s">
         <v>882</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="36" t="s">
         <v>883</v>
       </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38" t="s">
+      <c r="B21" s="37"/>
+      <c r="C21" s="37" t="s">
         <v>884</v>
       </c>
-      <c r="D21" s="38" t="s">
+      <c r="D21" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E21" s="38" t="s">
+      <c r="E21" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F21" s="38" t="s">
+      <c r="F21" s="37" t="s">
         <v>885</v>
       </c>
-      <c r="G21" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H21" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I21" s="39" t="s">
+      <c r="G21" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="38" t="s">
         <v>886</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="36" t="s">
         <v>887</v>
       </c>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38" t="s">
+      <c r="B22" s="37"/>
+      <c r="C22" s="37" t="s">
         <v>827</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="D22" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E22" s="38" t="s">
+      <c r="E22" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F22" s="38" t="s">
+      <c r="F22" s="37" t="s">
         <v>888</v>
       </c>
-      <c r="G22" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H22" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I22" s="39" t="s">
+      <c r="G22" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H22" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="38" t="s">
         <v>889</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="37" t="s">
+      <c r="A23" s="36" t="s">
         <v>890</v>
       </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38" t="s">
+      <c r="B23" s="37"/>
+      <c r="C23" s="37" t="s">
         <v>832</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D23" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E23" s="38" t="s">
+      <c r="E23" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F23" s="38" t="s">
+      <c r="F23" s="37" t="s">
         <v>891</v>
       </c>
-      <c r="G23" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H23" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I23" s="39" t="s">
+      <c r="G23" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H23" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="38" t="s">
         <v>892</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="36" t="s">
         <v>893</v>
       </c>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38" t="s">
+      <c r="B24" s="37"/>
+      <c r="C24" s="37" t="s">
         <v>894</v>
       </c>
-      <c r="D24" s="38" t="s">
+      <c r="D24" s="37" t="s">
         <v>843</v>
       </c>
-      <c r="E24" s="38" t="s">
+      <c r="E24" s="37" t="s">
         <v>844</v>
       </c>
-      <c r="F24" s="38" t="s">
+      <c r="F24" s="37" t="s">
         <v>895</v>
       </c>
-      <c r="G24" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="H24" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="I24" s="39" t="s">
+      <c r="G24" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" s="38" t="s">
         <v>896</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="40" t="s">
+      <c r="A25" s="39" t="s">
         <v>897</v>
       </c>
-      <c r="B25" s="41"/>
-      <c r="C25" s="41" t="s">
+      <c r="B25" s="40"/>
+      <c r="C25" s="40" t="s">
         <v>837</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E25" s="41" t="s">
+      <c r="E25" s="40" t="s">
         <v>844</v>
       </c>
-      <c r="F25" s="41" t="s">
+      <c r="F25" s="40" t="s">
         <v>898</v>
       </c>
-      <c r="G25" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="42" t="s">
+      <c r="G25" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="41" t="s">
         <v>899</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="39" t="s">
         <v>900</v>
       </c>
-      <c r="B26" s="41"/>
-      <c r="C26" s="41" t="s">
+      <c r="B26" s="40"/>
+      <c r="C26" s="40" t="s">
         <v>901</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E26" s="41" t="s">
+      <c r="E26" s="40" t="s">
         <v>902</v>
       </c>
-      <c r="F26" s="41" t="s">
+      <c r="F26" s="40" t="s">
         <v>903</v>
       </c>
-      <c r="G26" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I26" s="42" t="s">
+      <c r="G26" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="41" t="s">
         <v>904</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="39" t="s">
         <v>905</v>
       </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="41" t="s">
+      <c r="B27" s="40"/>
+      <c r="C27" s="40" t="s">
         <v>906</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E27" s="41" t="s">
+      <c r="E27" s="40" t="s">
         <v>907</v>
       </c>
-      <c r="F27" s="41" t="s">
+      <c r="F27" s="40" t="s">
         <v>908</v>
       </c>
-      <c r="G27" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H27" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I27" s="42" t="s">
+      <c r="G27" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H27" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="41" t="s">
         <v>909</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="40" t="s">
+      <c r="A28" s="39" t="s">
         <v>910</v>
       </c>
-      <c r="B28" s="41"/>
-      <c r="C28" s="41" t="s">
+      <c r="B28" s="40"/>
+      <c r="C28" s="40" t="s">
         <v>911</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E28" s="41" t="s">
+      <c r="E28" s="40" t="s">
         <v>912</v>
       </c>
-      <c r="F28" s="41" t="s">
+      <c r="F28" s="40" t="s">
         <v>913</v>
       </c>
-      <c r="G28" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="42" t="s">
+      <c r="G28" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="41" t="s">
         <v>914</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="39" t="s">
         <v>915</v>
       </c>
-      <c r="B29" s="41"/>
-      <c r="C29" s="41" t="s">
+      <c r="B29" s="40"/>
+      <c r="C29" s="40" t="s">
         <v>916</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E29" s="41" t="s">
+      <c r="E29" s="40" t="s">
         <v>917</v>
       </c>
-      <c r="F29" s="41" t="s">
+      <c r="F29" s="40" t="s">
         <v>918</v>
       </c>
-      <c r="G29" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H29" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29" s="42" t="s">
+      <c r="G29" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="41" t="s">
         <v>919</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="40" t="s">
+      <c r="A30" s="39" t="s">
         <v>920</v>
       </c>
-      <c r="B30" s="41"/>
-      <c r="C30" s="41" t="s">
+      <c r="B30" s="40"/>
+      <c r="C30" s="40" t="s">
         <v>921</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E30" s="41" t="s">
+      <c r="E30" s="40" t="s">
         <v>922</v>
       </c>
-      <c r="F30" s="41" t="s">
+      <c r="F30" s="40" t="s">
         <v>923</v>
       </c>
-      <c r="G30" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="42" t="s">
+      <c r="G30" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H30" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="41" t="s">
         <v>924</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="40" t="s">
+      <c r="A31" s="39" t="s">
         <v>925</v>
       </c>
-      <c r="B31" s="41"/>
-      <c r="C31" s="41" t="s">
+      <c r="B31" s="40"/>
+      <c r="C31" s="40" t="s">
         <v>832</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E31" s="41" t="s">
+      <c r="E31" s="40" t="s">
         <v>926</v>
       </c>
-      <c r="F31" s="41" t="s">
+      <c r="F31" s="40" t="s">
         <v>927</v>
       </c>
-      <c r="G31" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H31" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I31" s="42" t="s">
+      <c r="G31" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H31" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="41" t="s">
         <v>928</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="40" t="s">
+      <c r="A32" s="39" t="s">
         <v>929</v>
       </c>
-      <c r="B32" s="41"/>
-      <c r="C32" s="41" t="s">
+      <c r="B32" s="40"/>
+      <c r="C32" s="40" t="s">
         <v>930</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E32" s="41" t="s">
+      <c r="E32" s="40" t="s">
         <v>931</v>
       </c>
-      <c r="F32" s="41" t="s">
+      <c r="F32" s="40" t="s">
         <v>932</v>
       </c>
-      <c r="G32" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32" s="42" t="s">
+      <c r="G32" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" s="41" t="s">
         <v>933</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="40" t="s">
+      <c r="A33" s="39" t="s">
         <v>934</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="41" t="s">
+      <c r="B33" s="40"/>
+      <c r="C33" s="40" t="s">
         <v>935</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="40" t="s">
         <v>843</v>
       </c>
-      <c r="E33" s="41" t="s">
+      <c r="E33" s="40" t="s">
         <v>936</v>
       </c>
-      <c r="F33" s="41" t="s">
+      <c r="F33" s="40" t="s">
         <v>937</v>
       </c>
-      <c r="G33" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H33" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="I33" s="42" t="s">
+      <c r="G33" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H33" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="41" t="s">
         <v>938</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: correct Stage 6 Pass 009 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,12 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1802" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="948">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
   <si>
-    <t>Stage 1 evidence map derived from legacy code/configuration only. Target and SDD columns remain open until owner-approved design work begins.</t>
+    <t>Legacy evidence map with Stage 5 SDD coverage complete. Destination implementation remains open until each approved delivery slice is built and accepted.</t>
   </si>
   <si>
     <t>Green</t>
@@ -33,7 +33,7 @@
     <t>Red</t>
   </si>
   <si>
-    <t>Missed: source exists, destination does not implement it, SDD does not cover/defer it.</t>
+    <t>Open: source is evidenced and SDD-covered, but destination implementation is not complete and is not deferred.</t>
   </si>
   <si>
     <t>Orange</t>
@@ -105,10 +105,10 @@
     <t>Access, sessions, and channel navigation</t>
   </si>
   <si>
-    <t>Not Passed - Missed</t>
-  </si>
-  <si>
-    <t>Legacy behavior is evidenced; target implementation and SDD coverage have not started.</t>
+    <t>Not Passed - Open</t>
+  </si>
+  <si>
+    <t>Legacy behavior is evidenced and covered by SDD; target implementation has not started.</t>
   </si>
   <si>
     <t>CICS operator opens the banking menu</t>
@@ -507,7 +507,7 @@
     <t>A provider failure is reported and no partial customer is created.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/CRECUST.cbl:363-384,958; Runtime: static-only</t>
+    <t>legacy/src/base/cics/cobol/CRECUST.cbl:473-493,758-814,889-922; Runtime: static-only</t>
   </si>
   <si>
     <t>Customer creation fails transactionally</t>
@@ -987,7 +987,10 @@
     <t>ACCOUNT and PROCTRAN are updated consistently or rolled back.</t>
   </si>
   <si>
-    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl ACCOUNT update and PROCTRAN insert; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-cash; harness: simulation/test; basis: legacy/src/base/cics/cobol/DBCRFUN.cbl:200-555; legacy/src/base/cics/copy/PAYDBCR.cpy</t>
+    <t>legacy/src/base/cics/cobol/DBCRFUN.cbl ACCOUNT update and PROCTRAN insert; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decision D-006: persist balance changes and immutable transaction/audit records atomically.</t>
   </si>
   <si>
     <t>IMS customer deposits or withdraws</t>
@@ -1065,7 +1068,7 @@
     <t>DB2 history is attempted first, IMS history is inserted next, and the account is replaced last; failures can expose partial-write risk according to the coded status handling.</t>
   </si>
   <si>
-    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:326-367,454-554; legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:140; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.ims-transaction; harness: simulation/test; basis: legacy/src/base/ims/cobol/IBTRAN.cbl:290-383; legacy/src/base/ims/LoadData/ACCOUNT.data; legacy/src/base/ims/LoadData/CUSTACCS.data; legacy/src/base/ims/LoadData/HISTORY.data</t>
+    <t>legacy/src/base/ims/cobol/IBTRAN.cbl:326-367,454-554; legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:140; Runtime: static-only</t>
   </si>
   <si>
     <t>Deviation D-006: make balance, history, and audit persistence atomic.</t>
@@ -1281,6 +1284,9 @@
     <t>legacy/src/base/cics/cobol/XFRFUN.cbl:998-1450; Runtime: static-only</t>
   </si>
   <si>
+    <t>Decision D-006: debit, credit, and immutable transaction/audit persistence are atomic.</t>
+  </si>
+  <si>
     <t>Transfer writes transaction evidence</t>
   </si>
   <si>
@@ -1296,6 +1302,9 @@
     <t>legacy/src/base/cics/cobol/XFRFUN.cbl:1563-1639; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
   </si>
   <si>
+    <t>Decision D-006: processed-transfer evidence is committed atomically with both balance mutations.</t>
+  </si>
+  <si>
     <t>Transfer overdraft behavior requires owner decision</t>
   </si>
   <si>
@@ -1356,6 +1365,9 @@
     <t>legacy/src/api/src/main/api/openapi.yaml:275-345; operations ...customers...; zosAssets/INQCUST and UPDCUST; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
+    <t>Decision D-008: expose supported customer capabilities through target REST resources, not path parity.</t>
+  </si>
+  <si>
     <t>External client retrieves CICS accounts and balances</t>
   </si>
   <si>
@@ -1404,6 +1416,9 @@
     <t>legacy/src/api/src/main/api/openapi.yaml:31-245; zosAssets/IBGCUDAT,IBSCUDAT,IBACSUM,IBTRAN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
+    <t>Decision D-008: expose supported IMS-backed capabilities through unified target REST resources.</t>
+  </si>
+  <si>
     <t>External client lists all accounts</t>
   </si>
   <si>
@@ -1467,6 +1482,9 @@
     <t>legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:45-47; Runtime: static-only</t>
   </si>
   <si>
+    <t>Decision D-008: target history resources preserve supported behavior without reproducing legacy route defects.</t>
+  </si>
+  <si>
     <t>API client receives standard failures</t>
   </si>
   <si>
@@ -1515,6 +1533,9 @@
     <t>legacy/src/api/src/main/api/openapi.yaml:246-274; legacy/src/api/src/main/operations/%2Fcustomers/post/operation.yaml; legacy/src/api/src/main/zosAssets/CRECUST/zosAsset.yaml; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
   </si>
   <si>
+    <t>Decision D-008: customer creation is exposed as a supported target capability, not legacy path parity.</t>
+  </si>
+  <si>
     <t>IMS client requests recent history through IBGHIST</t>
   </si>
   <si>
@@ -1746,7 +1767,7 @@
     <t>Static files are returned and index.html redirects the browser to admin.html.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js:14-51; legacy/src/frontend/index.html redirects to admin.html; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
+    <t>legacy/src/frontend/server.js:14-51; legacy/src/frontend/index.html redirects to admin.html; Runtime: static-only</t>
   </si>
   <si>
     <t>Deviation D-001/D-002/D-014: secure same-origin Angular/API shell replaces the unauthenticated proxy panel.</t>
@@ -1764,7 +1785,7 @@
     <t>Requests and responses are streamed to/from API_BASE_URL.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js proxy paths; config.js base URL; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
+    <t>legacy/src/frontend/server.js proxy paths; config.js base URL; Runtime: static-only</t>
   </si>
   <si>
     <t>Web static file is missing</t>
@@ -1809,7 +1830,7 @@
     <t>No application login challenge is presented; target access control requires explicit owner approval rather than silent inheritance.</t>
   </si>
   <si>
-    <t>legacy/src/frontend/server.js:1-111; legacy/src/frontend/admin.html:1-103; no authentication middleware or login page is present under legacy/src/frontend; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.web-edge; harness: simulation/test; basis: legacy/src/frontend/server.js; legacy/src/frontend/index.html; legacy/src/frontend/admin.html</t>
+    <t>legacy/src/frontend/server.js:1-111; legacy/src/frontend/admin.html:1-103; no authentication middleware or login page is present under legacy/src/frontend; Runtime: static-only</t>
   </si>
   <si>
     <t>UF-011</t>
@@ -1854,7 +1875,7 @@
     <t>legacy/src/base/ims/cobol/LOADCUST.cbl; Runtime: static-only</t>
   </si>
   <si>
-    <t>Deviation D-013: explicit EF migrations and import/demo command replace IBM loaders and DB2 preparation.</t>
+    <t>Decisions D-013/D-021: staged validation and atomic promotion replace partial legacy loading.</t>
   </si>
   <si>
     <t>Operator loads IMS accounts</t>
@@ -1935,6 +1956,9 @@
     <t>legacy/.setup/setup/populate-ims-tables.sh:27-52; legacy/src/base/ims/LoadData/ACCTYPE.data; legacy/src/base/ims/LoadData/CUSTTYPE.data; legacy/src/base/ims/LoadData/TSTATTYP.data; legacy/src/base/ims/LoadData/TTYPE.data; Runtime: static-only</t>
   </si>
   <si>
+    <t>Decisions D-013/D-021: explicit import validates supported reference data before atomic promotion.</t>
+  </si>
+  <si>
     <t>Operator prepares DB2 structures and access</t>
   </si>
   <si>
@@ -2544,7 +2568,7 @@
     <t>R1-D-001</t>
   </si>
   <si>
-    <t>8-14,113</t>
+    <t>8-14,113-117</t>
   </si>
   <si>
     <t>decision</t>
@@ -2562,7 +2586,7 @@
     <t>R1-D-002</t>
   </si>
   <si>
-    <t>15-20,109,117</t>
+    <t>15-20,109,113-117</t>
   </si>
   <si>
     <t>Owner-approved target decision D-002 recorded in Stage 4.</t>
@@ -2586,7 +2610,7 @@
     <t>R1-D-004</t>
   </si>
   <si>
-    <t>75-78,84</t>
+    <t>72-78,84</t>
   </si>
   <si>
     <t>Owner-approved target decision D-004 recorded in Stage 4.</t>
@@ -2598,7 +2622,7 @@
     <t>R1-D-005</t>
   </si>
   <si>
-    <t>72-74</t>
+    <t>72-78</t>
   </si>
   <si>
     <t>Owner-approved target decision D-005 recorded in Stage 4.</t>
@@ -2610,7 +2634,7 @@
     <t>R1-D-006</t>
   </si>
   <si>
-    <t>63,68,82-83</t>
+    <t>63,68,82-83,134</t>
   </si>
   <si>
     <t>Owner-approved target decision D-006 recorded in Stage 4.</t>
@@ -2634,7 +2658,7 @@
     <t>R1-D-008</t>
   </si>
   <si>
-    <t>87-98</t>
+    <t>87-88,90-98</t>
   </si>
   <si>
     <t>Owner-approved target decision D-008 recorded in Stage 4.</t>
@@ -2646,7 +2670,7 @@
     <t>R1-D-009</t>
   </si>
   <si>
-    <t>34,36,39,53,56,58</t>
+    <t>38-39,53,56,58</t>
   </si>
   <si>
     <t>Owner-approved target decision D-009 recorded in Stage 4.</t>
@@ -2700,7 +2724,7 @@
     <t>R1-D-014</t>
   </si>
   <si>
-    <t>114-116,128-153</t>
+    <t>113-117,128-132,134-135,137-149,151-153</t>
   </si>
   <si>
     <t>Owner-approved target decision D-014 recorded in Stage 4.</t>
@@ -2712,6 +2736,9 @@
     <t>R1-D-015</t>
   </si>
   <si>
+    <t>128-132,135,137-149,151-153</t>
+  </si>
+  <si>
     <t>Owner-approved target decision D-015 recorded in Stage 4.</t>
   </si>
   <si>
@@ -2757,7 +2784,7 @@
     <t>Name search is unsupported and failed lookup can retain stale customer state.</t>
   </si>
   <si>
-    <t>Target normalized search is implemented; failed lookup clears stale state and disables mutation.</t>
+    <t>Target implements normalized search; failed lookup clears stale state and disables mutation.</t>
   </si>
   <si>
     <t>analysis/stage-04-requirements-revision.md#d-018</t>
@@ -5688,7 +5715,9 @@
         <v>323</v>
       </c>
       <c r="I63" s="20"/>
-      <c r="J63" s="20"/>
+      <c r="J63" s="20" t="s">
+        <v>324</v>
+      </c>
       <c r="K63" s="20"/>
       <c r="L63" s="20" t="s">
         <v>36</v>
@@ -5703,25 +5732,25 @@
     <row r="64" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A64" s="18"/>
       <c r="B64" s="19" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C64" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D64" s="20" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F64" s="20" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G64" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H64" s="20" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I64" s="20"/>
       <c r="J64" s="20"/>
@@ -5739,25 +5768,25 @@
     <row r="65" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A65" s="18"/>
       <c r="B65" s="19" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C65" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D65" s="20" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E65" s="20" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F65" s="20" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G65" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H65" s="20" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="I65" s="20"/>
       <c r="J65" s="20"/>
@@ -5775,25 +5804,25 @@
     <row r="66" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A66" s="18"/>
       <c r="B66" s="19" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C66" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D66" s="20" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E66" s="20" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F66" s="20" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H66" s="20" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="I66" s="20"/>
       <c r="J66" s="20"/>
@@ -5811,29 +5840,29 @@
     <row r="67" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A67" s="18"/>
       <c r="B67" s="19" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C67" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D67" s="20" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E67" s="20" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F67" s="20" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G67" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H67" s="20" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="I67" s="20"/>
       <c r="J67" s="20" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K67" s="20"/>
       <c r="L67" s="20" t="s">
@@ -5849,29 +5878,29 @@
     <row r="68" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A68" s="18"/>
       <c r="B68" s="19" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C68" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D68" s="20" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E68" s="20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F68" s="20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G68" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H68" s="20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I68" s="20"/>
       <c r="J68" s="20" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K68" s="20"/>
       <c r="L68" s="20" t="s">
@@ -5887,29 +5916,29 @@
     <row r="69" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A69" s="18"/>
       <c r="B69" s="19" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C69" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D69" s="20" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E69" s="20" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F69" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G69" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H69" s="20" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="I69" s="20"/>
       <c r="J69" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K69" s="20"/>
       <c r="L69" s="20" t="s">
@@ -5925,25 +5954,25 @@
     <row r="70" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A70" s="18"/>
       <c r="B70" s="19" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C70" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D70" s="20" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E70" s="20" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F70" s="20" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G70" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="I70" s="20"/>
       <c r="J70" s="20"/>
@@ -5961,29 +5990,29 @@
     <row r="71" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A71" s="18"/>
       <c r="B71" s="19" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C71" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D71" s="20" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E71" s="20" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F71" s="20" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G71" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H71" s="20" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I71" s="20"/>
       <c r="J71" s="20" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K71" s="20"/>
       <c r="L71" s="20" t="s">
@@ -5999,29 +6028,29 @@
     <row r="72" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A72" s="18"/>
       <c r="B72" s="19" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C72" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D72" s="20" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E72" s="20" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F72" s="20" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="G72" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H72" s="20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="I72" s="20"/>
       <c r="J72" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K72" s="20"/>
       <c r="L72" s="20" t="s">
@@ -6037,29 +6066,29 @@
     <row r="73" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A73" s="18"/>
       <c r="B73" s="19" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C73" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D73" s="20" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E73" s="20" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F73" s="20" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G73" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H73" s="20" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="I73" s="20"/>
       <c r="J73" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K73" s="20"/>
       <c r="L73" s="20" t="s">
@@ -6075,29 +6104,29 @@
     <row r="74" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A74" s="18"/>
       <c r="B74" s="19" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C74" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D74" s="20" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E74" s="20" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F74" s="20" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G74" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H74" s="20" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="I74" s="20"/>
       <c r="J74" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K74" s="20"/>
       <c r="L74" s="20" t="s">
@@ -6113,29 +6142,29 @@
     <row r="75" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A75" s="18"/>
       <c r="B75" s="19" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C75" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D75" s="20" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E75" s="20" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G75" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H75" s="20" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I75" s="20"/>
       <c r="J75" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K75" s="20"/>
       <c r="L75" s="20" t="s">
@@ -6151,29 +6180,29 @@
     <row r="76" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A76" s="18"/>
       <c r="B76" s="19" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C76" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D76" s="20" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F76" s="20" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G76" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H76" s="20" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I76" s="20"/>
       <c r="J76" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K76" s="20"/>
       <c r="L76" s="20" t="s">
@@ -6189,29 +6218,29 @@
     <row r="77" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A77" s="18"/>
       <c r="B77" s="19" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C77" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D77" s="20" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E77" s="20" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F77" s="20" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G77" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H77" s="20" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I77" s="20"/>
       <c r="J77" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K77" s="20"/>
       <c r="L77" s="20" t="s">
@@ -6227,29 +6256,29 @@
     <row r="78" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A78" s="18"/>
       <c r="B78" s="19" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C78" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="20" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E78" s="20" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F78" s="20" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G78" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H78" s="20" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I78" s="20"/>
       <c r="J78" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K78" s="20"/>
       <c r="L78" s="20" t="s">
@@ -6264,10 +6293,10 @@
     </row>
     <row r="79" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C79" s="17" t="s">
         <v>29</v>
@@ -6289,29 +6318,29 @@
     <row r="80" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A80" s="18"/>
       <c r="B80" s="19" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C80" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D80" s="20" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E80" s="20" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F80" s="20" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G80" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H80" s="20" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="I80" s="20"/>
       <c r="J80" s="20" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K80" s="20"/>
       <c r="L80" s="20" t="s">
@@ -6321,31 +6350,31 @@
         <v>39</v>
       </c>
       <c r="N80" s="20" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="81" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A81" s="18"/>
       <c r="B81" s="19" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C81" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D81" s="20" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E81" s="20" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F81" s="20" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G81" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H81" s="20" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="I81" s="20"/>
       <c r="J81" s="20"/>
@@ -6357,34 +6386,36 @@
         <v>39</v>
       </c>
       <c r="N81" s="20" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="82" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A82" s="18"/>
       <c r="B82" s="19" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C82" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E82" s="20" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F82" s="20" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G82" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H82" s="20" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I82" s="20"/>
-      <c r="J82" s="20"/>
+      <c r="J82" s="20" t="s">
+        <v>422</v>
+      </c>
       <c r="K82" s="20"/>
       <c r="L82" s="20" t="s">
         <v>36</v>
@@ -6393,34 +6424,36 @@
         <v>39</v>
       </c>
       <c r="N82" s="20" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="83" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="18"/>
       <c r="B83" s="19" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C83" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D83" s="20" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="E83" s="20" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="F83" s="20" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="G83" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H83" s="20" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="I83" s="20"/>
-      <c r="J83" s="20"/>
+      <c r="J83" s="20" t="s">
+        <v>428</v>
+      </c>
       <c r="K83" s="20"/>
       <c r="L83" s="20" t="s">
         <v>36</v>
@@ -6429,35 +6462,35 @@
         <v>39</v>
       </c>
       <c r="N83" s="20" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="84" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="18"/>
       <c r="B84" s="19" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="C84" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E84" s="20" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="F84" s="20" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="G84" s="20" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="H84" s="20" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="I84" s="20"/>
       <c r="J84" s="20" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="K84" s="20"/>
       <c r="L84" s="20" t="s">
@@ -6467,35 +6500,35 @@
         <v>39</v>
       </c>
       <c r="N84" s="20" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="85" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="C85" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D85" s="20" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E85" s="20" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F85" s="20" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="G85" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H85" s="20" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="I85" s="20"/>
       <c r="J85" s="20" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="K85" s="20"/>
       <c r="L85" s="20" t="s">
@@ -6505,15 +6538,15 @@
         <v>39</v>
       </c>
       <c r="N85" s="20" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="B86" s="17" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C86" s="17" t="s">
         <v>29</v>
@@ -6535,28 +6568,30 @@
     <row r="87" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="C87" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D87" s="20" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="E87" s="20" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F87" s="20" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G87" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H87" s="20" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="I87" s="20"/>
-      <c r="J87" s="20"/>
+      <c r="J87" s="20" t="s">
+        <v>449</v>
+      </c>
       <c r="K87" s="20"/>
       <c r="L87" s="20" t="s">
         <v>36</v>
@@ -6571,29 +6606,29 @@
     <row r="88" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="C88" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="E88" s="20" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="F88" s="20" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="G88" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H88" s="20" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="I88" s="20"/>
       <c r="J88" s="20" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="K88" s="20"/>
       <c r="L88" s="20" t="s">
@@ -6609,29 +6644,29 @@
     <row r="89" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="C89" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="F89" s="20" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="G89" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H89" s="20" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="I89" s="20"/>
       <c r="J89" s="20" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K89" s="20"/>
       <c r="L89" s="20" t="s">
@@ -6647,28 +6682,30 @@
     <row r="90" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="C90" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D90" s="20" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="E90" s="20" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="F90" s="20" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="G90" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H90" s="20" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="I90" s="20"/>
-      <c r="J90" s="20"/>
+      <c r="J90" s="20" t="s">
+        <v>466</v>
+      </c>
       <c r="K90" s="20"/>
       <c r="L90" s="20" t="s">
         <v>36</v>
@@ -6683,29 +6720,29 @@
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="18"/>
       <c r="B91" s="19" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="C91" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D91" s="20" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="E91" s="20" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="F91" s="20" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="G91" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H91" s="20" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="I91" s="20"/>
       <c r="J91" s="20" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="K91" s="20"/>
       <c r="L91" s="20" t="s">
@@ -6715,35 +6752,35 @@
         <v>39</v>
       </c>
       <c r="N91" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="92" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="C92" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D92" s="20" t="s">
+        <v>475</v>
+      </c>
+      <c r="E92" s="20" t="s">
+        <v>476</v>
+      </c>
+      <c r="F92" s="20" t="s">
         <v>470</v>
-      </c>
-      <c r="E92" s="20" t="s">
-        <v>471</v>
-      </c>
-      <c r="F92" s="20" t="s">
-        <v>465</v>
       </c>
       <c r="G92" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H92" s="20" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="I92" s="20"/>
       <c r="J92" s="20" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="K92" s="20"/>
       <c r="L92" s="20" t="s">
@@ -6753,35 +6790,35 @@
         <v>39</v>
       </c>
       <c r="N92" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="18"/>
       <c r="B93" s="19" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C93" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D93" s="20" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E93" s="20" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="F93" s="20" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="G93" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H93" s="20" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="I93" s="20"/>
       <c r="J93" s="20" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="K93" s="20"/>
       <c r="L93" s="20" t="s">
@@ -6791,34 +6828,36 @@
         <v>39</v>
       </c>
       <c r="N93" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="18"/>
       <c r="B94" s="19" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="C94" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D94" s="20" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="E94" s="20" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="F94" s="20" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="G94" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H94" s="20" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="I94" s="20"/>
-      <c r="J94" s="20"/>
+      <c r="J94" s="20" t="s">
+        <v>488</v>
+      </c>
       <c r="K94" s="20"/>
       <c r="L94" s="20" t="s">
         <v>36</v>
@@ -6827,35 +6866,35 @@
         <v>39</v>
       </c>
       <c r="N94" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="C95" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D95" s="20" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="E95" s="20" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="F95" s="20" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="G95" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H95" s="20" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="I95" s="20"/>
       <c r="J95" s="20" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="K95" s="20"/>
       <c r="L95" s="20" t="s">
@@ -6865,35 +6904,35 @@
         <v>39</v>
       </c>
       <c r="N95" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="96" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D96" s="20" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="E96" s="20" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="F96" s="20" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="G96" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H96" s="20" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="I96" s="20"/>
       <c r="J96" s="20" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="K96" s="20"/>
       <c r="L96" s="20" t="s">
@@ -6903,34 +6942,36 @@
         <v>39</v>
       </c>
       <c r="N96" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="97" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="C97" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D97" s="20" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="E97" s="20" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="F97" s="20" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="G97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H97" s="20" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="I97" s="20"/>
-      <c r="J97" s="20"/>
+      <c r="J97" s="20" t="s">
+        <v>505</v>
+      </c>
       <c r="K97" s="20"/>
       <c r="L97" s="20" t="s">
         <v>36</v>
@@ -6945,28 +6986,30 @@
     <row r="98" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="C98" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D98" s="20" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="E98" s="20" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
       <c r="F98" s="20" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
       <c r="G98" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H98" s="20" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="I98" s="20"/>
-      <c r="J98" s="20"/>
+      <c r="J98" s="20" t="s">
+        <v>488</v>
+      </c>
       <c r="K98" s="20"/>
       <c r="L98" s="20" t="s">
         <v>36</v>
@@ -6975,15 +7018,15 @@
         <v>39</v>
       </c>
       <c r="N98" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="B99" s="17" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="C99" s="17" t="s">
         <v>29</v>
@@ -7005,29 +7048,29 @@
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="18"/>
       <c r="B100" s="19" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="C100" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D100" s="20" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
       <c r="E100" s="20" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="F100" s="20" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="G100" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H100" s="20" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="I100" s="20"/>
       <c r="J100" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K100" s="20"/>
       <c r="L100" s="20" t="s">
@@ -7037,35 +7080,35 @@
         <v>39</v>
       </c>
       <c r="N100" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="18"/>
       <c r="B101" s="19" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="C101" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D101" s="20" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="E101" s="20" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="F101" s="20" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="G101" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H101" s="20" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
       <c r="I101" s="20"/>
       <c r="J101" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K101" s="20"/>
       <c r="L101" s="20" t="s">
@@ -7075,35 +7118,35 @@
         <v>39</v>
       </c>
       <c r="N101" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D102" s="20" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="E102" s="20" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="F102" s="20" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="G102" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H102" s="20" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
       <c r="I102" s="20"/>
       <c r="J102" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K102" s="20"/>
       <c r="L102" s="20" t="s">
@@ -7113,35 +7156,35 @@
         <v>39</v>
       </c>
       <c r="N102" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="C103" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D103" s="20" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="E103" s="20" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="F103" s="20" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="G103" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H103" s="20" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="I103" s="20"/>
       <c r="J103" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K103" s="20"/>
       <c r="L103" s="20" t="s">
@@ -7151,35 +7194,35 @@
         <v>39</v>
       </c>
       <c r="N103" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D104" s="20" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="E104" s="20" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="F104" s="20" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="G104" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H104" s="20" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="I104" s="20"/>
       <c r="J104" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K104" s="20"/>
       <c r="L104" s="20" t="s">
@@ -7189,35 +7232,35 @@
         <v>39</v>
       </c>
       <c r="N104" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="18"/>
       <c r="B105" s="19" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="C105" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D105" s="20" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="E105" s="20" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="F105" s="20" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="G105" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H105" s="20" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="I105" s="20"/>
       <c r="J105" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K105" s="20"/>
       <c r="L105" s="20" t="s">
@@ -7227,35 +7270,35 @@
         <v>39</v>
       </c>
       <c r="N105" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="C106" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D106" s="20" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="E106" s="20" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="F106" s="20" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="G106" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H106" s="20" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="I106" s="20"/>
       <c r="J106" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K106" s="20"/>
       <c r="L106" s="20" t="s">
@@ -7265,35 +7308,35 @@
         <v>39</v>
       </c>
       <c r="N106" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="C107" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D107" s="20" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="E107" s="20" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
       <c r="F107" s="20" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="G107" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H107" s="20" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="I107" s="20"/>
       <c r="J107" s="20" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="K107" s="20"/>
       <c r="L107" s="20" t="s">
@@ -7303,15 +7346,15 @@
         <v>39</v>
       </c>
       <c r="N107" s="20" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
     </row>
     <row r="108" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="B108" s="17" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="C108" s="17" t="s">
         <v>29</v>
@@ -7333,29 +7376,29 @@
     <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="C109" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="E109" s="20" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="F109" s="20" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="I109" s="20"/>
       <c r="J109" s="20" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="K109" s="20"/>
       <c r="L109" s="20" t="s">
@@ -7371,29 +7414,29 @@
     <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="C110" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="F110" s="20" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="G110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="I110" s="20"/>
       <c r="J110" s="20" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="K110" s="20"/>
       <c r="L110" s="20" t="s">
@@ -7409,29 +7452,29 @@
     <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="C111" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D111" s="20" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="E111" s="20" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="F111" s="20" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="G111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
       <c r="I111" s="20"/>
       <c r="J111" s="20" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="K111" s="20"/>
       <c r="L111" s="20" t="s">
@@ -7447,29 +7490,29 @@
     <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
       <c r="C112" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
       <c r="F112" s="20" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="G112" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="I112" s="20"/>
       <c r="J112" s="20" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="K112" s="20"/>
       <c r="L112" s="20" t="s">
@@ -7485,29 +7528,29 @@
     <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="C113" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>575</v>
+        <v>582</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>576</v>
+        <v>583</v>
       </c>
       <c r="I113" s="20"/>
       <c r="J113" s="20" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="K113" s="20"/>
       <c r="L113" s="20" t="s">
@@ -7523,29 +7566,29 @@
     <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>578</v>
+        <v>585</v>
       </c>
       <c r="C114" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D114" s="20" t="s">
-        <v>579</v>
+        <v>586</v>
       </c>
       <c r="E114" s="20" t="s">
-        <v>580</v>
+        <v>587</v>
       </c>
       <c r="F114" s="20" t="s">
-        <v>581</v>
+        <v>588</v>
       </c>
       <c r="G114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="20" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
       <c r="I114" s="20"/>
       <c r="J114" s="20" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="K114" s="20"/>
       <c r="L114" s="20" t="s">
@@ -7561,29 +7604,29 @@
     <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="C115" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D115" s="20" t="s">
-        <v>584</v>
+        <v>591</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>585</v>
+        <v>592</v>
       </c>
       <c r="F115" s="20" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
       <c r="G115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="20" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
       <c r="I115" s="20"/>
       <c r="J115" s="20" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="K115" s="20"/>
       <c r="L115" s="20" t="s">
@@ -7599,29 +7642,29 @@
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="18"/>
       <c r="B116" s="19" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
       <c r="C116" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D116" s="20" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
       <c r="E116" s="20" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="F116" s="20" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="G116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H116" s="20" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
       <c r="I116" s="20"/>
       <c r="J116" s="20" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="K116" s="20"/>
       <c r="L116" s="20" t="s">
@@ -7637,29 +7680,29 @@
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
       <c r="B117" s="19" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
       <c r="C117" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="E117" s="20" t="s">
-        <v>595</v>
+        <v>602</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>596</v>
+        <v>603</v>
       </c>
       <c r="G117" s="20" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
       <c r="I117" s="20"/>
       <c r="J117" s="20" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="K117" s="20"/>
       <c r="L117" s="20" t="s">
@@ -7674,10 +7717,10 @@
     </row>
     <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="17" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
       <c r="B118" s="17" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
       <c r="C118" s="17" t="s">
         <v>29</v>
@@ -7699,29 +7742,29 @@
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="19" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D119" s="20" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
       <c r="E119" s="20" t="s">
-        <v>602</v>
+        <v>609</v>
       </c>
       <c r="F119" s="20" t="s">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="G119" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="20" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
       <c r="I119" s="20"/>
       <c r="J119" s="20" t="s">
-        <v>605</v>
+        <v>612</v>
       </c>
       <c r="K119" s="20"/>
       <c r="L119" s="20" t="s">
@@ -7731,35 +7774,35 @@
         <v>39</v>
       </c>
       <c r="N119" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="19" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D120" s="20" t="s">
-        <v>608</v>
+        <v>615</v>
       </c>
       <c r="E120" s="20" t="s">
-        <v>609</v>
+        <v>616</v>
       </c>
       <c r="F120" s="20" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="G120" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="20" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
       <c r="I120" s="20"/>
       <c r="J120" s="20" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="K120" s="20"/>
       <c r="L120" s="20" t="s">
@@ -7769,35 +7812,35 @@
         <v>39</v>
       </c>
       <c r="N120" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
       <c r="B121" s="19" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
       <c r="C121" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D121" s="20" t="s">
-        <v>614</v>
+        <v>621</v>
       </c>
       <c r="E121" s="20" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="F121" s="20" t="s">
-        <v>616</v>
+        <v>623</v>
       </c>
       <c r="G121" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="20" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
       <c r="I121" s="20"/>
       <c r="J121" s="20" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="K121" s="20"/>
       <c r="L121" s="20" t="s">
@@ -7807,35 +7850,35 @@
         <v>39</v>
       </c>
       <c r="N121" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="19" t="s">
-        <v>618</v>
+        <v>625</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D122" s="20" t="s">
-        <v>619</v>
+        <v>626</v>
       </c>
       <c r="E122" s="20" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
       <c r="F122" s="20" t="s">
-        <v>621</v>
+        <v>628</v>
       </c>
       <c r="G122" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="20" t="s">
-        <v>622</v>
+        <v>629</v>
       </c>
       <c r="I122" s="20"/>
       <c r="J122" s="20" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="K122" s="20"/>
       <c r="L122" s="20" t="s">
@@ -7845,35 +7888,35 @@
         <v>39</v>
       </c>
       <c r="N122" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="19" t="s">
-        <v>623</v>
+        <v>630</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D123" s="20" t="s">
-        <v>624</v>
+        <v>631</v>
       </c>
       <c r="E123" s="20" t="s">
-        <v>625</v>
+        <v>632</v>
       </c>
       <c r="F123" s="20" t="s">
-        <v>626</v>
+        <v>633</v>
       </c>
       <c r="G123" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H123" s="20" t="s">
-        <v>627</v>
+        <v>634</v>
       </c>
       <c r="I123" s="20"/>
       <c r="J123" s="20" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="K123" s="20"/>
       <c r="L123" s="20" t="s">
@@ -7883,35 +7926,35 @@
         <v>39</v>
       </c>
       <c r="N123" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="19" t="s">
-        <v>628</v>
+        <v>635</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D124" s="20" t="s">
-        <v>629</v>
+        <v>636</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>630</v>
+        <v>637</v>
       </c>
       <c r="F124" s="20" t="s">
-        <v>631</v>
+        <v>638</v>
       </c>
       <c r="G124" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H124" s="20" t="s">
-        <v>632</v>
+        <v>639</v>
       </c>
       <c r="I124" s="20"/>
       <c r="J124" s="20" t="s">
-        <v>633</v>
+        <v>640</v>
       </c>
       <c r="K124" s="20"/>
       <c r="L124" s="20" t="s">
@@ -7921,35 +7964,35 @@
         <v>39</v>
       </c>
       <c r="N124" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="19" t="s">
-        <v>634</v>
+        <v>641</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D125" s="20" t="s">
-        <v>635</v>
+        <v>642</v>
       </c>
       <c r="E125" s="20" t="s">
-        <v>636</v>
+        <v>643</v>
       </c>
       <c r="F125" s="20" t="s">
-        <v>637</v>
+        <v>644</v>
       </c>
       <c r="G125" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H125" s="20" t="s">
-        <v>638</v>
+        <v>645</v>
       </c>
       <c r="I125" s="20"/>
       <c r="J125" s="20" t="s">
-        <v>612</v>
+        <v>646</v>
       </c>
       <c r="K125" s="20"/>
       <c r="L125" s="20" t="s">
@@ -7959,35 +8002,35 @@
         <v>39</v>
       </c>
       <c r="N125" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="19" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D126" s="20" t="s">
-        <v>640</v>
+        <v>648</v>
       </c>
       <c r="E126" s="20" t="s">
-        <v>641</v>
+        <v>649</v>
       </c>
       <c r="F126" s="20" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="G126" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="20" t="s">
-        <v>643</v>
+        <v>651</v>
       </c>
       <c r="I126" s="20"/>
       <c r="J126" s="20" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="K126" s="20"/>
       <c r="L126" s="20" t="s">
@@ -7997,15 +8040,15 @@
         <v>39</v>
       </c>
       <c r="N126" s="20" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
     </row>
     <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="17" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="B127" s="17" t="s">
-        <v>646</v>
+        <v>654</v>
       </c>
       <c r="C127" s="17" t="s">
         <v>29</v>
@@ -8027,29 +8070,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>647</v>
+        <v>655</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D128" s="20" t="s">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="E128" s="20" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="F128" s="20" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
       <c r="G128" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="20" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="I128" s="20"/>
       <c r="J128" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K128" s="20"/>
       <c r="L128" s="20" t="s">
@@ -8059,35 +8102,35 @@
         <v>39</v>
       </c>
       <c r="N128" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D129" s="20" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="E129" s="20" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="F129" s="20" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="G129" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="20" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="I129" s="20"/>
       <c r="J129" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K129" s="20"/>
       <c r="L129" s="20" t="s">
@@ -8097,35 +8140,35 @@
         <v>39</v>
       </c>
       <c r="N129" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="18"/>
       <c r="B130" s="19" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D130" s="20" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="E130" s="20" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="F130" s="20" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="G130" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="20" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="I130" s="20"/>
       <c r="J130" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K130" s="20"/>
       <c r="L130" s="20" t="s">
@@ -8135,35 +8178,35 @@
         <v>39</v>
       </c>
       <c r="N130" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D131" s="20" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="E131" s="20" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="F131" s="20" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="G131" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H131" s="20" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="I131" s="20"/>
       <c r="J131" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K131" s="20"/>
       <c r="L131" s="20" t="s">
@@ -8173,35 +8216,35 @@
         <v>39</v>
       </c>
       <c r="N131" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D132" s="20" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="E132" s="20" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="F132" s="20" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="G132" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="20" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="I132" s="20"/>
       <c r="J132" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K132" s="20"/>
       <c r="L132" s="20" t="s">
@@ -8211,35 +8254,35 @@
         <v>39</v>
       </c>
       <c r="N132" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D133" s="20" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="E133" s="20" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="F133" s="20" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="G133" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H133" s="20" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="I133" s="20"/>
       <c r="J133" s="20" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="K133" s="20"/>
       <c r="L133" s="20" t="s">
@@ -8249,35 +8292,35 @@
         <v>39</v>
       </c>
       <c r="N133" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D134" s="20" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="E134" s="20" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="F134" s="20" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="G134" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="20" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="I134" s="20"/>
       <c r="J134" s="20" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="K134" s="20"/>
       <c r="L134" s="20" t="s">
@@ -8287,35 +8330,35 @@
         <v>39</v>
       </c>
       <c r="N134" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D135" s="20" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="E135" s="20" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="F135" s="20" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
       <c r="G135" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H135" s="20" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="I135" s="20"/>
       <c r="J135" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K135" s="20"/>
       <c r="L135" s="20" t="s">
@@ -8325,35 +8368,35 @@
         <v>39</v>
       </c>
       <c r="N135" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D136" s="20" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="E136" s="20" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
       <c r="F136" s="20" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="G136" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H136" s="20" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="I136" s="20"/>
       <c r="J136" s="20" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="K136" s="20"/>
       <c r="L136" s="20" t="s">
@@ -8363,35 +8406,35 @@
         <v>39</v>
       </c>
       <c r="N136" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D137" s="20" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="E137" s="20" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="F137" s="20" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="G137" s="20" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="H137" s="20" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="I137" s="20"/>
       <c r="J137" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K137" s="20"/>
       <c r="L137" s="20" t="s">
@@ -8401,35 +8444,35 @@
         <v>39</v>
       </c>
       <c r="N137" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D138" s="20" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="E138" s="20" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="F138" s="20" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="G138" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="20" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="I138" s="20"/>
       <c r="J138" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K138" s="20"/>
       <c r="L138" s="20" t="s">
@@ -8439,35 +8482,35 @@
         <v>39</v>
       </c>
       <c r="N138" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D139" s="20" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="E139" s="20" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="F139" s="20" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="G139" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="20" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="I139" s="20"/>
       <c r="J139" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K139" s="20"/>
       <c r="L139" s="20" t="s">
@@ -8477,35 +8520,35 @@
         <v>39</v>
       </c>
       <c r="N139" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D140" s="20" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="E140" s="20" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="F140" s="20" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="G140" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="20" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="I140" s="20"/>
       <c r="J140" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K140" s="20"/>
       <c r="L140" s="20" t="s">
@@ -8515,35 +8558,35 @@
         <v>39</v>
       </c>
       <c r="N140" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D141" s="20" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="E141" s="20" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="F141" s="20" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="G141" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="20" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="I141" s="20"/>
       <c r="J141" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K141" s="20"/>
       <c r="L141" s="20" t="s">
@@ -8553,35 +8596,35 @@
         <v>39</v>
       </c>
       <c r="N141" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D142" s="20" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="E142" s="20" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="F142" s="20" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="G142" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="I142" s="20"/>
       <c r="J142" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K142" s="20"/>
       <c r="L142" s="20" t="s">
@@ -8591,35 +8634,35 @@
         <v>39</v>
       </c>
       <c r="N142" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D143" s="20" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="E143" s="20" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="F143" s="20" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="G143" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="20" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="I143" s="20"/>
       <c r="J143" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K143" s="20"/>
       <c r="L143" s="20" t="s">
@@ -8629,35 +8672,35 @@
         <v>39</v>
       </c>
       <c r="N143" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D144" s="20" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="E144" s="20" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="F144" s="20" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="G144" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H144" s="20" t="s">
-        <v>736</v>
+        <v>744</v>
       </c>
       <c r="I144" s="20"/>
       <c r="J144" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K144" s="20"/>
       <c r="L144" s="20" t="s">
@@ -8667,35 +8710,35 @@
         <v>39</v>
       </c>
       <c r="N144" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>737</v>
+        <v>745</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D145" s="20" t="s">
-        <v>738</v>
+        <v>746</v>
       </c>
       <c r="E145" s="20" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="F145" s="20" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="G145" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="20" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="I145" s="20"/>
       <c r="J145" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K145" s="20"/>
       <c r="L145" s="20" t="s">
@@ -8705,35 +8748,35 @@
         <v>39</v>
       </c>
       <c r="N145" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D146" s="20" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="E146" s="20" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="F146" s="20" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="G146" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="20" t="s">
-        <v>746</v>
+        <v>754</v>
       </c>
       <c r="I146" s="20"/>
       <c r="J146" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K146" s="20"/>
       <c r="L146" s="20" t="s">
@@ -8743,35 +8786,35 @@
         <v>39</v>
       </c>
       <c r="N146" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D147" s="20" t="s">
-        <v>748</v>
+        <v>756</v>
       </c>
       <c r="E147" s="20" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="F147" s="20" t="s">
-        <v>750</v>
+        <v>758</v>
       </c>
       <c r="G147" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="20" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="I147" s="20"/>
       <c r="J147" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K147" s="20"/>
       <c r="L147" s="20" t="s">
@@ -8781,35 +8824,35 @@
         <v>39</v>
       </c>
       <c r="N147" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>752</v>
+        <v>760</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D148" s="20" t="s">
-        <v>753</v>
+        <v>761</v>
       </c>
       <c r="E148" s="20" t="s">
-        <v>754</v>
+        <v>762</v>
       </c>
       <c r="F148" s="20" t="s">
-        <v>755</v>
+        <v>763</v>
       </c>
       <c r="G148" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="20" t="s">
-        <v>756</v>
+        <v>764</v>
       </c>
       <c r="I148" s="20"/>
       <c r="J148" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K148" s="20"/>
       <c r="L148" s="20" t="s">
@@ -8819,35 +8862,35 @@
         <v>39</v>
       </c>
       <c r="N148" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>757</v>
+        <v>765</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D149" s="20" t="s">
-        <v>758</v>
+        <v>766</v>
       </c>
       <c r="E149" s="20" t="s">
-        <v>759</v>
+        <v>767</v>
       </c>
       <c r="F149" s="20" t="s">
-        <v>760</v>
+        <v>768</v>
       </c>
       <c r="G149" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="20" t="s">
-        <v>761</v>
+        <v>769</v>
       </c>
       <c r="I149" s="20"/>
       <c r="J149" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K149" s="20"/>
       <c r="L149" s="20" t="s">
@@ -8857,35 +8900,35 @@
         <v>39</v>
       </c>
       <c r="N149" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>762</v>
+        <v>770</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D150" s="20" t="s">
-        <v>763</v>
+        <v>771</v>
       </c>
       <c r="E150" s="20" t="s">
-        <v>764</v>
+        <v>772</v>
       </c>
       <c r="F150" s="20" t="s">
-        <v>765</v>
+        <v>773</v>
       </c>
       <c r="G150" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H150" s="20" t="s">
-        <v>766</v>
+        <v>774</v>
       </c>
       <c r="I150" s="20"/>
       <c r="J150" s="20" t="s">
-        <v>767</v>
+        <v>775</v>
       </c>
       <c r="K150" s="20"/>
       <c r="L150" s="20" t="s">
@@ -8895,35 +8938,35 @@
         <v>39</v>
       </c>
       <c r="N150" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>768</v>
+        <v>776</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D151" s="20" t="s">
-        <v>769</v>
+        <v>777</v>
       </c>
       <c r="E151" s="20" t="s">
-        <v>770</v>
+        <v>778</v>
       </c>
       <c r="F151" s="20" t="s">
-        <v>771</v>
+        <v>779</v>
       </c>
       <c r="G151" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H151" s="20" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="I151" s="20"/>
       <c r="J151" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K151" s="20"/>
       <c r="L151" s="20" t="s">
@@ -8933,35 +8976,35 @@
         <v>39</v>
       </c>
       <c r="N151" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>773</v>
+        <v>781</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D152" s="20" t="s">
-        <v>774</v>
+        <v>782</v>
       </c>
       <c r="E152" s="20" t="s">
-        <v>775</v>
+        <v>783</v>
       </c>
       <c r="F152" s="20" t="s">
-        <v>776</v>
+        <v>784</v>
       </c>
       <c r="G152" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H152" s="20" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="I152" s="20"/>
       <c r="J152" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K152" s="20"/>
       <c r="L152" s="20" t="s">
@@ -8971,35 +9014,35 @@
         <v>39</v>
       </c>
       <c r="N152" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>778</v>
+        <v>786</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D153" s="20" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="E153" s="20" t="s">
-        <v>780</v>
+        <v>788</v>
       </c>
       <c r="F153" s="20" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
       <c r="G153" s="20" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="H153" s="20" t="s">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="I153" s="20"/>
       <c r="J153" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="K153" s="20"/>
       <c r="L153" s="20" t="s">
@@ -9009,7 +9052,7 @@
         <v>39</v>
       </c>
       <c r="N153" s="20" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
   </sheetData>
@@ -9042,51 +9085,51 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>783</v>
+        <v>791</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>785</v>
+        <v>793</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>786</v>
+        <v>794</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>788</v>
+        <v>796</v>
       </c>
       <c r="G1" s="22" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="22" t="s">
-        <v>789</v>
+        <v>797</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
-        <v>791</v>
+        <v>799</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>792</v>
+        <v>800</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>793</v>
+        <v>801</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>795</v>
+        <v>803</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>796</v>
+        <v>804</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>36</v>
@@ -9095,27 +9138,27 @@
         <v>39</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>797</v>
+        <v>805</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>801</v>
+        <v>809</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>802</v>
+        <v>810</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>36</v>
@@ -9124,27 +9167,27 @@
         <v>39</v>
       </c>
       <c r="I3" s="29" t="s">
-        <v>803</v>
+        <v>811</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
-        <v>804</v>
+        <v>812</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>806</v>
+        <v>814</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>807</v>
+        <v>815</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>808</v>
+        <v>816</v>
       </c>
       <c r="G4" s="28" t="s">
         <v>36</v>
@@ -9153,27 +9196,27 @@
         <v>39</v>
       </c>
       <c r="I4" s="29" t="s">
-        <v>809</v>
+        <v>817</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>810</v>
+        <v>818</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>811</v>
+        <v>819</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>812</v>
+        <v>820</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>813</v>
+        <v>821</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
       <c r="G5" s="28" t="s">
         <v>36</v>
@@ -9182,27 +9225,27 @@
         <v>39</v>
       </c>
       <c r="I5" s="29" t="s">
-        <v>815</v>
+        <v>823</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>816</v>
+        <v>824</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>817</v>
+        <v>825</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>819</v>
+        <v>827</v>
       </c>
       <c r="G6" s="28" t="s">
         <v>36</v>
@@ -9211,27 +9254,27 @@
         <v>39</v>
       </c>
       <c r="I6" s="29" t="s">
-        <v>820</v>
+        <v>828</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
-        <v>821</v>
+        <v>829</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>822</v>
+        <v>830</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>824</v>
+        <v>832</v>
       </c>
       <c r="G7" s="28" t="s">
         <v>36</v>
@@ -9240,27 +9283,27 @@
         <v>39</v>
       </c>
       <c r="I7" s="29" t="s">
-        <v>825</v>
+        <v>833</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>827</v>
+        <v>835</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>828</v>
+        <v>836</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>829</v>
+        <v>837</v>
       </c>
       <c r="G8" s="28" t="s">
         <v>36</v>
@@ -9269,27 +9312,27 @@
         <v>39</v>
       </c>
       <c r="I8" s="29" t="s">
-        <v>830</v>
+        <v>838</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>833</v>
+        <v>841</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>834</v>
+        <v>842</v>
       </c>
       <c r="G9" s="28" t="s">
         <v>36</v>
@@ -9298,27 +9341,27 @@
         <v>39</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>835</v>
+        <v>843</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
-        <v>836</v>
+        <v>844</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>837</v>
+        <v>845</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>838</v>
+        <v>846</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
       <c r="G10" s="31" t="s">
         <v>36</v>
@@ -9327,25 +9370,25 @@
         <v>39</v>
       </c>
       <c r="I10" s="32" t="s">
-        <v>840</v>
+        <v>848</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>841</v>
+        <v>849</v>
       </c>
       <c r="B11" s="34"/>
       <c r="C11" s="34" t="s">
-        <v>842</v>
+        <v>850</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F11" s="34" t="s">
-        <v>845</v>
+        <v>853</v>
       </c>
       <c r="G11" s="34" t="s">
         <v>36</v>
@@ -9354,25 +9397,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="35" t="s">
-        <v>846</v>
+        <v>854</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="36" t="s">
-        <v>847</v>
+        <v>855</v>
       </c>
       <c r="B12" s="37"/>
       <c r="C12" s="37" t="s">
-        <v>848</v>
+        <v>856</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>849</v>
+        <v>857</v>
       </c>
       <c r="G12" s="37" t="s">
         <v>36</v>
@@ -9381,25 +9424,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>850</v>
+        <v>858</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="36" t="s">
-        <v>851</v>
+        <v>859</v>
       </c>
       <c r="B13" s="37"/>
       <c r="C13" s="37" t="s">
+        <v>860</v>
+      </c>
+      <c r="D13" s="37" t="s">
+        <v>851</v>
+      </c>
+      <c r="E13" s="37" t="s">
         <v>852</v>
       </c>
-      <c r="D13" s="37" t="s">
-        <v>843</v>
-      </c>
-      <c r="E13" s="37" t="s">
-        <v>844</v>
-      </c>
       <c r="F13" s="37" t="s">
-        <v>853</v>
+        <v>861</v>
       </c>
       <c r="G13" s="37" t="s">
         <v>36</v>
@@ -9408,25 +9451,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>854</v>
+        <v>862</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="B14" s="37"/>
       <c r="C14" s="37" t="s">
-        <v>856</v>
+        <v>864</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>857</v>
+        <v>865</v>
       </c>
       <c r="G14" s="37" t="s">
         <v>36</v>
@@ -9435,25 +9478,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="36" t="s">
-        <v>859</v>
+        <v>867</v>
       </c>
       <c r="B15" s="37"/>
       <c r="C15" s="37" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
       <c r="G15" s="37" t="s">
         <v>36</v>
@@ -9462,25 +9505,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="36" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="B16" s="37"/>
       <c r="C16" s="37" t="s">
-        <v>864</v>
+        <v>872</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="G16" s="37" t="s">
         <v>36</v>
@@ -9489,25 +9532,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="36" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
       <c r="B17" s="37"/>
       <c r="C17" s="37" t="s">
-        <v>868</v>
+        <v>876</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="G17" s="37" t="s">
         <v>36</v>
@@ -9516,25 +9559,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>870</v>
+        <v>878</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="36" t="s">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="B18" s="37"/>
       <c r="C18" s="37" t="s">
-        <v>872</v>
+        <v>880</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="G18" s="37" t="s">
         <v>36</v>
@@ -9543,25 +9586,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="38" t="s">
-        <v>874</v>
+        <v>882</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="36" t="s">
-        <v>875</v>
+        <v>883</v>
       </c>
       <c r="B19" s="37"/>
       <c r="C19" s="37" t="s">
-        <v>876</v>
+        <v>884</v>
       </c>
       <c r="D19" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F19" s="37" t="s">
-        <v>877</v>
+        <v>885</v>
       </c>
       <c r="G19" s="37" t="s">
         <v>36</v>
@@ -9570,25 +9613,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>878</v>
+        <v>886</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="36" t="s">
-        <v>879</v>
+        <v>887</v>
       </c>
       <c r="B20" s="37"/>
       <c r="C20" s="37" t="s">
-        <v>880</v>
+        <v>888</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="G20" s="37" t="s">
         <v>36</v>
@@ -9597,25 +9640,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="38" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="36" t="s">
-        <v>883</v>
+        <v>891</v>
       </c>
       <c r="B21" s="37"/>
       <c r="C21" s="37" t="s">
-        <v>884</v>
+        <v>892</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F21" s="37" t="s">
-        <v>885</v>
+        <v>893</v>
       </c>
       <c r="G21" s="37" t="s">
         <v>36</v>
@@ -9624,25 +9667,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>886</v>
+        <v>894</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="36" t="s">
-        <v>887</v>
+        <v>895</v>
       </c>
       <c r="B22" s="37"/>
       <c r="C22" s="37" t="s">
-        <v>827</v>
+        <v>835</v>
       </c>
       <c r="D22" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>888</v>
+        <v>896</v>
       </c>
       <c r="G22" s="37" t="s">
         <v>36</v>
@@ -9651,25 +9694,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>889</v>
+        <v>897</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="36" t="s">
-        <v>890</v>
+        <v>898</v>
       </c>
       <c r="B23" s="37"/>
       <c r="C23" s="37" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
       <c r="D23" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F23" s="37" t="s">
-        <v>891</v>
+        <v>899</v>
       </c>
       <c r="G23" s="37" t="s">
         <v>36</v>
@@ -9678,25 +9721,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>892</v>
+        <v>900</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="36" t="s">
-        <v>893</v>
+        <v>901</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="37" t="s">
-        <v>894</v>
+        <v>902</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>895</v>
+        <v>903</v>
       </c>
       <c r="G24" s="37" t="s">
         <v>36</v>
@@ -9705,25 +9748,25 @@
         <v>36</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>896</v>
+        <v>904</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
-        <v>897</v>
+        <v>905</v>
       </c>
       <c r="B25" s="40"/>
       <c r="C25" s="40" t="s">
-        <v>837</v>
+        <v>906</v>
       </c>
       <c r="D25" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F25" s="40" t="s">
-        <v>898</v>
+        <v>907</v>
       </c>
       <c r="G25" s="40" t="s">
         <v>36</v>
@@ -9732,25 +9775,25 @@
         <v>36</v>
       </c>
       <c r="I25" s="41" t="s">
-        <v>899</v>
+        <v>908</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="39" t="s">
-        <v>900</v>
+        <v>909</v>
       </c>
       <c r="B26" s="40"/>
       <c r="C26" s="40" t="s">
-        <v>901</v>
+        <v>910</v>
       </c>
       <c r="D26" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>902</v>
+        <v>911</v>
       </c>
       <c r="F26" s="40" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="G26" s="40" t="s">
         <v>36</v>
@@ -9759,25 +9802,25 @@
         <v>36</v>
       </c>
       <c r="I26" s="41" t="s">
-        <v>904</v>
+        <v>913</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>905</v>
+        <v>914</v>
       </c>
       <c r="B27" s="40"/>
       <c r="C27" s="40" t="s">
-        <v>906</v>
+        <v>915</v>
       </c>
       <c r="D27" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>907</v>
+        <v>916</v>
       </c>
       <c r="F27" s="40" t="s">
-        <v>908</v>
+        <v>917</v>
       </c>
       <c r="G27" s="40" t="s">
         <v>36</v>
@@ -9786,25 +9829,25 @@
         <v>36</v>
       </c>
       <c r="I27" s="41" t="s">
-        <v>909</v>
+        <v>918</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>910</v>
+        <v>919</v>
       </c>
       <c r="B28" s="40"/>
       <c r="C28" s="40" t="s">
-        <v>911</v>
+        <v>920</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>912</v>
+        <v>921</v>
       </c>
       <c r="F28" s="40" t="s">
-        <v>913</v>
+        <v>922</v>
       </c>
       <c r="G28" s="40" t="s">
         <v>36</v>
@@ -9813,25 +9856,25 @@
         <v>36</v>
       </c>
       <c r="I28" s="41" t="s">
-        <v>914</v>
+        <v>923</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>915</v>
+        <v>924</v>
       </c>
       <c r="B29" s="40"/>
       <c r="C29" s="40" t="s">
-        <v>916</v>
+        <v>925</v>
       </c>
       <c r="D29" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>917</v>
+        <v>926</v>
       </c>
       <c r="F29" s="40" t="s">
-        <v>918</v>
+        <v>927</v>
       </c>
       <c r="G29" s="40" t="s">
         <v>36</v>
@@ -9840,25 +9883,25 @@
         <v>36</v>
       </c>
       <c r="I29" s="41" t="s">
-        <v>919</v>
+        <v>928</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="39" t="s">
-        <v>920</v>
+        <v>929</v>
       </c>
       <c r="B30" s="40"/>
       <c r="C30" s="40" t="s">
-        <v>921</v>
+        <v>930</v>
       </c>
       <c r="D30" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>922</v>
+        <v>931</v>
       </c>
       <c r="F30" s="40" t="s">
-        <v>923</v>
+        <v>932</v>
       </c>
       <c r="G30" s="40" t="s">
         <v>36</v>
@@ -9867,25 +9910,25 @@
         <v>36</v>
       </c>
       <c r="I30" s="41" t="s">
-        <v>924</v>
+        <v>933</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="39" t="s">
-        <v>925</v>
+        <v>934</v>
       </c>
       <c r="B31" s="40"/>
       <c r="C31" s="40" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
       <c r="D31" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>926</v>
+        <v>935</v>
       </c>
       <c r="F31" s="40" t="s">
-        <v>927</v>
+        <v>936</v>
       </c>
       <c r="G31" s="40" t="s">
         <v>36</v>
@@ -9894,25 +9937,25 @@
         <v>36</v>
       </c>
       <c r="I31" s="41" t="s">
-        <v>928</v>
+        <v>937</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="39" t="s">
-        <v>929</v>
+        <v>938</v>
       </c>
       <c r="B32" s="40"/>
       <c r="C32" s="40" t="s">
-        <v>930</v>
+        <v>939</v>
       </c>
       <c r="D32" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E32" s="40" t="s">
-        <v>931</v>
+        <v>940</v>
       </c>
       <c r="F32" s="40" t="s">
-        <v>932</v>
+        <v>941</v>
       </c>
       <c r="G32" s="40" t="s">
         <v>36</v>
@@ -9921,25 +9964,25 @@
         <v>36</v>
       </c>
       <c r="I32" s="41" t="s">
-        <v>933</v>
+        <v>942</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="39" t="s">
-        <v>934</v>
+        <v>943</v>
       </c>
       <c r="B33" s="40"/>
       <c r="C33" s="40" t="s">
-        <v>935</v>
+        <v>944</v>
       </c>
       <c r="D33" s="40" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>936</v>
+        <v>945</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>937</v>
+        <v>946</v>
       </c>
       <c r="G33" s="40" t="s">
         <v>36</v>
@@ -9948,7 +9991,7 @@
         <v>36</v>
       </c>
       <c r="I33" s="41" t="s">
-        <v>938</v>
+        <v>947</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: correct Stage 6 Pass 010 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="948">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1811" uniqueCount="949">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1269,6 +1269,9 @@
     <t>legacy/src/base/cics/cobol/BNK1TFN.cbl:988-1204; XFRFUN.cbl inquiry sections; Runtime: static-only</t>
   </si>
   <si>
+    <t>Decision D-005: generic transfers allow transactional products only; loan and mortgage movements use dedicated operations.</t>
+  </si>
+  <si>
     <t>Transfer updates both accounts atomically</t>
   </si>
   <si>
@@ -2622,7 +2625,7 @@
     <t>R1-D-005</t>
   </si>
   <si>
-    <t>72-78</t>
+    <t>72-78,81</t>
   </si>
   <si>
     <t>Owner-approved target decision D-005 recorded in Stage 4.</t>
@@ -3587,7 +3590,7 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3685,7 +3688,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>27</v>
       </c>
@@ -4203,7 +4206,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>105</v>
       </c>
@@ -4447,7 +4450,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>141</v>
       </c>
@@ -4877,7 +4880,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="40" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
         <v>202</v>
       </c>
@@ -5195,7 +5198,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="49" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
         <v>248</v>
       </c>
@@ -5559,7 +5562,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="59" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="17" t="s">
         <v>301</v>
       </c>
@@ -6291,7 +6294,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="79" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
         <v>403</v>
       </c>
@@ -6377,7 +6380,9 @@
         <v>416</v>
       </c>
       <c r="I81" s="20"/>
-      <c r="J81" s="20"/>
+      <c r="J81" s="20" t="s">
+        <v>417</v>
+      </c>
       <c r="K81" s="20"/>
       <c r="L81" s="20" t="s">
         <v>36</v>
@@ -6392,29 +6397,29 @@
     <row r="82" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A82" s="18"/>
       <c r="B82" s="19" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C82" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D82" s="20" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E82" s="20" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F82" s="20" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G82" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H82" s="20" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="I82" s="20"/>
       <c r="J82" s="20" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="K82" s="20"/>
       <c r="L82" s="20" t="s">
@@ -6430,29 +6435,29 @@
     <row r="83" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="18"/>
       <c r="B83" s="19" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C83" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D83" s="20" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="E83" s="20" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F83" s="20" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G83" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H83" s="20" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="I83" s="20"/>
       <c r="J83" s="20" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K83" s="20"/>
       <c r="L83" s="20" t="s">
@@ -6468,29 +6473,29 @@
     <row r="84" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="18"/>
       <c r="B84" s="19" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C84" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E84" s="20" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F84" s="20" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G84" s="20" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H84" s="20" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="I84" s="20"/>
       <c r="J84" s="20" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K84" s="20"/>
       <c r="L84" s="20" t="s">
@@ -6506,29 +6511,29 @@
     <row r="85" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C85" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D85" s="20" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E85" s="20" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F85" s="20" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G85" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H85" s="20" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I85" s="20"/>
       <c r="J85" s="20" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="K85" s="20"/>
       <c r="L85" s="20" t="s">
@@ -6541,12 +6546,12 @@
         <v>411</v>
       </c>
     </row>
-    <row r="86" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B86" s="17" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C86" s="17" t="s">
         <v>29</v>
@@ -6568,29 +6573,29 @@
     <row r="87" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C87" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D87" s="20" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E87" s="20" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F87" s="20" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G87" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H87" s="20" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I87" s="20"/>
       <c r="J87" s="20" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K87" s="20"/>
       <c r="L87" s="20" t="s">
@@ -6606,29 +6611,29 @@
     <row r="88" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C88" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E88" s="20" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F88" s="20" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G88" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H88" s="20" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="I88" s="20"/>
       <c r="J88" s="20" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K88" s="20"/>
       <c r="L88" s="20" t="s">
@@ -6644,25 +6649,25 @@
     <row r="89" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C89" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F89" s="20" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="G89" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H89" s="20" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I89" s="20"/>
       <c r="J89" s="20" t="s">
@@ -6682,29 +6687,29 @@
     <row r="90" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C90" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D90" s="20" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E90" s="20" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F90" s="20" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G90" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H90" s="20" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="I90" s="20"/>
       <c r="J90" s="20" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K90" s="20"/>
       <c r="L90" s="20" t="s">
@@ -6720,29 +6725,29 @@
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="18"/>
       <c r="B91" s="19" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C91" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D91" s="20" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E91" s="20" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F91" s="20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G91" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H91" s="20" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="I91" s="20"/>
       <c r="J91" s="20" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K91" s="20"/>
       <c r="L91" s="20" t="s">
@@ -6752,35 +6757,35 @@
         <v>39</v>
       </c>
       <c r="N91" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="92" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C92" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D92" s="20" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F92" s="20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G92" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H92" s="20" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="I92" s="20"/>
       <c r="J92" s="20" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K92" s="20"/>
       <c r="L92" s="20" t="s">
@@ -6790,35 +6795,35 @@
         <v>39</v>
       </c>
       <c r="N92" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="18"/>
       <c r="B93" s="19" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C93" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D93" s="20" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E93" s="20" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F93" s="20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G93" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H93" s="20" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I93" s="20"/>
       <c r="J93" s="20" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K93" s="20"/>
       <c r="L93" s="20" t="s">
@@ -6828,35 +6833,35 @@
         <v>39</v>
       </c>
       <c r="N93" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="18"/>
       <c r="B94" s="19" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C94" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D94" s="20" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E94" s="20" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F94" s="20" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G94" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H94" s="20" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="I94" s="20"/>
       <c r="J94" s="20" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="K94" s="20"/>
       <c r="L94" s="20" t="s">
@@ -6866,35 +6871,35 @@
         <v>39</v>
       </c>
       <c r="N94" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C95" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D95" s="20" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E95" s="20" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F95" s="20" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="G95" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H95" s="20" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="I95" s="20"/>
       <c r="J95" s="20" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K95" s="20"/>
       <c r="L95" s="20" t="s">
@@ -6904,35 +6909,35 @@
         <v>39</v>
       </c>
       <c r="N95" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="96" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D96" s="20" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E96" s="20" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F96" s="20" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G96" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H96" s="20" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="I96" s="20"/>
       <c r="J96" s="20" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="K96" s="20"/>
       <c r="L96" s="20" t="s">
@@ -6942,35 +6947,35 @@
         <v>39</v>
       </c>
       <c r="N96" s="20" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="97" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C97" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D97" s="20" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E97" s="20" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F97" s="20" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H97" s="20" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="I97" s="20"/>
       <c r="J97" s="20" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="K97" s="20"/>
       <c r="L97" s="20" t="s">
@@ -6986,29 +6991,29 @@
     <row r="98" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C98" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D98" s="20" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E98" s="20" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F98" s="20" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="G98" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H98" s="20" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="I98" s="20"/>
       <c r="J98" s="20" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="K98" s="20"/>
       <c r="L98" s="20" t="s">
@@ -7018,15 +7023,15 @@
         <v>39</v>
       </c>
       <c r="N98" s="20" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="99" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="99" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B99" s="17" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C99" s="17" t="s">
         <v>29</v>
@@ -7048,29 +7053,29 @@
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="18"/>
       <c r="B100" s="19" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C100" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D100" s="20" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E100" s="20" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F100" s="20" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G100" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H100" s="20" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="I100" s="20"/>
       <c r="J100" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K100" s="20"/>
       <c r="L100" s="20" t="s">
@@ -7080,35 +7085,35 @@
         <v>39</v>
       </c>
       <c r="N100" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="18"/>
       <c r="B101" s="19" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C101" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D101" s="20" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E101" s="20" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F101" s="20" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="G101" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H101" s="20" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="I101" s="20"/>
       <c r="J101" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K101" s="20"/>
       <c r="L101" s="20" t="s">
@@ -7118,35 +7123,35 @@
         <v>39</v>
       </c>
       <c r="N101" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D102" s="20" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E102" s="20" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F102" s="20" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="G102" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H102" s="20" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="I102" s="20"/>
       <c r="J102" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K102" s="20"/>
       <c r="L102" s="20" t="s">
@@ -7156,35 +7161,35 @@
         <v>39</v>
       </c>
       <c r="N102" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C103" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D103" s="20" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E103" s="20" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F103" s="20" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="G103" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H103" s="20" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="I103" s="20"/>
       <c r="J103" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K103" s="20"/>
       <c r="L103" s="20" t="s">
@@ -7194,35 +7199,35 @@
         <v>39</v>
       </c>
       <c r="N103" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D104" s="20" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E104" s="20" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F104" s="20" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="G104" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H104" s="20" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="I104" s="20"/>
       <c r="J104" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K104" s="20"/>
       <c r="L104" s="20" t="s">
@@ -7232,35 +7237,35 @@
         <v>39</v>
       </c>
       <c r="N104" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="18"/>
       <c r="B105" s="19" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="C105" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D105" s="20" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E105" s="20" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F105" s="20" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G105" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H105" s="20" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="I105" s="20"/>
       <c r="J105" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K105" s="20"/>
       <c r="L105" s="20" t="s">
@@ -7270,35 +7275,35 @@
         <v>39</v>
       </c>
       <c r="N105" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C106" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D106" s="20" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E106" s="20" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F106" s="20" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="G106" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H106" s="20" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="I106" s="20"/>
       <c r="J106" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K106" s="20"/>
       <c r="L106" s="20" t="s">
@@ -7308,35 +7313,35 @@
         <v>39</v>
       </c>
       <c r="N106" s="20" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C107" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D107" s="20" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="E107" s="20" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="F107" s="20" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="G107" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H107" s="20" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="I107" s="20"/>
       <c r="J107" s="20" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="K107" s="20"/>
       <c r="L107" s="20" t="s">
@@ -7346,15 +7351,15 @@
         <v>39</v>
       </c>
       <c r="N107" s="20" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="108" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="108" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B108" s="17" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C108" s="17" t="s">
         <v>29</v>
@@ -7376,29 +7381,29 @@
     <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C109" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E109" s="20" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F109" s="20" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="I109" s="20"/>
       <c r="J109" s="20" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="K109" s="20"/>
       <c r="L109" s="20" t="s">
@@ -7414,29 +7419,29 @@
     <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C110" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F110" s="20" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="I110" s="20"/>
       <c r="J110" s="20" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="K110" s="20"/>
       <c r="L110" s="20" t="s">
@@ -7452,29 +7457,29 @@
     <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C111" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D111" s="20" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E111" s="20" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F111" s="20" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="I111" s="20"/>
       <c r="J111" s="20" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="K111" s="20"/>
       <c r="L111" s="20" t="s">
@@ -7490,29 +7495,29 @@
     <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C112" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="F112" s="20" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="G112" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="I112" s="20"/>
       <c r="J112" s="20" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="K112" s="20"/>
       <c r="L112" s="20" t="s">
@@ -7528,29 +7533,29 @@
     <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C113" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="I113" s="20"/>
       <c r="J113" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="K113" s="20"/>
       <c r="L113" s="20" t="s">
@@ -7566,29 +7571,29 @@
     <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C114" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D114" s="20" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E114" s="20" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F114" s="20" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="20" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="I114" s="20"/>
       <c r="J114" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="K114" s="20"/>
       <c r="L114" s="20" t="s">
@@ -7604,29 +7609,29 @@
     <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C115" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D115" s="20" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F115" s="20" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="G115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="20" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="I115" s="20"/>
       <c r="J115" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="K115" s="20"/>
       <c r="L115" s="20" t="s">
@@ -7642,29 +7647,29 @@
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="18"/>
       <c r="B116" s="19" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C116" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D116" s="20" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E116" s="20" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="F116" s="20" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="G116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H116" s="20" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="I116" s="20"/>
       <c r="J116" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="K116" s="20"/>
       <c r="L116" s="20" t="s">
@@ -7680,29 +7685,29 @@
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
       <c r="B117" s="19" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="C117" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E117" s="20" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="G117" s="20" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="I117" s="20"/>
       <c r="J117" s="20" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="K117" s="20"/>
       <c r="L117" s="20" t="s">
@@ -7715,12 +7720,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="118" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="118" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="17" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B118" s="17" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C118" s="17" t="s">
         <v>29</v>
@@ -7742,29 +7747,29 @@
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="19" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D119" s="20" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E119" s="20" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="F119" s="20" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="G119" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="20" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="I119" s="20"/>
       <c r="J119" s="20" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="K119" s="20"/>
       <c r="L119" s="20" t="s">
@@ -7774,35 +7779,35 @@
         <v>39</v>
       </c>
       <c r="N119" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="19" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D120" s="20" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E120" s="20" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F120" s="20" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G120" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="20" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="I120" s="20"/>
       <c r="J120" s="20" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="K120" s="20"/>
       <c r="L120" s="20" t="s">
@@ -7812,35 +7817,35 @@
         <v>39</v>
       </c>
       <c r="N120" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
       <c r="B121" s="19" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C121" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D121" s="20" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E121" s="20" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F121" s="20" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="G121" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="20" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="I121" s="20"/>
       <c r="J121" s="20" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="K121" s="20"/>
       <c r="L121" s="20" t="s">
@@ -7850,35 +7855,35 @@
         <v>39</v>
       </c>
       <c r="N121" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="19" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D122" s="20" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E122" s="20" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="F122" s="20" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="G122" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="20" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="I122" s="20"/>
       <c r="J122" s="20" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="K122" s="20"/>
       <c r="L122" s="20" t="s">
@@ -7888,35 +7893,35 @@
         <v>39</v>
       </c>
       <c r="N122" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="19" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D123" s="20" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="E123" s="20" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="F123" s="20" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="G123" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H123" s="20" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="I123" s="20"/>
       <c r="J123" s="20" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="K123" s="20"/>
       <c r="L123" s="20" t="s">
@@ -7926,35 +7931,35 @@
         <v>39</v>
       </c>
       <c r="N123" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="19" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D124" s="20" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="F124" s="20" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="G124" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H124" s="20" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="I124" s="20"/>
       <c r="J124" s="20" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="K124" s="20"/>
       <c r="L124" s="20" t="s">
@@ -7964,35 +7969,35 @@
         <v>39</v>
       </c>
       <c r="N124" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="19" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D125" s="20" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E125" s="20" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="F125" s="20" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G125" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H125" s="20" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="I125" s="20"/>
       <c r="J125" s="20" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="K125" s="20"/>
       <c r="L125" s="20" t="s">
@@ -8002,35 +8007,35 @@
         <v>39</v>
       </c>
       <c r="N125" s="20" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="19" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D126" s="20" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="E126" s="20" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="F126" s="20" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="G126" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="20" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="I126" s="20"/>
       <c r="J126" s="20" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="K126" s="20"/>
       <c r="L126" s="20" t="s">
@@ -8040,15 +8045,15 @@
         <v>39</v>
       </c>
       <c r="N126" s="20" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="127" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="17" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B127" s="17" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C127" s="17" t="s">
         <v>29</v>
@@ -8070,29 +8075,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D128" s="20" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E128" s="20" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F128" s="20" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G128" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="20" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="I128" s="20"/>
       <c r="J128" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K128" s="20"/>
       <c r="L128" s="20" t="s">
@@ -8102,35 +8107,35 @@
         <v>39</v>
       </c>
       <c r="N128" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D129" s="20" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E129" s="20" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="F129" s="20" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="G129" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="20" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I129" s="20"/>
       <c r="J129" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K129" s="20"/>
       <c r="L129" s="20" t="s">
@@ -8140,35 +8145,35 @@
         <v>39</v>
       </c>
       <c r="N129" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="18"/>
       <c r="B130" s="19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D130" s="20" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E130" s="20" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F130" s="20" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="G130" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="20" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="I130" s="20"/>
       <c r="J130" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K130" s="20"/>
       <c r="L130" s="20" t="s">
@@ -8178,35 +8183,35 @@
         <v>39</v>
       </c>
       <c r="N130" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D131" s="20" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E131" s="20" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F131" s="20" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G131" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H131" s="20" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="I131" s="20"/>
       <c r="J131" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K131" s="20"/>
       <c r="L131" s="20" t="s">
@@ -8216,35 +8221,35 @@
         <v>39</v>
       </c>
       <c r="N131" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D132" s="20" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="E132" s="20" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F132" s="20" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="G132" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="20" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="I132" s="20"/>
       <c r="J132" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K132" s="20"/>
       <c r="L132" s="20" t="s">
@@ -8254,35 +8259,35 @@
         <v>39</v>
       </c>
       <c r="N132" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D133" s="20" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="E133" s="20" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="F133" s="20" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="G133" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H133" s="20" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="I133" s="20"/>
       <c r="J133" s="20" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="K133" s="20"/>
       <c r="L133" s="20" t="s">
@@ -8292,35 +8297,35 @@
         <v>39</v>
       </c>
       <c r="N133" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D134" s="20" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E134" s="20" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F134" s="20" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G134" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="20" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="I134" s="20"/>
       <c r="J134" s="20" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="K134" s="20"/>
       <c r="L134" s="20" t="s">
@@ -8330,35 +8335,35 @@
         <v>39</v>
       </c>
       <c r="N134" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D135" s="20" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="E135" s="20" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="F135" s="20" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="G135" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H135" s="20" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="I135" s="20"/>
       <c r="J135" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K135" s="20"/>
       <c r="L135" s="20" t="s">
@@ -8368,35 +8373,35 @@
         <v>39</v>
       </c>
       <c r="N135" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D136" s="20" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E136" s="20" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F136" s="20" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G136" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H136" s="20" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="I136" s="20"/>
       <c r="J136" s="20" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="K136" s="20"/>
       <c r="L136" s="20" t="s">
@@ -8406,35 +8411,35 @@
         <v>39</v>
       </c>
       <c r="N136" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D137" s="20" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E137" s="20" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F137" s="20" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G137" s="20" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H137" s="20" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="I137" s="20"/>
       <c r="J137" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K137" s="20"/>
       <c r="L137" s="20" t="s">
@@ -8444,35 +8449,35 @@
         <v>39</v>
       </c>
       <c r="N137" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D138" s="20" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="E138" s="20" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="F138" s="20" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="G138" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="20" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="I138" s="20"/>
       <c r="J138" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K138" s="20"/>
       <c r="L138" s="20" t="s">
@@ -8482,35 +8487,35 @@
         <v>39</v>
       </c>
       <c r="N138" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D139" s="20" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="E139" s="20" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="F139" s="20" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="G139" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="20" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="I139" s="20"/>
       <c r="J139" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K139" s="20"/>
       <c r="L139" s="20" t="s">
@@ -8520,35 +8525,35 @@
         <v>39</v>
       </c>
       <c r="N139" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D140" s="20" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E140" s="20" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F140" s="20" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="G140" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="20" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="I140" s="20"/>
       <c r="J140" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K140" s="20"/>
       <c r="L140" s="20" t="s">
@@ -8558,35 +8563,35 @@
         <v>39</v>
       </c>
       <c r="N140" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D141" s="20" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="E141" s="20" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="F141" s="20" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="G141" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="20" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="I141" s="20"/>
       <c r="J141" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K141" s="20"/>
       <c r="L141" s="20" t="s">
@@ -8596,35 +8601,35 @@
         <v>39</v>
       </c>
       <c r="N141" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D142" s="20" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E142" s="20" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="F142" s="20" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="G142" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="I142" s="20"/>
       <c r="J142" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K142" s="20"/>
       <c r="L142" s="20" t="s">
@@ -8634,35 +8639,35 @@
         <v>39</v>
       </c>
       <c r="N142" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D143" s="20" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="E143" s="20" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="F143" s="20" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="G143" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="20" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="I143" s="20"/>
       <c r="J143" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K143" s="20"/>
       <c r="L143" s="20" t="s">
@@ -8672,35 +8677,35 @@
         <v>39</v>
       </c>
       <c r="N143" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D144" s="20" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="E144" s="20" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="F144" s="20" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="G144" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H144" s="20" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="I144" s="20"/>
       <c r="J144" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K144" s="20"/>
       <c r="L144" s="20" t="s">
@@ -8710,35 +8715,35 @@
         <v>39</v>
       </c>
       <c r="N144" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D145" s="20" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="E145" s="20" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="F145" s="20" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="G145" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="20" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="I145" s="20"/>
       <c r="J145" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K145" s="20"/>
       <c r="L145" s="20" t="s">
@@ -8748,35 +8753,35 @@
         <v>39</v>
       </c>
       <c r="N145" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D146" s="20" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="E146" s="20" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="F146" s="20" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="G146" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="20" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="I146" s="20"/>
       <c r="J146" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K146" s="20"/>
       <c r="L146" s="20" t="s">
@@ -8786,35 +8791,35 @@
         <v>39</v>
       </c>
       <c r="N146" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D147" s="20" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="E147" s="20" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="F147" s="20" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="G147" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="20" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="I147" s="20"/>
       <c r="J147" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K147" s="20"/>
       <c r="L147" s="20" t="s">
@@ -8824,35 +8829,35 @@
         <v>39</v>
       </c>
       <c r="N147" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D148" s="20" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="E148" s="20" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="F148" s="20" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="G148" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="20" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="I148" s="20"/>
       <c r="J148" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K148" s="20"/>
       <c r="L148" s="20" t="s">
@@ -8862,35 +8867,35 @@
         <v>39</v>
       </c>
       <c r="N148" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D149" s="20" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="E149" s="20" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="F149" s="20" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="G149" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="20" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="I149" s="20"/>
       <c r="J149" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K149" s="20"/>
       <c r="L149" s="20" t="s">
@@ -8900,35 +8905,35 @@
         <v>39</v>
       </c>
       <c r="N149" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D150" s="20" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="E150" s="20" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="F150" s="20" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="G150" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H150" s="20" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="I150" s="20"/>
       <c r="J150" s="20" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="K150" s="20"/>
       <c r="L150" s="20" t="s">
@@ -8938,35 +8943,35 @@
         <v>39</v>
       </c>
       <c r="N150" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D151" s="20" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="E151" s="20" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="F151" s="20" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="G151" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H151" s="20" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="I151" s="20"/>
       <c r="J151" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K151" s="20"/>
       <c r="L151" s="20" t="s">
@@ -8976,35 +8981,35 @@
         <v>39</v>
       </c>
       <c r="N151" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>95</v>
       </c>
       <c r="D152" s="20" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="E152" s="20" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="F152" s="20" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="G152" s="20" t="s">
         <v>132</v>
       </c>
       <c r="H152" s="20" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="I152" s="20"/>
       <c r="J152" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K152" s="20"/>
       <c r="L152" s="20" t="s">
@@ -9014,35 +9019,35 @@
         <v>39</v>
       </c>
       <c r="N152" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>42</v>
       </c>
       <c r="D153" s="20" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="E153" s="20" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="F153" s="20" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="G153" s="20" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H153" s="20" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="I153" s="20"/>
       <c r="J153" s="20" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="K153" s="20"/>
       <c r="L153" s="20" t="s">
@@ -9052,7 +9057,7 @@
         <v>39</v>
       </c>
       <c r="N153" s="20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
   </sheetData>
@@ -9083,53 +9088,53 @@
     <col min="9" max="9" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="G1" s="22" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="22" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>36</v>
@@ -9138,27 +9143,27 @@
         <v>39</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>36</v>
@@ -9167,27 +9172,27 @@
         <v>39</v>
       </c>
       <c r="I3" s="29" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="G4" s="28" t="s">
         <v>36</v>
@@ -9196,27 +9201,27 @@
         <v>39</v>
       </c>
       <c r="I4" s="29" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="G5" s="28" t="s">
         <v>36</v>
@@ -9225,27 +9230,27 @@
         <v>39</v>
       </c>
       <c r="I5" s="29" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B6" s="28" t="s">
         <v>403</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="G6" s="28" t="s">
         <v>36</v>
@@ -9254,27 +9259,27 @@
         <v>39</v>
       </c>
       <c r="I6" s="29" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="G7" s="28" t="s">
         <v>36</v>
@@ -9283,27 +9288,27 @@
         <v>39</v>
       </c>
       <c r="I7" s="29" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="G8" s="28" t="s">
         <v>36</v>
@@ -9312,27 +9317,27 @@
         <v>39</v>
       </c>
       <c r="I8" s="29" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="G9" s="28" t="s">
         <v>36</v>
@@ -9341,27 +9346,27 @@
         <v>39</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="G10" s="31" t="s">
         <v>36</v>
@@ -9370,25 +9375,25 @@
         <v>39</v>
       </c>
       <c r="I10" s="32" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="B11" s="34"/>
       <c r="C11" s="34" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F11" s="34" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="G11" s="34" t="s">
         <v>36</v>
@@ -9397,25 +9402,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="35" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="36" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="B12" s="37"/>
       <c r="C12" s="37" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="G12" s="37" t="s">
         <v>36</v>
@@ -9424,25 +9429,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="36" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B13" s="37"/>
       <c r="C13" s="37" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="G13" s="37" t="s">
         <v>36</v>
@@ -9451,25 +9456,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B14" s="37"/>
       <c r="C14" s="37" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="G14" s="37" t="s">
         <v>36</v>
@@ -9478,25 +9483,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="36" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B15" s="37"/>
       <c r="C15" s="37" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="G15" s="37" t="s">
         <v>36</v>
@@ -9505,25 +9510,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="36" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B16" s="37"/>
       <c r="C16" s="37" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="G16" s="37" t="s">
         <v>36</v>
@@ -9532,25 +9537,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="36" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="B17" s="37"/>
       <c r="C17" s="37" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="G17" s="37" t="s">
         <v>36</v>
@@ -9559,25 +9564,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="36" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B18" s="37"/>
       <c r="C18" s="37" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="G18" s="37" t="s">
         <v>36</v>
@@ -9586,25 +9591,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="38" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="36" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="B19" s="37"/>
       <c r="C19" s="37" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="D19" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F19" s="37" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="G19" s="37" t="s">
         <v>36</v>
@@ -9613,25 +9618,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="36" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="B20" s="37"/>
       <c r="C20" s="37" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="G20" s="37" t="s">
         <v>36</v>
@@ -9640,25 +9645,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="38" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="36" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="B21" s="37"/>
       <c r="C21" s="37" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F21" s="37" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="G21" s="37" t="s">
         <v>36</v>
@@ -9667,25 +9672,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="36" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="B22" s="37"/>
       <c r="C22" s="37" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="D22" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="G22" s="37" t="s">
         <v>36</v>
@@ -9694,25 +9699,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="36" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B23" s="37"/>
       <c r="C23" s="37" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="D23" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F23" s="37" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="G23" s="37" t="s">
         <v>36</v>
@@ -9721,25 +9726,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="36" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B24" s="37"/>
       <c r="C24" s="37" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="G24" s="37" t="s">
         <v>36</v>
@@ -9748,25 +9753,25 @@
         <v>36</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B25" s="40"/>
       <c r="C25" s="40" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="D25" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F25" s="40" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="G25" s="40" t="s">
         <v>36</v>
@@ -9775,25 +9780,25 @@
         <v>36</v>
       </c>
       <c r="I25" s="41" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="39" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B26" s="40"/>
       <c r="C26" s="40" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="D26" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="F26" s="40" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="G26" s="40" t="s">
         <v>36</v>
@@ -9802,25 +9807,25 @@
         <v>36</v>
       </c>
       <c r="I26" s="41" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B27" s="40"/>
       <c r="C27" s="40" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="D27" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="F27" s="40" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="G27" s="40" t="s">
         <v>36</v>
@@ -9829,25 +9834,25 @@
         <v>36</v>
       </c>
       <c r="I27" s="41" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="39" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="B28" s="40"/>
       <c r="C28" s="40" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="F28" s="40" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="G28" s="40" t="s">
         <v>36</v>
@@ -9856,25 +9861,25 @@
         <v>36</v>
       </c>
       <c r="I28" s="41" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="39" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B29" s="40"/>
       <c r="C29" s="40" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="D29" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="F29" s="40" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="G29" s="40" t="s">
         <v>36</v>
@@ -9883,25 +9888,25 @@
         <v>36</v>
       </c>
       <c r="I29" s="41" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="39" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="B30" s="40"/>
       <c r="C30" s="40" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="D30" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="F30" s="40" t="s">
-        <v>932</v>
+        <v>933</v>
       </c>
       <c r="G30" s="40" t="s">
         <v>36</v>
@@ -9910,25 +9915,25 @@
         <v>36</v>
       </c>
       <c r="I30" s="41" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="39" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="B31" s="40"/>
       <c r="C31" s="40" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="D31" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="F31" s="40" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="G31" s="40" t="s">
         <v>36</v>
@@ -9937,25 +9942,25 @@
         <v>36</v>
       </c>
       <c r="I31" s="41" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="39" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B32" s="40"/>
       <c r="C32" s="40" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="D32" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E32" s="40" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="F32" s="40" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="G32" s="40" t="s">
         <v>36</v>
@@ -9964,25 +9969,25 @@
         <v>36</v>
       </c>
       <c r="I32" s="41" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="39" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="B33" s="40"/>
       <c r="C33" s="40" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="D33" s="40" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="G33" s="40" t="s">
         <v>36</v>
@@ -9991,7 +9996,7 @@
         <v>36</v>
       </c>
       <c r="I33" s="41" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: correct Stage 6 Pass 011 findings
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -39,13 +39,13 @@
     <t>Orange</t>
   </si>
   <si>
-    <t>Known gap, partial behavior, or deferred/planned decision.</t>
+    <t>Deferred: source is evidenced and SDD-covered; an explicit owner-approved deferral and reason are recorded.</t>
   </si>
   <si>
     <t>White</t>
   </si>
   <si>
-    <t>Review/neutral: not fully closed, but not classified as missed or deferred.</t>
+    <t>Neutral formatting only; it does not express lifecycle status.</t>
   </si>
   <si>
     <t>SOURCE / LEGACY CODE</t>
@@ -3590,7 +3590,7 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" ht="54" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -9088,7 +9088,7 @@
     <col min="9" max="9" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>792</v>
       </c>

</xml_diff>

<commit_message>
Document Feature 005 peer review and workbook closure
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1994" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="1059">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1485,130 +1485,148 @@
     <t>Funds transfer</t>
   </si>
   <si>
+    <t>CICS operator transfers funds</t>
+  </si>
+  <si>
+    <t>Transfer a numeric amount from one account to another.</t>
+  </si>
+  <si>
+    <t>The operator supplies source/destination account numbers and amount; the program supplies the configured bank sort code internally.</t>
+  </si>
+  <si>
+    <t>Both resulting balances are displayed after success.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl; XFRFUN.cbl; BNK1TFM.bms; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
+  </si>
+  <si>
+    <t>Decision D-020: implemented by the authenticated internal-transfer command; configured account sort codes are never operator input.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/InternalTransfersController.cs; modern/backend/src/BankOfZ.Application/Transactions/InternalTransferService.cs; modern/backend/tests/BankOfZ.IntegrationTests/InternalTransferApiTests.cs; modern/frontend/bank-of-z-ui/src/app/accounts/account-detail.component.ts; modern/frontend/bank-of-z-ui/e2e/secure-access.spec.ts; deployed /z-bank-new/</t>
+  </si>
+  <si>
+    <t>specs/005-funds-transfers/spec.md; plan.md; tasks.md</t>
+  </si>
+  <si>
+    <t>Transfer input is invalid</t>
+  </si>
+  <si>
+    <t>Validate transfer input, then rely on the CICS unit of work while accounts are selected and updated in account-number order.</t>
+  </si>
+  <si>
+    <t>One account can be updated before a missing second account is discovered; rollback supplies atomic recovery.</t>
+  </si>
+  <si>
+    <t>Input errors are reported; transactional lookup/update failure rolls back the unit of work.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl:988-1204; XFRFUN.cbl inquiry sections; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decision D-005: generic transfers validate distinct accounts, positive two-decimal amounts, ownership, active status, currency, and transactional products.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Application/Transactions/InternalTransferService.cs; modern/backend/tests/BankOfZ.UnitTests/Transactions/InternalTransferServiceTests.cs; modern/backend/tests/BankOfZ.IntegrationTests/InternalTransferApiTests.cs; modern/frontend/bank-of-z-ui/src/app/accounts/account-detail.component.spec.ts</t>
+  </si>
+  <si>
+    <t>Transfer updates both accounts atomically</t>
+  </si>
+  <si>
+    <t>Debit source, credit destination, and rollback if either update cannot complete.</t>
+  </si>
+  <si>
+    <t>A transfer must not leave money changed on one side only.</t>
+  </si>
+  <si>
+    <t>Both account updates commit, otherwise a CICS syncpoint rollback is performed.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:998-1450; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decision D-006: debit, credit, paired immutable history, audit, and idempotency commit in one serializable SQL transaction.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Infrastructure/Transactions/InternalTransferRepository.cs; modern/backend/tests/BankOfZ.IntegrationTests/InternalTransferApiTests.cs; modern/backend/src/BankOfZ.Infrastructure/Persistence/Migrations/20260723094211_AddInternalTransfers.cs</t>
+  </si>
+  <si>
+    <t>Transfer writes transaction evidence</t>
+  </si>
+  <si>
+    <t>Write processed-transaction evidence for the transfer.</t>
+  </si>
+  <si>
+    <t>Transfers appear in downstream statement/history processing.</t>
+  </si>
+  <si>
+    <t>PROCTRAN receives transfer type, amount, counterparty sort code/account, date, time, and reference.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:1563-1639; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
+  </si>
+  <si>
+    <t>Decision D-006: paired Modern ledger records use distinct references and one transfer correlation ID, with matching audit evidence.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Transactions/BookedTransaction.cs; modern/backend/src/BankOfZ.Infrastructure/Persistence/Configurations/BookedTransactionConfiguration.cs; modern/backend/src/BankOfZ.Infrastructure/Transactions/InternalTransferRepository.cs; modern/backend/tests/BankOfZ.IntegrationTests/InternalTransferApiTests.cs</t>
+  </si>
+  <si>
+    <t>Transfer overdraft behavior requires owner decision</t>
+  </si>
+  <si>
+    <t>Preserve the observed transfer calculation or explicitly define a replacement funds/overdraft rule.</t>
+  </si>
+  <si>
+    <t>The transfer code reads overdraft metadata but no clear pre-transfer limit rejection was found.</t>
+  </si>
+  <si>
+    <t>Treat current overdraft enforcement as inferred/unverified until executable legacy observation is available.</t>
+  </si>
+  <si>
+    <t>Inferred</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:10-22 explicitly states that no overdraft-limit checking is made; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
+  </si>
+  <si>
+    <t>Deviation D-004: available balance plus overdraft is enforced before debit; rejection leaves both accounts and history unchanged.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Accounts/Account.cs; modern/backend/src/BankOfZ.Application/Transactions/InternalTransferService.cs; modern/backend/tests/BankOfZ.UnitTests/Transactions/InternalTransferServiceTests.cs; modern/backend/tests/BankOfZ.IntegrationTests/InternalTransferApiTests.cs</t>
+  </si>
+  <si>
+    <t>Bank-to-bank transfer screen is a non-deployed surface</t>
+  </si>
+  <si>
+    <t>Record the BNK1B2M transfer screen and BNK1B2B program definition without treating them as executable legacy behavior.</t>
+  </si>
+  <si>
+    <t>A bank-to-bank transfer surface is present in definitions, but its COBOL implementation and transaction binding are absent.</t>
+  </si>
+  <si>
+    <t>The surface is classified Partial and excluded from the default deployment; no successful transfer is claimed.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/bms/BNK1B2M.bms; legacy/.setup/zconfig/bank-of-z-definitions.yaml:51,143; legacy/.setup/deploy/Development.yml:16-18; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Deviation D-011: only internal account-to-account transfer is exposed; the non-deployed bank-to-bank legacy surface remains intentionally unsupported.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/InternalTransfersController.cs; modern/backend/src/BankOfZ.Application/Transactions/InternalTransferService.cs; specs/005-funds-transfers/spec.md</t>
+  </si>
+  <si>
+    <t>UF-008</t>
+  </si>
+  <si>
+    <t>Transaction history and external account APIs</t>
+  </si>
+  <si>
     <t>Not Passed - Open</t>
   </si>
   <si>
     <t>Legacy behavior is evidenced and covered by SDD; target implementation has not started.</t>
-  </si>
-  <si>
-    <t>CICS operator transfers funds</t>
-  </si>
-  <si>
-    <t>Transfer a numeric amount from one account to another.</t>
-  </si>
-  <si>
-    <t>The operator supplies source/destination account numbers and amount; the program supplies the configured bank sort code internally.</t>
-  </si>
-  <si>
-    <t>Both resulting balances are displayed after success.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl; XFRFUN.cbl; BNK1TFM.bms; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
-  </si>
-  <si>
-    <t>Decision D-020: target derives sort codes from account/bank configuration.</t>
-  </si>
-  <si>
-    <t>specs/005-funds-transfers/spec.md; plan.md; tasks.md</t>
-  </si>
-  <si>
-    <t>Transfer input is invalid</t>
-  </si>
-  <si>
-    <t>Validate transfer input, then rely on the CICS unit of work while accounts are selected and updated in account-number order.</t>
-  </si>
-  <si>
-    <t>One account can be updated before a missing second account is discovered; rollback supplies atomic recovery.</t>
-  </si>
-  <si>
-    <t>Input errors are reported; transactional lookup/update failure rolls back the unit of work.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/cobol/BNK1TFN.cbl:988-1204; XFRFUN.cbl inquiry sections; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decision D-005: generic transfers allow transactional products only; loan and mortgage movements use dedicated operations.</t>
-  </si>
-  <si>
-    <t>Transfer updates both accounts atomically</t>
-  </si>
-  <si>
-    <t>Debit source, credit destination, and rollback if either update cannot complete.</t>
-  </si>
-  <si>
-    <t>A transfer must not leave money changed on one side only.</t>
-  </si>
-  <si>
-    <t>Both account updates commit, otherwise a CICS syncpoint rollback is performed.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:998-1450; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decision D-006: debit, credit, and immutable transaction/audit persistence are atomic.</t>
-  </si>
-  <si>
-    <t>Transfer writes transaction evidence</t>
-  </si>
-  <si>
-    <t>Write processed-transaction evidence for the transfer.</t>
-  </si>
-  <si>
-    <t>Transfers appear in downstream statement/history processing.</t>
-  </si>
-  <si>
-    <t>PROCTRAN receives transfer type, amount, counterparty sort code/account, date, time, and reference.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:1563-1639; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
-  </si>
-  <si>
-    <t>Decision D-006: processed-transfer evidence is committed atomically with both balance mutations.</t>
-  </si>
-  <si>
-    <t>Transfer overdraft behavior requires owner decision</t>
-  </si>
-  <si>
-    <t>Preserve the observed transfer calculation or explicitly define a replacement funds/overdraft rule.</t>
-  </si>
-  <si>
-    <t>The transfer code reads overdraft metadata but no clear pre-transfer limit rejection was found.</t>
-  </si>
-  <si>
-    <t>Treat current overdraft enforcement as inferred/unverified until executable legacy observation is available.</t>
-  </si>
-  <si>
-    <t>Inferred</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/cobol/XFRFUN.cbl:10-22 explicitly states that no overdraft-limit checking is made; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.cics-transfer; harness: simulation/test; basis: legacy/src/base/cics/cobol/XFRFUN.cbl:150-1700; legacy/src/base/cics/copy/XFRFUN.cpy</t>
-  </si>
-  <si>
-    <t>Deviation D-004: enforce available-funds/overdraft policy before transfer.</t>
-  </si>
-  <si>
-    <t>Bank-to-bank transfer screen is a non-deployed surface</t>
-  </si>
-  <si>
-    <t>Record the BNK1B2M transfer screen and BNK1B2B program definition without treating them as executable legacy behavior.</t>
-  </si>
-  <si>
-    <t>A bank-to-bank transfer surface is present in definitions, but its COBOL implementation and transaction binding are absent.</t>
-  </si>
-  <si>
-    <t>The surface is classified Partial and excluded from the default deployment; no successful transfer is claimed.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/bms/BNK1B2M.bms; legacy/.setup/zconfig/bank-of-z-definitions.yaml:51,143; legacy/.setup/deploy/Development.yml:16-18; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Deviation D-011: non-deployed bank-to-bank surface is not ported.</t>
-  </si>
-  <si>
-    <t>UF-008</t>
-  </si>
-  <si>
-    <t>Transaction history and external account APIs</t>
   </si>
   <si>
     <t>External client retrieves a CICS customer</t>
@@ -6920,103 +6938,111 @@
       </c>
     </row>
     <row r="79" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A79" s="21" t="s">
+      <c r="A79" s="17" t="s">
         <v>487</v>
       </c>
-      <c r="B79" s="21" t="s">
+      <c r="B79" s="17" t="s">
         <v>488</v>
       </c>
-      <c r="C79" s="21" t="s">
-        <v>489</v>
-      </c>
-      <c r="D79" s="21" t="s">
-        <v>490</v>
-      </c>
-      <c r="E79" s="21"/>
-      <c r="F79" s="21"/>
-      <c r="G79" s="21"/>
-      <c r="H79" s="21"/>
-      <c r="I79" s="21"/>
-      <c r="J79" s="21"/>
-      <c r="K79" s="21"/>
-      <c r="L79" s="21"/>
-      <c r="M79" s="21"/>
-      <c r="N79" s="21"/>
+      <c r="C79" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D79" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E79" s="17"/>
+      <c r="F79" s="17"/>
+      <c r="G79" s="17"/>
+      <c r="H79" s="17"/>
+      <c r="I79" s="17"/>
+      <c r="J79" s="17"/>
+      <c r="K79" s="17"/>
+      <c r="L79" s="17"/>
+      <c r="M79" s="17"/>
+      <c r="N79" s="17"/>
     </row>
     <row r="80" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A80" s="18"/>
       <c r="B80" s="19" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C80" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D80" s="22" t="s">
+      <c r="D80" s="20" t="s">
+        <v>490</v>
+      </c>
+      <c r="E80" s="20" t="s">
+        <v>491</v>
+      </c>
+      <c r="F80" s="20" t="s">
         <v>492</v>
       </c>
-      <c r="E80" s="22" t="s">
+      <c r="G80" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H80" s="20" t="s">
         <v>493</v>
       </c>
-      <c r="F80" s="22" t="s">
+      <c r="I80" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J80" s="20" t="s">
         <v>494</v>
       </c>
-      <c r="G80" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H80" s="22" t="s">
+      <c r="K80" s="20" t="s">
         <v>495</v>
       </c>
-      <c r="I80" s="22"/>
-      <c r="J80" s="22" t="s">
+      <c r="L80" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M80" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N80" s="20" t="s">
         <v>496</v>
-      </c>
-      <c r="K80" s="22"/>
-      <c r="L80" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M80" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N80" s="22" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="81" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A81" s="18"/>
       <c r="B81" s="19" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C81" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D81" s="22" t="s">
+      <c r="D81" s="20" t="s">
+        <v>498</v>
+      </c>
+      <c r="E81" s="20" t="s">
         <v>499</v>
       </c>
-      <c r="E81" s="22" t="s">
+      <c r="F81" s="20" t="s">
         <v>500</v>
       </c>
-      <c r="F81" s="22" t="s">
+      <c r="G81" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H81" s="20" t="s">
         <v>501</v>
       </c>
-      <c r="G81" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H81" s="22" t="s">
+      <c r="I81" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J81" s="20" t="s">
         <v>502</v>
       </c>
-      <c r="I81" s="22"/>
-      <c r="J81" s="22" t="s">
+      <c r="K81" s="20" t="s">
         <v>503</v>
       </c>
-      <c r="K81" s="22"/>
-      <c r="L81" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M81" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N81" s="22" t="s">
-        <v>497</v>
+      <c r="L81" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M81" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N81" s="20" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="82" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
@@ -7027,162 +7053,178 @@
       <c r="C82" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D82" s="22" t="s">
+      <c r="D82" s="20" t="s">
         <v>505</v>
       </c>
-      <c r="E82" s="22" t="s">
+      <c r="E82" s="20" t="s">
         <v>506</v>
       </c>
-      <c r="F82" s="22" t="s">
+      <c r="F82" s="20" t="s">
         <v>507</v>
       </c>
-      <c r="G82" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H82" s="22" t="s">
+      <c r="G82" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H82" s="20" t="s">
         <v>508</v>
       </c>
-      <c r="I82" s="22"/>
-      <c r="J82" s="22" t="s">
+      <c r="I82" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J82" s="20" t="s">
         <v>509</v>
       </c>
-      <c r="K82" s="22"/>
-      <c r="L82" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M82" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N82" s="22" t="s">
-        <v>497</v>
+      <c r="K82" s="20" t="s">
+        <v>510</v>
+      </c>
+      <c r="L82" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M82" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N82" s="20" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="83" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A83" s="18"/>
       <c r="B83" s="19" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C83" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D83" s="22" t="s">
-        <v>511</v>
-      </c>
-      <c r="E83" s="22" t="s">
+      <c r="D83" s="20" t="s">
         <v>512</v>
       </c>
-      <c r="F83" s="22" t="s">
+      <c r="E83" s="20" t="s">
         <v>513</v>
       </c>
-      <c r="G83" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H83" s="22" t="s">
+      <c r="F83" s="20" t="s">
         <v>514</v>
       </c>
-      <c r="I83" s="22"/>
-      <c r="J83" s="22" t="s">
+      <c r="G83" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H83" s="20" t="s">
         <v>515</v>
       </c>
-      <c r="K83" s="22"/>
-      <c r="L83" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M83" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N83" s="22" t="s">
-        <v>497</v>
+      <c r="I83" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J83" s="20" t="s">
+        <v>516</v>
+      </c>
+      <c r="K83" s="20" t="s">
+        <v>517</v>
+      </c>
+      <c r="L83" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M83" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N83" s="20" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="84" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A84" s="18"/>
       <c r="B84" s="19" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C84" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D84" s="22" t="s">
-        <v>517</v>
-      </c>
-      <c r="E84" s="22" t="s">
-        <v>518</v>
-      </c>
-      <c r="F84" s="22" t="s">
+      <c r="D84" s="20" t="s">
         <v>519</v>
       </c>
-      <c r="G84" s="22" t="s">
+      <c r="E84" s="20" t="s">
         <v>520</v>
       </c>
-      <c r="H84" s="22" t="s">
+      <c r="F84" s="20" t="s">
         <v>521</v>
       </c>
-      <c r="I84" s="22"/>
-      <c r="J84" s="22" t="s">
+      <c r="G84" s="20" t="s">
         <v>522</v>
       </c>
-      <c r="K84" s="22"/>
-      <c r="L84" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M84" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N84" s="22" t="s">
-        <v>497</v>
+      <c r="H84" s="20" t="s">
+        <v>523</v>
+      </c>
+      <c r="I84" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J84" s="20" t="s">
+        <v>524</v>
+      </c>
+      <c r="K84" s="20" t="s">
+        <v>525</v>
+      </c>
+      <c r="L84" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M84" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N84" s="20" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="85" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A85" s="18"/>
       <c r="B85" s="19" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C85" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D85" s="22" t="s">
-        <v>524</v>
-      </c>
-      <c r="E85" s="22" t="s">
-        <v>525</v>
-      </c>
-      <c r="F85" s="22" t="s">
-        <v>526</v>
-      </c>
-      <c r="G85" s="22" t="s">
+      <c r="D85" s="20" t="s">
+        <v>527</v>
+      </c>
+      <c r="E85" s="20" t="s">
+        <v>528</v>
+      </c>
+      <c r="F85" s="20" t="s">
+        <v>529</v>
+      </c>
+      <c r="G85" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H85" s="22" t="s">
-        <v>527</v>
-      </c>
-      <c r="I85" s="22"/>
-      <c r="J85" s="22" t="s">
-        <v>528</v>
-      </c>
-      <c r="K85" s="22"/>
-      <c r="L85" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M85" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N85" s="22" t="s">
-        <v>497</v>
+      <c r="H85" s="20" t="s">
+        <v>530</v>
+      </c>
+      <c r="I85" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J85" s="20" t="s">
+        <v>531</v>
+      </c>
+      <c r="K85" s="20" t="s">
+        <v>532</v>
+      </c>
+      <c r="L85" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M85" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N85" s="20" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="86" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="21" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="B86" s="21" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="C86" s="21" t="s">
-        <v>489</v>
+        <v>535</v>
       </c>
       <c r="D86" s="21" t="s">
-        <v>490</v>
+        <v>536</v>
       </c>
       <c r="E86" s="21"/>
       <c r="F86" s="21"/>
@@ -7198,34 +7240,34 @@
     <row r="87" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C87" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D87" s="20" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="E87" s="20" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="F87" s="20" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="G87" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H87" s="20" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="I87" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J87" s="20" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="K87" s="20" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="L87" s="20" t="s">
         <v>36</v>
@@ -7240,34 +7282,34 @@
     <row r="88" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="C88" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D88" s="20" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="E88" s="20" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="F88" s="20" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="G88" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H88" s="20" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="I88" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J88" s="20" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="K88" s="20" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="L88" s="20" t="s">
         <v>36</v>
@@ -7282,31 +7324,31 @@
     <row r="89" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="C89" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="F89" s="20" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="G89" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H89" s="20" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="I89" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J89" s="20" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="K89" s="20" t="s">
         <v>377</v>
@@ -7324,31 +7366,31 @@
     <row r="90" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="C90" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D90" s="20" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="E90" s="20" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="F90" s="20" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="G90" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H90" s="20" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="I90" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J90" s="20" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="K90" s="20" t="s">
         <v>153</v>
@@ -7366,29 +7408,29 @@
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="18"/>
       <c r="B91" s="19" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="C91" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D91" s="22" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="E91" s="22" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="F91" s="22" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="G91" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H91" s="22" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="I91" s="22"/>
       <c r="J91" s="22" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="K91" s="22"/>
       <c r="L91" s="22" t="s">
@@ -7398,35 +7440,35 @@
         <v>40</v>
       </c>
       <c r="N91" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="92" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="C92" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D92" s="22" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="E92" s="22" t="s">
+        <v>572</v>
+      </c>
+      <c r="F92" s="22" t="s">
         <v>566</v>
-      </c>
-      <c r="F92" s="22" t="s">
-        <v>560</v>
       </c>
       <c r="G92" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H92" s="22" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="I92" s="22"/>
       <c r="J92" s="22" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="K92" s="22"/>
       <c r="L92" s="22" t="s">
@@ -7436,35 +7478,35 @@
         <v>40</v>
       </c>
       <c r="N92" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A93" s="18"/>
       <c r="B93" s="19" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="C93" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D93" s="22" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="E93" s="22" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="F93" s="22" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="G93" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H93" s="22" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="I93" s="22"/>
       <c r="J93" s="22" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="K93" s="22"/>
       <c r="L93" s="22" t="s">
@@ -7474,35 +7516,35 @@
         <v>40</v>
       </c>
       <c r="N93" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="18"/>
       <c r="B94" s="19" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="C94" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D94" s="22" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="E94" s="22" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="F94" s="22" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="G94" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H94" s="22" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="I94" s="22"/>
       <c r="J94" s="22" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="K94" s="22"/>
       <c r="L94" s="22" t="s">
@@ -7512,35 +7554,35 @@
         <v>40</v>
       </c>
       <c r="N94" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="C95" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D95" s="22" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="E95" s="22" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="F95" s="22" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="G95" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H95" s="22" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="I95" s="22"/>
       <c r="J95" s="22" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="K95" s="22"/>
       <c r="L95" s="22" t="s">
@@ -7550,35 +7592,35 @@
         <v>40</v>
       </c>
       <c r="N95" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="96" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D96" s="22" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="E96" s="22" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="F96" s="22" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="G96" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H96" s="22" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="I96" s="22"/>
       <c r="J96" s="22" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="K96" s="22"/>
       <c r="L96" s="22" t="s">
@@ -7588,40 +7630,40 @@
         <v>40</v>
       </c>
       <c r="N96" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="97" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="C97" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D97" s="20" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="E97" s="20" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="F97" s="20" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="G97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H97" s="20" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="I97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J97" s="20" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="K97" s="20" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="L97" s="20" t="s">
         <v>36</v>
@@ -7636,29 +7678,29 @@
     <row r="98" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="C98" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D98" s="22" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="E98" s="22" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="F98" s="22" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="G98" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H98" s="22" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="I98" s="22"/>
       <c r="J98" s="22" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="K98" s="22"/>
       <c r="L98" s="22" t="s">
@@ -7668,21 +7710,21 @@
         <v>40</v>
       </c>
       <c r="N98" s="22" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="99" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="21" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="B99" s="21" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="C99" s="21" t="s">
-        <v>489</v>
+        <v>535</v>
       </c>
       <c r="D99" s="21" t="s">
-        <v>490</v>
+        <v>536</v>
       </c>
       <c r="E99" s="21"/>
       <c r="F99" s="21"/>
@@ -7698,29 +7740,29 @@
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="18"/>
       <c r="B100" s="19" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="C100" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D100" s="22" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="E100" s="22" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="F100" s="22" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="G100" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H100" s="22" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="I100" s="22"/>
       <c r="J100" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K100" s="22"/>
       <c r="L100" s="22" t="s">
@@ -7730,35 +7772,35 @@
         <v>40</v>
       </c>
       <c r="N100" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="18"/>
       <c r="B101" s="19" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="C101" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D101" s="22" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="E101" s="22" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="F101" s="22" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="G101" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H101" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="I101" s="22"/>
       <c r="J101" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K101" s="22"/>
       <c r="L101" s="22" t="s">
@@ -7768,35 +7810,35 @@
         <v>40</v>
       </c>
       <c r="N101" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D102" s="22" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="E102" s="22" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="F102" s="22" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="G102" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H102" s="22" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="I102" s="22"/>
       <c r="J102" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K102" s="22"/>
       <c r="L102" s="22" t="s">
@@ -7806,35 +7848,35 @@
         <v>40</v>
       </c>
       <c r="N102" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="C103" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D103" s="22" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="E103" s="22" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="F103" s="22" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="G103" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H103" s="22" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="I103" s="22"/>
       <c r="J103" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K103" s="22"/>
       <c r="L103" s="22" t="s">
@@ -7844,35 +7886,35 @@
         <v>40</v>
       </c>
       <c r="N103" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D104" s="22" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="E104" s="22" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="F104" s="22" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="G104" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H104" s="22" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="I104" s="22"/>
       <c r="J104" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K104" s="22"/>
       <c r="L104" s="22" t="s">
@@ -7882,35 +7924,35 @@
         <v>40</v>
       </c>
       <c r="N104" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="18"/>
       <c r="B105" s="19" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="C105" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D105" s="22" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="E105" s="22" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="F105" s="22" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="G105" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H105" s="22" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="I105" s="22"/>
       <c r="J105" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K105" s="22"/>
       <c r="L105" s="22" t="s">
@@ -7920,35 +7962,35 @@
         <v>40</v>
       </c>
       <c r="N105" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="C106" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D106" s="22" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="E106" s="22" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="F106" s="22" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="G106" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H106" s="22" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="I106" s="22"/>
       <c r="J106" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K106" s="22"/>
       <c r="L106" s="22" t="s">
@@ -7958,35 +8000,35 @@
         <v>40</v>
       </c>
       <c r="N106" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="C107" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D107" s="22" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="E107" s="22" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="F107" s="22" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="G107" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H107" s="22" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="I107" s="22"/>
       <c r="J107" s="22" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="K107" s="22"/>
       <c r="L107" s="22" t="s">
@@ -7996,15 +8038,15 @@
         <v>40</v>
       </c>
       <c r="N107" s="22" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="108" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="B108" s="17" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="C108" s="17" t="s">
         <v>29</v>
@@ -8026,34 +8068,34 @@
     <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="C109" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="E109" s="20" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="F109" s="20" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="I109" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J109" s="20" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="K109" s="20" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="L109" s="20" t="s">
         <v>36</v>
@@ -8068,34 +8110,34 @@
     <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C110" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="F110" s="20" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="G110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="I110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J110" s="20" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="K110" s="20" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="L110" s="20" t="s">
         <v>36</v>
@@ -8110,34 +8152,34 @@
     <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="C111" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D111" s="20" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="E111" s="20" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="F111" s="20" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="G111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="I111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J111" s="20" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="K111" s="20" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="L111" s="20" t="s">
         <v>36</v>
@@ -8152,34 +8194,34 @@
     <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="C112" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="F112" s="20" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="G112" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="I112" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J112" s="20" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="K112" s="20" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="L112" s="20" t="s">
         <v>36</v>
@@ -8194,34 +8236,34 @@
     <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="C113" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="I113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J113" s="20" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="K113" s="20" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="L113" s="20" t="s">
         <v>36</v>
@@ -8236,34 +8278,34 @@
     <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="C114" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D114" s="20" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="E114" s="20" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="F114" s="20" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="G114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="20" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="I114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J114" s="20" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="K114" s="20" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="L114" s="20" t="s">
         <v>36</v>
@@ -8278,31 +8320,31 @@
     <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="C115" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D115" s="20" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="F115" s="20" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="G115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="20" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="I115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J115" s="20" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="K115" s="20" t="s">
         <v>56</v>
@@ -8320,34 +8362,34 @@
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="18"/>
       <c r="B116" s="19" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="C116" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D116" s="20" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="E116" s="20" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="F116" s="20" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="G116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H116" s="20" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="I116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J116" s="20" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="K116" s="20" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="L116" s="20" t="s">
         <v>36</v>
@@ -8362,34 +8404,34 @@
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
       <c r="B117" s="19" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="C117" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="E117" s="20" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="G117" s="20" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="I117" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J117" s="20" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="K117" s="20" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="L117" s="20" t="s">
         <v>36</v>
@@ -8403,16 +8445,16 @@
     </row>
     <row r="118" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="21" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="B118" s="21" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="C118" s="21" t="s">
-        <v>489</v>
+        <v>535</v>
       </c>
       <c r="D118" s="21" t="s">
-        <v>490</v>
+        <v>536</v>
       </c>
       <c r="E118" s="21"/>
       <c r="F118" s="21"/>
@@ -8428,29 +8470,29 @@
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="19" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D119" s="22" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="E119" s="22" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="F119" s="22" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="G119" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="22" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="I119" s="22"/>
       <c r="J119" s="22" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="K119" s="22"/>
       <c r="L119" s="22" t="s">
@@ -8460,35 +8502,35 @@
         <v>40</v>
       </c>
       <c r="N119" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="19" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D120" s="22" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="E120" s="22" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="F120" s="22" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="G120" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="22" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="I120" s="22"/>
       <c r="J120" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="K120" s="22"/>
       <c r="L120" s="22" t="s">
@@ -8498,35 +8540,35 @@
         <v>40</v>
       </c>
       <c r="N120" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
       <c r="B121" s="19" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="C121" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D121" s="22" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="E121" s="22" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="F121" s="22" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="G121" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="22" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="I121" s="22"/>
       <c r="J121" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="K121" s="22"/>
       <c r="L121" s="22" t="s">
@@ -8536,35 +8578,35 @@
         <v>40</v>
       </c>
       <c r="N121" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="19" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D122" s="22" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="E122" s="22" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="F122" s="22" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="G122" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="22" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="I122" s="22"/>
       <c r="J122" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="K122" s="22"/>
       <c r="L122" s="22" t="s">
@@ -8574,35 +8616,35 @@
         <v>40</v>
       </c>
       <c r="N122" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="19" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D123" s="22" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="E123" s="22" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="F123" s="22" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="G123" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H123" s="22" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="I123" s="22"/>
       <c r="J123" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="K123" s="22"/>
       <c r="L123" s="22" t="s">
@@ -8612,35 +8654,35 @@
         <v>40</v>
       </c>
       <c r="N123" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="19" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D124" s="22" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="E124" s="22" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="F124" s="22" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
       <c r="G124" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H124" s="22" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="I124" s="22"/>
       <c r="J124" s="22" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="K124" s="22"/>
       <c r="L124" s="22" t="s">
@@ -8650,35 +8692,35 @@
         <v>40</v>
       </c>
       <c r="N124" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="19" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D125" s="22" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="E125" s="22" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="F125" s="22" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="G125" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H125" s="22" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="I125" s="22"/>
       <c r="J125" s="22" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="K125" s="22"/>
       <c r="L125" s="22" t="s">
@@ -8688,35 +8730,35 @@
         <v>40</v>
       </c>
       <c r="N125" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="19" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D126" s="22" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="E126" s="22" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="F126" s="22" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="G126" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="22" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="I126" s="22"/>
       <c r="J126" s="22" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="K126" s="22"/>
       <c r="L126" s="22" t="s">
@@ -8726,21 +8768,21 @@
         <v>40</v>
       </c>
       <c r="N126" s="22" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="21" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="B127" s="21" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="C127" s="21" t="s">
-        <v>489</v>
+        <v>535</v>
       </c>
       <c r="D127" s="21" t="s">
-        <v>490</v>
+        <v>536</v>
       </c>
       <c r="E127" s="21"/>
       <c r="F127" s="21"/>
@@ -8756,29 +8798,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D128" s="22" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="E128" s="22" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="F128" s="22" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="G128" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="22" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="I128" s="22"/>
       <c r="J128" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K128" s="22"/>
       <c r="L128" s="22" t="s">
@@ -8788,35 +8830,35 @@
         <v>40</v>
       </c>
       <c r="N128" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D129" s="22" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="E129" s="22" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="F129" s="22" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="G129" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="I129" s="22"/>
       <c r="J129" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K129" s="22"/>
       <c r="L129" s="22" t="s">
@@ -8826,35 +8868,35 @@
         <v>40</v>
       </c>
       <c r="N129" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="18"/>
       <c r="B130" s="19" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D130" s="22" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="E130" s="22" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="F130" s="22" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="G130" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="22" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="I130" s="22"/>
       <c r="J130" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K130" s="22"/>
       <c r="L130" s="22" t="s">
@@ -8864,35 +8906,35 @@
         <v>40</v>
       </c>
       <c r="N130" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D131" s="22" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="E131" s="22" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="F131" s="22" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
       <c r="G131" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H131" s="22" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="I131" s="22"/>
       <c r="J131" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K131" s="22"/>
       <c r="L131" s="22" t="s">
@@ -8902,35 +8944,35 @@
         <v>40</v>
       </c>
       <c r="N131" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D132" s="22" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="E132" s="22" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="F132" s="22" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="G132" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="22" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="I132" s="22"/>
       <c r="J132" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K132" s="22"/>
       <c r="L132" s="22" t="s">
@@ -8940,35 +8982,35 @@
         <v>40</v>
       </c>
       <c r="N132" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D133" s="22" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="E133" s="22" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="F133" s="22" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="G133" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H133" s="22" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="I133" s="22"/>
       <c r="J133" s="22" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="K133" s="22"/>
       <c r="L133" s="22" t="s">
@@ -8978,35 +9020,35 @@
         <v>40</v>
       </c>
       <c r="N133" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D134" s="22" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="E134" s="22" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
       <c r="F134" s="22" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="G134" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="22" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="I134" s="22"/>
       <c r="J134" s="22" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="K134" s="22"/>
       <c r="L134" s="22" t="s">
@@ -9016,35 +9058,35 @@
         <v>40</v>
       </c>
       <c r="N134" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D135" s="22" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="E135" s="22" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
       <c r="F135" s="22" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
       <c r="G135" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H135" s="22" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="I135" s="22"/>
       <c r="J135" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K135" s="22"/>
       <c r="L135" s="22" t="s">
@@ -9054,35 +9096,35 @@
         <v>40</v>
       </c>
       <c r="N135" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D136" s="22" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="E136" s="22" t="s">
-        <v>806</v>
+        <v>812</v>
       </c>
       <c r="F136" s="22" t="s">
-        <v>807</v>
+        <v>813</v>
       </c>
       <c r="G136" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H136" s="22" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="I136" s="22"/>
       <c r="J136" s="22" t="s">
-        <v>809</v>
+        <v>815</v>
       </c>
       <c r="K136" s="22"/>
       <c r="L136" s="22" t="s">
@@ -9092,35 +9134,35 @@
         <v>40</v>
       </c>
       <c r="N136" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D137" s="22" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="E137" s="22" t="s">
-        <v>812</v>
+        <v>818</v>
       </c>
       <c r="F137" s="22" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
       <c r="G137" s="22" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="H137" s="22" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
       <c r="I137" s="22"/>
       <c r="J137" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K137" s="22"/>
       <c r="L137" s="22" t="s">
@@ -9130,35 +9172,35 @@
         <v>40</v>
       </c>
       <c r="N137" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D138" s="22" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="E138" s="22" t="s">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="F138" s="22" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
       <c r="G138" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="22" t="s">
-        <v>819</v>
+        <v>825</v>
       </c>
       <c r="I138" s="22"/>
       <c r="J138" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K138" s="22"/>
       <c r="L138" s="22" t="s">
@@ -9168,35 +9210,35 @@
         <v>40</v>
       </c>
       <c r="N138" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D139" s="22" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="E139" s="22" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
       <c r="F139" s="22" t="s">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="G139" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="22" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
       <c r="I139" s="22"/>
       <c r="J139" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K139" s="22"/>
       <c r="L139" s="22" t="s">
@@ -9206,35 +9248,35 @@
         <v>40</v>
       </c>
       <c r="N139" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D140" s="22" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="E140" s="22" t="s">
-        <v>827</v>
+        <v>833</v>
       </c>
       <c r="F140" s="22" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="G140" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="22" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
       <c r="I140" s="22"/>
       <c r="J140" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K140" s="22"/>
       <c r="L140" s="22" t="s">
@@ -9244,35 +9286,35 @@
         <v>40</v>
       </c>
       <c r="N140" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D141" s="22" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="E141" s="22" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
       <c r="F141" s="22" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="G141" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="22" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
       <c r="I141" s="22"/>
       <c r="J141" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K141" s="22"/>
       <c r="L141" s="22" t="s">
@@ -9282,35 +9324,35 @@
         <v>40</v>
       </c>
       <c r="N141" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>835</v>
+        <v>841</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D142" s="22" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
       <c r="E142" s="22" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="F142" s="22" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="G142" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="22" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="I142" s="22"/>
       <c r="J142" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K142" s="22"/>
       <c r="L142" s="22" t="s">
@@ -9320,35 +9362,35 @@
         <v>40</v>
       </c>
       <c r="N142" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D143" s="22" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="E143" s="22" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
       <c r="F143" s="22" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
       <c r="G143" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="22" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="I143" s="22"/>
       <c r="J143" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K143" s="22"/>
       <c r="L143" s="22" t="s">
@@ -9358,35 +9400,35 @@
         <v>40</v>
       </c>
       <c r="N143" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D144" s="22" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="E144" s="22" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="F144" s="22" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="G144" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H144" s="22" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="I144" s="22"/>
       <c r="J144" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K144" s="22"/>
       <c r="L144" s="22" t="s">
@@ -9396,35 +9438,35 @@
         <v>40</v>
       </c>
       <c r="N144" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D145" s="22" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="E145" s="22" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="F145" s="22" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="G145" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="22" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="I145" s="22"/>
       <c r="J145" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K145" s="22"/>
       <c r="L145" s="22" t="s">
@@ -9434,35 +9476,35 @@
         <v>40</v>
       </c>
       <c r="N145" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D146" s="22" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="E146" s="22" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="F146" s="22" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="G146" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="22" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="I146" s="22"/>
       <c r="J146" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K146" s="22"/>
       <c r="L146" s="22" t="s">
@@ -9472,35 +9514,35 @@
         <v>40</v>
       </c>
       <c r="N146" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D147" s="22" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="E147" s="22" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="F147" s="22" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="G147" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="22" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="I147" s="22"/>
       <c r="J147" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K147" s="22"/>
       <c r="L147" s="22" t="s">
@@ -9510,35 +9552,35 @@
         <v>40</v>
       </c>
       <c r="N147" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D148" s="22" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
       <c r="E148" s="22" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
       <c r="F148" s="22" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="G148" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="22" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="I148" s="22"/>
       <c r="J148" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K148" s="22"/>
       <c r="L148" s="22" t="s">
@@ -9548,35 +9590,35 @@
         <v>40</v>
       </c>
       <c r="N148" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D149" s="22" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="E149" s="22" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="F149" s="22" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="G149" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="22" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="I149" s="22"/>
       <c r="J149" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K149" s="22"/>
       <c r="L149" s="22" t="s">
@@ -9586,35 +9628,35 @@
         <v>40</v>
       </c>
       <c r="N149" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D150" s="22" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="E150" s="22" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="F150" s="22" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="G150" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H150" s="22" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="I150" s="22"/>
       <c r="J150" s="22" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="K150" s="22"/>
       <c r="L150" s="22" t="s">
@@ -9624,35 +9666,35 @@
         <v>40</v>
       </c>
       <c r="N150" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D151" s="22" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
       <c r="E151" s="22" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="F151" s="22" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="G151" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H151" s="22" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
       <c r="I151" s="22"/>
       <c r="J151" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K151" s="22"/>
       <c r="L151" s="22" t="s">
@@ -9662,35 +9704,35 @@
         <v>40</v>
       </c>
       <c r="N151" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D152" s="22" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="E152" s="22" t="s">
-        <v>888</v>
+        <v>894</v>
       </c>
       <c r="F152" s="22" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="G152" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H152" s="22" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="I152" s="22"/>
       <c r="J152" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K152" s="22"/>
       <c r="L152" s="22" t="s">
@@ -9700,35 +9742,35 @@
         <v>40</v>
       </c>
       <c r="N152" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D153" s="22" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
       <c r="E153" s="22" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
       <c r="F153" s="22" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="G153" s="22" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="H153" s="22" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="I153" s="22"/>
       <c r="J153" s="22" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="K153" s="22"/>
       <c r="L153" s="22" t="s">
@@ -9738,7 +9780,7 @@
         <v>40</v>
       </c>
       <c r="N153" s="22" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
   </sheetData>
@@ -9771,51 +9813,51 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>897</v>
+        <v>903</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>898</v>
+        <v>904</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>899</v>
+        <v>905</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="G1" s="24" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="24" t="s">
-        <v>902</v>
+        <v>908</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>909</v>
+        <v>915</v>
       </c>
       <c r="G2" s="27" t="s">
         <v>36</v>
@@ -9824,27 +9866,27 @@
         <v>36</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
-        <v>911</v>
+        <v>917</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>912</v>
+        <v>918</v>
       </c>
       <c r="C3" s="30" t="s">
+        <v>919</v>
+      </c>
+      <c r="D3" s="30" t="s">
         <v>913</v>
       </c>
-      <c r="D3" s="30" t="s">
-        <v>907</v>
-      </c>
       <c r="E3" s="30" t="s">
-        <v>914</v>
+        <v>920</v>
       </c>
       <c r="F3" s="30" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
       <c r="G3" s="30" t="s">
         <v>36</v>
@@ -9853,27 +9895,27 @@
         <v>36</v>
       </c>
       <c r="I3" s="31" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
-        <v>917</v>
+        <v>923</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>919</v>
+        <v>925</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
       <c r="G4" s="30" t="s">
         <v>36</v>
@@ -9882,27 +9924,27 @@
         <v>36</v>
       </c>
       <c r="I4" s="31" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>36</v>
@@ -9911,27 +9953,27 @@
         <v>36</v>
       </c>
       <c r="I5" s="31" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="32" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>487</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>930</v>
+        <v>936</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>931</v>
+        <v>937</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>932</v>
+        <v>938</v>
       </c>
       <c r="G6" s="33" t="s">
         <v>36</v>
@@ -9940,27 +9982,27 @@
         <v>40</v>
       </c>
       <c r="I6" s="34" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>935</v>
+        <v>941</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
       <c r="G7" s="33" t="s">
         <v>36</v>
@@ -9969,27 +10011,27 @@
         <v>40</v>
       </c>
       <c r="I7" s="34" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
-        <v>939</v>
+        <v>945</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>941</v>
+        <v>947</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="G8" s="33" t="s">
         <v>36</v>
@@ -9998,27 +10040,27 @@
         <v>40</v>
       </c>
       <c r="I8" s="34" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="G9" s="33" t="s">
         <v>36</v>
@@ -10027,27 +10069,27 @@
         <v>40</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="B10" s="36" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="G10" s="36" t="s">
         <v>36</v>
@@ -10056,25 +10098,25 @@
         <v>40</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="B11" s="27"/>
       <c r="C11" s="27" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="G11" s="27" t="s">
         <v>36</v>
@@ -10083,25 +10125,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="30" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>36</v>
@@ -10110,25 +10152,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="B13" s="30"/>
       <c r="C13" s="30" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E13" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="G13" s="30" t="s">
         <v>36</v>
@@ -10137,25 +10179,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="30" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
       <c r="G14" s="30" t="s">
         <v>36</v>
@@ -10164,25 +10206,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="31" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="B15" s="30"/>
       <c r="C15" s="30" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E15" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="G15" s="30" t="s">
         <v>36</v>
@@ -10191,25 +10233,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="30" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
       <c r="G16" s="30" t="s">
         <v>36</v>
@@ -10218,25 +10260,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="31" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="29" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
       <c r="B17" s="30"/>
       <c r="C17" s="30" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="G17" s="30" t="s">
         <v>36</v>
@@ -10245,25 +10287,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="G18" s="30" t="s">
         <v>36</v>
@@ -10272,25 +10314,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="31" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="29" t="s">
-        <v>988</v>
+        <v>994</v>
       </c>
       <c r="B19" s="30"/>
       <c r="C19" s="30" t="s">
-        <v>989</v>
+        <v>995</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
       <c r="G19" s="30" t="s">
         <v>36</v>
@@ -10299,25 +10341,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
-        <v>992</v>
+        <v>998</v>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="30" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="G20" s="30" t="s">
         <v>36</v>
@@ -10326,25 +10368,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="31" t="s">
-        <v>995</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="29" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="B21" s="30"/>
       <c r="C21" s="30" t="s">
-        <v>997</v>
+        <v>1003</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E21" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F21" s="30" t="s">
-        <v>998</v>
+        <v>1004</v>
       </c>
       <c r="G21" s="30" t="s">
         <v>36</v>
@@ -10353,25 +10395,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>999</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="G22" s="30" t="s">
         <v>36</v>
@@ -10380,25 +10422,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="31" t="s">
-        <v>1002</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
-        <v>1003</v>
+        <v>1009</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F23" s="30" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="G23" s="30" t="s">
         <v>36</v>
@@ -10407,25 +10449,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>1005</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
-        <v>1006</v>
+        <v>1012</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30" t="s">
-        <v>1007</v>
+        <v>1013</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>1008</v>
+        <v>1014</v>
       </c>
       <c r="G24" s="30" t="s">
         <v>36</v>
@@ -10434,25 +10476,25 @@
         <v>36</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>1009</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="39" t="s">
-        <v>1011</v>
+        <v>1017</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>1012</v>
+        <v>1018</v>
       </c>
       <c r="G25" s="39" t="s">
         <v>36</v>
@@ -10461,25 +10503,25 @@
         <v>36</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>1013</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="38" t="s">
-        <v>1014</v>
+        <v>1020</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="39" t="s">
-        <v>1015</v>
+        <v>1021</v>
       </c>
       <c r="D26" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E26" s="39" t="s">
-        <v>1016</v>
+        <v>1022</v>
       </c>
       <c r="F26" s="39" t="s">
-        <v>1017</v>
+        <v>1023</v>
       </c>
       <c r="G26" s="39" t="s">
         <v>36</v>
@@ -10488,25 +10530,25 @@
         <v>36</v>
       </c>
       <c r="I26" s="40" t="s">
-        <v>1018</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="38" t="s">
-        <v>1019</v>
+        <v>1025</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39" t="s">
-        <v>1020</v>
+        <v>1026</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>1021</v>
+        <v>1027</v>
       </c>
       <c r="F27" s="39" t="s">
-        <v>1022</v>
+        <v>1028</v>
       </c>
       <c r="G27" s="39" t="s">
         <v>36</v>
@@ -10515,25 +10557,25 @@
         <v>36</v>
       </c>
       <c r="I27" s="40" t="s">
-        <v>1023</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>1024</v>
+        <v>1030</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39" t="s">
-        <v>1025</v>
+        <v>1031</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E28" s="39" t="s">
-        <v>1026</v>
+        <v>1032</v>
       </c>
       <c r="F28" s="39" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="G28" s="39" t="s">
         <v>36</v>
@@ -10542,25 +10584,25 @@
         <v>36</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
-        <v>1029</v>
+        <v>1035</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39" t="s">
-        <v>1030</v>
+        <v>1036</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>1031</v>
+        <v>1037</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>1032</v>
+        <v>1038</v>
       </c>
       <c r="G29" s="39" t="s">
         <v>36</v>
@@ -10569,25 +10611,25 @@
         <v>36</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>1033</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
-        <v>1034</v>
+        <v>1040</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="39" t="s">
-        <v>1035</v>
+        <v>1041</v>
       </c>
       <c r="D30" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E30" s="39" t="s">
-        <v>1036</v>
+        <v>1042</v>
       </c>
       <c r="F30" s="39" t="s">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="G30" s="39" t="s">
         <v>36</v>
@@ -10596,25 +10638,25 @@
         <v>36</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>1038</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="38" t="s">
-        <v>1039</v>
+        <v>1045</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="D31" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="F31" s="39" t="s">
-        <v>1041</v>
+        <v>1047</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>36</v>
@@ -10623,25 +10665,25 @@
         <v>36</v>
       </c>
       <c r="I31" s="40" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="38" t="s">
-        <v>1043</v>
+        <v>1049</v>
       </c>
       <c r="B32" s="39"/>
       <c r="C32" s="39" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
       <c r="D32" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E32" s="39" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="F32" s="39" t="s">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="G32" s="39" t="s">
         <v>36</v>
@@ -10650,25 +10692,25 @@
         <v>36</v>
       </c>
       <c r="I32" s="40" t="s">
-        <v>1047</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="38" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39" t="s">
-        <v>1049</v>
+        <v>1055</v>
       </c>
       <c r="D33" s="39" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>1050</v>
+        <v>1056</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="G33" s="39" t="s">
         <v>36</v>
@@ -10677,7 +10719,7 @@
         <v>36</v>
       </c>
       <c r="I33" s="40" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement transaction history slice
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="1059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="1065">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1623,231 +1623,249 @@
     <t>Transaction history and external account APIs</t>
   </si>
   <si>
+    <t>External client retrieves a CICS customer</t>
+  </si>
+  <si>
+    <t>Expose CICS customer inquiry and update through z/OS Connect.</t>
+  </si>
+  <si>
+    <t>REST clients can access the core CICS customer programs.</t>
+  </si>
+  <si>
+    <t>GET and PUT success mappings reach INQCUST/UPDCUST, but the PUT 401/403 response selections reference missing generated files.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:275-345; operations ...customers...; zosAssets/INQCUST and UPDCUST; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+  </si>
+  <si>
+    <t>D-008 implemented: supported customer inquiry/update are exposed through unified target REST resources and Problem Details.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/CustomersController.cs; modern/backend/src/BankOfZ.Api/ErrorHandling/CustomerExceptionHandler.cs; CustomerApiTests.cs</t>
+  </si>
+  <si>
+    <t>External client retrieves CICS accounts and balances</t>
+  </si>
+  <si>
+    <t>Expose customer accounts, single account, and balances through z/OS Connect.</t>
+  </si>
+  <si>
+    <t>REST clients can inspect the CICS account portfolio.</t>
+  </si>
+  <si>
+    <t>Success mappings return account/balance schemas, but three selected 400 response files are absent.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:346-478; zosAssets/INQACCCU and INQACC; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-008 implemented: supported account list/detail resources return typed balances and stable Problem Details instead of missing generated response mappings.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/AccountsController.cs; modern/backend/src/BankOfZ.Api/ErrorHandling/AccountExceptionHandler.cs; AccountApiTests.cs</t>
+  </si>
+  <si>
+    <t>External client deposits to CICS</t>
+  </si>
+  <si>
+    <t>Expose the CICS deposit operation with a positive amount and six-digit sort code.</t>
+  </si>
+  <si>
+    <t>REST clients can add funds through the same balance logic.</t>
+  </si>
+  <si>
+    <t>The DBCRFUN-backed mapping returns the updated account/balance response.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:479-517,1025; zosAssets/DBCRFUN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+  </si>
+  <si>
+    <t>Decision D-020: target derives the sort code from account/bank configuration instead of trusting request input. The external legacy CICS deposit surface is replaced by the authenticated target API; sort code is derived from the account.</t>
+  </si>
+  <si>
+    <t>External client uses IMS customer/account APIs</t>
+  </si>
+  <si>
+    <t>Expose IMS get/update customer, accounts, balances, and deposit routes.</t>
+  </si>
+  <si>
+    <t>REST clients can reach the IMS channel without terminal messages.</t>
+  </si>
+  <si>
+    <t>Operations map to IBGCUDAT, IBSCUDAT, IBACSUM, and IBTRAN.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:31-245; zosAssets/IBGCUDAT,IBSCUDAT,IBACSUM,IBTRAN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+  </si>
+  <si>
+    <t>D-008 implemented: IMS-provenance customer capabilities use the same supported target resource, not path parity.</t>
+  </si>
+  <si>
+    <t>External client lists all accounts</t>
+  </si>
+  <si>
+    <t>Declare account collection filtering without claiming a working backend mapping.</t>
+  </si>
+  <si>
+    <t>OpenAPI publishes GET /accounts, but the operation directory has no operation.yaml.</t>
+  </si>
+  <si>
+    <t>The contract exists; deployable mapping is absent.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:379-412; operations/%2Faccounts/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+  </si>
+  <si>
+    <t>Deviation D-008: unbound all-account route is not recreated without a target business use case.</t>
+  </si>
+  <si>
+    <t>specs/006-transaction-history/spec.md; modern/backend/src/BankOfZ.Api/Controllers/AccountsController.cs</t>
+  </si>
+  <si>
+    <t>specs/006-transaction-history/spec.md; plan.md; tasks.md</t>
+  </si>
+  <si>
+    <t>External client lists account transactions</t>
+  </si>
+  <si>
+    <t>Declare paged transaction history without claiming a working backend mapping.</t>
+  </si>
+  <si>
+    <t>OpenAPI and the JS client publish the route, but no z/OS operation mapping exists.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:518-579; js/api.js:260-279; operations/...transactions/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+  </si>
+  <si>
+    <t>Decision D-008: provide supported unified history resources, not missing legacy mappings.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/TransactionHistoryController.cs; modern/backend/src/BankOfZ.Application/Transactions/TransactionHistoryService.cs; modern/frontend/bank-of-z-ui/src/app/accounts/transaction-history.component.ts; TransactionHistoryApiTests.cs; secure-access.spec.ts</t>
+  </si>
+  <si>
+    <t>External client retrieves one transaction</t>
+  </si>
+  <si>
+    <t>Declare transaction detail without claiming a working backend mapping.</t>
+  </si>
+  <si>
+    <t>The route is published but has no operation mapping.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:580-615; js/api.js:286-292; operations/...transactionId/get (no operation.yaml); Runtime: static-only</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/TransactionHistoryController.cs; modern/frontend/bank-of-z-ui/src/app/accounts/transaction-history-detail.component.ts; TransactionHistoryApiTests.cs; secure-access.spec.ts</t>
+  </si>
+  <si>
+    <t>Java history service reads recent activity</t>
+  </si>
+  <si>
+    <t>Return the latest 50 history rows for an account in reverse chronological order.</t>
+  </si>
+  <si>
+    <t>The Java/DB2 integration provides bounded recent transaction history.</t>
+  </si>
+  <si>
+    <t>At most 50 records are returned, newest first.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:45-47; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decision D-008: target history resources preserve supported behavior without reproducing legacy route defects.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Application/Transactions/TransactionHistoryService.cs; modern/backend/src/BankOfZ.Infrastructure/Transactions/TransactionHistoryRepository.cs; TransactionHistoryServiceTests.cs; TransactionHistoryApiTests.cs</t>
+  </si>
+  <si>
+    <t>API client receives standard failures</t>
+  </si>
+  <si>
+    <t>Represent validation, authentication, authorization, not-found, and server failures.</t>
+  </si>
+  <si>
+    <t>External consumers need stable error classes.</t>
+  </si>
+  <si>
+    <t>The contract declares standard failures, but five bound and three unbound response selections reference missing generated YAML artifacts.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Deviation D-008: target Problem Details replace missing generated response files.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/ErrorHandling/TransactionHistoryExceptionHandler.cs; modern/backend/src/BankOfZ.Api/Controllers/TransactionHistoryController.cs; TransactionHistoryApiTests.cs</t>
+  </si>
+  <si>
+    <t>Generated API mappings select missing response files</t>
+  </si>
+  <si>
+    <t>Record generated response selections whose referenced sibling YAML artifacts are absent.</t>
+  </si>
+  <si>
+    <t>Five missing files affect bound CICS account/customer operations; three more occur in already-unbound account/transaction routes.</t>
+  </si>
+  <si>
+    <t>Those selected error/fallback responses are not deployable from the supplied artifacts and must not be treated as complete API behavior.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Fbalances/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D/put/response_mapping.yaml:8-10; legacy/src/api/src/main/operations/%2Faccounts/get/response_mapping.yaml:3; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Ftransactions/get/response_mapping.yaml:3; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Ftransactions%2F%7BtransactionId%7D/get/response_mapping.yaml:3; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>External client creates a CICS customer</t>
+  </si>
+  <si>
+    <t>Expose CICS customer creation through POST /customers and the CRECUST z/OS asset.</t>
+  </si>
+  <si>
+    <t>REST clients can onboard a customer without using the web form or 3270 screen.</t>
+  </si>
+  <si>
+    <t>A successful response returns the created customer identity; mapped failures use the declared API responses.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:246-274; legacy/src/api/src/main/operations/%2Fcustomers/post/operation.yaml; legacy/src/api/src/main/zosAssets/CRECUST/zosAsset.yaml; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
+  </si>
+  <si>
+    <t>D-008 implemented: POST /api/customers provides supported onboarding with stable success and failure contracts.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/CustomersController.cs; modern/backend/src/BankOfZ.Api/Contracts/CreateCustomerRequest.cs; CustomerApiTests.cs</t>
+  </si>
+  <si>
+    <t>IMS client requests recent history through IBGHIST</t>
+  </si>
+  <si>
+    <t>Accept an IMS IBGHIST message containing an account number and return at most 50 recent DB2 history records.</t>
+  </si>
+  <si>
+    <t>IBGHIST is a separately deployed Java message-processing transaction, not only an internal repository service.</t>
+  </si>
+  <si>
+    <t>Success returns count/details; controller exceptions may populate MSG-OUT, while JDBC/DB2 failures can be swallowed as null without a response.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/deploy/ims_spoc.jcl.j2:84-86,95,108-109; legacy/src/base/ims/java/src/main/java/nazare/jmp/controller/QueryTransaction.java:28-131; legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:45-47; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Application/Transactions/TransactionHistoryService.cs; modern/backend/src/BankOfZ.Infrastructure/Transactions/TransactionHistoryRepository.cs; modern/backend/src/BankOfZ.Domain/Transactions/BookedTransaction.cs; TransactionHistoryApiTests.cs</t>
+  </si>
+  <si>
+    <t>UF-009</t>
+  </si>
+  <si>
+    <t>Monthly statements and reporting</t>
+  </si>
+  <si>
     <t>Not Passed - Open</t>
   </si>
   <si>
     <t>Legacy behavior is evidenced and covered by SDD; target implementation has not started.</t>
   </si>
   <si>
-    <t>External client retrieves a CICS customer</t>
-  </si>
-  <si>
-    <t>Expose CICS customer inquiry and update through z/OS Connect.</t>
-  </si>
-  <si>
-    <t>REST clients can access the core CICS customer programs.</t>
-  </si>
-  <si>
-    <t>GET and PUT success mappings reach INQCUST/UPDCUST, but the PUT 401/403 response selections reference missing generated files.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:275-345; operations ...customers...; zosAssets/INQCUST and UPDCUST; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
-  </si>
-  <si>
-    <t>D-008 implemented: supported customer inquiry/update are exposed through unified target REST resources and Problem Details.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Api/Controllers/CustomersController.cs; modern/backend/src/BankOfZ.Api/ErrorHandling/CustomerExceptionHandler.cs; CustomerApiTests.cs</t>
-  </si>
-  <si>
-    <t>External client retrieves CICS accounts and balances</t>
-  </si>
-  <si>
-    <t>Expose customer accounts, single account, and balances through z/OS Connect.</t>
-  </si>
-  <si>
-    <t>REST clients can inspect the CICS account portfolio.</t>
-  </si>
-  <si>
-    <t>Success mappings return account/balance schemas, but three selected 400 response files are absent.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:346-478; zosAssets/INQACCCU and INQACC; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-008 implemented: supported account list/detail resources return typed balances and stable Problem Details instead of missing generated response mappings.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Api/Controllers/AccountsController.cs; modern/backend/src/BankOfZ.Api/ErrorHandling/AccountExceptionHandler.cs; AccountApiTests.cs</t>
-  </si>
-  <si>
-    <t>External client deposits to CICS</t>
-  </si>
-  <si>
-    <t>Expose the CICS deposit operation with a positive amount and six-digit sort code.</t>
-  </si>
-  <si>
-    <t>REST clients can add funds through the same balance logic.</t>
-  </si>
-  <si>
-    <t>The DBCRFUN-backed mapping returns the updated account/balance response.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:479-517,1025; zosAssets/DBCRFUN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
-  </si>
-  <si>
-    <t>Decision D-020: target derives the sort code from account/bank configuration instead of trusting request input. The external legacy CICS deposit surface is replaced by the authenticated target API; sort code is derived from the account.</t>
-  </si>
-  <si>
-    <t>External client uses IMS customer/account APIs</t>
-  </si>
-  <si>
-    <t>Expose IMS get/update customer, accounts, balances, and deposit routes.</t>
-  </si>
-  <si>
-    <t>REST clients can reach the IMS channel without terminal messages.</t>
-  </si>
-  <si>
-    <t>Operations map to IBGCUDAT, IBSCUDAT, IBACSUM, and IBTRAN.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:31-245; zosAssets/IBGCUDAT,IBSCUDAT,IBACSUM,IBTRAN; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
-  </si>
-  <si>
-    <t>D-008 implemented: IMS-provenance customer capabilities use the same supported target resource, not path parity.</t>
-  </si>
-  <si>
-    <t>External client lists all accounts</t>
-  </si>
-  <si>
-    <t>Declare account collection filtering without claiming a working backend mapping.</t>
-  </si>
-  <si>
-    <t>OpenAPI publishes GET /accounts, but the operation directory has no operation.yaml.</t>
-  </si>
-  <si>
-    <t>The contract exists; deployable mapping is absent.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:379-412; operations/%2Faccounts/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
-  </si>
-  <si>
-    <t>Deviation D-008: unbound all-account route is not recreated without a target business use case.</t>
-  </si>
-  <si>
-    <t>specs/006-transaction-history/spec.md; plan.md; tasks.md</t>
-  </si>
-  <si>
-    <t>External client lists account transactions</t>
-  </si>
-  <si>
-    <t>Declare paged transaction history without claiming a working backend mapping.</t>
-  </si>
-  <si>
-    <t>OpenAPI and the JS client publish the route, but no z/OS operation mapping exists.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:518-579; js/api.js:260-279; operations/...transactions/get (no operation.yaml); Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
-  </si>
-  <si>
-    <t>Decision D-008: provide supported unified history resources, not missing legacy mappings.</t>
-  </si>
-  <si>
-    <t>External client retrieves one transaction</t>
-  </si>
-  <si>
-    <t>Declare transaction detail without claiming a working backend mapping.</t>
-  </si>
-  <si>
-    <t>The route is published but has no operation mapping.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:580-615; js/api.js:286-292; operations/...transactionId/get (no operation.yaml); Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Java history service reads recent activity</t>
-  </si>
-  <si>
-    <t>Return the latest 50 history rows for an account in reverse chronological order.</t>
-  </si>
-  <si>
-    <t>The Java/DB2 integration provides bounded recent transaction history.</t>
-  </si>
-  <si>
-    <t>At most 50 records are returned, newest first.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:45-47; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decision D-008: target history resources preserve supported behavior without reproducing legacy route defects.</t>
-  </si>
-  <si>
-    <t>API client receives standard failures</t>
-  </si>
-  <si>
-    <t>Represent validation, authentication, authorization, not-found, and server failures.</t>
-  </si>
-  <si>
-    <t>External consumers need stable error classes.</t>
-  </si>
-  <si>
-    <t>The contract declares standard failures, but five bound and three unbound response selections reference missing generated YAML artifacts.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml response sections and Error schema; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Deviation D-008: target Problem Details replace missing generated response files.</t>
-  </si>
-  <si>
-    <t>Generated API mappings select missing response files</t>
-  </si>
-  <si>
-    <t>Record generated response selections whose referenced sibling YAML artifacts are absent.</t>
-  </si>
-  <si>
-    <t>Five missing files affect bound CICS account/customer operations; three more occur in already-unbound account/transaction routes.</t>
-  </si>
-  <si>
-    <t>Those selected error/fallback responses are not deployable from the supplied artifacts and must not be treated as complete API behavior.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Fbalances/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_mapping.yaml:7; legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D/put/response_mapping.yaml:8-10; legacy/src/api/src/main/operations/%2Faccounts/get/response_mapping.yaml:3; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Ftransactions/get/response_mapping.yaml:3; legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D%2Ftransactions%2F%7BtransactionId%7D/get/response_mapping.yaml:3; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>External client creates a CICS customer</t>
-  </si>
-  <si>
-    <t>Expose CICS customer creation through POST /customers and the CRECUST z/OS asset.</t>
-  </si>
-  <si>
-    <t>REST clients can onboard a customer without using the web form or 3270 screen.</t>
-  </si>
-  <si>
-    <t>A successful response returns the created customer identity; mapped failures use the declared API responses.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:246-274; legacy/src/api/src/main/operations/%2Fcustomers/post/operation.yaml; legacy/src/api/src/main/zosAssets/CRECUST/zosAsset.yaml; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.api-contract; harness: simulation/test; basis: legacy/src/api/src/main/api/openapi.yaml; legacy/src/frontend/js/api.js</t>
-  </si>
-  <si>
-    <t>D-008 implemented: POST /api/customers provides supported onboarding with stable success and failure contracts.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Api/Controllers/CustomersController.cs; modern/backend/src/BankOfZ.Api/Contracts/CreateCustomerRequest.cs; CustomerApiTests.cs</t>
-  </si>
-  <si>
-    <t>IMS client requests recent history through IBGHIST</t>
-  </si>
-  <si>
-    <t>Accept an IMS IBGHIST message containing an account number and return at most 50 recent DB2 history records.</t>
-  </si>
-  <si>
-    <t>IBGHIST is a separately deployed Java message-processing transaction, not only an internal repository service.</t>
-  </si>
-  <si>
-    <t>Success returns count/details; controller exceptions may populate MSG-OUT, while JDBC/DB2 failures can be swallowed as null without a response.</t>
-  </si>
-  <si>
-    <t>legacy/.setup/deploy/ims_spoc.jcl.j2:84-86,95,108-109; legacy/src/base/ims/java/src/main/java/nazare/jmp/controller/QueryTransaction.java:28-131; legacy/src/base/ims/java/src/main/java/nazare/jmp/history/TransactionService.java:45-47; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>UF-009</t>
-  </si>
-  <si>
-    <t>Monthly statements and reporting</t>
-  </si>
-  <si>
     <t>Operator runs the monthly statement job</t>
   </si>
   <si>
@@ -2835,7 +2853,7 @@
     <t>Implement Feature 005 funds transfers.</t>
   </si>
   <si>
-    <t>Not checked: target implementation has not started. specs/005-funds-transfers/</t>
+    <t>Feature 005 delivered and browser-accepted. specs/005-funds-transfers/; analysis/reviews/feature-005-implementation-review.md; analysis/stage-08-feature-005-delivery.md; analysis/stage-09-feature-005-live-revision.md; deployed /z-bank-new/</t>
   </si>
   <si>
     <t>R1-G06</t>
@@ -2850,7 +2868,7 @@
     <t>Implement Feature 006 supported transaction history.</t>
   </si>
   <si>
-    <t>Not checked: target implementation has not started. specs/006-transaction-history/</t>
+    <t>Feature 006 implemented and peer-reviewed. specs/006-transaction-history/; analysis/reviews/feature-006-implementation-review.md; modern/backend/src/BankOfZ.Api/Controllers/TransactionHistoryController.cs; modern/frontend/bank-of-z-ui/src/app/accounts/transaction-history.component.ts; TransactionHistoryApiTests.cs; secure-access.spec.ts</t>
   </si>
   <si>
     <t>R1-G07</t>
@@ -7214,60 +7232,60 @@
       </c>
     </row>
     <row r="86" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A86" s="21" t="s">
+      <c r="A86" s="17" t="s">
         <v>533</v>
       </c>
-      <c r="B86" s="21" t="s">
+      <c r="B86" s="17" t="s">
         <v>534</v>
       </c>
-      <c r="C86" s="21" t="s">
-        <v>535</v>
-      </c>
-      <c r="D86" s="21" t="s">
-        <v>536</v>
-      </c>
-      <c r="E86" s="21"/>
-      <c r="F86" s="21"/>
-      <c r="G86" s="21"/>
-      <c r="H86" s="21"/>
-      <c r="I86" s="21"/>
-      <c r="J86" s="21"/>
-      <c r="K86" s="21"/>
-      <c r="L86" s="21"/>
-      <c r="M86" s="21"/>
-      <c r="N86" s="21"/>
+      <c r="C86" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D86" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E86" s="17"/>
+      <c r="F86" s="17"/>
+      <c r="G86" s="17"/>
+      <c r="H86" s="17"/>
+      <c r="I86" s="17"/>
+      <c r="J86" s="17"/>
+      <c r="K86" s="17"/>
+      <c r="L86" s="17"/>
+      <c r="M86" s="17"/>
+      <c r="N86" s="17"/>
     </row>
     <row r="87" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A87" s="18"/>
       <c r="B87" s="19" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C87" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D87" s="20" t="s">
+        <v>536</v>
+      </c>
+      <c r="E87" s="20" t="s">
+        <v>537</v>
+      </c>
+      <c r="F87" s="20" t="s">
         <v>538</v>
-      </c>
-      <c r="E87" s="20" t="s">
-        <v>539</v>
-      </c>
-      <c r="F87" s="20" t="s">
-        <v>540</v>
       </c>
       <c r="G87" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H87" s="20" t="s">
+        <v>539</v>
+      </c>
+      <c r="I87" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J87" s="20" t="s">
+        <v>540</v>
+      </c>
+      <c r="K87" s="20" t="s">
         <v>541</v>
-      </c>
-      <c r="I87" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="J87" s="20" t="s">
-        <v>542</v>
-      </c>
-      <c r="K87" s="20" t="s">
-        <v>543</v>
       </c>
       <c r="L87" s="20" t="s">
         <v>36</v>
@@ -7282,34 +7300,34 @@
     <row r="88" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A88" s="18"/>
       <c r="B88" s="19" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C88" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D88" s="20" t="s">
+        <v>543</v>
+      </c>
+      <c r="E88" s="20" t="s">
+        <v>544</v>
+      </c>
+      <c r="F88" s="20" t="s">
         <v>545</v>
-      </c>
-      <c r="E88" s="20" t="s">
-        <v>546</v>
-      </c>
-      <c r="F88" s="20" t="s">
-        <v>547</v>
       </c>
       <c r="G88" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H88" s="20" t="s">
+        <v>546</v>
+      </c>
+      <c r="I88" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J88" s="20" t="s">
+        <v>547</v>
+      </c>
+      <c r="K88" s="20" t="s">
         <v>548</v>
-      </c>
-      <c r="I88" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="J88" s="20" t="s">
-        <v>549</v>
-      </c>
-      <c r="K88" s="20" t="s">
-        <v>550</v>
       </c>
       <c r="L88" s="20" t="s">
         <v>36</v>
@@ -7324,31 +7342,31 @@
     <row r="89" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A89" s="18"/>
       <c r="B89" s="19" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C89" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D89" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="E89" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="F89" s="20" t="s">
         <v>552</v>
       </c>
-      <c r="E89" s="20" t="s">
+      <c r="G89" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H89" s="20" t="s">
         <v>553</v>
       </c>
-      <c r="F89" s="20" t="s">
+      <c r="I89" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J89" s="20" t="s">
         <v>554</v>
-      </c>
-      <c r="G89" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H89" s="20" t="s">
-        <v>555</v>
-      </c>
-      <c r="I89" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="J89" s="20" t="s">
-        <v>556</v>
       </c>
       <c r="K89" s="20" t="s">
         <v>377</v>
@@ -7366,31 +7384,31 @@
     <row r="90" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A90" s="18"/>
       <c r="B90" s="19" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C90" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D90" s="20" t="s">
+        <v>556</v>
+      </c>
+      <c r="E90" s="20" t="s">
+        <v>557</v>
+      </c>
+      <c r="F90" s="20" t="s">
         <v>558</v>
       </c>
-      <c r="E90" s="20" t="s">
+      <c r="G90" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H90" s="20" t="s">
         <v>559</v>
       </c>
-      <c r="F90" s="20" t="s">
+      <c r="I90" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J90" s="20" t="s">
         <v>560</v>
-      </c>
-      <c r="G90" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="H90" s="20" t="s">
-        <v>561</v>
-      </c>
-      <c r="I90" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="J90" s="20" t="s">
-        <v>562</v>
       </c>
       <c r="K90" s="20" t="s">
         <v>153</v>
@@ -7408,77 +7426,85 @@
     <row r="91" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A91" s="18"/>
       <c r="B91" s="19" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="C91" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D91" s="22" t="s">
+      <c r="D91" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="E91" s="20" t="s">
+        <v>563</v>
+      </c>
+      <c r="F91" s="20" t="s">
         <v>564</v>
       </c>
-      <c r="E91" s="22" t="s">
+      <c r="G91" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="H91" s="20" t="s">
         <v>565</v>
       </c>
-      <c r="F91" s="22" t="s">
+      <c r="I91" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J91" s="20" t="s">
         <v>566</v>
       </c>
-      <c r="G91" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="H91" s="22" t="s">
+      <c r="K91" s="20" t="s">
         <v>567</v>
       </c>
-      <c r="I91" s="22"/>
-      <c r="J91" s="22" t="s">
+      <c r="L91" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M91" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N91" s="20" t="s">
         <v>568</v>
-      </c>
-      <c r="K91" s="22"/>
-      <c r="L91" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M91" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N91" s="22" t="s">
-        <v>569</v>
       </c>
     </row>
     <row r="92" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A92" s="18"/>
       <c r="B92" s="19" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C92" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D92" s="22" t="s">
+      <c r="D92" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="E92" s="20" t="s">
         <v>571</v>
       </c>
-      <c r="E92" s="22" t="s">
+      <c r="F92" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="G92" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="H92" s="20" t="s">
         <v>572</v>
       </c>
-      <c r="F92" s="22" t="s">
-        <v>566</v>
-      </c>
-      <c r="G92" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="H92" s="22" t="s">
+      <c r="I92" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J92" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="I92" s="22"/>
-      <c r="J92" s="22" t="s">
+      <c r="K92" s="20" t="s">
         <v>574</v>
       </c>
-      <c r="K92" s="22"/>
-      <c r="L92" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M92" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N92" s="22" t="s">
-        <v>569</v>
+      <c r="L92" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M92" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N92" s="20" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="93" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
@@ -7489,181 +7515,197 @@
       <c r="C93" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D93" s="22" t="s">
+      <c r="D93" s="20" t="s">
         <v>576</v>
       </c>
-      <c r="E93" s="22" t="s">
+      <c r="E93" s="20" t="s">
         <v>577</v>
       </c>
-      <c r="F93" s="22" t="s">
-        <v>566</v>
-      </c>
-      <c r="G93" s="22" t="s">
+      <c r="F93" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="G93" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H93" s="22" t="s">
+      <c r="H93" s="20" t="s">
         <v>578</v>
       </c>
-      <c r="I93" s="22"/>
-      <c r="J93" s="22" t="s">
-        <v>574</v>
-      </c>
-      <c r="K93" s="22"/>
-      <c r="L93" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M93" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N93" s="22" t="s">
-        <v>569</v>
+      <c r="I93" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J93" s="20" t="s">
+        <v>573</v>
+      </c>
+      <c r="K93" s="20" t="s">
+        <v>579</v>
+      </c>
+      <c r="L93" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M93" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N93" s="20" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="94" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A94" s="18"/>
       <c r="B94" s="19" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C94" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D94" s="22" t="s">
-        <v>580</v>
-      </c>
-      <c r="E94" s="22" t="s">
+      <c r="D94" s="20" t="s">
         <v>581</v>
       </c>
-      <c r="F94" s="22" t="s">
+      <c r="E94" s="20" t="s">
         <v>582</v>
       </c>
-      <c r="G94" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H94" s="22" t="s">
+      <c r="F94" s="20" t="s">
         <v>583</v>
       </c>
-      <c r="I94" s="22"/>
-      <c r="J94" s="22" t="s">
+      <c r="G94" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H94" s="20" t="s">
         <v>584</v>
       </c>
-      <c r="K94" s="22"/>
-      <c r="L94" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M94" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N94" s="22" t="s">
-        <v>569</v>
+      <c r="I94" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J94" s="20" t="s">
+        <v>585</v>
+      </c>
+      <c r="K94" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="L94" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M94" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N94" s="20" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="95" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A95" s="18"/>
       <c r="B95" s="19" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="C95" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D95" s="22" t="s">
-        <v>586</v>
-      </c>
-      <c r="E95" s="22" t="s">
-        <v>587</v>
-      </c>
-      <c r="F95" s="22" t="s">
+      <c r="D95" s="20" t="s">
         <v>588</v>
       </c>
-      <c r="G95" s="22" t="s">
+      <c r="E95" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="F95" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="G95" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H95" s="22" t="s">
-        <v>589</v>
-      </c>
-      <c r="I95" s="22"/>
-      <c r="J95" s="22" t="s">
-        <v>590</v>
-      </c>
-      <c r="K95" s="22"/>
-      <c r="L95" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M95" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N95" s="22" t="s">
-        <v>569</v>
+      <c r="H95" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="I95" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J95" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="K95" s="20" t="s">
+        <v>593</v>
+      </c>
+      <c r="L95" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M95" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N95" s="20" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="96" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A96" s="18"/>
       <c r="B96" s="19" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D96" s="22" t="s">
+      <c r="D96" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="E96" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="F96" s="20" t="s">
+        <v>597</v>
+      </c>
+      <c r="G96" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="H96" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="I96" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J96" s="20" t="s">
         <v>592</v>
       </c>
-      <c r="E96" s="22" t="s">
+      <c r="K96" s="20" t="s">
         <v>593</v>
       </c>
-      <c r="F96" s="22" t="s">
-        <v>594</v>
-      </c>
-      <c r="G96" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="H96" s="22" t="s">
-        <v>595</v>
-      </c>
-      <c r="I96" s="22"/>
-      <c r="J96" s="22" t="s">
-        <v>590</v>
-      </c>
-      <c r="K96" s="22"/>
-      <c r="L96" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M96" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N96" s="22" t="s">
-        <v>569</v>
+      <c r="L96" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M96" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N96" s="20" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="97" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A97" s="18"/>
       <c r="B97" s="19" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="C97" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D97" s="20" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="E97" s="20" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="F97" s="20" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="G97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H97" s="20" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="I97" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J97" s="20" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="K97" s="20" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="L97" s="20" t="s">
         <v>36</v>
@@ -7678,53 +7720,57 @@
     <row r="98" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A98" s="18"/>
       <c r="B98" s="19" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="C98" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D98" s="22" t="s">
-        <v>604</v>
-      </c>
-      <c r="E98" s="22" t="s">
-        <v>605</v>
-      </c>
-      <c r="F98" s="22" t="s">
-        <v>606</v>
-      </c>
-      <c r="G98" s="22" t="s">
+      <c r="D98" s="20" t="s">
+        <v>607</v>
+      </c>
+      <c r="E98" s="20" t="s">
+        <v>608</v>
+      </c>
+      <c r="F98" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="G98" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H98" s="22" t="s">
-        <v>607</v>
-      </c>
-      <c r="I98" s="22"/>
-      <c r="J98" s="22" t="s">
-        <v>584</v>
-      </c>
-      <c r="K98" s="22"/>
-      <c r="L98" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M98" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N98" s="22" t="s">
-        <v>569</v>
+      <c r="H98" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="I98" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J98" s="20" t="s">
+        <v>585</v>
+      </c>
+      <c r="K98" s="20" t="s">
+        <v>611</v>
+      </c>
+      <c r="L98" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M98" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N98" s="20" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="99" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="21" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="B99" s="21" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="C99" s="21" t="s">
-        <v>535</v>
+        <v>614</v>
       </c>
       <c r="D99" s="21" t="s">
-        <v>536</v>
+        <v>615</v>
       </c>
       <c r="E99" s="21"/>
       <c r="F99" s="21"/>
@@ -7740,29 +7786,29 @@
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="18"/>
       <c r="B100" s="19" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="C100" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D100" s="22" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="E100" s="22" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="F100" s="22" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="G100" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H100" s="22" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="I100" s="22"/>
       <c r="J100" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K100" s="22"/>
       <c r="L100" s="22" t="s">
@@ -7772,35 +7818,35 @@
         <v>40</v>
       </c>
       <c r="N100" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="18"/>
       <c r="B101" s="19" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="C101" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D101" s="22" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="E101" s="22" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="F101" s="22" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="G101" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H101" s="22" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="I101" s="22"/>
       <c r="J101" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K101" s="22"/>
       <c r="L101" s="22" t="s">
@@ -7810,35 +7856,35 @@
         <v>40</v>
       </c>
       <c r="N101" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D102" s="22" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="E102" s="22" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="F102" s="22" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="G102" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H102" s="22" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="I102" s="22"/>
       <c r="J102" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K102" s="22"/>
       <c r="L102" s="22" t="s">
@@ -7848,35 +7894,35 @@
         <v>40</v>
       </c>
       <c r="N102" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="C103" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D103" s="22" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="E103" s="22" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F103" s="22" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="G103" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H103" s="22" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="I103" s="22"/>
       <c r="J103" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K103" s="22"/>
       <c r="L103" s="22" t="s">
@@ -7886,35 +7932,35 @@
         <v>40</v>
       </c>
       <c r="N103" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D104" s="22" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="E104" s="22" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="F104" s="22" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="G104" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H104" s="22" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="I104" s="22"/>
       <c r="J104" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K104" s="22"/>
       <c r="L104" s="22" t="s">
@@ -7924,35 +7970,35 @@
         <v>40</v>
       </c>
       <c r="N104" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="18"/>
       <c r="B105" s="19" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="C105" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D105" s="22" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="E105" s="22" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="F105" s="22" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="G105" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H105" s="22" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="I105" s="22"/>
       <c r="J105" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K105" s="22"/>
       <c r="L105" s="22" t="s">
@@ -7962,35 +8008,35 @@
         <v>40</v>
       </c>
       <c r="N105" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="C106" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D106" s="22" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="E106" s="22" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="F106" s="22" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="G106" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H106" s="22" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="I106" s="22"/>
       <c r="J106" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K106" s="22"/>
       <c r="L106" s="22" t="s">
@@ -8000,35 +8046,35 @@
         <v>40</v>
       </c>
       <c r="N106" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="C107" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D107" s="22" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="E107" s="22" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="F107" s="22" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G107" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H107" s="22" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="I107" s="22"/>
       <c r="J107" s="22" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="K107" s="22"/>
       <c r="L107" s="22" t="s">
@@ -8038,15 +8084,15 @@
         <v>40</v>
       </c>
       <c r="N107" s="22" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="108" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="B108" s="17" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="C108" s="17" t="s">
         <v>29</v>
@@ -8068,34 +8114,34 @@
     <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="C109" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="E109" s="20" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="F109" s="20" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="I109" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J109" s="20" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="K109" s="20" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="L109" s="20" t="s">
         <v>36</v>
@@ -8110,34 +8156,34 @@
     <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="C110" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="F110" s="20" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="G110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="I110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J110" s="20" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="K110" s="20" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="L110" s="20" t="s">
         <v>36</v>
@@ -8152,34 +8198,34 @@
     <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="C111" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D111" s="20" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="E111" s="20" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="F111" s="20" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="G111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="I111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J111" s="20" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="K111" s="20" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="L111" s="20" t="s">
         <v>36</v>
@@ -8194,34 +8240,34 @@
     <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="C112" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="F112" s="20" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="G112" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="I112" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J112" s="20" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="K112" s="20" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="L112" s="20" t="s">
         <v>36</v>
@@ -8236,34 +8282,34 @@
     <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="C113" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="I113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J113" s="20" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="K113" s="20" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="L113" s="20" t="s">
         <v>36</v>
@@ -8278,34 +8324,34 @@
     <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="C114" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D114" s="20" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="E114" s="20" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="F114" s="20" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="G114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="20" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="I114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J114" s="20" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="K114" s="20" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="L114" s="20" t="s">
         <v>36</v>
@@ -8320,31 +8366,31 @@
     <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="C115" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D115" s="20" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="F115" s="20" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="G115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="20" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="I115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J115" s="20" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="K115" s="20" t="s">
         <v>56</v>
@@ -8362,34 +8408,34 @@
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="18"/>
       <c r="B116" s="19" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="C116" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D116" s="20" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="E116" s="20" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="F116" s="20" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="G116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H116" s="20" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="I116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J116" s="20" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="K116" s="20" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="L116" s="20" t="s">
         <v>36</v>
@@ -8404,34 +8450,34 @@
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
       <c r="B117" s="19" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="C117" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="E117" s="20" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="G117" s="20" t="s">
         <v>522</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="I117" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J117" s="20" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="K117" s="20" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="L117" s="20" t="s">
         <v>36</v>
@@ -8445,16 +8491,16 @@
     </row>
     <row r="118" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="21" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="B118" s="21" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="C118" s="21" t="s">
-        <v>535</v>
+        <v>614</v>
       </c>
       <c r="D118" s="21" t="s">
-        <v>536</v>
+        <v>615</v>
       </c>
       <c r="E118" s="21"/>
       <c r="F118" s="21"/>
@@ -8470,29 +8516,29 @@
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="19" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D119" s="22" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="E119" s="22" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="F119" s="22" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="G119" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="22" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="I119" s="22"/>
       <c r="J119" s="22" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="K119" s="22"/>
       <c r="L119" s="22" t="s">
@@ -8502,35 +8548,35 @@
         <v>40</v>
       </c>
       <c r="N119" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="19" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D120" s="22" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="E120" s="22" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="F120" s="22" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="G120" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="22" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="I120" s="22"/>
       <c r="J120" s="22" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="K120" s="22"/>
       <c r="L120" s="22" t="s">
@@ -8540,35 +8586,35 @@
         <v>40</v>
       </c>
       <c r="N120" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
       <c r="B121" s="19" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="C121" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D121" s="22" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="E121" s="22" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="F121" s="22" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="G121" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="22" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="I121" s="22"/>
       <c r="J121" s="22" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="K121" s="22"/>
       <c r="L121" s="22" t="s">
@@ -8578,35 +8624,35 @@
         <v>40</v>
       </c>
       <c r="N121" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="19" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D122" s="22" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="E122" s="22" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="F122" s="22" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="G122" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="22" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="I122" s="22"/>
       <c r="J122" s="22" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="K122" s="22"/>
       <c r="L122" s="22" t="s">
@@ -8616,35 +8662,35 @@
         <v>40</v>
       </c>
       <c r="N122" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="19" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D123" s="22" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="E123" s="22" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
       <c r="F123" s="22" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="G123" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H123" s="22" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="I123" s="22"/>
       <c r="J123" s="22" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="K123" s="22"/>
       <c r="L123" s="22" t="s">
@@ -8654,35 +8700,35 @@
         <v>40</v>
       </c>
       <c r="N123" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="19" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D124" s="22" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="E124" s="22" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="F124" s="22" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="G124" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H124" s="22" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="I124" s="22"/>
       <c r="J124" s="22" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="K124" s="22"/>
       <c r="L124" s="22" t="s">
@@ -8692,35 +8738,35 @@
         <v>40</v>
       </c>
       <c r="N124" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="19" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D125" s="22" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="E125" s="22" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="F125" s="22" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="G125" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H125" s="22" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="I125" s="22"/>
       <c r="J125" s="22" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="K125" s="22"/>
       <c r="L125" s="22" t="s">
@@ -8730,35 +8776,35 @@
         <v>40</v>
       </c>
       <c r="N125" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="19" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D126" s="22" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="E126" s="22" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="F126" s="22" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="G126" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="22" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="I126" s="22"/>
       <c r="J126" s="22" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="K126" s="22"/>
       <c r="L126" s="22" t="s">
@@ -8768,21 +8814,21 @@
         <v>40</v>
       </c>
       <c r="N126" s="22" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="21" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="B127" s="21" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="C127" s="21" t="s">
-        <v>535</v>
+        <v>614</v>
       </c>
       <c r="D127" s="21" t="s">
-        <v>536</v>
+        <v>615</v>
       </c>
       <c r="E127" s="21"/>
       <c r="F127" s="21"/>
@@ -8798,29 +8844,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D128" s="22" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="E128" s="22" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="F128" s="22" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="G128" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="22" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="I128" s="22"/>
       <c r="J128" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K128" s="22"/>
       <c r="L128" s="22" t="s">
@@ -8830,35 +8876,35 @@
         <v>40</v>
       </c>
       <c r="N128" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D129" s="22" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="E129" s="22" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="F129" s="22" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="G129" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="22" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="I129" s="22"/>
       <c r="J129" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K129" s="22"/>
       <c r="L129" s="22" t="s">
@@ -8868,35 +8914,35 @@
         <v>40</v>
       </c>
       <c r="N129" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="18"/>
       <c r="B130" s="19" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D130" s="22" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="E130" s="22" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
       <c r="F130" s="22" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="G130" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="22" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="I130" s="22"/>
       <c r="J130" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K130" s="22"/>
       <c r="L130" s="22" t="s">
@@ -8906,35 +8952,35 @@
         <v>40</v>
       </c>
       <c r="N130" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D131" s="22" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="E131" s="22" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="F131" s="22" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="G131" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H131" s="22" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="I131" s="22"/>
       <c r="J131" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K131" s="22"/>
       <c r="L131" s="22" t="s">
@@ -8944,35 +8990,35 @@
         <v>40</v>
       </c>
       <c r="N131" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D132" s="22" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="E132" s="22" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="F132" s="22" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="G132" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="22" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="I132" s="22"/>
       <c r="J132" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K132" s="22"/>
       <c r="L132" s="22" t="s">
@@ -8982,35 +9028,35 @@
         <v>40</v>
       </c>
       <c r="N132" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D133" s="22" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="E133" s="22" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
       <c r="F133" s="22" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="G133" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H133" s="22" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="I133" s="22"/>
       <c r="J133" s="22" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="K133" s="22"/>
       <c r="L133" s="22" t="s">
@@ -9020,35 +9066,35 @@
         <v>40</v>
       </c>
       <c r="N133" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D134" s="22" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="E134" s="22" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
       <c r="F134" s="22" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
       <c r="G134" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="22" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="I134" s="22"/>
       <c r="J134" s="22" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
       <c r="K134" s="22"/>
       <c r="L134" s="22" t="s">
@@ -9058,35 +9104,35 @@
         <v>40</v>
       </c>
       <c r="N134" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D135" s="22" t="s">
-        <v>806</v>
+        <v>812</v>
       </c>
       <c r="E135" s="22" t="s">
-        <v>807</v>
+        <v>813</v>
       </c>
       <c r="F135" s="22" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="G135" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H135" s="22" t="s">
-        <v>809</v>
+        <v>815</v>
       </c>
       <c r="I135" s="22"/>
       <c r="J135" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K135" s="22"/>
       <c r="L135" s="22" t="s">
@@ -9096,35 +9142,35 @@
         <v>40</v>
       </c>
       <c r="N135" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D136" s="22" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="E136" s="22" t="s">
-        <v>812</v>
+        <v>818</v>
       </c>
       <c r="F136" s="22" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
       <c r="G136" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H136" s="22" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
       <c r="I136" s="22"/>
       <c r="J136" s="22" t="s">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="K136" s="22"/>
       <c r="L136" s="22" t="s">
@@ -9134,35 +9180,35 @@
         <v>40</v>
       </c>
       <c r="N136" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D137" s="22" t="s">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="E137" s="22" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
       <c r="F137" s="22" t="s">
-        <v>819</v>
+        <v>825</v>
       </c>
       <c r="G137" s="22" t="s">
         <v>522</v>
       </c>
       <c r="H137" s="22" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
       <c r="I137" s="22"/>
       <c r="J137" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K137" s="22"/>
       <c r="L137" s="22" t="s">
@@ -9172,35 +9218,35 @@
         <v>40</v>
       </c>
       <c r="N137" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D138" s="22" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
       <c r="E138" s="22" t="s">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="F138" s="22" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
       <c r="G138" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="22" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="I138" s="22"/>
       <c r="J138" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K138" s="22"/>
       <c r="L138" s="22" t="s">
@@ -9210,35 +9256,35 @@
         <v>40</v>
       </c>
       <c r="N138" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D139" s="22" t="s">
-        <v>827</v>
+        <v>833</v>
       </c>
       <c r="E139" s="22" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="F139" s="22" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
       <c r="G139" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="22" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
       <c r="I139" s="22"/>
       <c r="J139" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K139" s="22"/>
       <c r="L139" s="22" t="s">
@@ -9248,35 +9294,35 @@
         <v>40</v>
       </c>
       <c r="N139" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D140" s="22" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
       <c r="E140" s="22" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="F140" s="22" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
       <c r="G140" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="22" t="s">
-        <v>835</v>
+        <v>841</v>
       </c>
       <c r="I140" s="22"/>
       <c r="J140" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K140" s="22"/>
       <c r="L140" s="22" t="s">
@@ -9286,35 +9332,35 @@
         <v>40</v>
       </c>
       <c r="N140" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D141" s="22" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="E141" s="22" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="F141" s="22" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="G141" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="22" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="I141" s="22"/>
       <c r="J141" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K141" s="22"/>
       <c r="L141" s="22" t="s">
@@ -9324,35 +9370,35 @@
         <v>40</v>
       </c>
       <c r="N141" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D142" s="22" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
       <c r="E142" s="22" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
       <c r="F142" s="22" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="G142" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="22" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="I142" s="22"/>
       <c r="J142" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K142" s="22"/>
       <c r="L142" s="22" t="s">
@@ -9362,35 +9408,35 @@
         <v>40</v>
       </c>
       <c r="N142" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D143" s="22" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="E143" s="22" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="F143" s="22" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="G143" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="22" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="I143" s="22"/>
       <c r="J143" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K143" s="22"/>
       <c r="L143" s="22" t="s">
@@ -9400,35 +9446,35 @@
         <v>40</v>
       </c>
       <c r="N143" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D144" s="22" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="E144" s="22" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="F144" s="22" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="G144" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H144" s="22" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="I144" s="22"/>
       <c r="J144" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K144" s="22"/>
       <c r="L144" s="22" t="s">
@@ -9438,35 +9484,35 @@
         <v>40</v>
       </c>
       <c r="N144" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D145" s="22" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="E145" s="22" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="F145" s="22" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="G145" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="22" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="I145" s="22"/>
       <c r="J145" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K145" s="22"/>
       <c r="L145" s="22" t="s">
@@ -9476,35 +9522,35 @@
         <v>40</v>
       </c>
       <c r="N145" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D146" s="22" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="E146" s="22" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="F146" s="22" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="G146" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="22" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="I146" s="22"/>
       <c r="J146" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K146" s="22"/>
       <c r="L146" s="22" t="s">
@@ -9514,35 +9560,35 @@
         <v>40</v>
       </c>
       <c r="N146" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D147" s="22" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
       <c r="E147" s="22" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="F147" s="22" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="G147" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="22" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="I147" s="22"/>
       <c r="J147" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K147" s="22"/>
       <c r="L147" s="22" t="s">
@@ -9552,35 +9598,35 @@
         <v>40</v>
       </c>
       <c r="N147" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D148" s="22" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="E148" s="22" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="F148" s="22" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="G148" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="22" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="I148" s="22"/>
       <c r="J148" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K148" s="22"/>
       <c r="L148" s="22" t="s">
@@ -9590,35 +9636,35 @@
         <v>40</v>
       </c>
       <c r="N148" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D149" s="22" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="E149" s="22" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="F149" s="22" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="G149" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="22" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="I149" s="22"/>
       <c r="J149" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K149" s="22"/>
       <c r="L149" s="22" t="s">
@@ -9628,35 +9674,35 @@
         <v>40</v>
       </c>
       <c r="N149" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D150" s="22" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
       <c r="E150" s="22" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="F150" s="22" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="G150" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H150" s="22" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
       <c r="I150" s="22"/>
       <c r="J150" s="22" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="K150" s="22"/>
       <c r="L150" s="22" t="s">
@@ -9666,35 +9712,35 @@
         <v>40</v>
       </c>
       <c r="N150" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D151" s="22" t="s">
-        <v>888</v>
+        <v>894</v>
       </c>
       <c r="E151" s="22" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="F151" s="22" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="G151" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H151" s="22" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="I151" s="22"/>
       <c r="J151" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K151" s="22"/>
       <c r="L151" s="22" t="s">
@@ -9704,35 +9750,35 @@
         <v>40</v>
       </c>
       <c r="N151" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D152" s="22" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
       <c r="E152" s="22" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="F152" s="22" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="G152" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H152" s="22" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
       <c r="I152" s="22"/>
       <c r="J152" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K152" s="22"/>
       <c r="L152" s="22" t="s">
@@ -9742,35 +9788,35 @@
         <v>40</v>
       </c>
       <c r="N152" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>897</v>
+        <v>903</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D153" s="22" t="s">
-        <v>898</v>
+        <v>904</v>
       </c>
       <c r="E153" s="22" t="s">
-        <v>899</v>
+        <v>905</v>
       </c>
       <c r="F153" s="22" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="G153" s="22" t="s">
         <v>522</v>
       </c>
       <c r="H153" s="22" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="I153" s="22"/>
       <c r="J153" s="22" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="K153" s="22"/>
       <c r="L153" s="22" t="s">
@@ -9780,7 +9826,7 @@
         <v>40</v>
       </c>
       <c r="N153" s="22" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
   </sheetData>
@@ -9813,51 +9859,51 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>902</v>
+        <v>908</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="G1" s="24" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="24" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>909</v>
+        <v>915</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>911</v>
+        <v>917</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>912</v>
+        <v>918</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>914</v>
+        <v>920</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
       <c r="G2" s="27" t="s">
         <v>36</v>
@@ -9866,27 +9912,27 @@
         <v>36</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
-        <v>917</v>
+        <v>923</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="C3" s="30" t="s">
+        <v>925</v>
+      </c>
+      <c r="D3" s="30" t="s">
         <v>919</v>
       </c>
-      <c r="D3" s="30" t="s">
-        <v>913</v>
-      </c>
       <c r="E3" s="30" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="F3" s="30" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
       <c r="G3" s="30" t="s">
         <v>36</v>
@@ -9895,27 +9941,27 @@
         <v>36</v>
       </c>
       <c r="I3" s="31" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="G4" s="30" t="s">
         <v>36</v>
@@ -9924,27 +9970,27 @@
         <v>36</v>
       </c>
       <c r="I4" s="31" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>930</v>
+        <v>936</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>931</v>
+        <v>937</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>932</v>
+        <v>938</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>36</v>
@@ -9953,85 +9999,85 @@
         <v>36</v>
       </c>
       <c r="I5" s="31" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="32" t="s">
-        <v>935</v>
-      </c>
-      <c r="B6" s="33" t="s">
+      <c r="A6" s="29" t="s">
+        <v>941</v>
+      </c>
+      <c r="B6" s="30" t="s">
         <v>487</v>
       </c>
-      <c r="C6" s="33" t="s">
-        <v>936</v>
-      </c>
-      <c r="D6" s="33" t="s">
-        <v>913</v>
-      </c>
-      <c r="E6" s="33" t="s">
-        <v>937</v>
-      </c>
-      <c r="F6" s="33" t="s">
-        <v>938</v>
-      </c>
-      <c r="G6" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="34" t="s">
-        <v>939</v>
+      <c r="C6" s="30" t="s">
+        <v>942</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>919</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>943</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>944</v>
+      </c>
+      <c r="G6" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="31" t="s">
+        <v>945</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
-        <v>940</v>
-      </c>
-      <c r="B7" s="33" t="s">
+      <c r="A7" s="29" t="s">
+        <v>946</v>
+      </c>
+      <c r="B7" s="30" t="s">
         <v>533</v>
       </c>
-      <c r="C7" s="33" t="s">
-        <v>941</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>913</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>942</v>
-      </c>
-      <c r="F7" s="33" t="s">
-        <v>943</v>
-      </c>
-      <c r="G7" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="I7" s="34" t="s">
-        <v>944</v>
+      <c r="C7" s="30" t="s">
+        <v>947</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>919</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>948</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>949</v>
+      </c>
+      <c r="G7" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="31" t="s">
+        <v>950</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="G8" s="33" t="s">
         <v>36</v>
@@ -10040,27 +10086,27 @@
         <v>40</v>
       </c>
       <c r="I8" s="34" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="G9" s="33" t="s">
         <v>36</v>
@@ -10069,27 +10115,27 @@
         <v>40</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="B10" s="36" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="G10" s="36" t="s">
         <v>36</v>
@@ -10098,25 +10144,25 @@
         <v>40</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="B11" s="27"/>
       <c r="C11" s="27" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="G11" s="27" t="s">
         <v>36</v>
@@ -10125,25 +10171,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="30" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>36</v>
@@ -10152,25 +10198,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
       <c r="B13" s="30"/>
       <c r="C13" s="30" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E13" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="G13" s="30" t="s">
         <v>36</v>
@@ -10179,25 +10225,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="30" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="G14" s="30" t="s">
         <v>36</v>
@@ -10206,25 +10252,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="31" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
       <c r="B15" s="30"/>
       <c r="C15" s="30" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E15" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
       <c r="G15" s="30" t="s">
         <v>36</v>
@@ -10233,25 +10279,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="30" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="G16" s="30" t="s">
         <v>36</v>
@@ -10260,25 +10306,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="31" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="29" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="B17" s="30"/>
       <c r="C17" s="30" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>988</v>
+        <v>994</v>
       </c>
       <c r="G17" s="30" t="s">
         <v>36</v>
@@ -10287,25 +10333,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>989</v>
+        <v>995</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>992</v>
+        <v>998</v>
       </c>
       <c r="G18" s="30" t="s">
         <v>36</v>
@@ -10314,25 +10360,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="31" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="29" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="B19" s="30"/>
       <c r="C19" s="30" t="s">
-        <v>995</v>
+        <v>1001</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="G19" s="30" t="s">
         <v>36</v>
@@ -10341,25 +10387,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>997</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
-        <v>998</v>
+        <v>1004</v>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="30" t="s">
-        <v>999</v>
+        <v>1005</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
       <c r="G20" s="30" t="s">
         <v>36</v>
@@ -10368,25 +10414,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="31" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="29" t="s">
-        <v>1002</v>
+        <v>1008</v>
       </c>
       <c r="B21" s="30"/>
       <c r="C21" s="30" t="s">
-        <v>1003</v>
+        <v>1009</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E21" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F21" s="30" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="G21" s="30" t="s">
         <v>36</v>
@@ -10395,25 +10441,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>1005</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
-        <v>1006</v>
+        <v>1012</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>1007</v>
+        <v>1013</v>
       </c>
       <c r="G22" s="30" t="s">
         <v>36</v>
@@ -10422,25 +10468,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="31" t="s">
-        <v>1008</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
-        <v>1009</v>
+        <v>1015</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F23" s="30" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="G23" s="30" t="s">
         <v>36</v>
@@ -10449,25 +10495,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>1011</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
-        <v>1012</v>
+        <v>1018</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30" t="s">
-        <v>1013</v>
+        <v>1019</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>1014</v>
+        <v>1020</v>
       </c>
       <c r="G24" s="30" t="s">
         <v>36</v>
@@ -10476,25 +10522,25 @@
         <v>36</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>1015</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>1016</v>
+        <v>1022</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="39" t="s">
-        <v>1017</v>
+        <v>1023</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>1018</v>
+        <v>1024</v>
       </c>
       <c r="G25" s="39" t="s">
         <v>36</v>
@@ -10503,25 +10549,25 @@
         <v>36</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>1019</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="38" t="s">
-        <v>1020</v>
+        <v>1026</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="39" t="s">
-        <v>1021</v>
+        <v>1027</v>
       </c>
       <c r="D26" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E26" s="39" t="s">
-        <v>1022</v>
+        <v>1028</v>
       </c>
       <c r="F26" s="39" t="s">
-        <v>1023</v>
+        <v>1029</v>
       </c>
       <c r="G26" s="39" t="s">
         <v>36</v>
@@ -10530,25 +10576,25 @@
         <v>36</v>
       </c>
       <c r="I26" s="40" t="s">
-        <v>1024</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="38" t="s">
-        <v>1025</v>
+        <v>1031</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39" t="s">
-        <v>1026</v>
+        <v>1032</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="F27" s="39" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="G27" s="39" t="s">
         <v>36</v>
@@ -10557,25 +10603,25 @@
         <v>36</v>
       </c>
       <c r="I27" s="40" t="s">
-        <v>1029</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>1030</v>
+        <v>1036</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39" t="s">
-        <v>1031</v>
+        <v>1037</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E28" s="39" t="s">
-        <v>1032</v>
+        <v>1038</v>
       </c>
       <c r="F28" s="39" t="s">
-        <v>1033</v>
+        <v>1039</v>
       </c>
       <c r="G28" s="39" t="s">
         <v>36</v>
@@ -10584,25 +10630,25 @@
         <v>36</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>1034</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
-        <v>1035</v>
+        <v>1041</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39" t="s">
-        <v>1036</v>
+        <v>1042</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>1038</v>
+        <v>1044</v>
       </c>
       <c r="G29" s="39" t="s">
         <v>36</v>
@@ -10611,25 +10657,25 @@
         <v>36</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>1039</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="39" t="s">
-        <v>1041</v>
+        <v>1047</v>
       </c>
       <c r="D30" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E30" s="39" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="F30" s="39" t="s">
-        <v>1043</v>
+        <v>1049</v>
       </c>
       <c r="G30" s="39" t="s">
         <v>36</v>
@@ -10638,25 +10684,25 @@
         <v>36</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="38" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="D31" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="F31" s="39" t="s">
-        <v>1047</v>
+        <v>1053</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>36</v>
@@ -10665,25 +10711,25 @@
         <v>36</v>
       </c>
       <c r="I31" s="40" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="38" t="s">
-        <v>1049</v>
+        <v>1055</v>
       </c>
       <c r="B32" s="39"/>
       <c r="C32" s="39" t="s">
-        <v>1050</v>
+        <v>1056</v>
       </c>
       <c r="D32" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E32" s="39" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="F32" s="39" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="G32" s="39" t="s">
         <v>36</v>
@@ -10692,25 +10738,25 @@
         <v>36</v>
       </c>
       <c r="I32" s="40" t="s">
-        <v>1053</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="38" t="s">
-        <v>1054</v>
+        <v>1060</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="D33" s="39" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="G33" s="39" t="s">
         <v>36</v>
@@ -10719,7 +10765,7 @@
         <v>36</v>
       </c>
       <c r="I33" s="40" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add monthly statement generation and UI
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="1065">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2036" uniqueCount="1088">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -1860,336 +1860,402 @@
     <t>Monthly statements and reporting</t>
   </si>
   <si>
+    <t>Operator runs the monthly statement job</t>
+  </si>
+  <si>
+    <t>Generate statements for all accounts of a sort code and reporting month.</t>
+  </si>
+  <si>
+    <t>The JCL supplies YYYYMM and sort code to the PL/I batch program.</t>
+  </si>
+  <si>
+    <t>BNKSTMT processes matching accounts and writes formatted statements to SYSPRINT.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/jcl/BNKSTMT.jcl:1-22; pli/BNKSTMT.pli:18-27,187-205; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Explicit operator bulk generation replaces JCL. The configured bank sort code selects all retained accounts and failed-only retry is supported.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Controllers/StatementsController.cs; modern/backend/src/BankOfZ.Application/Statements/StatementService.cs; modern/backend/tests/BankOfZ.IntegrationTests/StatementApiTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-001, FR-007; plan.md; tasks.md T002-T006</t>
+  </si>
+  <si>
+    <t>Statement parameters are missing</t>
+  </si>
+  <si>
+    <t>Use coded defaults when the date/sort-code input file is unavailable.</t>
+  </si>
+  <si>
+    <t>The batch does not fail solely because a parameter card is absent.</t>
+  </si>
+  <si>
+    <t>Default sort code 123456 and calculated/default statement period are used with diagnostic output.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:210-292; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Approved deviation D-012: the target requires an explicit year/month and derives sort code from configuration; missing or future periods are rejected instead of silently defaulted.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Contracts/GenerateStatementRequest.cs; modern/backend/src/BankOfZ.Application/Statements/StatementOptions.cs; StatementService.cs; StatementApiTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-001, FR-002; plan.md; analysis/stage-04-requirements-revision.md D-012</t>
+  </si>
+  <si>
+    <t>Statement includes customer and account identity</t>
+  </si>
+  <si>
+    <t>Print customer name/address/phone and account number/type/interest/overdraft.</t>
+  </si>
+  <si>
+    <t>The recipient can identify the owner and product.</t>
+  </si>
+  <si>
+    <t>Customer and account information sections are printed.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:430-635; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>The immutable statement snapshot includes customer contact details and account identity, product, currency, interest, and overdraft fields.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Statements/StatementSnapshot.cs; modern/frontend/bank-of-z-ui/src/app/statements/statement.component.html; StatementServiceTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-003, FR-006; plan.md; tasks.md T001, T004, T007</t>
+  </si>
+  <si>
+    <t>Statement lists period transactions</t>
+  </si>
+  <si>
+    <t>Print dated transaction history for the selected statement period.</t>
+  </si>
+  <si>
+    <t>The statement explains balance movement.</t>
+  </si>
+  <si>
+    <t>Each transaction includes date, time, type, reference, description, and amount; balances appear in the statement summary.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:638-779; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Booked period transactions are ordered deterministically and shown with date, reference, description, direction, and amount.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Application/Statements/StatementService.cs; modern/frontend/bank-of-z-ui/src/app/statements/statement.component.html; StatementServiceTests.cs; StatementApiTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-003; Calculation Decisions; tasks.md T001-T003, T007-T008</t>
+  </si>
+  <si>
+    <t>Statement period has no transactions</t>
+  </si>
+  <si>
+    <t>Print an explicit empty-history message.</t>
+  </si>
+  <si>
+    <t>A quiet account still receives an understandable statement.</t>
+  </si>
+  <si>
+    <t>NO TRANSACTIONS FOR THIS PERIOD is printed.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:719-725; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
+  </si>
+  <si>
+    <t>An empty period publishes a valid zero-activity statement with an explicit no-transactions message.</t>
+  </si>
+  <si>
+    <t>modern/frontend/bank-of-z-ui/src/app/statements/statement.component.html; modern/backend/tests/BankOfZ.UnitTests/Statements/StatementServiceTests.cs; modern/backend/tests/BankOfZ.IntegrationTests/StatementApiTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-005; tasks.md T001-T003, T007</t>
+  </si>
+  <si>
+    <t>Statement prints financial summary</t>
+  </si>
+  <si>
+    <t>Calculate and print opening balance, credits, debits, closing/available balance, and transaction count.</t>
+  </si>
+  <si>
+    <t>The recipient can reconcile the period at a glance.</t>
+  </si>
+  <si>
+    <t>A statement summary is printed with all totals.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:782-859; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Opening, credit, debit, closing, available balance, and count are snapshotted and reconciliation failure prevents publication.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Statements/StatementSnapshot.cs; modern/backend/src/BankOfZ.Application/Statements/StatementService.cs; StatementServiceTests.cs; StatementApiTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-004, FR-009; Calculation Decisions; tasks.md T001-T004</t>
+  </si>
+  <si>
+    <t>Statement paginates and closes</t>
+  </si>
+  <si>
+    <t>Repeat headers on page breaks and print an end-of-statement footer.</t>
+  </si>
+  <si>
+    <t>Long histories remain readable as a report.</t>
+  </si>
+  <si>
+    <t>Page headers and the closing footer are produced.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:519-560,862-905; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Approved deviation D-012: responsive HTML and print CSS replace fixed printer pagination while preserving headers and statement closure information.</t>
+  </si>
+  <si>
+    <t>modern/frontend/bank-of-z-ui/src/app/statements/statement.component.html; modern/frontend/bank-of-z-ui/src/app/statements/statement.component.scss; statement.component.spec.ts</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-010; plan.md; analysis/stage-04-requirements-revision.md D-012</t>
+  </si>
+  <si>
+    <t>Statement database operation fails</t>
+  </si>
+  <si>
+    <t>Report cursor, fetch, or customer lookup failures without silently printing trusted totals.</t>
+  </si>
+  <si>
+    <t>Batch failures are visible to the operator through job output.</t>
+  </si>
+  <si>
+    <t>SQLCODE diagnostics/warnings are written to SYSPRINT and processing follows the coded branch.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/batch/pli/BNKSTMT.pli:328-389,475-502,670-704; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Source, reconciliation, and persistence failures publish no partial statement; bulk results isolate the account and durable audit diagnostics support retry.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Application/Statements/StatementService.cs; modern/backend/src/BankOfZ.Infrastructure/Statements/StatementRepository.cs; modern/backend/src/BankOfZ.Api/ErrorHandling/StatementExceptionHandler.cs; StatementApiTests.cs</t>
+  </si>
+  <si>
+    <t>specs/007-monthly-statements/spec.md FR-007, FR-009; Calculation Decisions; tasks.md T002-T006</t>
+  </si>
+  <si>
+    <t>UF-010</t>
+  </si>
+  <si>
+    <t>API security, mapping, and web edge behavior</t>
+  </si>
+  <si>
+    <t>API consumer presents OAuth scopes</t>
+  </si>
+  <si>
+    <t>Declare OAuth2 authorization-code security and account/customer scopes.</t>
+  </si>
+  <si>
+    <t>The OpenAPI contract documents protected banking resources.</t>
+  </si>
+  <si>
+    <t>Consumers see the required scopes and authorization/token endpoints.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/api/openapi.yaml:25,616-635; auth.bankofz.example.com is a placeholder endpoint; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-002: no placeholder OAuth provider or scopes are advertised; the slice uses secure same-origin Identity sessions.</t>
+  </si>
+  <si>
+    <t>specs/001-secure-access-shell/spec.md FR-012; modern/backend/src/BankOfZ.Api/Program.cs</t>
+  </si>
+  <si>
+    <t>CICS single-account API normalizes account type</t>
+  </si>
+  <si>
+    <t>Translate the CICS single-account response into API product categories.</t>
+  </si>
+  <si>
+    <t>Only the single-account CICS mapping applies the documented normalization.</t>
+  </si>
+  <si>
+    <t>ISA maps to SAVINGS, MORTGAGE maps to LOAN, and all other values map to CURRENT.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D/get/response_200.yaml:10-15; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-007 implemented: CICS single-account product codes map through one explicit target AccountType enum.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Accounts/LegacyAccountTypeMapper.cs; modern/backend/tests/BankOfZ.UnitTests/Accounts/AccountTests.cs</t>
+  </si>
+  <si>
+    <t>CICS account-list API passes raw account types</t>
+  </si>
+  <si>
+    <t>Expose the route-specific CICS customer-account list mapping without assuming single-account normalization.</t>
+  </si>
+  <si>
+    <t>The list mapping passes the legacy account type directly to API consumers.</t>
+  </si>
+  <si>
+    <t>Raw CICS account type values are returned by the customer account-list route.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_200.yaml:16-20; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-007 implemented: portfolio responses use the same normalized product enum as account details rather than raw CICS values.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Accounts/LegacyAccountTypeMapper.cs; modern/backend/src/BankOfZ.Api/Controllers/AccountsController.cs; AccountApiTests.cs</t>
+  </si>
+  <si>
+    <t>IMS account API emits schema-invalid CHECKING type</t>
+  </si>
+  <si>
+    <t>Preserve or explicitly correct the route-specific IMS mapping for current/checking accounts.</t>
+  </si>
+  <si>
+    <t>IMS mappings convert type c to CHECKING even though the OpenAPI Account.accountType enum omits CHECKING.</t>
+  </si>
+  <si>
+    <t>The list mapping emits CHECKING; the single-account mapping references $item without a foreach and is not proven valid.</t>
+  </si>
+  <si>
+    <t>legacy/src/api/src/main/operations/%2Fims%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_200.yaml:16-20; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BaccountId%7D/get/response_200.yaml:11-15; legacy/src/api/src/main/api/openapi.yaml; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-007 implemented: IMS checking/current variants normalize to CURRENT, eliminating the schema-invalid CHECKING response.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Domain/Accounts/LegacyAccountTypeMapper.cs; modern/backend/tests/BankOfZ.UnitTests/Accounts/AccountTests.cs; AccountApiTests.cs</t>
+  </si>
+  <si>
+    <t>Web server serves the static UI</t>
+  </si>
+  <si>
+    <t>Serve Bank of Z assets and redirect the root index page to the administration control panel.</t>
+  </si>
+  <si>
+    <t>A browser can open the control-panel application.</t>
+  </si>
+  <si>
+    <t>Static files are returned and index.html redirects the browser to admin.html.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/server.js:14-51; legacy/src/frontend/index.html redirects to admin.html; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-001/D-002/D-014: Angular is served at /z-bank-new/ and the deployed HTTPS page passed browser smoke.</t>
+  </si>
+  <si>
+    <t>modern/frontend/bank-of-z-ui/Dockerfile; nginx.conf; deploy/nginx-z-bank.conf; https://legacy-transformation-demo.olsys.dev/z-bank-new/</t>
+  </si>
+  <si>
+    <t>Web server proxies API traffic</t>
+  </si>
+  <si>
+    <t>Proxy API/customer/account/IMS paths to the configured z/OS Connect base URL.</t>
+  </si>
+  <si>
+    <t>The browser uses one frontend origin for static content and banking calls.</t>
+  </si>
+  <si>
+    <t>Requests and responses are streamed to/from API_BASE_URL.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/server.js proxy paths; config.js base URL; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-001/D-002/D-014: browser API traffic uses the same origin and nginx proxies it to the internal API container.</t>
+  </si>
+  <si>
+    <t>modern/frontend/bank-of-z-ui/nginx.conf; modern/compose.yaml; deployed /z-bank-new/api/session HTTP 200</t>
+  </si>
+  <si>
+    <t>Web static file is missing</t>
+  </si>
+  <si>
+    <t>Return a 404 instead of another page for an unknown static path.</t>
+  </si>
+  <si>
+    <t>Broken links are distinguishable from the application landing page.</t>
+  </si>
+  <si>
+    <t>HTTP 404 is returned.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/server.js missing-file branch; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-001/D-002/D-014: unknown Angular routes render the explicit not-found component rather than the landing page.</t>
+  </si>
+  <si>
+    <t>Web proxy target is unavailable</t>
+  </si>
+  <si>
+    <t>Return a structured gateway failure when z/OS Connect cannot be reached.</t>
+  </si>
+  <si>
+    <t>Frontend availability does not disguise backend unavailability.</t>
+  </si>
+  <si>
+    <t>HTTP 502 with JSON error information is returned.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/server.js proxy error handler; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-001/D-002/D-014: unavailable API calls render a recoverable unavailable view without stack details.</t>
+  </si>
+  <si>
+    <t>modern/frontend/bank-of-z-ui/src/app/core/session.service.ts; src/app/pages/unavailable.component.ts; error-pages.spec.ts</t>
+  </si>
+  <si>
+    <t>Web control panel has no application authentication</t>
+  </si>
+  <si>
+    <t>Treat the absence of login, session, and authorization enforcement in the web server and pages as a security decision for the replacement.</t>
+  </si>
+  <si>
+    <t>The legacy web channel serves administration pages and proxies banking calls without identifying the operator.</t>
+  </si>
+  <si>
+    <t>No application login challenge is presented; target access control requires explicit owner approval rather than silent inheritance.</t>
+  </si>
+  <si>
+    <t>legacy/src/frontend/server.js:1-111; legacy/src/frontend/admin.html:1-103; no authentication middleware or login page is present under legacy/src/frontend; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>D-001/D-002/D-014: the public control surface now requires Identity authentication and API-enforced roles.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Api/Program.cs; Controllers/AccessProbeController.cs; tests/BankOfZ.IntegrationTests/SessionApiTests.cs</t>
+  </si>
+  <si>
+    <t>UF-011</t>
+  </si>
+  <si>
+    <t>Data initialization</t>
+  </si>
+  <si>
     <t>Not Passed - Open</t>
   </si>
   <si>
     <t>Legacy behavior is evidenced and covered by SDD; target implementation has not started.</t>
   </si>
   <si>
-    <t>Operator runs the monthly statement job</t>
-  </si>
-  <si>
-    <t>Generate statements for all accounts of a sort code and reporting month.</t>
-  </si>
-  <si>
-    <t>The JCL supplies YYYYMM and sort code to the PL/I batch program.</t>
-  </si>
-  <si>
-    <t>BNKSTMT processes matching accounts and writes formatted statements to SYSPRINT.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/jcl/BNKSTMT.jcl:1-22; pli/BNKSTMT.pli:18-27,187-205; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decision D-012: preserve statement content and period behavior through an explicit modern job/API without JCL or fixed-width pagination.</t>
-  </si>
-  <si>
-    <t>specs/007-monthly-statements/spec.md; plan.md; tasks.md</t>
-  </si>
-  <si>
-    <t>Statement parameters are missing</t>
-  </si>
-  <si>
-    <t>Use coded defaults when the date/sort-code input file is unavailable.</t>
-  </si>
-  <si>
-    <t>The batch does not fail solely because a parameter card is absent.</t>
-  </si>
-  <si>
-    <t>Default sort code 123456 and calculated/default statement period are used with diagnostic output.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:210-292; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Statement includes customer and account identity</t>
-  </si>
-  <si>
-    <t>Print customer name/address/phone and account number/type/interest/overdraft.</t>
-  </si>
-  <si>
-    <t>The recipient can identify the owner and product.</t>
-  </si>
-  <si>
-    <t>Customer and account information sections are printed.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:430-635; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Statement lists period transactions</t>
-  </si>
-  <si>
-    <t>Print dated transaction history for the selected statement period.</t>
-  </si>
-  <si>
-    <t>The statement explains balance movement.</t>
-  </si>
-  <si>
-    <t>Each transaction includes date, time, type, reference, description, and amount; balances appear in the statement summary.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:638-779; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Statement period has no transactions</t>
-  </si>
-  <si>
-    <t>Print an explicit empty-history message.</t>
-  </si>
-  <si>
-    <t>A quiet account still receives an understandable statement.</t>
-  </si>
-  <si>
-    <t>NO TRANSACTIONS FOR THIS PERIOD is printed.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:719-725; Runtime: simulated — simulation/fixtures/legacy-fixture.json#evidence.monthly-statement; harness: simulation/test; basis: legacy/src/base/batch/pli/BNKSTMT.pli; legacy/src/base/batch/jcl/BNKSTMT.jcl</t>
-  </si>
-  <si>
-    <t>Statement prints financial summary</t>
-  </si>
-  <si>
-    <t>Calculate and print opening balance, credits, debits, closing/available balance, and transaction count.</t>
-  </si>
-  <si>
-    <t>The recipient can reconcile the period at a glance.</t>
-  </si>
-  <si>
-    <t>A statement summary is printed with all totals.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:782-859; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Statement paginates and closes</t>
-  </si>
-  <si>
-    <t>Repeat headers on page breaks and print an end-of-statement footer.</t>
-  </si>
-  <si>
-    <t>Long histories remain readable as a report.</t>
-  </si>
-  <si>
-    <t>Page headers and the closing footer are produced.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:519-560,862-905; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Statement database operation fails</t>
-  </si>
-  <si>
-    <t>Report cursor, fetch, or customer lookup failures without silently printing trusted totals.</t>
-  </si>
-  <si>
-    <t>Batch failures are visible to the operator through job output.</t>
-  </si>
-  <si>
-    <t>SQLCODE diagnostics/warnings are written to SYSPRINT and processing follows the coded branch.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/batch/pli/BNKSTMT.pli:328-389,475-502,670-704; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>UF-010</t>
-  </si>
-  <si>
-    <t>API security, mapping, and web edge behavior</t>
-  </si>
-  <si>
-    <t>API consumer presents OAuth scopes</t>
-  </si>
-  <si>
-    <t>Declare OAuth2 authorization-code security and account/customer scopes.</t>
-  </si>
-  <si>
-    <t>The OpenAPI contract documents protected banking resources.</t>
-  </si>
-  <si>
-    <t>Consumers see the required scopes and authorization/token endpoints.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/api/openapi.yaml:25,616-635; auth.bankofz.example.com is a placeholder endpoint; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-002: no placeholder OAuth provider or scopes are advertised; the slice uses secure same-origin Identity sessions.</t>
-  </si>
-  <si>
-    <t>specs/001-secure-access-shell/spec.md FR-012; modern/backend/src/BankOfZ.Api/Program.cs</t>
-  </si>
-  <si>
-    <t>CICS single-account API normalizes account type</t>
-  </si>
-  <si>
-    <t>Translate the CICS single-account response into API product categories.</t>
-  </si>
-  <si>
-    <t>Only the single-account CICS mapping applies the documented normalization.</t>
-  </si>
-  <si>
-    <t>ISA maps to SAVINGS, MORTGAGE maps to LOAN, and all other values map to CURRENT.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/operations/%2Faccounts%2F%7BaccountId%7D/get/response_200.yaml:10-15; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-007 implemented: CICS single-account product codes map through one explicit target AccountType enum.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Domain/Accounts/LegacyAccountTypeMapper.cs; modern/backend/tests/BankOfZ.UnitTests/Accounts/AccountTests.cs</t>
-  </si>
-  <si>
-    <t>CICS account-list API passes raw account types</t>
-  </si>
-  <si>
-    <t>Expose the route-specific CICS customer-account list mapping without assuming single-account normalization.</t>
-  </si>
-  <si>
-    <t>The list mapping passes the legacy account type directly to API consumers.</t>
-  </si>
-  <si>
-    <t>Raw CICS account type values are returned by the customer account-list route.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/operations/%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_200.yaml:16-20; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-007 implemented: portfolio responses use the same normalized product enum as account details rather than raw CICS values.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Domain/Accounts/LegacyAccountTypeMapper.cs; modern/backend/src/BankOfZ.Api/Controllers/AccountsController.cs; AccountApiTests.cs</t>
-  </si>
-  <si>
-    <t>IMS account API emits schema-invalid CHECKING type</t>
-  </si>
-  <si>
-    <t>Preserve or explicitly correct the route-specific IMS mapping for current/checking accounts.</t>
-  </si>
-  <si>
-    <t>IMS mappings convert type c to CHECKING even though the OpenAPI Account.accountType enum omits CHECKING.</t>
-  </si>
-  <si>
-    <t>The list mapping emits CHECKING; the single-account mapping references $item without a foreach and is not proven valid.</t>
-  </si>
-  <si>
-    <t>legacy/src/api/src/main/operations/%2Fims%2Fcustomers%2F%7BcustomerId%7D%2Faccounts/get/response_200.yaml:16-20; legacy/src/api/src/main/operations/%2Fims%2Faccounts%2F%7BaccountId%7D/get/response_200.yaml:11-15; legacy/src/api/src/main/api/openapi.yaml; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-007 implemented: IMS checking/current variants normalize to CURRENT, eliminating the schema-invalid CHECKING response.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Domain/Accounts/LegacyAccountTypeMapper.cs; modern/backend/tests/BankOfZ.UnitTests/Accounts/AccountTests.cs; AccountApiTests.cs</t>
-  </si>
-  <si>
-    <t>Web server serves the static UI</t>
-  </si>
-  <si>
-    <t>Serve Bank of Z assets and redirect the root index page to the administration control panel.</t>
-  </si>
-  <si>
-    <t>A browser can open the control-panel application.</t>
-  </si>
-  <si>
-    <t>Static files are returned and index.html redirects the browser to admin.html.</t>
-  </si>
-  <si>
-    <t>legacy/src/frontend/server.js:14-51; legacy/src/frontend/index.html redirects to admin.html; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-001/D-002/D-014: Angular is served at /z-bank-new/ and the deployed HTTPS page passed browser smoke.</t>
-  </si>
-  <si>
-    <t>modern/frontend/bank-of-z-ui/Dockerfile; nginx.conf; deploy/nginx-z-bank.conf; https://legacy-transformation-demo.olsys.dev/z-bank-new/</t>
-  </si>
-  <si>
-    <t>Web server proxies API traffic</t>
-  </si>
-  <si>
-    <t>Proxy API/customer/account/IMS paths to the configured z/OS Connect base URL.</t>
-  </si>
-  <si>
-    <t>The browser uses one frontend origin for static content and banking calls.</t>
-  </si>
-  <si>
-    <t>Requests and responses are streamed to/from API_BASE_URL.</t>
-  </si>
-  <si>
-    <t>legacy/src/frontend/server.js proxy paths; config.js base URL; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-001/D-002/D-014: browser API traffic uses the same origin and nginx proxies it to the internal API container.</t>
-  </si>
-  <si>
-    <t>modern/frontend/bank-of-z-ui/nginx.conf; modern/compose.yaml; deployed /z-bank-new/api/session HTTP 200</t>
-  </si>
-  <si>
-    <t>Web static file is missing</t>
-  </si>
-  <si>
-    <t>Return a 404 instead of another page for an unknown static path.</t>
-  </si>
-  <si>
-    <t>Broken links are distinguishable from the application landing page.</t>
-  </si>
-  <si>
-    <t>HTTP 404 is returned.</t>
-  </si>
-  <si>
-    <t>legacy/src/frontend/server.js missing-file branch; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-001/D-002/D-014: unknown Angular routes render the explicit not-found component rather than the landing page.</t>
-  </si>
-  <si>
-    <t>Web proxy target is unavailable</t>
-  </si>
-  <si>
-    <t>Return a structured gateway failure when z/OS Connect cannot be reached.</t>
-  </si>
-  <si>
-    <t>Frontend availability does not disguise backend unavailability.</t>
-  </si>
-  <si>
-    <t>HTTP 502 with JSON error information is returned.</t>
-  </si>
-  <si>
-    <t>legacy/src/frontend/server.js proxy error handler; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-001/D-002/D-014: unavailable API calls render a recoverable unavailable view without stack details.</t>
-  </si>
-  <si>
-    <t>modern/frontend/bank-of-z-ui/src/app/core/session.service.ts; src/app/pages/unavailable.component.ts; error-pages.spec.ts</t>
-  </si>
-  <si>
-    <t>Web control panel has no application authentication</t>
-  </si>
-  <si>
-    <t>Treat the absence of login, session, and authorization enforcement in the web server and pages as a security decision for the replacement.</t>
-  </si>
-  <si>
-    <t>The legacy web channel serves administration pages and proxies banking calls without identifying the operator.</t>
-  </si>
-  <si>
-    <t>No application login challenge is presented; target access control requires explicit owner approval rather than silent inheritance.</t>
-  </si>
-  <si>
-    <t>legacy/src/frontend/server.js:1-111; legacy/src/frontend/admin.html:1-103; no authentication middleware or login page is present under legacy/src/frontend; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>D-001/D-002/D-014: the public control surface now requires Identity authentication and API-enforced roles.</t>
-  </si>
-  <si>
-    <t>modern/backend/src/BankOfZ.Api/Program.cs; Controllers/AccessProbeController.cs; tests/BankOfZ.IntegrationTests/SessionApiTests.cs</t>
-  </si>
-  <si>
-    <t>UF-011</t>
-  </si>
-  <si>
-    <t>Data initialization</t>
-  </si>
-  <si>
     <t>Operator initializes CICS DB2 banking data</t>
   </si>
   <si>
@@ -2883,7 +2949,7 @@
     <t>Implement Feature 007 monthly statements.</t>
   </si>
   <si>
-    <t>Not checked: target implementation has not started. specs/007-monthly-statements/</t>
+    <t>Feature 007 implemented and verified. specs/007-monthly-statements/; analysis/reviews/feature-007-implementation-review.md; modern/backend/src/BankOfZ.Api/Controllers/StatementsController.cs; modern/frontend/bank-of-z-ui/src/app/statements/statement.component.ts; StatementApiTests.cs; monthly-statements.spec.ts</t>
   </si>
   <si>
     <t>R1-G08</t>
@@ -3055,6 +3121,9 @@
   </si>
   <si>
     <t>R1-D-012</t>
+  </si>
+  <si>
+    <t>101,106</t>
   </si>
   <si>
     <t>Owner-approved target decision D-012 recorded in Stage 4.</t>
@@ -7760,339 +7829,371 @@
       </c>
     </row>
     <row r="99" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A99" s="21" t="s">
+      <c r="A99" s="17" t="s">
         <v>612</v>
       </c>
-      <c r="B99" s="21" t="s">
+      <c r="B99" s="17" t="s">
         <v>613</v>
       </c>
-      <c r="C99" s="21" t="s">
-        <v>614</v>
-      </c>
-      <c r="D99" s="21" t="s">
-        <v>615</v>
-      </c>
-      <c r="E99" s="21"/>
-      <c r="F99" s="21"/>
-      <c r="G99" s="21"/>
-      <c r="H99" s="21"/>
-      <c r="I99" s="21"/>
-      <c r="J99" s="21"/>
-      <c r="K99" s="21"/>
-      <c r="L99" s="21"/>
-      <c r="M99" s="21"/>
-      <c r="N99" s="21"/>
+      <c r="C99" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D99" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E99" s="17"/>
+      <c r="F99" s="17"/>
+      <c r="G99" s="17"/>
+      <c r="H99" s="17"/>
+      <c r="I99" s="17"/>
+      <c r="J99" s="17"/>
+      <c r="K99" s="17"/>
+      <c r="L99" s="17"/>
+      <c r="M99" s="17"/>
+      <c r="N99" s="17"/>
     </row>
     <row r="100" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A100" s="18"/>
       <c r="B100" s="19" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C100" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D100" s="22" t="s">
+      <c r="D100" s="20" t="s">
+        <v>615</v>
+      </c>
+      <c r="E100" s="20" t="s">
+        <v>616</v>
+      </c>
+      <c r="F100" s="20" t="s">
         <v>617</v>
       </c>
-      <c r="E100" s="22" t="s">
+      <c r="G100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H100" s="20" t="s">
         <v>618</v>
       </c>
-      <c r="F100" s="22" t="s">
+      <c r="I100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J100" s="20" t="s">
         <v>619</v>
       </c>
-      <c r="G100" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H100" s="22" t="s">
+      <c r="K100" s="20" t="s">
         <v>620</v>
       </c>
-      <c r="I100" s="22"/>
-      <c r="J100" s="22" t="s">
+      <c r="L100" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M100" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N100" s="20" t="s">
         <v>621</v>
-      </c>
-      <c r="K100" s="22"/>
-      <c r="L100" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M100" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N100" s="22" t="s">
-        <v>622</v>
       </c>
     </row>
     <row r="101" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A101" s="18"/>
       <c r="B101" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C101" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D101" s="22" t="s">
+      <c r="D101" s="20" t="s">
+        <v>623</v>
+      </c>
+      <c r="E101" s="20" t="s">
         <v>624</v>
       </c>
-      <c r="E101" s="22" t="s">
+      <c r="F101" s="20" t="s">
         <v>625</v>
       </c>
-      <c r="F101" s="22" t="s">
+      <c r="G101" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H101" s="20" t="s">
         <v>626</v>
       </c>
-      <c r="G101" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H101" s="22" t="s">
+      <c r="I101" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J101" s="20" t="s">
         <v>627</v>
       </c>
-      <c r="I101" s="22"/>
-      <c r="J101" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K101" s="22"/>
-      <c r="L101" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M101" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N101" s="22" t="s">
-        <v>622</v>
+      <c r="K101" s="20" t="s">
+        <v>628</v>
+      </c>
+      <c r="L101" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M101" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N101" s="20" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="102" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A102" s="18"/>
       <c r="B102" s="19" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="C102" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D102" s="22" t="s">
-        <v>629</v>
-      </c>
-      <c r="E102" s="22" t="s">
-        <v>630</v>
-      </c>
-      <c r="F102" s="22" t="s">
+      <c r="D102" s="20" t="s">
         <v>631</v>
       </c>
-      <c r="G102" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H102" s="22" t="s">
+      <c r="E102" s="20" t="s">
         <v>632</v>
       </c>
-      <c r="I102" s="22"/>
-      <c r="J102" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K102" s="22"/>
-      <c r="L102" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M102" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N102" s="22" t="s">
-        <v>622</v>
+      <c r="F102" s="20" t="s">
+        <v>633</v>
+      </c>
+      <c r="G102" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H102" s="20" t="s">
+        <v>634</v>
+      </c>
+      <c r="I102" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J102" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="K102" s="20" t="s">
+        <v>636</v>
+      </c>
+      <c r="L102" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M102" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N102" s="20" t="s">
+        <v>637</v>
       </c>
     </row>
     <row r="103" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A103" s="18"/>
       <c r="B103" s="19" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="C103" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D103" s="22" t="s">
-        <v>634</v>
-      </c>
-      <c r="E103" s="22" t="s">
-        <v>635</v>
-      </c>
-      <c r="F103" s="22" t="s">
-        <v>636</v>
-      </c>
-      <c r="G103" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H103" s="22" t="s">
-        <v>637</v>
-      </c>
-      <c r="I103" s="22"/>
-      <c r="J103" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K103" s="22"/>
-      <c r="L103" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M103" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N103" s="22" t="s">
-        <v>622</v>
+      <c r="D103" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="E103" s="20" t="s">
+        <v>640</v>
+      </c>
+      <c r="F103" s="20" t="s">
+        <v>641</v>
+      </c>
+      <c r="G103" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H103" s="20" t="s">
+        <v>642</v>
+      </c>
+      <c r="I103" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J103" s="20" t="s">
+        <v>643</v>
+      </c>
+      <c r="K103" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="L103" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M103" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N103" s="20" t="s">
+        <v>645</v>
       </c>
     </row>
     <row r="104" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A104" s="18"/>
       <c r="B104" s="19" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
       <c r="C104" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D104" s="22" t="s">
-        <v>639</v>
-      </c>
-      <c r="E104" s="22" t="s">
-        <v>640</v>
-      </c>
-      <c r="F104" s="22" t="s">
-        <v>641</v>
-      </c>
-      <c r="G104" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H104" s="22" t="s">
-        <v>642</v>
-      </c>
-      <c r="I104" s="22"/>
-      <c r="J104" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K104" s="22"/>
-      <c r="L104" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M104" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N104" s="22" t="s">
-        <v>622</v>
+      <c r="D104" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="E104" s="20" t="s">
+        <v>648</v>
+      </c>
+      <c r="F104" s="20" t="s">
+        <v>649</v>
+      </c>
+      <c r="G104" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H104" s="20" t="s">
+        <v>650</v>
+      </c>
+      <c r="I104" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J104" s="20" t="s">
+        <v>651</v>
+      </c>
+      <c r="K104" s="20" t="s">
+        <v>652</v>
+      </c>
+      <c r="L104" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M104" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N104" s="20" t="s">
+        <v>653</v>
       </c>
     </row>
     <row r="105" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A105" s="18"/>
       <c r="B105" s="19" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="C105" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D105" s="22" t="s">
-        <v>644</v>
-      </c>
-      <c r="E105" s="22" t="s">
-        <v>645</v>
-      </c>
-      <c r="F105" s="22" t="s">
-        <v>646</v>
-      </c>
-      <c r="G105" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H105" s="22" t="s">
-        <v>647</v>
-      </c>
-      <c r="I105" s="22"/>
-      <c r="J105" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K105" s="22"/>
-      <c r="L105" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M105" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N105" s="22" t="s">
-        <v>622</v>
+      <c r="D105" s="20" t="s">
+        <v>655</v>
+      </c>
+      <c r="E105" s="20" t="s">
+        <v>656</v>
+      </c>
+      <c r="F105" s="20" t="s">
+        <v>657</v>
+      </c>
+      <c r="G105" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H105" s="20" t="s">
+        <v>658</v>
+      </c>
+      <c r="I105" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J105" s="20" t="s">
+        <v>659</v>
+      </c>
+      <c r="K105" s="20" t="s">
+        <v>660</v>
+      </c>
+      <c r="L105" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M105" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N105" s="20" t="s">
+        <v>661</v>
       </c>
     </row>
     <row r="106" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A106" s="18"/>
       <c r="B106" s="19" t="s">
-        <v>648</v>
+        <v>662</v>
       </c>
       <c r="C106" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D106" s="22" t="s">
-        <v>649</v>
-      </c>
-      <c r="E106" s="22" t="s">
-        <v>650</v>
-      </c>
-      <c r="F106" s="22" t="s">
-        <v>651</v>
-      </c>
-      <c r="G106" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H106" s="22" t="s">
-        <v>652</v>
-      </c>
-      <c r="I106" s="22"/>
-      <c r="J106" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K106" s="22"/>
-      <c r="L106" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M106" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N106" s="22" t="s">
-        <v>622</v>
+      <c r="D106" s="20" t="s">
+        <v>663</v>
+      </c>
+      <c r="E106" s="20" t="s">
+        <v>664</v>
+      </c>
+      <c r="F106" s="20" t="s">
+        <v>665</v>
+      </c>
+      <c r="G106" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H106" s="20" t="s">
+        <v>666</v>
+      </c>
+      <c r="I106" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J106" s="20" t="s">
+        <v>667</v>
+      </c>
+      <c r="K106" s="20" t="s">
+        <v>668</v>
+      </c>
+      <c r="L106" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M106" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N106" s="20" t="s">
+        <v>669</v>
       </c>
     </row>
     <row r="107" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A107" s="18"/>
       <c r="B107" s="19" t="s">
-        <v>653</v>
+        <v>670</v>
       </c>
       <c r="C107" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D107" s="22" t="s">
-        <v>654</v>
-      </c>
-      <c r="E107" s="22" t="s">
-        <v>655</v>
-      </c>
-      <c r="F107" s="22" t="s">
-        <v>656</v>
-      </c>
-      <c r="G107" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H107" s="22" t="s">
-        <v>657</v>
-      </c>
-      <c r="I107" s="22"/>
-      <c r="J107" s="22" t="s">
-        <v>621</v>
-      </c>
-      <c r="K107" s="22"/>
-      <c r="L107" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M107" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N107" s="22" t="s">
-        <v>622</v>
+      <c r="D107" s="20" t="s">
+        <v>671</v>
+      </c>
+      <c r="E107" s="20" t="s">
+        <v>672</v>
+      </c>
+      <c r="F107" s="20" t="s">
+        <v>673</v>
+      </c>
+      <c r="G107" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H107" s="20" t="s">
+        <v>674</v>
+      </c>
+      <c r="I107" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J107" s="20" t="s">
+        <v>675</v>
+      </c>
+      <c r="K107" s="20" t="s">
+        <v>676</v>
+      </c>
+      <c r="L107" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M107" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N107" s="20" t="s">
+        <v>677</v>
       </c>
     </row>
     <row r="108" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>658</v>
+        <v>678</v>
       </c>
       <c r="B108" s="17" t="s">
-        <v>659</v>
+        <v>679</v>
       </c>
       <c r="C108" s="17" t="s">
         <v>29</v>
@@ -8114,34 +8215,34 @@
     <row r="109" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A109" s="18"/>
       <c r="B109" s="19" t="s">
-        <v>660</v>
+        <v>680</v>
       </c>
       <c r="C109" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>661</v>
+        <v>681</v>
       </c>
       <c r="E109" s="20" t="s">
-        <v>662</v>
+        <v>682</v>
       </c>
       <c r="F109" s="20" t="s">
-        <v>663</v>
+        <v>683</v>
       </c>
       <c r="G109" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H109" s="20" t="s">
-        <v>664</v>
+        <v>684</v>
       </c>
       <c r="I109" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J109" s="20" t="s">
-        <v>665</v>
+        <v>685</v>
       </c>
       <c r="K109" s="20" t="s">
-        <v>666</v>
+        <v>686</v>
       </c>
       <c r="L109" s="20" t="s">
         <v>36</v>
@@ -8156,34 +8257,34 @@
     <row r="110" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A110" s="18"/>
       <c r="B110" s="19" t="s">
-        <v>667</v>
+        <v>687</v>
       </c>
       <c r="C110" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>668</v>
+        <v>688</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>669</v>
+        <v>689</v>
       </c>
       <c r="F110" s="20" t="s">
-        <v>670</v>
+        <v>690</v>
       </c>
       <c r="G110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H110" s="20" t="s">
-        <v>671</v>
+        <v>691</v>
       </c>
       <c r="I110" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J110" s="20" t="s">
-        <v>672</v>
+        <v>692</v>
       </c>
       <c r="K110" s="20" t="s">
-        <v>673</v>
+        <v>693</v>
       </c>
       <c r="L110" s="20" t="s">
         <v>36</v>
@@ -8198,34 +8299,34 @@
     <row r="111" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A111" s="18"/>
       <c r="B111" s="19" t="s">
-        <v>674</v>
+        <v>694</v>
       </c>
       <c r="C111" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D111" s="20" t="s">
-        <v>675</v>
+        <v>695</v>
       </c>
       <c r="E111" s="20" t="s">
-        <v>676</v>
+        <v>696</v>
       </c>
       <c r="F111" s="20" t="s">
-        <v>677</v>
+        <v>697</v>
       </c>
       <c r="G111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H111" s="20" t="s">
-        <v>678</v>
+        <v>698</v>
       </c>
       <c r="I111" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J111" s="20" t="s">
-        <v>679</v>
+        <v>699</v>
       </c>
       <c r="K111" s="20" t="s">
-        <v>680</v>
+        <v>700</v>
       </c>
       <c r="L111" s="20" t="s">
         <v>36</v>
@@ -8240,34 +8341,34 @@
     <row r="112" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A112" s="18"/>
       <c r="B112" s="19" t="s">
-        <v>681</v>
+        <v>701</v>
       </c>
       <c r="C112" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>682</v>
+        <v>702</v>
       </c>
       <c r="E112" s="20" t="s">
-        <v>683</v>
+        <v>703</v>
       </c>
       <c r="F112" s="20" t="s">
-        <v>684</v>
+        <v>704</v>
       </c>
       <c r="G112" s="20" t="s">
         <v>158</v>
       </c>
       <c r="H112" s="20" t="s">
-        <v>685</v>
+        <v>705</v>
       </c>
       <c r="I112" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J112" s="20" t="s">
-        <v>686</v>
+        <v>706</v>
       </c>
       <c r="K112" s="20" t="s">
-        <v>687</v>
+        <v>707</v>
       </c>
       <c r="L112" s="20" t="s">
         <v>36</v>
@@ -8282,34 +8383,34 @@
     <row r="113" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A113" s="18"/>
       <c r="B113" s="19" t="s">
-        <v>688</v>
+        <v>708</v>
       </c>
       <c r="C113" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>689</v>
+        <v>709</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>690</v>
+        <v>710</v>
       </c>
       <c r="F113" s="20" t="s">
-        <v>691</v>
+        <v>711</v>
       </c>
       <c r="G113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H113" s="20" t="s">
-        <v>692</v>
+        <v>712</v>
       </c>
       <c r="I113" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J113" s="20" t="s">
-        <v>693</v>
+        <v>713</v>
       </c>
       <c r="K113" s="20" t="s">
-        <v>694</v>
+        <v>714</v>
       </c>
       <c r="L113" s="20" t="s">
         <v>36</v>
@@ -8324,34 +8425,34 @@
     <row r="114" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A114" s="18"/>
       <c r="B114" s="19" t="s">
-        <v>695</v>
+        <v>715</v>
       </c>
       <c r="C114" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D114" s="20" t="s">
-        <v>696</v>
+        <v>716</v>
       </c>
       <c r="E114" s="20" t="s">
-        <v>697</v>
+        <v>717</v>
       </c>
       <c r="F114" s="20" t="s">
-        <v>698</v>
+        <v>718</v>
       </c>
       <c r="G114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H114" s="20" t="s">
-        <v>699</v>
+        <v>719</v>
       </c>
       <c r="I114" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J114" s="20" t="s">
-        <v>700</v>
+        <v>720</v>
       </c>
       <c r="K114" s="20" t="s">
-        <v>701</v>
+        <v>721</v>
       </c>
       <c r="L114" s="20" t="s">
         <v>36</v>
@@ -8366,31 +8467,31 @@
     <row r="115" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A115" s="18"/>
       <c r="B115" s="19" t="s">
-        <v>702</v>
+        <v>722</v>
       </c>
       <c r="C115" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D115" s="20" t="s">
-        <v>703</v>
+        <v>723</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>704</v>
+        <v>724</v>
       </c>
       <c r="F115" s="20" t="s">
-        <v>705</v>
+        <v>725</v>
       </c>
       <c r="G115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H115" s="20" t="s">
-        <v>706</v>
+        <v>726</v>
       </c>
       <c r="I115" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J115" s="20" t="s">
-        <v>707</v>
+        <v>727</v>
       </c>
       <c r="K115" s="20" t="s">
         <v>56</v>
@@ -8408,34 +8509,34 @@
     <row r="116" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A116" s="18"/>
       <c r="B116" s="19" t="s">
-        <v>708</v>
+        <v>728</v>
       </c>
       <c r="C116" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D116" s="20" t="s">
-        <v>709</v>
+        <v>729</v>
       </c>
       <c r="E116" s="20" t="s">
-        <v>710</v>
+        <v>730</v>
       </c>
       <c r="F116" s="20" t="s">
-        <v>711</v>
+        <v>731</v>
       </c>
       <c r="G116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="H116" s="20" t="s">
-        <v>712</v>
+        <v>732</v>
       </c>
       <c r="I116" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J116" s="20" t="s">
-        <v>713</v>
+        <v>733</v>
       </c>
       <c r="K116" s="20" t="s">
-        <v>714</v>
+        <v>734</v>
       </c>
       <c r="L116" s="20" t="s">
         <v>36</v>
@@ -8450,34 +8551,34 @@
     <row r="117" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A117" s="18"/>
       <c r="B117" s="19" t="s">
-        <v>715</v>
+        <v>735</v>
       </c>
       <c r="C117" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D117" s="20" t="s">
-        <v>716</v>
+        <v>736</v>
       </c>
       <c r="E117" s="20" t="s">
-        <v>717</v>
+        <v>737</v>
       </c>
       <c r="F117" s="20" t="s">
-        <v>718</v>
+        <v>738</v>
       </c>
       <c r="G117" s="20" t="s">
         <v>522</v>
       </c>
       <c r="H117" s="20" t="s">
-        <v>719</v>
+        <v>739</v>
       </c>
       <c r="I117" s="20" t="s">
         <v>36</v>
       </c>
       <c r="J117" s="20" t="s">
-        <v>720</v>
+        <v>740</v>
       </c>
       <c r="K117" s="20" t="s">
-        <v>721</v>
+        <v>741</v>
       </c>
       <c r="L117" s="20" t="s">
         <v>36</v>
@@ -8491,16 +8592,16 @@
     </row>
     <row r="118" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="21" t="s">
-        <v>722</v>
+        <v>742</v>
       </c>
       <c r="B118" s="21" t="s">
-        <v>723</v>
+        <v>743</v>
       </c>
       <c r="C118" s="21" t="s">
-        <v>614</v>
+        <v>744</v>
       </c>
       <c r="D118" s="21" t="s">
-        <v>615</v>
+        <v>745</v>
       </c>
       <c r="E118" s="21"/>
       <c r="F118" s="21"/>
@@ -8516,29 +8617,29 @@
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="19" t="s">
-        <v>724</v>
+        <v>746</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D119" s="22" t="s">
-        <v>725</v>
+        <v>747</v>
       </c>
       <c r="E119" s="22" t="s">
-        <v>726</v>
+        <v>748</v>
       </c>
       <c r="F119" s="22" t="s">
-        <v>727</v>
+        <v>749</v>
       </c>
       <c r="G119" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H119" s="22" t="s">
-        <v>728</v>
+        <v>750</v>
       </c>
       <c r="I119" s="22"/>
       <c r="J119" s="22" t="s">
-        <v>729</v>
+        <v>751</v>
       </c>
       <c r="K119" s="22"/>
       <c r="L119" s="22" t="s">
@@ -8548,35 +8649,35 @@
         <v>40</v>
       </c>
       <c r="N119" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="19" t="s">
-        <v>731</v>
+        <v>753</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D120" s="22" t="s">
-        <v>732</v>
+        <v>754</v>
       </c>
       <c r="E120" s="22" t="s">
-        <v>733</v>
+        <v>755</v>
       </c>
       <c r="F120" s="22" t="s">
-        <v>734</v>
+        <v>756</v>
       </c>
       <c r="G120" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H120" s="22" t="s">
-        <v>735</v>
+        <v>757</v>
       </c>
       <c r="I120" s="22"/>
       <c r="J120" s="22" t="s">
-        <v>736</v>
+        <v>758</v>
       </c>
       <c r="K120" s="22"/>
       <c r="L120" s="22" t="s">
@@ -8586,35 +8687,35 @@
         <v>40</v>
       </c>
       <c r="N120" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A121" s="18"/>
       <c r="B121" s="19" t="s">
-        <v>737</v>
+        <v>759</v>
       </c>
       <c r="C121" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D121" s="22" t="s">
-        <v>738</v>
+        <v>760</v>
       </c>
       <c r="E121" s="22" t="s">
-        <v>739</v>
+        <v>761</v>
       </c>
       <c r="F121" s="22" t="s">
-        <v>740</v>
+        <v>762</v>
       </c>
       <c r="G121" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H121" s="22" t="s">
-        <v>741</v>
+        <v>763</v>
       </c>
       <c r="I121" s="22"/>
       <c r="J121" s="22" t="s">
-        <v>736</v>
+        <v>758</v>
       </c>
       <c r="K121" s="22"/>
       <c r="L121" s="22" t="s">
@@ -8624,35 +8725,35 @@
         <v>40</v>
       </c>
       <c r="N121" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="19" t="s">
-        <v>742</v>
+        <v>764</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D122" s="22" t="s">
-        <v>743</v>
+        <v>765</v>
       </c>
       <c r="E122" s="22" t="s">
-        <v>744</v>
+        <v>766</v>
       </c>
       <c r="F122" s="22" t="s">
-        <v>745</v>
+        <v>767</v>
       </c>
       <c r="G122" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H122" s="22" t="s">
-        <v>746</v>
+        <v>768</v>
       </c>
       <c r="I122" s="22"/>
       <c r="J122" s="22" t="s">
-        <v>736</v>
+        <v>758</v>
       </c>
       <c r="K122" s="22"/>
       <c r="L122" s="22" t="s">
@@ -8662,35 +8763,35 @@
         <v>40</v>
       </c>
       <c r="N122" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="19" t="s">
-        <v>747</v>
+        <v>769</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D123" s="22" t="s">
-        <v>748</v>
+        <v>770</v>
       </c>
       <c r="E123" s="22" t="s">
-        <v>749</v>
+        <v>771</v>
       </c>
       <c r="F123" s="22" t="s">
-        <v>750</v>
+        <v>772</v>
       </c>
       <c r="G123" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H123" s="22" t="s">
-        <v>751</v>
+        <v>773</v>
       </c>
       <c r="I123" s="22"/>
       <c r="J123" s="22" t="s">
-        <v>736</v>
+        <v>758</v>
       </c>
       <c r="K123" s="22"/>
       <c r="L123" s="22" t="s">
@@ -8700,35 +8801,35 @@
         <v>40</v>
       </c>
       <c r="N123" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="19" t="s">
-        <v>752</v>
+        <v>774</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D124" s="22" t="s">
-        <v>753</v>
+        <v>775</v>
       </c>
       <c r="E124" s="22" t="s">
-        <v>754</v>
+        <v>776</v>
       </c>
       <c r="F124" s="22" t="s">
-        <v>755</v>
+        <v>777</v>
       </c>
       <c r="G124" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H124" s="22" t="s">
-        <v>756</v>
+        <v>778</v>
       </c>
       <c r="I124" s="22"/>
       <c r="J124" s="22" t="s">
-        <v>757</v>
+        <v>779</v>
       </c>
       <c r="K124" s="22"/>
       <c r="L124" s="22" t="s">
@@ -8738,35 +8839,35 @@
         <v>40</v>
       </c>
       <c r="N124" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="19" t="s">
-        <v>758</v>
+        <v>780</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D125" s="22" t="s">
-        <v>759</v>
+        <v>781</v>
       </c>
       <c r="E125" s="22" t="s">
-        <v>760</v>
+        <v>782</v>
       </c>
       <c r="F125" s="22" t="s">
-        <v>761</v>
+        <v>783</v>
       </c>
       <c r="G125" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H125" s="22" t="s">
-        <v>762</v>
+        <v>784</v>
       </c>
       <c r="I125" s="22"/>
       <c r="J125" s="22" t="s">
-        <v>763</v>
+        <v>785</v>
       </c>
       <c r="K125" s="22"/>
       <c r="L125" s="22" t="s">
@@ -8776,35 +8877,35 @@
         <v>40</v>
       </c>
       <c r="N125" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="19" t="s">
-        <v>764</v>
+        <v>786</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D126" s="22" t="s">
-        <v>765</v>
+        <v>787</v>
       </c>
       <c r="E126" s="22" t="s">
-        <v>766</v>
+        <v>788</v>
       </c>
       <c r="F126" s="22" t="s">
-        <v>767</v>
+        <v>789</v>
       </c>
       <c r="G126" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H126" s="22" t="s">
-        <v>768</v>
+        <v>790</v>
       </c>
       <c r="I126" s="22"/>
       <c r="J126" s="22" t="s">
-        <v>769</v>
+        <v>791</v>
       </c>
       <c r="K126" s="22"/>
       <c r="L126" s="22" t="s">
@@ -8814,21 +8915,21 @@
         <v>40</v>
       </c>
       <c r="N126" s="22" t="s">
-        <v>730</v>
+        <v>752</v>
       </c>
     </row>
     <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="21" t="s">
-        <v>770</v>
+        <v>792</v>
       </c>
       <c r="B127" s="21" t="s">
-        <v>771</v>
+        <v>793</v>
       </c>
       <c r="C127" s="21" t="s">
-        <v>614</v>
+        <v>744</v>
       </c>
       <c r="D127" s="21" t="s">
-        <v>615</v>
+        <v>745</v>
       </c>
       <c r="E127" s="21"/>
       <c r="F127" s="21"/>
@@ -8844,29 +8945,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>772</v>
+        <v>794</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D128" s="22" t="s">
-        <v>773</v>
+        <v>795</v>
       </c>
       <c r="E128" s="22" t="s">
-        <v>774</v>
+        <v>796</v>
       </c>
       <c r="F128" s="22" t="s">
-        <v>775</v>
+        <v>797</v>
       </c>
       <c r="G128" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="22" t="s">
-        <v>776</v>
+        <v>798</v>
       </c>
       <c r="I128" s="22"/>
       <c r="J128" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K128" s="22"/>
       <c r="L128" s="22" t="s">
@@ -8876,35 +8977,35 @@
         <v>40</v>
       </c>
       <c r="N128" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>779</v>
+        <v>801</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D129" s="22" t="s">
-        <v>780</v>
+        <v>802</v>
       </c>
       <c r="E129" s="22" t="s">
-        <v>781</v>
+        <v>803</v>
       </c>
       <c r="F129" s="22" t="s">
-        <v>782</v>
+        <v>804</v>
       </c>
       <c r="G129" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="22" t="s">
-        <v>783</v>
+        <v>805</v>
       </c>
       <c r="I129" s="22"/>
       <c r="J129" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K129" s="22"/>
       <c r="L129" s="22" t="s">
@@ -8914,35 +9015,35 @@
         <v>40</v>
       </c>
       <c r="N129" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="18"/>
       <c r="B130" s="19" t="s">
-        <v>784</v>
+        <v>806</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D130" s="22" t="s">
-        <v>785</v>
+        <v>807</v>
       </c>
       <c r="E130" s="22" t="s">
-        <v>786</v>
+        <v>808</v>
       </c>
       <c r="F130" s="22" t="s">
-        <v>787</v>
+        <v>809</v>
       </c>
       <c r="G130" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="22" t="s">
-        <v>788</v>
+        <v>810</v>
       </c>
       <c r="I130" s="22"/>
       <c r="J130" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K130" s="22"/>
       <c r="L130" s="22" t="s">
@@ -8952,35 +9053,35 @@
         <v>40</v>
       </c>
       <c r="N130" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>789</v>
+        <v>811</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D131" s="22" t="s">
-        <v>790</v>
+        <v>812</v>
       </c>
       <c r="E131" s="22" t="s">
-        <v>791</v>
+        <v>813</v>
       </c>
       <c r="F131" s="22" t="s">
-        <v>792</v>
+        <v>814</v>
       </c>
       <c r="G131" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H131" s="22" t="s">
-        <v>793</v>
+        <v>815</v>
       </c>
       <c r="I131" s="22"/>
       <c r="J131" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K131" s="22"/>
       <c r="L131" s="22" t="s">
@@ -8990,35 +9091,35 @@
         <v>40</v>
       </c>
       <c r="N131" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>794</v>
+        <v>816</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D132" s="22" t="s">
-        <v>795</v>
+        <v>817</v>
       </c>
       <c r="E132" s="22" t="s">
-        <v>796</v>
+        <v>818</v>
       </c>
       <c r="F132" s="22" t="s">
-        <v>797</v>
+        <v>819</v>
       </c>
       <c r="G132" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="22" t="s">
-        <v>798</v>
+        <v>820</v>
       </c>
       <c r="I132" s="22"/>
       <c r="J132" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K132" s="22"/>
       <c r="L132" s="22" t="s">
@@ -9028,35 +9129,35 @@
         <v>40</v>
       </c>
       <c r="N132" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>799</v>
+        <v>821</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D133" s="22" t="s">
-        <v>800</v>
+        <v>822</v>
       </c>
       <c r="E133" s="22" t="s">
-        <v>801</v>
+        <v>823</v>
       </c>
       <c r="F133" s="22" t="s">
-        <v>802</v>
+        <v>824</v>
       </c>
       <c r="G133" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H133" s="22" t="s">
-        <v>803</v>
+        <v>825</v>
       </c>
       <c r="I133" s="22"/>
       <c r="J133" s="22" t="s">
-        <v>804</v>
+        <v>826</v>
       </c>
       <c r="K133" s="22"/>
       <c r="L133" s="22" t="s">
@@ -9066,35 +9167,35 @@
         <v>40</v>
       </c>
       <c r="N133" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>805</v>
+        <v>827</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D134" s="22" t="s">
-        <v>806</v>
+        <v>828</v>
       </c>
       <c r="E134" s="22" t="s">
-        <v>807</v>
+        <v>829</v>
       </c>
       <c r="F134" s="22" t="s">
-        <v>808</v>
+        <v>830</v>
       </c>
       <c r="G134" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="22" t="s">
-        <v>809</v>
+        <v>831</v>
       </c>
       <c r="I134" s="22"/>
       <c r="J134" s="22" t="s">
-        <v>810</v>
+        <v>832</v>
       </c>
       <c r="K134" s="22"/>
       <c r="L134" s="22" t="s">
@@ -9104,35 +9205,35 @@
         <v>40</v>
       </c>
       <c r="N134" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>811</v>
+        <v>833</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D135" s="22" t="s">
-        <v>812</v>
+        <v>834</v>
       </c>
       <c r="E135" s="22" t="s">
-        <v>813</v>
+        <v>835</v>
       </c>
       <c r="F135" s="22" t="s">
-        <v>814</v>
+        <v>836</v>
       </c>
       <c r="G135" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H135" s="22" t="s">
-        <v>815</v>
+        <v>837</v>
       </c>
       <c r="I135" s="22"/>
       <c r="J135" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K135" s="22"/>
       <c r="L135" s="22" t="s">
@@ -9142,35 +9243,35 @@
         <v>40</v>
       </c>
       <c r="N135" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>816</v>
+        <v>838</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D136" s="22" t="s">
-        <v>817</v>
+        <v>839</v>
       </c>
       <c r="E136" s="22" t="s">
-        <v>818</v>
+        <v>840</v>
       </c>
       <c r="F136" s="22" t="s">
-        <v>819</v>
+        <v>841</v>
       </c>
       <c r="G136" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H136" s="22" t="s">
-        <v>820</v>
+        <v>842</v>
       </c>
       <c r="I136" s="22"/>
       <c r="J136" s="22" t="s">
-        <v>821</v>
+        <v>843</v>
       </c>
       <c r="K136" s="22"/>
       <c r="L136" s="22" t="s">
@@ -9180,35 +9281,35 @@
         <v>40</v>
       </c>
       <c r="N136" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>822</v>
+        <v>844</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D137" s="22" t="s">
-        <v>823</v>
+        <v>845</v>
       </c>
       <c r="E137" s="22" t="s">
-        <v>824</v>
+        <v>846</v>
       </c>
       <c r="F137" s="22" t="s">
-        <v>825</v>
+        <v>847</v>
       </c>
       <c r="G137" s="22" t="s">
         <v>522</v>
       </c>
       <c r="H137" s="22" t="s">
-        <v>826</v>
+        <v>848</v>
       </c>
       <c r="I137" s="22"/>
       <c r="J137" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K137" s="22"/>
       <c r="L137" s="22" t="s">
@@ -9218,35 +9319,35 @@
         <v>40</v>
       </c>
       <c r="N137" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>827</v>
+        <v>849</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D138" s="22" t="s">
-        <v>828</v>
+        <v>850</v>
       </c>
       <c r="E138" s="22" t="s">
-        <v>829</v>
+        <v>851</v>
       </c>
       <c r="F138" s="22" t="s">
-        <v>830</v>
+        <v>852</v>
       </c>
       <c r="G138" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="22" t="s">
-        <v>831</v>
+        <v>853</v>
       </c>
       <c r="I138" s="22"/>
       <c r="J138" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K138" s="22"/>
       <c r="L138" s="22" t="s">
@@ -9256,35 +9357,35 @@
         <v>40</v>
       </c>
       <c r="N138" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>832</v>
+        <v>854</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D139" s="22" t="s">
-        <v>833</v>
+        <v>855</v>
       </c>
       <c r="E139" s="22" t="s">
-        <v>834</v>
+        <v>856</v>
       </c>
       <c r="F139" s="22" t="s">
-        <v>835</v>
+        <v>857</v>
       </c>
       <c r="G139" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="22" t="s">
-        <v>836</v>
+        <v>858</v>
       </c>
       <c r="I139" s="22"/>
       <c r="J139" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K139" s="22"/>
       <c r="L139" s="22" t="s">
@@ -9294,35 +9395,35 @@
         <v>40</v>
       </c>
       <c r="N139" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>837</v>
+        <v>859</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D140" s="22" t="s">
-        <v>838</v>
+        <v>860</v>
       </c>
       <c r="E140" s="22" t="s">
-        <v>839</v>
+        <v>861</v>
       </c>
       <c r="F140" s="22" t="s">
-        <v>840</v>
+        <v>862</v>
       </c>
       <c r="G140" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="22" t="s">
-        <v>841</v>
+        <v>863</v>
       </c>
       <c r="I140" s="22"/>
       <c r="J140" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K140" s="22"/>
       <c r="L140" s="22" t="s">
@@ -9332,35 +9433,35 @@
         <v>40</v>
       </c>
       <c r="N140" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>842</v>
+        <v>864</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D141" s="22" t="s">
-        <v>843</v>
+        <v>865</v>
       </c>
       <c r="E141" s="22" t="s">
-        <v>844</v>
+        <v>866</v>
       </c>
       <c r="F141" s="22" t="s">
-        <v>845</v>
+        <v>867</v>
       </c>
       <c r="G141" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="22" t="s">
-        <v>846</v>
+        <v>868</v>
       </c>
       <c r="I141" s="22"/>
       <c r="J141" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K141" s="22"/>
       <c r="L141" s="22" t="s">
@@ -9370,35 +9471,35 @@
         <v>40</v>
       </c>
       <c r="N141" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>847</v>
+        <v>869</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D142" s="22" t="s">
-        <v>848</v>
+        <v>870</v>
       </c>
       <c r="E142" s="22" t="s">
-        <v>849</v>
+        <v>871</v>
       </c>
       <c r="F142" s="22" t="s">
-        <v>850</v>
+        <v>872</v>
       </c>
       <c r="G142" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="22" t="s">
-        <v>851</v>
+        <v>873</v>
       </c>
       <c r="I142" s="22"/>
       <c r="J142" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K142" s="22"/>
       <c r="L142" s="22" t="s">
@@ -9408,35 +9509,35 @@
         <v>40</v>
       </c>
       <c r="N142" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>852</v>
+        <v>874</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D143" s="22" t="s">
-        <v>853</v>
+        <v>875</v>
       </c>
       <c r="E143" s="22" t="s">
-        <v>854</v>
+        <v>876</v>
       </c>
       <c r="F143" s="22" t="s">
-        <v>855</v>
+        <v>877</v>
       </c>
       <c r="G143" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="22" t="s">
-        <v>856</v>
+        <v>878</v>
       </c>
       <c r="I143" s="22"/>
       <c r="J143" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K143" s="22"/>
       <c r="L143" s="22" t="s">
@@ -9446,35 +9547,35 @@
         <v>40</v>
       </c>
       <c r="N143" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>857</v>
+        <v>879</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D144" s="22" t="s">
-        <v>858</v>
+        <v>880</v>
       </c>
       <c r="E144" s="22" t="s">
-        <v>859</v>
+        <v>881</v>
       </c>
       <c r="F144" s="22" t="s">
-        <v>860</v>
+        <v>882</v>
       </c>
       <c r="G144" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H144" s="22" t="s">
-        <v>861</v>
+        <v>883</v>
       </c>
       <c r="I144" s="22"/>
       <c r="J144" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K144" s="22"/>
       <c r="L144" s="22" t="s">
@@ -9484,35 +9585,35 @@
         <v>40</v>
       </c>
       <c r="N144" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>862</v>
+        <v>884</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D145" s="22" t="s">
-        <v>863</v>
+        <v>885</v>
       </c>
       <c r="E145" s="22" t="s">
-        <v>864</v>
+        <v>886</v>
       </c>
       <c r="F145" s="22" t="s">
-        <v>865</v>
+        <v>887</v>
       </c>
       <c r="G145" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="22" t="s">
-        <v>866</v>
+        <v>888</v>
       </c>
       <c r="I145" s="22"/>
       <c r="J145" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K145" s="22"/>
       <c r="L145" s="22" t="s">
@@ -9522,35 +9623,35 @@
         <v>40</v>
       </c>
       <c r="N145" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>867</v>
+        <v>889</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D146" s="22" t="s">
-        <v>868</v>
+        <v>890</v>
       </c>
       <c r="E146" s="22" t="s">
-        <v>869</v>
+        <v>891</v>
       </c>
       <c r="F146" s="22" t="s">
-        <v>870</v>
+        <v>892</v>
       </c>
       <c r="G146" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="22" t="s">
-        <v>871</v>
+        <v>893</v>
       </c>
       <c r="I146" s="22"/>
       <c r="J146" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K146" s="22"/>
       <c r="L146" s="22" t="s">
@@ -9560,35 +9661,35 @@
         <v>40</v>
       </c>
       <c r="N146" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>872</v>
+        <v>894</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D147" s="22" t="s">
-        <v>873</v>
+        <v>895</v>
       </c>
       <c r="E147" s="22" t="s">
-        <v>874</v>
+        <v>896</v>
       </c>
       <c r="F147" s="22" t="s">
-        <v>875</v>
+        <v>897</v>
       </c>
       <c r="G147" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="22" t="s">
-        <v>876</v>
+        <v>898</v>
       </c>
       <c r="I147" s="22"/>
       <c r="J147" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K147" s="22"/>
       <c r="L147" s="22" t="s">
@@ -9598,35 +9699,35 @@
         <v>40</v>
       </c>
       <c r="N147" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>877</v>
+        <v>899</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D148" s="22" t="s">
-        <v>878</v>
+        <v>900</v>
       </c>
       <c r="E148" s="22" t="s">
-        <v>879</v>
+        <v>901</v>
       </c>
       <c r="F148" s="22" t="s">
-        <v>880</v>
+        <v>902</v>
       </c>
       <c r="G148" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="22" t="s">
-        <v>881</v>
+        <v>903</v>
       </c>
       <c r="I148" s="22"/>
       <c r="J148" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K148" s="22"/>
       <c r="L148" s="22" t="s">
@@ -9636,35 +9737,35 @@
         <v>40</v>
       </c>
       <c r="N148" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>882</v>
+        <v>904</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D149" s="22" t="s">
-        <v>883</v>
+        <v>905</v>
       </c>
       <c r="E149" s="22" t="s">
-        <v>884</v>
+        <v>906</v>
       </c>
       <c r="F149" s="22" t="s">
-        <v>885</v>
+        <v>907</v>
       </c>
       <c r="G149" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="22" t="s">
-        <v>886</v>
+        <v>908</v>
       </c>
       <c r="I149" s="22"/>
       <c r="J149" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K149" s="22"/>
       <c r="L149" s="22" t="s">
@@ -9674,35 +9775,35 @@
         <v>40</v>
       </c>
       <c r="N149" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>887</v>
+        <v>909</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D150" s="22" t="s">
-        <v>888</v>
+        <v>910</v>
       </c>
       <c r="E150" s="22" t="s">
-        <v>889</v>
+        <v>911</v>
       </c>
       <c r="F150" s="22" t="s">
-        <v>890</v>
+        <v>912</v>
       </c>
       <c r="G150" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H150" s="22" t="s">
-        <v>891</v>
+        <v>913</v>
       </c>
       <c r="I150" s="22"/>
       <c r="J150" s="22" t="s">
-        <v>892</v>
+        <v>914</v>
       </c>
       <c r="K150" s="22"/>
       <c r="L150" s="22" t="s">
@@ -9712,35 +9813,35 @@
         <v>40</v>
       </c>
       <c r="N150" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>893</v>
+        <v>915</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D151" s="22" t="s">
-        <v>894</v>
+        <v>916</v>
       </c>
       <c r="E151" s="22" t="s">
-        <v>895</v>
+        <v>917</v>
       </c>
       <c r="F151" s="22" t="s">
-        <v>896</v>
+        <v>918</v>
       </c>
       <c r="G151" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H151" s="22" t="s">
-        <v>897</v>
+        <v>919</v>
       </c>
       <c r="I151" s="22"/>
       <c r="J151" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K151" s="22"/>
       <c r="L151" s="22" t="s">
@@ -9750,35 +9851,35 @@
         <v>40</v>
       </c>
       <c r="N151" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>898</v>
+        <v>920</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D152" s="22" t="s">
-        <v>899</v>
+        <v>921</v>
       </c>
       <c r="E152" s="22" t="s">
-        <v>900</v>
+        <v>922</v>
       </c>
       <c r="F152" s="22" t="s">
-        <v>901</v>
+        <v>923</v>
       </c>
       <c r="G152" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H152" s="22" t="s">
-        <v>902</v>
+        <v>924</v>
       </c>
       <c r="I152" s="22"/>
       <c r="J152" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K152" s="22"/>
       <c r="L152" s="22" t="s">
@@ -9788,35 +9889,35 @@
         <v>40</v>
       </c>
       <c r="N152" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>903</v>
+        <v>925</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D153" s="22" t="s">
-        <v>904</v>
+        <v>926</v>
       </c>
       <c r="E153" s="22" t="s">
-        <v>905</v>
+        <v>927</v>
       </c>
       <c r="F153" s="22" t="s">
-        <v>906</v>
+        <v>928</v>
       </c>
       <c r="G153" s="22" t="s">
         <v>522</v>
       </c>
       <c r="H153" s="22" t="s">
-        <v>907</v>
+        <v>929</v>
       </c>
       <c r="I153" s="22"/>
       <c r="J153" s="22" t="s">
-        <v>777</v>
+        <v>799</v>
       </c>
       <c r="K153" s="22"/>
       <c r="L153" s="22" t="s">
@@ -9826,7 +9927,7 @@
         <v>40</v>
       </c>
       <c r="N153" s="22" t="s">
-        <v>778</v>
+        <v>800</v>
       </c>
     </row>
   </sheetData>
@@ -9859,51 +9960,51 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>908</v>
+        <v>930</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>909</v>
+        <v>931</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>910</v>
+        <v>932</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>911</v>
+        <v>933</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>912</v>
+        <v>934</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>913</v>
+        <v>935</v>
       </c>
       <c r="G1" s="24" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="24" t="s">
-        <v>914</v>
+        <v>936</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>915</v>
+        <v>937</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>916</v>
+        <v>938</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>917</v>
+        <v>939</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>918</v>
+        <v>940</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>920</v>
+        <v>942</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>921</v>
+        <v>943</v>
       </c>
       <c r="G2" s="27" t="s">
         <v>36</v>
@@ -9912,27 +10013,27 @@
         <v>36</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>922</v>
+        <v>944</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
-        <v>923</v>
+        <v>945</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>924</v>
+        <v>946</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>925</v>
+        <v>947</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E3" s="30" t="s">
-        <v>926</v>
+        <v>948</v>
       </c>
       <c r="F3" s="30" t="s">
-        <v>927</v>
+        <v>949</v>
       </c>
       <c r="G3" s="30" t="s">
         <v>36</v>
@@ -9941,27 +10042,27 @@
         <v>36</v>
       </c>
       <c r="I3" s="31" t="s">
-        <v>928</v>
+        <v>950</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
-        <v>929</v>
+        <v>951</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>930</v>
+        <v>952</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>931</v>
+        <v>953</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>932</v>
+        <v>954</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>933</v>
+        <v>955</v>
       </c>
       <c r="G4" s="30" t="s">
         <v>36</v>
@@ -9970,27 +10071,27 @@
         <v>36</v>
       </c>
       <c r="I4" s="31" t="s">
-        <v>934</v>
+        <v>956</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
-        <v>935</v>
+        <v>957</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>936</v>
+        <v>958</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>937</v>
+        <v>959</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>938</v>
+        <v>960</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>939</v>
+        <v>961</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>36</v>
@@ -9999,27 +10100,27 @@
         <v>36</v>
       </c>
       <c r="I5" s="31" t="s">
-        <v>940</v>
+        <v>962</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
-        <v>941</v>
+        <v>963</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>487</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>942</v>
+        <v>964</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>943</v>
+        <v>965</v>
       </c>
       <c r="F6" s="30" t="s">
-        <v>944</v>
+        <v>966</v>
       </c>
       <c r="G6" s="30" t="s">
         <v>36</v>
@@ -10028,27 +10129,27 @@
         <v>36</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>945</v>
+        <v>967</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="29" t="s">
-        <v>946</v>
+        <v>968</v>
       </c>
       <c r="B7" s="30" t="s">
         <v>533</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>947</v>
+        <v>969</v>
       </c>
       <c r="D7" s="30" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>948</v>
+        <v>970</v>
       </c>
       <c r="F7" s="30" t="s">
-        <v>949</v>
+        <v>971</v>
       </c>
       <c r="G7" s="30" t="s">
         <v>36</v>
@@ -10057,56 +10158,56 @@
         <v>36</v>
       </c>
       <c r="I7" s="31" t="s">
-        <v>950</v>
+        <v>972</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
-        <v>951</v>
-      </c>
-      <c r="B8" s="33" t="s">
+      <c r="A8" s="29" t="s">
+        <v>973</v>
+      </c>
+      <c r="B8" s="30" t="s">
         <v>612</v>
       </c>
-      <c r="C8" s="33" t="s">
-        <v>952</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>919</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>953</v>
-      </c>
-      <c r="F8" s="33" t="s">
-        <v>954</v>
-      </c>
-      <c r="G8" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="34" t="s">
-        <v>955</v>
+      <c r="C8" s="30" t="s">
+        <v>974</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>941</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>975</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>976</v>
+      </c>
+      <c r="G8" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="31" t="s">
+        <v>977</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
-        <v>956</v>
+        <v>978</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>722</v>
+        <v>742</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>957</v>
+        <v>979</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>958</v>
+        <v>980</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>959</v>
+        <v>981</v>
       </c>
       <c r="G9" s="33" t="s">
         <v>36</v>
@@ -10115,27 +10216,27 @@
         <v>40</v>
       </c>
       <c r="I9" s="34" t="s">
-        <v>960</v>
+        <v>982</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
-        <v>961</v>
+        <v>983</v>
       </c>
       <c r="B10" s="36" t="s">
-        <v>770</v>
+        <v>792</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>962</v>
+        <v>984</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>919</v>
+        <v>941</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>963</v>
+        <v>985</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>964</v>
+        <v>986</v>
       </c>
       <c r="G10" s="36" t="s">
         <v>36</v>
@@ -10144,25 +10245,25 @@
         <v>40</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>965</v>
+        <v>987</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>966</v>
+        <v>988</v>
       </c>
       <c r="B11" s="27"/>
       <c r="C11" s="27" t="s">
-        <v>967</v>
+        <v>989</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>970</v>
+        <v>992</v>
       </c>
       <c r="G11" s="27" t="s">
         <v>36</v>
@@ -10171,25 +10272,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>971</v>
+        <v>993</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>972</v>
+        <v>994</v>
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="30" t="s">
-        <v>973</v>
+        <v>995</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>974</v>
+        <v>996</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>36</v>
@@ -10198,25 +10299,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>975</v>
+        <v>997</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
-        <v>976</v>
+        <v>998</v>
       </c>
       <c r="B13" s="30"/>
       <c r="C13" s="30" t="s">
-        <v>977</v>
+        <v>999</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E13" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>978</v>
+        <v>1000</v>
       </c>
       <c r="G13" s="30" t="s">
         <v>36</v>
@@ -10225,25 +10326,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>979</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
-        <v>980</v>
+        <v>1002</v>
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="30" t="s">
-        <v>981</v>
+        <v>1003</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>982</v>
+        <v>1004</v>
       </c>
       <c r="G14" s="30" t="s">
         <v>36</v>
@@ -10252,25 +10353,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="31" t="s">
-        <v>983</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
-        <v>984</v>
+        <v>1006</v>
       </c>
       <c r="B15" s="30"/>
       <c r="C15" s="30" t="s">
-        <v>985</v>
+        <v>1007</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E15" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>986</v>
+        <v>1008</v>
       </c>
       <c r="G15" s="30" t="s">
         <v>36</v>
@@ -10279,25 +10380,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>987</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
-        <v>988</v>
+        <v>1010</v>
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="30" t="s">
-        <v>989</v>
+        <v>1011</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>990</v>
+        <v>1012</v>
       </c>
       <c r="G16" s="30" t="s">
         <v>36</v>
@@ -10306,25 +10407,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="31" t="s">
-        <v>991</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="29" t="s">
-        <v>992</v>
+        <v>1014</v>
       </c>
       <c r="B17" s="30"/>
       <c r="C17" s="30" t="s">
-        <v>993</v>
+        <v>1015</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>994</v>
+        <v>1016</v>
       </c>
       <c r="G17" s="30" t="s">
         <v>36</v>
@@ -10333,25 +10434,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>995</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>996</v>
+        <v>1018</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30" t="s">
-        <v>997</v>
+        <v>1019</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>998</v>
+        <v>1020</v>
       </c>
       <c r="G18" s="30" t="s">
         <v>36</v>
@@ -10360,25 +10461,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="31" t="s">
-        <v>999</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="29" t="s">
-        <v>1000</v>
+        <v>1022</v>
       </c>
       <c r="B19" s="30"/>
       <c r="C19" s="30" t="s">
-        <v>1001</v>
+        <v>1023</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>1002</v>
+        <v>1024</v>
       </c>
       <c r="G19" s="30" t="s">
         <v>36</v>
@@ -10387,25 +10488,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>1003</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
-        <v>1004</v>
+        <v>1026</v>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="30" t="s">
-        <v>1005</v>
+        <v>1027</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>1006</v>
+        <v>1028</v>
       </c>
       <c r="G20" s="30" t="s">
         <v>36</v>
@@ -10414,25 +10515,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="31" t="s">
-        <v>1007</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="29" t="s">
-        <v>1008</v>
+        <v>1030</v>
       </c>
       <c r="B21" s="30"/>
       <c r="C21" s="30" t="s">
-        <v>1009</v>
+        <v>1031</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E21" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F21" s="30" t="s">
-        <v>1010</v>
+        <v>1032</v>
       </c>
       <c r="G21" s="30" t="s">
         <v>36</v>
@@ -10441,25 +10542,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>1011</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
-        <v>1012</v>
+        <v>1034</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30" t="s">
-        <v>952</v>
+        <v>1035</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>1013</v>
+        <v>1036</v>
       </c>
       <c r="G22" s="30" t="s">
         <v>36</v>
@@ -10468,25 +10569,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="31" t="s">
-        <v>1014</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
-        <v>1015</v>
+        <v>1038</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30" t="s">
-        <v>957</v>
+        <v>979</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F23" s="30" t="s">
-        <v>1016</v>
+        <v>1039</v>
       </c>
       <c r="G23" s="30" t="s">
         <v>36</v>
@@ -10495,25 +10596,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>1017</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
-        <v>1018</v>
+        <v>1041</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30" t="s">
-        <v>1019</v>
+        <v>1042</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>1020</v>
+        <v>1043</v>
       </c>
       <c r="G24" s="30" t="s">
         <v>36</v>
@@ -10522,25 +10623,25 @@
         <v>36</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>1021</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
-        <v>1022</v>
+        <v>1045</v>
       </c>
       <c r="B25" s="39"/>
       <c r="C25" s="39" t="s">
-        <v>1023</v>
+        <v>1046</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E25" s="39" t="s">
-        <v>969</v>
+        <v>991</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>1024</v>
+        <v>1047</v>
       </c>
       <c r="G25" s="39" t="s">
         <v>36</v>
@@ -10549,25 +10650,25 @@
         <v>36</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>1025</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="38" t="s">
-        <v>1026</v>
+        <v>1049</v>
       </c>
       <c r="B26" s="39"/>
       <c r="C26" s="39" t="s">
-        <v>1027</v>
+        <v>1050</v>
       </c>
       <c r="D26" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E26" s="39" t="s">
-        <v>1028</v>
+        <v>1051</v>
       </c>
       <c r="F26" s="39" t="s">
-        <v>1029</v>
+        <v>1052</v>
       </c>
       <c r="G26" s="39" t="s">
         <v>36</v>
@@ -10576,25 +10677,25 @@
         <v>36</v>
       </c>
       <c r="I26" s="40" t="s">
-        <v>1030</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="38" t="s">
-        <v>1031</v>
+        <v>1054</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39" t="s">
-        <v>1032</v>
+        <v>1055</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>1033</v>
+        <v>1056</v>
       </c>
       <c r="F27" s="39" t="s">
-        <v>1034</v>
+        <v>1057</v>
       </c>
       <c r="G27" s="39" t="s">
         <v>36</v>
@@ -10603,25 +10704,25 @@
         <v>36</v>
       </c>
       <c r="I27" s="40" t="s">
-        <v>1035</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
-        <v>1036</v>
+        <v>1059</v>
       </c>
       <c r="B28" s="39"/>
       <c r="C28" s="39" t="s">
-        <v>1037</v>
+        <v>1060</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E28" s="39" t="s">
-        <v>1038</v>
+        <v>1061</v>
       </c>
       <c r="F28" s="39" t="s">
-        <v>1039</v>
+        <v>1062</v>
       </c>
       <c r="G28" s="39" t="s">
         <v>36</v>
@@ -10630,25 +10731,25 @@
         <v>36</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>1040</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
-        <v>1041</v>
+        <v>1064</v>
       </c>
       <c r="B29" s="39"/>
       <c r="C29" s="39" t="s">
-        <v>1042</v>
+        <v>1065</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>1043</v>
+        <v>1066</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>1044</v>
+        <v>1067</v>
       </c>
       <c r="G29" s="39" t="s">
         <v>36</v>
@@ -10657,25 +10758,25 @@
         <v>36</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>1045</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
-        <v>1046</v>
+        <v>1069</v>
       </c>
       <c r="B30" s="39"/>
       <c r="C30" s="39" t="s">
-        <v>1047</v>
+        <v>1070</v>
       </c>
       <c r="D30" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E30" s="39" t="s">
-        <v>1048</v>
+        <v>1071</v>
       </c>
       <c r="F30" s="39" t="s">
-        <v>1049</v>
+        <v>1072</v>
       </c>
       <c r="G30" s="39" t="s">
         <v>36</v>
@@ -10684,25 +10785,25 @@
         <v>36</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>1050</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="38" t="s">
-        <v>1051</v>
+        <v>1074</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39" t="s">
-        <v>957</v>
+        <v>979</v>
       </c>
       <c r="D31" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E31" s="39" t="s">
-        <v>1052</v>
+        <v>1075</v>
       </c>
       <c r="F31" s="39" t="s">
-        <v>1053</v>
+        <v>1076</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>36</v>
@@ -10711,25 +10812,25 @@
         <v>36</v>
       </c>
       <c r="I31" s="40" t="s">
-        <v>1054</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="38" t="s">
-        <v>1055</v>
+        <v>1078</v>
       </c>
       <c r="B32" s="39"/>
       <c r="C32" s="39" t="s">
-        <v>1056</v>
+        <v>1079</v>
       </c>
       <c r="D32" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E32" s="39" t="s">
-        <v>1057</v>
+        <v>1080</v>
       </c>
       <c r="F32" s="39" t="s">
-        <v>1058</v>
+        <v>1081</v>
       </c>
       <c r="G32" s="39" t="s">
         <v>36</v>
@@ -10738,25 +10839,25 @@
         <v>36</v>
       </c>
       <c r="I32" s="40" t="s">
-        <v>1059</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="38" t="s">
-        <v>1060</v>
+        <v>1083</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39" t="s">
-        <v>1061</v>
+        <v>1084</v>
       </c>
       <c r="D33" s="39" t="s">
-        <v>968</v>
+        <v>990</v>
       </c>
       <c r="E33" s="39" t="s">
-        <v>1062</v>
+        <v>1085</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>1063</v>
+        <v>1086</v>
       </c>
       <c r="G33" s="39" t="s">
         <v>36</v>
@@ -10765,7 +10866,7 @@
         <v>36</v>
       </c>
       <c r="I33" s="40" t="s">
-        <v>1064</v>
+        <v>1087</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement explicit data initialization
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2036" uniqueCount="1088">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="1096">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -2250,156 +2250,180 @@
     <t>Data initialization</t>
   </si>
   <si>
+    <t>Operator initializes CICS DB2 banking data</t>
+  </si>
+  <si>
+    <t>Delete existing CUSTOMER/ACCOUNT/CONTROL rows, then generate and load a requested customer/account range.</t>
+  </si>
+  <si>
+    <t>The legacy demo utility is destructive and accepts start/end/step/random-seed parameters.</t>
+  </si>
+  <si>
+    <t>CUSTOMER and ACCOUNT rows are created according to start/end/step/random-seed parameters.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/cics/cobol/BANKDATA.cbl; legacy/.setup/jcl/cics/Db2-insert.j2; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decisions D-013/D-021: explicit guarded deterministic reset/import replaces destructive startup-style loading.</t>
+  </si>
+  <si>
+    <t>modern/backend/tools/BankOfZ.Setup/DemoResetService.cs; DemoPackageFactory.cs; SetupAuthorizationTests.cs; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>specs/008-data-initialization/spec.md; plan.md; tasks.md</t>
+  </si>
+  <si>
+    <t>Operator loads IMS customers</t>
+  </si>
+  <si>
+    <t>Load customer input records into the IMS customer segment.</t>
+  </si>
+  <si>
+    <t>The IMS datastore can be initialized from sequential input.</t>
+  </si>
+  <si>
+    <t>Valid input rows are inserted and loader diagnostics are emitted.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/LOADCUST.cbl; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decisions D-013/D-021: staged validation and atomic promotion replace partial legacy loading.</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Infrastructure/DataInitialization/DataImportService.cs; ImportPackageValidator.cs; Customer.cs; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>Operator loads IMS accounts</t>
+  </si>
+  <si>
+    <t>Load account input records into IMS account segments.</t>
+  </si>
+  <si>
+    <t>Customer portfolios can be initialized for IMS scenarios.</t>
+  </si>
+  <si>
+    <t>Valid account rows are inserted and loader diagnostics are emitted.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/LOADACCT.cbl; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>modern/backend/src/BankOfZ.Infrastructure/DataInitialization/DataImportService.cs; Account.cs; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>Operator loads IMS customer-account relationships</t>
+  </si>
+  <si>
+    <t>Load links between IMS customers and their account identifiers.</t>
+  </si>
+  <si>
+    <t>IMS account lookup depends on relationship segments in addition to customer and account records.</t>
+  </si>
+  <si>
+    <t>Valid relationship rows are inserted and loader diagnostics are emitted.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/LOADCUSA.cbl; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>ImportPackage.cs account.customerId ownership contract; ImportPackageValidator.cs FK validation; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>Operator loads IMS history</t>
+  </si>
+  <si>
+    <t>Load transaction-history input into IMS history segments.</t>
+  </si>
+  <si>
+    <t>Historical activity can be initialized with the account data.</t>
+  </si>
+  <si>
+    <t>Valid history rows are inserted and loader diagnostics are emitted.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/LOADHIST.cbl; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>BookedTransaction.cs; DataImportService.cs; ImportPackageValidator.cs running-balance validation; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>Operator loads IMS transaction-status data</t>
+  </si>
+  <si>
+    <t>Load transaction status, timing, and customer linkage into IMS status segments.</t>
+  </si>
+  <si>
+    <t>IMS transaction state data is prepared separately from financial history.</t>
+  </si>
+  <si>
+    <t>Valid status rows are inserted and loader diagnostics are emitted.</t>
+  </si>
+  <si>
+    <t>legacy/src/base/ims/cobol/LOADTSTA.cbl; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decisions D-013/D-021: target import includes legacy transaction-run status through staged atomic promotion.</t>
+  </si>
+  <si>
+    <t>LegacyTransactionRun.cs; LegacyTransactionRunConfiguration.cs; DataImportService.cs; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>Operator stages IMS reference data without loading it</t>
+  </si>
+  <si>
+    <t>Stage ACCTYPE, CUSTTYPE, TSTATTYP, and TTYPE inputs without claiming that the supplied population flow loads them.</t>
+  </si>
+  <si>
+    <t>The setup script creates datasets for four IMS reference-data files but submits loaders only for the five application datasets.</t>
+  </si>
+  <si>
+    <t>Reference inputs are staged, but no active loader job in the supplied population flow inserts them; this is a partial deployment surface.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/setup/populate-ims-tables.sh:27-52; legacy/src/base/ims/LoadData/ACCTYPE.data; legacy/src/base/ims/LoadData/CUSTTYPE.data; legacy/src/base/ims/LoadData/TSTATTYP.data; legacy/src/base/ims/LoadData/TTYPE.data; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decisions D-013/D-021: explicit import validates supported reference data before atomic promotion.</t>
+  </si>
+  <si>
+    <t>ImportReferenceValue.cs; ImportReferenceValueConfiguration.cs; DataImportService.cs; DataInitializationTests.cs</t>
+  </si>
+  <si>
+    <t>Operator prepares DB2 structures and access</t>
+  </si>
+  <si>
+    <t>Create/drop tables, grant access, and bind required plans through deployment JCL.</t>
+  </si>
+  <si>
+    <t>Programs require schema and plan preparation before transactions run.</t>
+  </si>
+  <si>
+    <t>The configured DB2 objects and plans are created/bound for CICS and IMS modules.</t>
+  </si>
+  <si>
+    <t>legacy/.setup/jcl/cics/Db2-*.j2; legacy/.setup/jcl/ims/Db2-*.j2; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>Decisions D-013/D-021: explicit migrations/import use least-privilege operator credentials, not PUBLIC grants.</t>
+  </si>
+  <si>
+    <t>20260723140526_AddDataInitialization.cs; DataInitializationMigrationTests.cs; DatabaseAccessProvisioner.cs; modern/README.md</t>
+  </si>
+  <si>
+    <t>UF-012</t>
+  </si>
+  <si>
+    <t>Runtime deployment, resilience, and security observations</t>
+  </si>
+  <si>
     <t>Not Passed - Open</t>
   </si>
   <si>
     <t>Legacy behavior is evidenced and covered by SDD; target implementation has not started.</t>
   </si>
   <si>
-    <t>Operator initializes CICS DB2 banking data</t>
-  </si>
-  <si>
-    <t>Delete existing CUSTOMER/ACCOUNT/CONTROL rows, then generate and load a requested customer/account range.</t>
-  </si>
-  <si>
-    <t>The legacy demo utility is destructive and accepts start/end/step/random-seed parameters.</t>
-  </si>
-  <si>
-    <t>CUSTOMER and ACCOUNT rows are created according to start/end/step/random-seed parameters.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/cics/cobol/BANKDATA.cbl; legacy/.setup/jcl/cics/Db2-insert.j2; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decisions D-013/D-021: explicit guarded deterministic reset/import replaces destructive startup-style loading.</t>
-  </si>
-  <si>
-    <t>specs/008-data-initialization/spec.md; plan.md; tasks.md</t>
-  </si>
-  <si>
-    <t>Operator loads IMS customers</t>
-  </si>
-  <si>
-    <t>Load customer input records into the IMS customer segment.</t>
-  </si>
-  <si>
-    <t>The IMS datastore can be initialized from sequential input.</t>
-  </si>
-  <si>
-    <t>Valid input rows are inserted and loader diagnostics are emitted.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/LOADCUST.cbl; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decisions D-013/D-021: staged validation and atomic promotion replace partial legacy loading.</t>
-  </si>
-  <si>
-    <t>Operator loads IMS accounts</t>
-  </si>
-  <si>
-    <t>Load account input records into IMS account segments.</t>
-  </si>
-  <si>
-    <t>Customer portfolios can be initialized for IMS scenarios.</t>
-  </si>
-  <si>
-    <t>Valid account rows are inserted and loader diagnostics are emitted.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/LOADACCT.cbl; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Operator loads IMS customer-account relationships</t>
-  </si>
-  <si>
-    <t>Load links between IMS customers and their account identifiers.</t>
-  </si>
-  <si>
-    <t>IMS account lookup depends on relationship segments in addition to customer and account records.</t>
-  </si>
-  <si>
-    <t>Valid relationship rows are inserted and loader diagnostics are emitted.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/LOADCUSA.cbl; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Operator loads IMS history</t>
-  </si>
-  <si>
-    <t>Load transaction-history input into IMS history segments.</t>
-  </si>
-  <si>
-    <t>Historical activity can be initialized with the account data.</t>
-  </si>
-  <si>
-    <t>Valid history rows are inserted and loader diagnostics are emitted.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/LOADHIST.cbl; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Operator loads IMS transaction-status data</t>
-  </si>
-  <si>
-    <t>Load transaction status, timing, and customer linkage into IMS status segments.</t>
-  </si>
-  <si>
-    <t>IMS transaction state data is prepared separately from financial history.</t>
-  </si>
-  <si>
-    <t>Valid status rows are inserted and loader diagnostics are emitted.</t>
-  </si>
-  <si>
-    <t>legacy/src/base/ims/cobol/LOADTSTA.cbl; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decisions D-013/D-021: target import includes legacy transaction-run status through staged atomic promotion.</t>
-  </si>
-  <si>
-    <t>Operator stages IMS reference data without loading it</t>
-  </si>
-  <si>
-    <t>Stage ACCTYPE, CUSTTYPE, TSTATTYP, and TTYPE inputs without claiming that the supplied population flow loads them.</t>
-  </si>
-  <si>
-    <t>The setup script creates datasets for four IMS reference-data files but submits loaders only for the five application datasets.</t>
-  </si>
-  <si>
-    <t>Reference inputs are staged, but no active loader job in the supplied population flow inserts them; this is a partial deployment surface.</t>
-  </si>
-  <si>
-    <t>legacy/.setup/setup/populate-ims-tables.sh:27-52; legacy/src/base/ims/LoadData/ACCTYPE.data; legacy/src/base/ims/LoadData/CUSTTYPE.data; legacy/src/base/ims/LoadData/TSTATTYP.data; legacy/src/base/ims/LoadData/TTYPE.data; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decisions D-013/D-021: explicit import validates supported reference data before atomic promotion.</t>
-  </si>
-  <si>
-    <t>Operator prepares DB2 structures and access</t>
-  </si>
-  <si>
-    <t>Create/drop tables, grant access, and bind required plans through deployment JCL.</t>
-  </si>
-  <si>
-    <t>Programs require schema and plan preparation before transactions run.</t>
-  </si>
-  <si>
-    <t>The configured DB2 objects and plans are created/bound for CICS and IMS modules.</t>
-  </si>
-  <si>
-    <t>legacy/.setup/jcl/cics/Db2-*.j2; legacy/.setup/jcl/ims/Db2-*.j2; Runtime: static-only</t>
-  </si>
-  <si>
-    <t>Decisions D-013/D-021: explicit migrations/import use least-privilege operator credentials, not PUBLIC grants.</t>
-  </si>
-  <si>
-    <t>UF-012</t>
-  </si>
-  <si>
-    <t>Runtime deployment, resilience, and security observations</t>
-  </si>
-  <si>
     <t>Operator starts web and z/OS Connect containers</t>
   </si>
   <si>
@@ -2964,7 +2988,7 @@
     <t>Implement Feature 008 explicit migrations and import.</t>
   </si>
   <si>
-    <t>Not checked: target implementation has not started. specs/008-data-initialization/</t>
+    <t>Feature 008 implemented and peer-reviewed. specs/008-data-initialization/; analysis/reviews/feature-008-implementation-review.md; modern/backend/tools/BankOfZ.Setup/; DataInitializationTests.cs; DataInitializationMigrationTests.cs</t>
   </si>
   <si>
     <t>R1-G09</t>
@@ -3629,7 +3653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3714,15 +3738,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8591,103 +8606,111 @@
       </c>
     </row>
     <row r="118" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A118" s="21" t="s">
+      <c r="A118" s="17" t="s">
         <v>742</v>
       </c>
-      <c r="B118" s="21" t="s">
+      <c r="B118" s="17" t="s">
         <v>743</v>
       </c>
-      <c r="C118" s="21" t="s">
-        <v>744</v>
-      </c>
-      <c r="D118" s="21" t="s">
-        <v>745</v>
-      </c>
-      <c r="E118" s="21"/>
-      <c r="F118" s="21"/>
-      <c r="G118" s="21"/>
-      <c r="H118" s="21"/>
-      <c r="I118" s="21"/>
-      <c r="J118" s="21"/>
-      <c r="K118" s="21"/>
-      <c r="L118" s="21"/>
-      <c r="M118" s="21"/>
-      <c r="N118" s="21"/>
+      <c r="C118" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D118" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E118" s="17"/>
+      <c r="F118" s="17"/>
+      <c r="G118" s="17"/>
+      <c r="H118" s="17"/>
+      <c r="I118" s="17"/>
+      <c r="J118" s="17"/>
+      <c r="K118" s="17"/>
+      <c r="L118" s="17"/>
+      <c r="M118" s="17"/>
+      <c r="N118" s="17"/>
     </row>
     <row r="119" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A119" s="18"/>
       <c r="B119" s="19" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="C119" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D119" s="22" t="s">
+      <c r="D119" s="20" t="s">
+        <v>745</v>
+      </c>
+      <c r="E119" s="20" t="s">
+        <v>746</v>
+      </c>
+      <c r="F119" s="20" t="s">
         <v>747</v>
       </c>
-      <c r="E119" s="22" t="s">
+      <c r="G119" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H119" s="20" t="s">
         <v>748</v>
       </c>
-      <c r="F119" s="22" t="s">
+      <c r="I119" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J119" s="20" t="s">
         <v>749</v>
       </c>
-      <c r="G119" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H119" s="22" t="s">
+      <c r="K119" s="20" t="s">
         <v>750</v>
       </c>
-      <c r="I119" s="22"/>
-      <c r="J119" s="22" t="s">
+      <c r="L119" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M119" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N119" s="20" t="s">
         <v>751</v>
-      </c>
-      <c r="K119" s="22"/>
-      <c r="L119" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M119" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N119" s="22" t="s">
-        <v>752</v>
       </c>
     </row>
     <row r="120" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A120" s="18"/>
       <c r="B120" s="19" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C120" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D120" s="22" t="s">
+      <c r="D120" s="20" t="s">
+        <v>753</v>
+      </c>
+      <c r="E120" s="20" t="s">
         <v>754</v>
       </c>
-      <c r="E120" s="22" t="s">
+      <c r="F120" s="20" t="s">
         <v>755</v>
       </c>
-      <c r="F120" s="22" t="s">
+      <c r="G120" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H120" s="20" t="s">
         <v>756</v>
       </c>
-      <c r="G120" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H120" s="22" t="s">
+      <c r="I120" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J120" s="20" t="s">
         <v>757</v>
       </c>
-      <c r="I120" s="22"/>
-      <c r="J120" s="22" t="s">
+      <c r="K120" s="20" t="s">
         <v>758</v>
       </c>
-      <c r="K120" s="22"/>
-      <c r="L120" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M120" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N120" s="22" t="s">
-        <v>752</v>
+      <c r="L120" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M120" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N120" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
@@ -8698,238 +8721,262 @@
       <c r="C121" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D121" s="22" t="s">
+      <c r="D121" s="20" t="s">
         <v>760</v>
       </c>
-      <c r="E121" s="22" t="s">
+      <c r="E121" s="20" t="s">
         <v>761</v>
       </c>
-      <c r="F121" s="22" t="s">
+      <c r="F121" s="20" t="s">
         <v>762</v>
       </c>
-      <c r="G121" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H121" s="22" t="s">
+      <c r="G121" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H121" s="20" t="s">
         <v>763</v>
       </c>
-      <c r="I121" s="22"/>
-      <c r="J121" s="22" t="s">
-        <v>758</v>
-      </c>
-      <c r="K121" s="22"/>
-      <c r="L121" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M121" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N121" s="22" t="s">
-        <v>752</v>
+      <c r="I121" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J121" s="20" t="s">
+        <v>757</v>
+      </c>
+      <c r="K121" s="20" t="s">
+        <v>764</v>
+      </c>
+      <c r="L121" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M121" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N121" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="122" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A122" s="18"/>
       <c r="B122" s="19" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="C122" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D122" s="22" t="s">
-        <v>765</v>
-      </c>
-      <c r="E122" s="22" t="s">
+      <c r="D122" s="20" t="s">
         <v>766</v>
       </c>
-      <c r="F122" s="22" t="s">
+      <c r="E122" s="20" t="s">
         <v>767</v>
       </c>
-      <c r="G122" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H122" s="22" t="s">
+      <c r="F122" s="20" t="s">
         <v>768</v>
       </c>
-      <c r="I122" s="22"/>
-      <c r="J122" s="22" t="s">
-        <v>758</v>
-      </c>
-      <c r="K122" s="22"/>
-      <c r="L122" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M122" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N122" s="22" t="s">
-        <v>752</v>
+      <c r="G122" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H122" s="20" t="s">
+        <v>769</v>
+      </c>
+      <c r="I122" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J122" s="20" t="s">
+        <v>757</v>
+      </c>
+      <c r="K122" s="20" t="s">
+        <v>770</v>
+      </c>
+      <c r="L122" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M122" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N122" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="123" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A123" s="18"/>
       <c r="B123" s="19" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="C123" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D123" s="22" t="s">
-        <v>770</v>
-      </c>
-      <c r="E123" s="22" t="s">
-        <v>771</v>
-      </c>
-      <c r="F123" s="22" t="s">
+      <c r="D123" s="20" t="s">
         <v>772</v>
       </c>
-      <c r="G123" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H123" s="22" t="s">
+      <c r="E123" s="20" t="s">
         <v>773</v>
       </c>
-      <c r="I123" s="22"/>
-      <c r="J123" s="22" t="s">
-        <v>758</v>
-      </c>
-      <c r="K123" s="22"/>
-      <c r="L123" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M123" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N123" s="22" t="s">
-        <v>752</v>
+      <c r="F123" s="20" t="s">
+        <v>774</v>
+      </c>
+      <c r="G123" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H123" s="20" t="s">
+        <v>775</v>
+      </c>
+      <c r="I123" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J123" s="20" t="s">
+        <v>757</v>
+      </c>
+      <c r="K123" s="20" t="s">
+        <v>776</v>
+      </c>
+      <c r="L123" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M123" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N123" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="124" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A124" s="18"/>
       <c r="B124" s="19" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="C124" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D124" s="22" t="s">
-        <v>775</v>
-      </c>
-      <c r="E124" s="22" t="s">
-        <v>776</v>
-      </c>
-      <c r="F124" s="22" t="s">
-        <v>777</v>
-      </c>
-      <c r="G124" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H124" s="22" t="s">
+      <c r="D124" s="20" t="s">
         <v>778</v>
       </c>
-      <c r="I124" s="22"/>
-      <c r="J124" s="22" t="s">
+      <c r="E124" s="20" t="s">
         <v>779</v>
       </c>
-      <c r="K124" s="22"/>
-      <c r="L124" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M124" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N124" s="22" t="s">
-        <v>752</v>
+      <c r="F124" s="20" t="s">
+        <v>780</v>
+      </c>
+      <c r="G124" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H124" s="20" t="s">
+        <v>781</v>
+      </c>
+      <c r="I124" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J124" s="20" t="s">
+        <v>782</v>
+      </c>
+      <c r="K124" s="20" t="s">
+        <v>783</v>
+      </c>
+      <c r="L124" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M124" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N124" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="125" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A125" s="18"/>
       <c r="B125" s="19" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="C125" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D125" s="22" t="s">
-        <v>781</v>
-      </c>
-      <c r="E125" s="22" t="s">
-        <v>782</v>
-      </c>
-      <c r="F125" s="22" t="s">
-        <v>783</v>
-      </c>
-      <c r="G125" s="22" t="s">
+      <c r="D125" s="20" t="s">
+        <v>785</v>
+      </c>
+      <c r="E125" s="20" t="s">
+        <v>786</v>
+      </c>
+      <c r="F125" s="20" t="s">
+        <v>787</v>
+      </c>
+      <c r="G125" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H125" s="22" t="s">
-        <v>784</v>
-      </c>
-      <c r="I125" s="22"/>
-      <c r="J125" s="22" t="s">
-        <v>785</v>
-      </c>
-      <c r="K125" s="22"/>
-      <c r="L125" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M125" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N125" s="22" t="s">
-        <v>752</v>
+      <c r="H125" s="20" t="s">
+        <v>788</v>
+      </c>
+      <c r="I125" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J125" s="20" t="s">
+        <v>789</v>
+      </c>
+      <c r="K125" s="20" t="s">
+        <v>790</v>
+      </c>
+      <c r="L125" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M125" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N125" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="126" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A126" s="18"/>
       <c r="B126" s="19" t="s">
-        <v>786</v>
+        <v>791</v>
       </c>
       <c r="C126" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D126" s="22" t="s">
-        <v>787</v>
-      </c>
-      <c r="E126" s="22" t="s">
-        <v>788</v>
-      </c>
-      <c r="F126" s="22" t="s">
-        <v>789</v>
-      </c>
-      <c r="G126" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H126" s="22" t="s">
-        <v>790</v>
-      </c>
-      <c r="I126" s="22"/>
-      <c r="J126" s="22" t="s">
-        <v>791</v>
-      </c>
-      <c r="K126" s="22"/>
-      <c r="L126" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M126" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N126" s="22" t="s">
-        <v>752</v>
+      <c r="D126" s="20" t="s">
+        <v>792</v>
+      </c>
+      <c r="E126" s="20" t="s">
+        <v>793</v>
+      </c>
+      <c r="F126" s="20" t="s">
+        <v>794</v>
+      </c>
+      <c r="G126" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H126" s="20" t="s">
+        <v>795</v>
+      </c>
+      <c r="I126" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J126" s="20" t="s">
+        <v>796</v>
+      </c>
+      <c r="K126" s="20" t="s">
+        <v>797</v>
+      </c>
+      <c r="L126" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M126" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N126" s="20" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="21" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="B127" s="21" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C127" s="21" t="s">
-        <v>744</v>
+        <v>800</v>
       </c>
       <c r="D127" s="21" t="s">
-        <v>745</v>
+        <v>801</v>
       </c>
       <c r="E127" s="21"/>
       <c r="F127" s="21"/>
@@ -8945,29 +8992,29 @@
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D128" s="22" t="s">
-        <v>795</v>
+        <v>803</v>
       </c>
       <c r="E128" s="22" t="s">
-        <v>796</v>
+        <v>804</v>
       </c>
       <c r="F128" s="22" t="s">
-        <v>797</v>
+        <v>805</v>
       </c>
       <c r="G128" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H128" s="22" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
       <c r="I128" s="22"/>
       <c r="J128" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K128" s="22"/>
       <c r="L128" s="22" t="s">
@@ -8977,35 +9024,35 @@
         <v>40</v>
       </c>
       <c r="N128" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>801</v>
+        <v>809</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D129" s="22" t="s">
-        <v>802</v>
+        <v>810</v>
       </c>
       <c r="E129" s="22" t="s">
-        <v>803</v>
+        <v>811</v>
       </c>
       <c r="F129" s="22" t="s">
-        <v>804</v>
+        <v>812</v>
       </c>
       <c r="G129" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H129" s="22" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="I129" s="22"/>
       <c r="J129" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K129" s="22"/>
       <c r="L129" s="22" t="s">
@@ -9015,35 +9062,35 @@
         <v>40</v>
       </c>
       <c r="N129" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A130" s="18"/>
       <c r="B130" s="19" t="s">
-        <v>806</v>
+        <v>814</v>
       </c>
       <c r="C130" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D130" s="22" t="s">
-        <v>807</v>
+        <v>815</v>
       </c>
       <c r="E130" s="22" t="s">
-        <v>808</v>
+        <v>816</v>
       </c>
       <c r="F130" s="22" t="s">
-        <v>809</v>
+        <v>817</v>
       </c>
       <c r="G130" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H130" s="22" t="s">
-        <v>810</v>
+        <v>818</v>
       </c>
       <c r="I130" s="22"/>
       <c r="J130" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K130" s="22"/>
       <c r="L130" s="22" t="s">
@@ -9053,35 +9100,35 @@
         <v>40</v>
       </c>
       <c r="N130" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>811</v>
+        <v>819</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D131" s="22" t="s">
-        <v>812</v>
+        <v>820</v>
       </c>
       <c r="E131" s="22" t="s">
-        <v>813</v>
+        <v>821</v>
       </c>
       <c r="F131" s="22" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
       <c r="G131" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H131" s="22" t="s">
-        <v>815</v>
+        <v>823</v>
       </c>
       <c r="I131" s="22"/>
       <c r="J131" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K131" s="22"/>
       <c r="L131" s="22" t="s">
@@ -9091,35 +9138,35 @@
         <v>40</v>
       </c>
       <c r="N131" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>816</v>
+        <v>824</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D132" s="22" t="s">
-        <v>817</v>
+        <v>825</v>
       </c>
       <c r="E132" s="22" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="F132" s="22" t="s">
-        <v>819</v>
+        <v>827</v>
       </c>
       <c r="G132" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H132" s="22" t="s">
-        <v>820</v>
+        <v>828</v>
       </c>
       <c r="I132" s="22"/>
       <c r="J132" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K132" s="22"/>
       <c r="L132" s="22" t="s">
@@ -9129,35 +9176,35 @@
         <v>40</v>
       </c>
       <c r="N132" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>821</v>
+        <v>829</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D133" s="22" t="s">
-        <v>822</v>
+        <v>830</v>
       </c>
       <c r="E133" s="22" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
       <c r="F133" s="22" t="s">
-        <v>824</v>
+        <v>832</v>
       </c>
       <c r="G133" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H133" s="22" t="s">
-        <v>825</v>
+        <v>833</v>
       </c>
       <c r="I133" s="22"/>
       <c r="J133" s="22" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="K133" s="22"/>
       <c r="L133" s="22" t="s">
@@ -9167,35 +9214,35 @@
         <v>40</v>
       </c>
       <c r="N133" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>827</v>
+        <v>835</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D134" s="22" t="s">
-        <v>828</v>
+        <v>836</v>
       </c>
       <c r="E134" s="22" t="s">
-        <v>829</v>
+        <v>837</v>
       </c>
       <c r="F134" s="22" t="s">
-        <v>830</v>
+        <v>838</v>
       </c>
       <c r="G134" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H134" s="22" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
       <c r="I134" s="22"/>
       <c r="J134" s="22" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
       <c r="K134" s="22"/>
       <c r="L134" s="22" t="s">
@@ -9205,35 +9252,35 @@
         <v>40</v>
       </c>
       <c r="N134" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>833</v>
+        <v>841</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D135" s="22" t="s">
-        <v>834</v>
+        <v>842</v>
       </c>
       <c r="E135" s="22" t="s">
-        <v>835</v>
+        <v>843</v>
       </c>
       <c r="F135" s="22" t="s">
-        <v>836</v>
+        <v>844</v>
       </c>
       <c r="G135" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H135" s="22" t="s">
-        <v>837</v>
+        <v>845</v>
       </c>
       <c r="I135" s="22"/>
       <c r="J135" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K135" s="22"/>
       <c r="L135" s="22" t="s">
@@ -9243,35 +9290,35 @@
         <v>40</v>
       </c>
       <c r="N135" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>838</v>
+        <v>846</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D136" s="22" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
       <c r="E136" s="22" t="s">
-        <v>840</v>
+        <v>848</v>
       </c>
       <c r="F136" s="22" t="s">
-        <v>841</v>
+        <v>849</v>
       </c>
       <c r="G136" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H136" s="22" t="s">
-        <v>842</v>
+        <v>850</v>
       </c>
       <c r="I136" s="22"/>
       <c r="J136" s="22" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="K136" s="22"/>
       <c r="L136" s="22" t="s">
@@ -9281,35 +9328,35 @@
         <v>40</v>
       </c>
       <c r="N136" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D137" s="22" t="s">
-        <v>845</v>
+        <v>853</v>
       </c>
       <c r="E137" s="22" t="s">
-        <v>846</v>
+        <v>854</v>
       </c>
       <c r="F137" s="22" t="s">
-        <v>847</v>
+        <v>855</v>
       </c>
       <c r="G137" s="22" t="s">
         <v>522</v>
       </c>
       <c r="H137" s="22" t="s">
-        <v>848</v>
+        <v>856</v>
       </c>
       <c r="I137" s="22"/>
       <c r="J137" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K137" s="22"/>
       <c r="L137" s="22" t="s">
@@ -9319,35 +9366,35 @@
         <v>40</v>
       </c>
       <c r="N137" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>849</v>
+        <v>857</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D138" s="22" t="s">
-        <v>850</v>
+        <v>858</v>
       </c>
       <c r="E138" s="22" t="s">
-        <v>851</v>
+        <v>859</v>
       </c>
       <c r="F138" s="22" t="s">
-        <v>852</v>
+        <v>860</v>
       </c>
       <c r="G138" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H138" s="22" t="s">
-        <v>853</v>
+        <v>861</v>
       </c>
       <c r="I138" s="22"/>
       <c r="J138" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K138" s="22"/>
       <c r="L138" s="22" t="s">
@@ -9357,35 +9404,35 @@
         <v>40</v>
       </c>
       <c r="N138" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>854</v>
+        <v>862</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D139" s="22" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="E139" s="22" t="s">
-        <v>856</v>
+        <v>864</v>
       </c>
       <c r="F139" s="22" t="s">
-        <v>857</v>
+        <v>865</v>
       </c>
       <c r="G139" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H139" s="22" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
       <c r="I139" s="22"/>
       <c r="J139" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K139" s="22"/>
       <c r="L139" s="22" t="s">
@@ -9395,35 +9442,35 @@
         <v>40</v>
       </c>
       <c r="N139" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>859</v>
+        <v>867</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D140" s="22" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="E140" s="22" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
       <c r="F140" s="22" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
       <c r="G140" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H140" s="22" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="I140" s="22"/>
       <c r="J140" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K140" s="22"/>
       <c r="L140" s="22" t="s">
@@ -9433,35 +9480,35 @@
         <v>40</v>
       </c>
       <c r="N140" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>864</v>
+        <v>872</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D141" s="22" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="E141" s="22" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
       <c r="F141" s="22" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
       <c r="G141" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H141" s="22" t="s">
-        <v>868</v>
+        <v>876</v>
       </c>
       <c r="I141" s="22"/>
       <c r="J141" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K141" s="22"/>
       <c r="L141" s="22" t="s">
@@ -9471,35 +9518,35 @@
         <v>40</v>
       </c>
       <c r="N141" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D142" s="22" t="s">
-        <v>870</v>
+        <v>878</v>
       </c>
       <c r="E142" s="22" t="s">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="F142" s="22" t="s">
-        <v>872</v>
+        <v>880</v>
       </c>
       <c r="G142" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H142" s="22" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="I142" s="22"/>
       <c r="J142" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K142" s="22"/>
       <c r="L142" s="22" t="s">
@@ -9509,35 +9556,35 @@
         <v>40</v>
       </c>
       <c r="N142" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>874</v>
+        <v>882</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D143" s="22" t="s">
-        <v>875</v>
+        <v>883</v>
       </c>
       <c r="E143" s="22" t="s">
-        <v>876</v>
+        <v>884</v>
       </c>
       <c r="F143" s="22" t="s">
-        <v>877</v>
+        <v>885</v>
       </c>
       <c r="G143" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H143" s="22" t="s">
-        <v>878</v>
+        <v>886</v>
       </c>
       <c r="I143" s="22"/>
       <c r="J143" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K143" s="22"/>
       <c r="L143" s="22" t="s">
@@ -9547,35 +9594,35 @@
         <v>40</v>
       </c>
       <c r="N143" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>879</v>
+        <v>887</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D144" s="22" t="s">
-        <v>880</v>
+        <v>888</v>
       </c>
       <c r="E144" s="22" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="F144" s="22" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
       <c r="G144" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H144" s="22" t="s">
-        <v>883</v>
+        <v>891</v>
       </c>
       <c r="I144" s="22"/>
       <c r="J144" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K144" s="22"/>
       <c r="L144" s="22" t="s">
@@ -9585,35 +9632,35 @@
         <v>40</v>
       </c>
       <c r="N144" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>884</v>
+        <v>892</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D145" s="22" t="s">
-        <v>885</v>
+        <v>893</v>
       </c>
       <c r="E145" s="22" t="s">
-        <v>886</v>
+        <v>894</v>
       </c>
       <c r="F145" s="22" t="s">
-        <v>887</v>
+        <v>895</v>
       </c>
       <c r="G145" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H145" s="22" t="s">
-        <v>888</v>
+        <v>896</v>
       </c>
       <c r="I145" s="22"/>
       <c r="J145" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K145" s="22"/>
       <c r="L145" s="22" t="s">
@@ -9623,35 +9670,35 @@
         <v>40</v>
       </c>
       <c r="N145" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>889</v>
+        <v>897</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D146" s="22" t="s">
-        <v>890</v>
+        <v>898</v>
       </c>
       <c r="E146" s="22" t="s">
-        <v>891</v>
+        <v>899</v>
       </c>
       <c r="F146" s="22" t="s">
-        <v>892</v>
+        <v>900</v>
       </c>
       <c r="G146" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H146" s="22" t="s">
-        <v>893</v>
+        <v>901</v>
       </c>
       <c r="I146" s="22"/>
       <c r="J146" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K146" s="22"/>
       <c r="L146" s="22" t="s">
@@ -9661,35 +9708,35 @@
         <v>40</v>
       </c>
       <c r="N146" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>894</v>
+        <v>902</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D147" s="22" t="s">
-        <v>895</v>
+        <v>903</v>
       </c>
       <c r="E147" s="22" t="s">
-        <v>896</v>
+        <v>904</v>
       </c>
       <c r="F147" s="22" t="s">
-        <v>897</v>
+        <v>905</v>
       </c>
       <c r="G147" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H147" s="22" t="s">
-        <v>898</v>
+        <v>906</v>
       </c>
       <c r="I147" s="22"/>
       <c r="J147" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K147" s="22"/>
       <c r="L147" s="22" t="s">
@@ -9699,35 +9746,35 @@
         <v>40</v>
       </c>
       <c r="N147" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>899</v>
+        <v>907</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D148" s="22" t="s">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="E148" s="22" t="s">
-        <v>901</v>
+        <v>909</v>
       </c>
       <c r="F148" s="22" t="s">
-        <v>902</v>
+        <v>910</v>
       </c>
       <c r="G148" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H148" s="22" t="s">
-        <v>903</v>
+        <v>911</v>
       </c>
       <c r="I148" s="22"/>
       <c r="J148" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K148" s="22"/>
       <c r="L148" s="22" t="s">
@@ -9737,35 +9784,35 @@
         <v>40</v>
       </c>
       <c r="N148" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>904</v>
+        <v>912</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D149" s="22" t="s">
-        <v>905</v>
+        <v>913</v>
       </c>
       <c r="E149" s="22" t="s">
-        <v>906</v>
+        <v>914</v>
       </c>
       <c r="F149" s="22" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="G149" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H149" s="22" t="s">
-        <v>908</v>
+        <v>916</v>
       </c>
       <c r="I149" s="22"/>
       <c r="J149" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K149" s="22"/>
       <c r="L149" s="22" t="s">
@@ -9775,35 +9822,35 @@
         <v>40</v>
       </c>
       <c r="N149" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>909</v>
+        <v>917</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D150" s="22" t="s">
-        <v>910</v>
+        <v>918</v>
       </c>
       <c r="E150" s="22" t="s">
-        <v>911</v>
+        <v>919</v>
       </c>
       <c r="F150" s="22" t="s">
-        <v>912</v>
+        <v>920</v>
       </c>
       <c r="G150" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H150" s="22" t="s">
-        <v>913</v>
+        <v>921</v>
       </c>
       <c r="I150" s="22"/>
       <c r="J150" s="22" t="s">
-        <v>914</v>
+        <v>922</v>
       </c>
       <c r="K150" s="22"/>
       <c r="L150" s="22" t="s">
@@ -9813,35 +9860,35 @@
         <v>40</v>
       </c>
       <c r="N150" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>915</v>
+        <v>923</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D151" s="22" t="s">
-        <v>916</v>
+        <v>924</v>
       </c>
       <c r="E151" s="22" t="s">
-        <v>917</v>
+        <v>925</v>
       </c>
       <c r="F151" s="22" t="s">
-        <v>918</v>
+        <v>926</v>
       </c>
       <c r="G151" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H151" s="22" t="s">
-        <v>919</v>
+        <v>927</v>
       </c>
       <c r="I151" s="22"/>
       <c r="J151" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K151" s="22"/>
       <c r="L151" s="22" t="s">
@@ -9851,35 +9898,35 @@
         <v>40</v>
       </c>
       <c r="N151" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>920</v>
+        <v>928</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>111</v>
       </c>
       <c r="D152" s="22" t="s">
-        <v>921</v>
+        <v>929</v>
       </c>
       <c r="E152" s="22" t="s">
-        <v>922</v>
+        <v>930</v>
       </c>
       <c r="F152" s="22" t="s">
-        <v>923</v>
+        <v>931</v>
       </c>
       <c r="G152" s="22" t="s">
         <v>158</v>
       </c>
       <c r="H152" s="22" t="s">
-        <v>924</v>
+        <v>932</v>
       </c>
       <c r="I152" s="22"/>
       <c r="J152" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K152" s="22"/>
       <c r="L152" s="22" t="s">
@@ -9889,35 +9936,35 @@
         <v>40</v>
       </c>
       <c r="N152" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>925</v>
+        <v>933</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>43</v>
       </c>
       <c r="D153" s="22" t="s">
-        <v>926</v>
+        <v>934</v>
       </c>
       <c r="E153" s="22" t="s">
-        <v>927</v>
+        <v>935</v>
       </c>
       <c r="F153" s="22" t="s">
-        <v>928</v>
+        <v>936</v>
       </c>
       <c r="G153" s="22" t="s">
         <v>522</v>
       </c>
       <c r="H153" s="22" t="s">
-        <v>929</v>
+        <v>937</v>
       </c>
       <c r="I153" s="22"/>
       <c r="J153" s="22" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="K153" s="22"/>
       <c r="L153" s="22" t="s">
@@ -9927,7 +9974,7 @@
         <v>40</v>
       </c>
       <c r="N153" s="22" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
     </row>
   </sheetData>
@@ -9960,51 +10007,51 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
-        <v>930</v>
+        <v>938</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>931</v>
+        <v>939</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>932</v>
+        <v>940</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>933</v>
+        <v>941</v>
       </c>
       <c r="E1" s="24" t="s">
-        <v>934</v>
+        <v>942</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>935</v>
+        <v>943</v>
       </c>
       <c r="G1" s="24" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="24" t="s">
-        <v>936</v>
+        <v>944</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>937</v>
+        <v>945</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>938</v>
+        <v>946</v>
       </c>
       <c r="B2" s="27" t="s">
-        <v>939</v>
+        <v>947</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>940</v>
+        <v>948</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>942</v>
+        <v>950</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>943</v>
+        <v>951</v>
       </c>
       <c r="G2" s="27" t="s">
         <v>36</v>
@@ -10013,27 +10060,27 @@
         <v>36</v>
       </c>
       <c r="I2" s="28" t="s">
-        <v>944</v>
+        <v>952</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
-        <v>945</v>
+        <v>953</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>947</v>
+        <v>955</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E3" s="30" t="s">
-        <v>948</v>
+        <v>956</v>
       </c>
       <c r="F3" s="30" t="s">
-        <v>949</v>
+        <v>957</v>
       </c>
       <c r="G3" s="30" t="s">
         <v>36</v>
@@ -10042,27 +10089,27 @@
         <v>36</v>
       </c>
       <c r="I3" s="31" t="s">
-        <v>950</v>
+        <v>958</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
-        <v>951</v>
+        <v>959</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>952</v>
+        <v>960</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>953</v>
+        <v>961</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>954</v>
+        <v>962</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>955</v>
+        <v>963</v>
       </c>
       <c r="G4" s="30" t="s">
         <v>36</v>
@@ -10071,27 +10118,27 @@
         <v>36</v>
       </c>
       <c r="I4" s="31" t="s">
-        <v>956</v>
+        <v>964</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
-        <v>957</v>
+        <v>965</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>958</v>
+        <v>966</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>959</v>
+        <v>967</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>960</v>
+        <v>968</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>961</v>
+        <v>969</v>
       </c>
       <c r="G5" s="30" t="s">
         <v>36</v>
@@ -10100,27 +10147,27 @@
         <v>36</v>
       </c>
       <c r="I5" s="31" t="s">
-        <v>962</v>
+        <v>970</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
-        <v>963</v>
+        <v>971</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>487</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>964</v>
+        <v>972</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>965</v>
+        <v>973</v>
       </c>
       <c r="F6" s="30" t="s">
-        <v>966</v>
+        <v>974</v>
       </c>
       <c r="G6" s="30" t="s">
         <v>36</v>
@@ -10129,27 +10176,27 @@
         <v>36</v>
       </c>
       <c r="I6" s="31" t="s">
-        <v>967</v>
+        <v>975</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="29" t="s">
-        <v>968</v>
+        <v>976</v>
       </c>
       <c r="B7" s="30" t="s">
         <v>533</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>969</v>
+        <v>977</v>
       </c>
       <c r="D7" s="30" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>970</v>
+        <v>978</v>
       </c>
       <c r="F7" s="30" t="s">
-        <v>971</v>
+        <v>979</v>
       </c>
       <c r="G7" s="30" t="s">
         <v>36</v>
@@ -10158,27 +10205,27 @@
         <v>36</v>
       </c>
       <c r="I7" s="31" t="s">
-        <v>972</v>
+        <v>980</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="29" t="s">
-        <v>973</v>
+        <v>981</v>
       </c>
       <c r="B8" s="30" t="s">
         <v>612</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>974</v>
+        <v>982</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>941</v>
+        <v>949</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>975</v>
+        <v>983</v>
       </c>
       <c r="F8" s="30" t="s">
-        <v>976</v>
+        <v>984</v>
       </c>
       <c r="G8" s="30" t="s">
         <v>36</v>
@@ -10187,83 +10234,83 @@
         <v>36</v>
       </c>
       <c r="I8" s="31" t="s">
-        <v>977</v>
+        <v>985</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
-        <v>978</v>
-      </c>
-      <c r="B9" s="33" t="s">
+      <c r="A9" s="29" t="s">
+        <v>986</v>
+      </c>
+      <c r="B9" s="30" t="s">
         <v>742</v>
       </c>
-      <c r="C9" s="33" t="s">
-        <v>979</v>
-      </c>
-      <c r="D9" s="33" t="s">
-        <v>941</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>980</v>
-      </c>
-      <c r="F9" s="33" t="s">
-        <v>981</v>
-      </c>
-      <c r="G9" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="I9" s="34" t="s">
-        <v>982</v>
+      <c r="C9" s="30" t="s">
+        <v>987</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>949</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>988</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>989</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="31" t="s">
+        <v>990</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="35" t="s">
-        <v>983</v>
-      </c>
-      <c r="B10" s="36" t="s">
-        <v>792</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>984</v>
-      </c>
-      <c r="D10" s="36" t="s">
-        <v>941</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>985</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>986</v>
-      </c>
-      <c r="G10" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="I10" s="37" t="s">
-        <v>987</v>
+      <c r="A10" s="32" t="s">
+        <v>991</v>
+      </c>
+      <c r="B10" s="33" t="s">
+        <v>798</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>992</v>
+      </c>
+      <c r="D10" s="33" t="s">
+        <v>949</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>993</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>994</v>
+      </c>
+      <c r="G10" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="34" t="s">
+        <v>995</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>988</v>
+        <v>996</v>
       </c>
       <c r="B11" s="27"/>
       <c r="C11" s="27" t="s">
-        <v>989</v>
+        <v>997</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>992</v>
+        <v>1000</v>
       </c>
       <c r="G11" s="27" t="s">
         <v>36</v>
@@ -10272,25 +10319,25 @@
         <v>36</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>993</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
-        <v>994</v>
+        <v>1002</v>
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="30" t="s">
-        <v>995</v>
+        <v>1003</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>36</v>
@@ -10299,25 +10346,25 @@
         <v>36</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>997</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
-        <v>998</v>
+        <v>1006</v>
       </c>
       <c r="B13" s="30"/>
       <c r="C13" s="30" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>998</v>
+      </c>
+      <c r="E13" s="30" t="s">
         <v>999</v>
       </c>
-      <c r="D13" s="30" t="s">
-        <v>990</v>
-      </c>
-      <c r="E13" s="30" t="s">
-        <v>991</v>
-      </c>
       <c r="F13" s="30" t="s">
-        <v>1000</v>
+        <v>1008</v>
       </c>
       <c r="G13" s="30" t="s">
         <v>36</v>
@@ -10326,25 +10373,25 @@
         <v>36</v>
       </c>
       <c r="I13" s="31" t="s">
-        <v>1001</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
-        <v>1002</v>
+        <v>1010</v>
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="30" t="s">
-        <v>1003</v>
+        <v>1011</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>1004</v>
+        <v>1012</v>
       </c>
       <c r="G14" s="30" t="s">
         <v>36</v>
@@ -10353,25 +10400,25 @@
         <v>36</v>
       </c>
       <c r="I14" s="31" t="s">
-        <v>1005</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
-        <v>1006</v>
+        <v>1014</v>
       </c>
       <c r="B15" s="30"/>
       <c r="C15" s="30" t="s">
-        <v>1007</v>
+        <v>1015</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E15" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>1008</v>
+        <v>1016</v>
       </c>
       <c r="G15" s="30" t="s">
         <v>36</v>
@@ -10380,25 +10427,25 @@
         <v>36</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>1009</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
-        <v>1010</v>
+        <v>1018</v>
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="30" t="s">
-        <v>1011</v>
+        <v>1019</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>1012</v>
+        <v>1020</v>
       </c>
       <c r="G16" s="30" t="s">
         <v>36</v>
@@ -10407,25 +10454,25 @@
         <v>36</v>
       </c>
       <c r="I16" s="31" t="s">
-        <v>1013</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="29" t="s">
-        <v>1014</v>
+        <v>1022</v>
       </c>
       <c r="B17" s="30"/>
       <c r="C17" s="30" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>1016</v>
+        <v>1024</v>
       </c>
       <c r="G17" s="30" t="s">
         <v>36</v>
@@ -10434,25 +10481,25 @@
         <v>36</v>
       </c>
       <c r="I17" s="31" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="30" t="s">
-        <v>1019</v>
+        <v>1027</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>1020</v>
+        <v>1028</v>
       </c>
       <c r="G18" s="30" t="s">
         <v>36</v>
@@ -10461,25 +10508,25 @@
         <v>36</v>
       </c>
       <c r="I18" s="31" t="s">
-        <v>1021</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="29" t="s">
-        <v>1022</v>
+        <v>1030</v>
       </c>
       <c r="B19" s="30"/>
       <c r="C19" s="30" t="s">
-        <v>1023</v>
+        <v>1031</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>1024</v>
+        <v>1032</v>
       </c>
       <c r="G19" s="30" t="s">
         <v>36</v>
@@ -10488,25 +10535,25 @@
         <v>36</v>
       </c>
       <c r="I19" s="31" t="s">
-        <v>1025</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
-        <v>1026</v>
+        <v>1034</v>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="30" t="s">
-        <v>1027</v>
+        <v>1035</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>1028</v>
+        <v>1036</v>
       </c>
       <c r="G20" s="30" t="s">
         <v>36</v>
@@ -10515,25 +10562,25 @@
         <v>36</v>
       </c>
       <c r="I20" s="31" t="s">
-        <v>1029</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="29" t="s">
-        <v>1030</v>
+        <v>1038</v>
       </c>
       <c r="B21" s="30"/>
       <c r="C21" s="30" t="s">
-        <v>1031</v>
+        <v>1039</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E21" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F21" s="30" t="s">
-        <v>1032</v>
+        <v>1040</v>
       </c>
       <c r="G21" s="30" t="s">
         <v>36</v>
@@ -10542,25 +10589,25 @@
         <v>36</v>
       </c>
       <c r="I21" s="31" t="s">
-        <v>1033</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
-        <v>1034</v>
+        <v>1042</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30" t="s">
-        <v>1035</v>
+        <v>1043</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>1036</v>
+        <v>1044</v>
       </c>
       <c r="G22" s="30" t="s">
         <v>36</v>
@@ -10569,25 +10616,25 @@
         <v>36</v>
       </c>
       <c r="I22" s="31" t="s">
-        <v>1037</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
-        <v>1038</v>
+        <v>1046</v>
       </c>
       <c r="B23" s="30"/>
       <c r="C23" s="30" t="s">
-        <v>979</v>
+        <v>987</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F23" s="30" t="s">
-        <v>1039</v>
+        <v>1047</v>
       </c>
       <c r="G23" s="30" t="s">
         <v>36</v>
@@ -10596,25 +10643,25 @@
         <v>36</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>1040</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
-        <v>1041</v>
+        <v>1049</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30" t="s">
-        <v>1042</v>
+        <v>1050</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>990</v>
+        <v>998</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>991</v>
+        <v>999</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>1043</v>
+        <v>1051</v>
       </c>
       <c r="G24" s="30" t="s">
         <v>36</v>
@@ -10623,250 +10670,250 @@
         <v>36</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>1044</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="38" t="s">
-        <v>1045</v>
-      </c>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39" t="s">
-        <v>1046</v>
-      </c>
-      <c r="D25" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E25" s="39" t="s">
-        <v>991</v>
-      </c>
-      <c r="F25" s="39" t="s">
-        <v>1047</v>
-      </c>
-      <c r="G25" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="40" t="s">
-        <v>1048</v>
+      <c r="A25" s="35" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D25" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E25" s="36" t="s">
+        <v>999</v>
+      </c>
+      <c r="F25" s="36" t="s">
+        <v>1055</v>
+      </c>
+      <c r="G25" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>1056</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="38" t="s">
-        <v>1049</v>
-      </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39" t="s">
-        <v>1050</v>
-      </c>
-      <c r="D26" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E26" s="39" t="s">
-        <v>1051</v>
-      </c>
-      <c r="F26" s="39" t="s">
-        <v>1052</v>
-      </c>
-      <c r="G26" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I26" s="40" t="s">
-        <v>1053</v>
+      <c r="A26" s="35" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D26" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E26" s="36" t="s">
+        <v>1059</v>
+      </c>
+      <c r="F26" s="36" t="s">
+        <v>1060</v>
+      </c>
+      <c r="G26" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="37" t="s">
+        <v>1061</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="38" t="s">
-        <v>1054</v>
-      </c>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39" t="s">
-        <v>1055</v>
-      </c>
-      <c r="D27" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E27" s="39" t="s">
-        <v>1056</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>1057</v>
-      </c>
-      <c r="G27" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H27" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I27" s="40" t="s">
-        <v>1058</v>
+      <c r="A27" s="35" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36" t="s">
+        <v>1063</v>
+      </c>
+      <c r="D27" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E27" s="36" t="s">
+        <v>1064</v>
+      </c>
+      <c r="F27" s="36" t="s">
+        <v>1065</v>
+      </c>
+      <c r="G27" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H27" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>1066</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="38" t="s">
-        <v>1059</v>
-      </c>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39" t="s">
-        <v>1060</v>
-      </c>
-      <c r="D28" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E28" s="39" t="s">
-        <v>1061</v>
-      </c>
-      <c r="F28" s="39" t="s">
-        <v>1062</v>
-      </c>
-      <c r="G28" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="40" t="s">
-        <v>1063</v>
+      <c r="A28" s="35" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D28" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E28" s="36" t="s">
+        <v>1069</v>
+      </c>
+      <c r="F28" s="36" t="s">
+        <v>1070</v>
+      </c>
+      <c r="G28" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="37" t="s">
+        <v>1071</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="38" t="s">
-        <v>1064</v>
-      </c>
-      <c r="B29" s="39"/>
-      <c r="C29" s="39" t="s">
-        <v>1065</v>
-      </c>
-      <c r="D29" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E29" s="39" t="s">
-        <v>1066</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>1067</v>
-      </c>
-      <c r="G29" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H29" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29" s="40" t="s">
-        <v>1068</v>
+      <c r="A29" s="35" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36" t="s">
+        <v>1073</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E29" s="36" t="s">
+        <v>1074</v>
+      </c>
+      <c r="F29" s="36" t="s">
+        <v>1075</v>
+      </c>
+      <c r="G29" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>1076</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="38" t="s">
-        <v>1069</v>
-      </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39" t="s">
-        <v>1070</v>
-      </c>
-      <c r="D30" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E30" s="39" t="s">
-        <v>1071</v>
-      </c>
-      <c r="F30" s="39" t="s">
-        <v>1072</v>
-      </c>
-      <c r="G30" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="40" t="s">
-        <v>1073</v>
+      <c r="A30" s="35" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36" t="s">
+        <v>1078</v>
+      </c>
+      <c r="D30" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E30" s="36" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F30" s="36" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G30" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H30" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>1081</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="38" t="s">
-        <v>1074</v>
-      </c>
-      <c r="B31" s="39"/>
-      <c r="C31" s="39" t="s">
-        <v>979</v>
-      </c>
-      <c r="D31" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E31" s="39" t="s">
-        <v>1075</v>
-      </c>
-      <c r="F31" s="39" t="s">
-        <v>1076</v>
-      </c>
-      <c r="G31" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H31" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I31" s="40" t="s">
-        <v>1077</v>
+      <c r="A31" s="35" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B31" s="36"/>
+      <c r="C31" s="36" t="s">
+        <v>987</v>
+      </c>
+      <c r="D31" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E31" s="36" t="s">
+        <v>1083</v>
+      </c>
+      <c r="F31" s="36" t="s">
+        <v>1084</v>
+      </c>
+      <c r="G31" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H31" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="37" t="s">
+        <v>1085</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="38" t="s">
-        <v>1078</v>
-      </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39" t="s">
-        <v>1079</v>
-      </c>
-      <c r="D32" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E32" s="39" t="s">
-        <v>1080</v>
-      </c>
-      <c r="F32" s="39" t="s">
-        <v>1081</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32" s="40" t="s">
-        <v>1082</v>
+      <c r="A32" s="35" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E32" s="36" t="s">
+        <v>1088</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>1089</v>
+      </c>
+      <c r="G32" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" s="37" t="s">
+        <v>1090</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="38" t="s">
-        <v>1083</v>
-      </c>
-      <c r="B33" s="39"/>
-      <c r="C33" s="39" t="s">
-        <v>1084</v>
-      </c>
-      <c r="D33" s="39" t="s">
-        <v>990</v>
-      </c>
-      <c r="E33" s="39" t="s">
-        <v>1085</v>
-      </c>
-      <c r="F33" s="39" t="s">
-        <v>1086</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="H33" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="I33" s="40" t="s">
-        <v>1087</v>
+      <c r="A33" s="35" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B33" s="36"/>
+      <c r="C33" s="36" t="s">
+        <v>1092</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>998</v>
+      </c>
+      <c r="E33" s="36" t="s">
+        <v>1093</v>
+      </c>
+      <c r="F33" s="36" t="s">
+        <v>1094</v>
+      </c>
+      <c r="G33" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="H33" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="37" t="s">
+        <v>1095</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement delivery and operations hardening
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="1096">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="1118">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -2418,12 +2418,6 @@
     <t>Runtime deployment, resilience, and security observations</t>
   </si>
   <si>
-    <t>Not Passed - Open</t>
-  </si>
-  <si>
-    <t>Legacy behavior is evidenced and covered by SDD; target implementation has not started.</t>
-  </si>
-  <si>
     <t>Operator starts web and z/OS Connect containers</t>
   </si>
   <si>
@@ -2442,6 +2436,9 @@
     <t>Deviation D-014/D-015: Docker Compose and secure modern operations replace IBM-only tooling; IBM runtime remains unverified.</t>
   </si>
   <si>
+    <t>modern/compose.yaml; modern/Dockerfile; modern/frontend/bank-of-z-ui/Dockerfile; modern/OPERATIONS.md</t>
+  </si>
+  <si>
     <t>specs/009-delivery-operations/spec.md; plan.md; tasks.md</t>
   </si>
   <si>
@@ -2460,6 +2457,9 @@
     <t>legacy/docker-compose.yaml environment; src/api/src/main/liberty/config/cics.xml and ims.xml; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/compose.yaml; SqlReadinessHealthCheck.cs; OperationalApiTests.cs; modern/OPERATIONS.md</t>
+  </si>
+  <si>
     <t>Operator deploys CICS transactions</t>
   </si>
   <si>
@@ -2475,6 +2475,9 @@
     <t>legacy/.setup/zconfig/bank-of-z-definitions.yaml:1-1156; legacy/.setup/setup/setup-cics-region.sh:120-190; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/compose.yaml; modern/OPERATIONS.md; modern/scripts/smoke-demo.sh</t>
+  </si>
+  <si>
     <t>Deployment enables INQACCTY without an implementation</t>
   </si>
   <si>
@@ -2490,6 +2493,9 @@
     <t>legacy/.setup/zconfig/bank-of-z-definitions.yaml:520-529; no INQACCTY implementation exists under legacy/src; Runtime: static-only</t>
   </si>
   <si>
+    <t>specs/009-delivery-operations/spec.md; modern/OPERATIONS.md (explicit do-not-port decision)</t>
+  </si>
+  <si>
     <t>Operator deploys IMS transactions</t>
   </si>
   <si>
@@ -2523,6 +2529,9 @@
     <t>Decision D-022: target bank identity is validated configuration; unused helpers are not ported.</t>
   </si>
   <si>
+    <t>BankIdentityOptions.cs; BankConfigurationController.cs; bank-identity.service.ts; OperationalApiTests.cs</t>
+  </si>
+  <si>
     <t>CICS program encounters an unrecoverable error</t>
   </si>
   <si>
@@ -2541,6 +2550,9 @@
     <t>Decisions D-006/D-014: target financial/audit writes roll back atomically and emit correlated diagnostics.</t>
   </si>
   <si>
+    <t>CorrelationMiddleware.cs; Program.cs; OperationalApiTests.cs; AccountServiceIntegrationTests.cs</t>
+  </si>
+  <si>
     <t>History diagnostic client uses TLS</t>
   </si>
   <si>
@@ -2556,6 +2568,9 @@
     <t>legacy/src/base/ims/java/src/main/java/nazare/jmp/controller/IMSBankHistory.java trust manager/hostname verifier; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/frontend/bank-of-z-ui/nginx.conf; e2e/operations.spec.ts; modern/OPERATIONS.md</t>
+  </si>
+  <si>
     <t>History diagnostic client queries fixed account 1501</t>
   </si>
   <si>
@@ -2574,6 +2589,9 @@
     <t>Decision D-022: fixed-account diagnostic utilities are not ported as banking capabilities.</t>
   </si>
   <si>
+    <t>specs/009-delivery-operations/spec.md; modern/OPERATIONS.md (fixed-account diagnostic excluded)</t>
+  </si>
+  <si>
     <t>Team attempts a standalone local run</t>
   </si>
   <si>
@@ -2589,6 +2607,9 @@
     <t>legacy/docker-compose.yaml only defines frontend and z/OS Connect; all core mappings require external CICS/IMS endpoints; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/compose.yaml; modern/.env.example; modern/README.md; modern/scripts/smoke-demo.sh</t>
+  </si>
+  <si>
     <t>Operator deploys the frontend as a Liberty WAR on z/OS</t>
   </si>
   <si>
@@ -2604,6 +2625,9 @@
     <t>legacy/.setup/build/groovy/VanillaFrontend.groovy:124-135; legacy/.setup/setup/setup-frontend-server.sh:68-102; legacy/src/frontend/config.js:14-20; legacy/.setup/setup/setup-zosconnect-server.sh:139-157; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/frontend/bank-of-z-ui/Dockerfile; nginx.conf; modern/compose.yaml</t>
+  </si>
+  <si>
     <t>Operator provisions IMS runtime datasets and metadata</t>
   </si>
   <si>
@@ -2619,6 +2643,9 @@
     <t>legacy/.setup/jcl/ims/Ims-recon.j2; legacy/.setup/jcl/ims/Ims-deloldrecon.j2; legacy/.setup/jcl/ims/Ims-dynalloc.j2; legacy/.setup/deploy/ims_maclib.jcl.j2; legacy/.setup/deploy/deployment-method.yml:334-338; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/OPERATIONS.md; modern/backend/tools/BankOfZ.Setup; verify-restart-persistence.sh</t>
+  </si>
+  <si>
     <t>Operator prepares CICS startup and TCP/IP integration</t>
   </si>
   <si>
@@ -2634,6 +2661,9 @@
     <t>legacy/.setup/jcl/cics/plt-create.j2:21-29; legacy/.setup/jcl/cics/tcpip-create.j2; legacy/.setup/setup/setup-cics-region.sh:164-172; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/frontend/bank-of-z-ui/nginx.conf; modern/compose.yaml; e2e/operations.spec.ts</t>
+  </si>
+  <si>
     <t>Operator orchestrates remote Bank of Z setup</t>
   </si>
   <si>
@@ -2649,6 +2679,9 @@
     <t>legacy/.setup/setup-local.sh:22-50; legacy/.setup/setup-remote.sh:24-68; legacy/.setup/setup-common.sh:466-590; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/OPERATIONS.md; modern/compose.yaml; smoke-demo.sh; verify-restart-persistence.sh</t>
+  </si>
+  <si>
     <t>Operator validates the IBM installation prerequisites</t>
   </si>
   <si>
@@ -2664,6 +2697,9 @@
     <t>legacy/.setup/setup/validate-install.sh:73-253; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/scripts/verify-delivery.mjs; modern/OPERATIONS.md; modern/.env.example</t>
+  </si>
+  <si>
     <t>Operator builds and packages Bank of Z with DBB</t>
   </si>
   <si>
@@ -2679,6 +2715,9 @@
     <t>legacy/.setup/pipeline-common.sh:128-247; legacy/.setup/tasks/task-dbb-build.sh; legacy/dbb-app.yaml:276-370; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/Dockerfile; modern/frontend/bank-of-z-ui/Dockerfile; .github/workflows/modern-feature-001.yml</t>
+  </si>
+  <si>
     <t>Operator runs Z Code Scan</t>
   </si>
   <si>
@@ -2694,6 +2733,9 @@
     <t>legacy/.setup/pipeline-common.sh:25-98; legacy/.setup/tasks/task-zcodescan-static-scan.sh; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/scripts/scan-secrets.mjs; .github/workflows/modern-feature-001.yml</t>
+  </si>
+  <si>
     <t>Operator deploys build outputs with Wazi Deploy</t>
   </si>
   <si>
@@ -2709,6 +2751,9 @@
     <t>legacy/.setup/tasks/task-wazi-deploy.sh; legacy/.setup/deploy/deployment-method.yml:104-501; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/compose.yaml; modern/OPERATIONS.md; .github/workflows/modern-feature-001.yml</t>
+  </si>
+  <si>
     <t>Operator provisions and refreshes native z/OS Connect</t>
   </si>
   <si>
@@ -2724,6 +2769,9 @@
     <t>legacy/.setup/setup/setup-zosconnect-server.sh:31-167; legacy/.setup/deploy/deployment-method.yml:304-501; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/compose.yaml; modern/OPERATIONS.md; SqlReadinessHealthCheck.cs</t>
+  </si>
+  <si>
     <t>Developer runs pre-commit secret detection</t>
   </si>
   <si>
@@ -2739,6 +2787,9 @@
     <t>legacy/.pre-commit-config.yaml:14-21; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/scripts/scan-secrets.mjs; scan-secrets.sh; .github/workflows/modern-feature-001.yml</t>
+  </si>
+  <si>
     <t>Developer downloads and installs configured VSIX tools</t>
   </si>
   <si>
@@ -2754,6 +2805,9 @@
     <t>legacy/scripts/download-vsix.js:176-238; legacy/scripts/install-vscode-vsix.js:133-227; legacy/scripts/install-bobide-vsix.js:132-225; Runtime: static-only</t>
   </si>
   <si>
+    <t>specs/009-delivery-operations/spec.md; modern/OPERATIONS.md (IBM-only editor tooling excluded)</t>
+  </si>
+  <si>
     <t>Developer connects zOpenDebug to a parked session</t>
   </si>
   <si>
@@ -2769,6 +2823,9 @@
     <t>legacy/.vscode/launch.json:6-15; Runtime: static-only</t>
   </si>
   <si>
+    <t>specs/009-delivery-operations/spec.md; modern/OPERATIONS.md (IBM-only debugger flow excluded)</t>
+  </si>
+  <si>
     <t>Documentation operator regenerates the site TOC</t>
   </si>
   <si>
@@ -2787,6 +2844,9 @@
     <t>Decision D-022: the broken, uninvoked TOC generator is not ported.</t>
   </si>
   <si>
+    <t>specs/009-delivery-operations/spec.md; modern/OPERATIONS.md (broken TOC generator excluded)</t>
+  </si>
+  <si>
     <t>Zowe management connections bypass certificate verification</t>
   </si>
   <si>
@@ -2817,6 +2877,9 @@
     <t>legacy/.setup/zconfig/cics-region.yaml:56-82; legacy/.setup/setup/setup-cics-region.sh:125-140; Runtime: static-only</t>
   </si>
   <si>
+    <t>modern/compose.yaml internal network and least-privilege SQL users; modern/OPERATIONS.md</t>
+  </si>
+  <si>
     <t>IBM MQ is documented but not evidenced in runtime banking code</t>
   </si>
   <si>
@@ -2830,6 +2893,9 @@
   </si>
   <si>
     <t>legacy/.setup/build/datasets.yaml.j2:52-66 contains optional MQ library placeholders; no MQCONN/MQOPEN/MQPUT/MQGET calls are present under legacy/src; Runtime: static-only</t>
+  </si>
+  <si>
+    <t>specs/009-delivery-operations/spec.md; modern/OPERATIONS.md (MQ residual risk and non-port decision)</t>
   </si>
   <si>
     <t>ID</t>
@@ -3310,7 +3376,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -3360,12 +3426,6 @@
       <b/>
       <color rgb="FF000000"/>
       <sz val="10"/>
-      <name val="Carlito"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF7F0000"/>
-      <sz val="11"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -3438,12 +3498,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -3653,7 +3713,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3707,19 +3767,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3740,13 +3794,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8966,103 +9020,111 @@
       </c>
     </row>
     <row r="127" ht="40" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A127" s="21" t="s">
+      <c r="A127" s="17" t="s">
         <v>798</v>
       </c>
-      <c r="B127" s="21" t="s">
+      <c r="B127" s="17" t="s">
         <v>799</v>
       </c>
-      <c r="C127" s="21" t="s">
-        <v>800</v>
-      </c>
-      <c r="D127" s="21" t="s">
-        <v>801</v>
-      </c>
-      <c r="E127" s="21"/>
-      <c r="F127" s="21"/>
-      <c r="G127" s="21"/>
-      <c r="H127" s="21"/>
-      <c r="I127" s="21"/>
-      <c r="J127" s="21"/>
-      <c r="K127" s="21"/>
-      <c r="L127" s="21"/>
-      <c r="M127" s="21"/>
-      <c r="N127" s="21"/>
+      <c r="C127" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D127" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E127" s="17"/>
+      <c r="F127" s="17"/>
+      <c r="G127" s="17"/>
+      <c r="H127" s="17"/>
+      <c r="I127" s="17"/>
+      <c r="J127" s="17"/>
+      <c r="K127" s="17"/>
+      <c r="L127" s="17"/>
+      <c r="M127" s="17"/>
+      <c r="N127" s="17"/>
     </row>
     <row r="128" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A128" s="18"/>
       <c r="B128" s="19" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="C128" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D128" s="22" t="s">
+      <c r="D128" s="20" t="s">
+        <v>801</v>
+      </c>
+      <c r="E128" s="20" t="s">
+        <v>802</v>
+      </c>
+      <c r="F128" s="20" t="s">
         <v>803</v>
       </c>
-      <c r="E128" s="22" t="s">
+      <c r="G128" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H128" s="20" t="s">
         <v>804</v>
       </c>
-      <c r="F128" s="22" t="s">
+      <c r="I128" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J128" s="20" t="s">
         <v>805</v>
       </c>
-      <c r="G128" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H128" s="22" t="s">
+      <c r="K128" s="20" t="s">
         <v>806</v>
       </c>
-      <c r="I128" s="22"/>
-      <c r="J128" s="22" t="s">
+      <c r="L128" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M128" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N128" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K128" s="22"/>
-      <c r="L128" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M128" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N128" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="129" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A129" s="18"/>
       <c r="B129" s="19" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="C129" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D129" s="22" t="s">
+      <c r="D129" s="20" t="s">
+        <v>809</v>
+      </c>
+      <c r="E129" s="20" t="s">
         <v>810</v>
       </c>
-      <c r="E129" s="22" t="s">
+      <c r="F129" s="20" t="s">
         <v>811</v>
       </c>
-      <c r="F129" s="22" t="s">
+      <c r="G129" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H129" s="20" t="s">
         <v>812</v>
       </c>
-      <c r="G129" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H129" s="22" t="s">
+      <c r="I129" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J129" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K129" s="20" t="s">
         <v>813</v>
       </c>
-      <c r="I129" s="22"/>
-      <c r="J129" s="22" t="s">
+      <c r="L129" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M129" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N129" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K129" s="22"/>
-      <c r="L129" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M129" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N129" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="130" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
@@ -9073,908 +9135,1004 @@
       <c r="C130" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D130" s="22" t="s">
+      <c r="D130" s="20" t="s">
         <v>815</v>
       </c>
-      <c r="E130" s="22" t="s">
+      <c r="E130" s="20" t="s">
         <v>816</v>
       </c>
-      <c r="F130" s="22" t="s">
+      <c r="F130" s="20" t="s">
         <v>817</v>
       </c>
-      <c r="G130" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H130" s="22" t="s">
+      <c r="G130" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H130" s="20" t="s">
         <v>818</v>
       </c>
-      <c r="I130" s="22"/>
-      <c r="J130" s="22" t="s">
+      <c r="I130" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J130" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K130" s="20" t="s">
+        <v>819</v>
+      </c>
+      <c r="L130" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M130" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N130" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K130" s="22"/>
-      <c r="L130" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M130" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N130" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="131" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A131" s="18"/>
       <c r="B131" s="19" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="C131" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D131" s="22" t="s">
-        <v>820</v>
-      </c>
-      <c r="E131" s="22" t="s">
+      <c r="D131" s="20" t="s">
         <v>821</v>
       </c>
-      <c r="F131" s="22" t="s">
+      <c r="E131" s="20" t="s">
         <v>822</v>
       </c>
-      <c r="G131" s="22" t="s">
+      <c r="F131" s="20" t="s">
+        <v>823</v>
+      </c>
+      <c r="G131" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H131" s="22" t="s">
-        <v>823</v>
-      </c>
-      <c r="I131" s="22"/>
-      <c r="J131" s="22" t="s">
+      <c r="H131" s="20" t="s">
+        <v>824</v>
+      </c>
+      <c r="I131" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J131" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K131" s="20" t="s">
+        <v>825</v>
+      </c>
+      <c r="L131" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M131" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N131" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K131" s="22"/>
-      <c r="L131" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M131" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N131" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="132" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A132" s="18"/>
       <c r="B132" s="19" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="C132" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D132" s="22" t="s">
-        <v>825</v>
-      </c>
-      <c r="E132" s="22" t="s">
-        <v>826</v>
-      </c>
-      <c r="F132" s="22" t="s">
+      <c r="D132" s="20" t="s">
         <v>827</v>
       </c>
-      <c r="G132" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H132" s="22" t="s">
+      <c r="E132" s="20" t="s">
         <v>828</v>
       </c>
-      <c r="I132" s="22"/>
-      <c r="J132" s="22" t="s">
+      <c r="F132" s="20" t="s">
+        <v>829</v>
+      </c>
+      <c r="G132" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H132" s="20" t="s">
+        <v>830</v>
+      </c>
+      <c r="I132" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J132" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K132" s="20" t="s">
+        <v>819</v>
+      </c>
+      <c r="L132" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M132" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N132" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K132" s="22"/>
-      <c r="L132" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M132" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N132" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="133" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A133" s="18"/>
       <c r="B133" s="19" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="C133" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D133" s="22" t="s">
-        <v>830</v>
-      </c>
-      <c r="E133" s="22" t="s">
-        <v>831</v>
-      </c>
-      <c r="F133" s="22" t="s">
+      <c r="D133" s="20" t="s">
         <v>832</v>
       </c>
-      <c r="G133" s="22" t="s">
+      <c r="E133" s="20" t="s">
+        <v>833</v>
+      </c>
+      <c r="F133" s="20" t="s">
+        <v>834</v>
+      </c>
+      <c r="G133" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H133" s="22" t="s">
-        <v>833</v>
-      </c>
-      <c r="I133" s="22"/>
-      <c r="J133" s="22" t="s">
-        <v>834</v>
-      </c>
-      <c r="K133" s="22"/>
-      <c r="L133" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M133" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N133" s="22" t="s">
-        <v>808</v>
+      <c r="H133" s="20" t="s">
+        <v>835</v>
+      </c>
+      <c r="I133" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J133" s="20" t="s">
+        <v>836</v>
+      </c>
+      <c r="K133" s="20" t="s">
+        <v>837</v>
+      </c>
+      <c r="L133" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M133" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N133" s="20" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="134" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A134" s="18"/>
       <c r="B134" s="19" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="C134" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D134" s="22" t="s">
-        <v>836</v>
-      </c>
-      <c r="E134" s="22" t="s">
-        <v>837</v>
-      </c>
-      <c r="F134" s="22" t="s">
-        <v>838</v>
-      </c>
-      <c r="G134" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H134" s="22" t="s">
+      <c r="D134" s="20" t="s">
         <v>839</v>
       </c>
-      <c r="I134" s="22"/>
-      <c r="J134" s="22" t="s">
+      <c r="E134" s="20" t="s">
         <v>840</v>
       </c>
-      <c r="K134" s="22"/>
-      <c r="L134" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M134" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N134" s="22" t="s">
-        <v>808</v>
+      <c r="F134" s="20" t="s">
+        <v>841</v>
+      </c>
+      <c r="G134" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H134" s="20" t="s">
+        <v>842</v>
+      </c>
+      <c r="I134" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J134" s="20" t="s">
+        <v>843</v>
+      </c>
+      <c r="K134" s="20" t="s">
+        <v>844</v>
+      </c>
+      <c r="L134" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M134" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N134" s="20" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="135" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A135" s="18"/>
       <c r="B135" s="19" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="C135" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D135" s="22" t="s">
-        <v>842</v>
-      </c>
-      <c r="E135" s="22" t="s">
-        <v>843</v>
-      </c>
-      <c r="F135" s="22" t="s">
-        <v>844</v>
-      </c>
-      <c r="G135" s="22" t="s">
+      <c r="D135" s="20" t="s">
+        <v>846</v>
+      </c>
+      <c r="E135" s="20" t="s">
+        <v>847</v>
+      </c>
+      <c r="F135" s="20" t="s">
+        <v>848</v>
+      </c>
+      <c r="G135" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H135" s="22" t="s">
-        <v>845</v>
-      </c>
-      <c r="I135" s="22"/>
-      <c r="J135" s="22" t="s">
+      <c r="H135" s="20" t="s">
+        <v>849</v>
+      </c>
+      <c r="I135" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J135" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K135" s="20" t="s">
+        <v>850</v>
+      </c>
+      <c r="L135" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M135" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N135" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K135" s="22"/>
-      <c r="L135" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M135" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N135" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="136" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A136" s="18"/>
       <c r="B136" s="19" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="C136" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D136" s="22" t="s">
-        <v>847</v>
-      </c>
-      <c r="E136" s="22" t="s">
-        <v>848</v>
-      </c>
-      <c r="F136" s="22" t="s">
-        <v>849</v>
-      </c>
-      <c r="G136" s="22" t="s">
+      <c r="D136" s="20" t="s">
+        <v>852</v>
+      </c>
+      <c r="E136" s="20" t="s">
+        <v>853</v>
+      </c>
+      <c r="F136" s="20" t="s">
+        <v>854</v>
+      </c>
+      <c r="G136" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H136" s="22" t="s">
-        <v>850</v>
-      </c>
-      <c r="I136" s="22"/>
-      <c r="J136" s="22" t="s">
-        <v>851</v>
-      </c>
-      <c r="K136" s="22"/>
-      <c r="L136" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M136" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N136" s="22" t="s">
-        <v>808</v>
+      <c r="H136" s="20" t="s">
+        <v>855</v>
+      </c>
+      <c r="I136" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J136" s="20" t="s">
+        <v>856</v>
+      </c>
+      <c r="K136" s="20" t="s">
+        <v>857</v>
+      </c>
+      <c r="L136" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M136" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N136" s="20" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="137" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A137" s="18"/>
       <c r="B137" s="19" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="C137" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D137" s="22" t="s">
-        <v>853</v>
-      </c>
-      <c r="E137" s="22" t="s">
-        <v>854</v>
-      </c>
-      <c r="F137" s="22" t="s">
-        <v>855</v>
-      </c>
-      <c r="G137" s="22" t="s">
+      <c r="D137" s="20" t="s">
+        <v>859</v>
+      </c>
+      <c r="E137" s="20" t="s">
+        <v>860</v>
+      </c>
+      <c r="F137" s="20" t="s">
+        <v>861</v>
+      </c>
+      <c r="G137" s="20" t="s">
         <v>522</v>
       </c>
-      <c r="H137" s="22" t="s">
-        <v>856</v>
-      </c>
-      <c r="I137" s="22"/>
-      <c r="J137" s="22" t="s">
+      <c r="H137" s="20" t="s">
+        <v>862</v>
+      </c>
+      <c r="I137" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J137" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K137" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="L137" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M137" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N137" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K137" s="22"/>
-      <c r="L137" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M137" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N137" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="138" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A138" s="18"/>
       <c r="B138" s="19" t="s">
-        <v>857</v>
+        <v>864</v>
       </c>
       <c r="C138" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D138" s="22" t="s">
-        <v>858</v>
-      </c>
-      <c r="E138" s="22" t="s">
-        <v>859</v>
-      </c>
-      <c r="F138" s="22" t="s">
-        <v>860</v>
-      </c>
-      <c r="G138" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H138" s="22" t="s">
-        <v>861</v>
-      </c>
-      <c r="I138" s="22"/>
-      <c r="J138" s="22" t="s">
+      <c r="D138" s="20" t="s">
+        <v>865</v>
+      </c>
+      <c r="E138" s="20" t="s">
+        <v>866</v>
+      </c>
+      <c r="F138" s="20" t="s">
+        <v>867</v>
+      </c>
+      <c r="G138" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H138" s="20" t="s">
+        <v>868</v>
+      </c>
+      <c r="I138" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J138" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K138" s="20" t="s">
+        <v>869</v>
+      </c>
+      <c r="L138" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M138" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N138" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K138" s="22"/>
-      <c r="L138" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M138" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N138" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="139" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A139" s="18"/>
       <c r="B139" s="19" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
       <c r="C139" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D139" s="22" t="s">
-        <v>863</v>
-      </c>
-      <c r="E139" s="22" t="s">
-        <v>864</v>
-      </c>
-      <c r="F139" s="22" t="s">
-        <v>865</v>
-      </c>
-      <c r="G139" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H139" s="22" t="s">
-        <v>866</v>
-      </c>
-      <c r="I139" s="22"/>
-      <c r="J139" s="22" t="s">
+      <c r="D139" s="20" t="s">
+        <v>871</v>
+      </c>
+      <c r="E139" s="20" t="s">
+        <v>872</v>
+      </c>
+      <c r="F139" s="20" t="s">
+        <v>873</v>
+      </c>
+      <c r="G139" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H139" s="20" t="s">
+        <v>874</v>
+      </c>
+      <c r="I139" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J139" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K139" s="20" t="s">
+        <v>875</v>
+      </c>
+      <c r="L139" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M139" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N139" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K139" s="22"/>
-      <c r="L139" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M139" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N139" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="140" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A140" s="18"/>
       <c r="B140" s="19" t="s">
-        <v>867</v>
+        <v>876</v>
       </c>
       <c r="C140" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D140" s="22" t="s">
-        <v>868</v>
-      </c>
-      <c r="E140" s="22" t="s">
-        <v>869</v>
-      </c>
-      <c r="F140" s="22" t="s">
-        <v>870</v>
-      </c>
-      <c r="G140" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H140" s="22" t="s">
-        <v>871</v>
-      </c>
-      <c r="I140" s="22"/>
-      <c r="J140" s="22" t="s">
+      <c r="D140" s="20" t="s">
+        <v>877</v>
+      </c>
+      <c r="E140" s="20" t="s">
+        <v>878</v>
+      </c>
+      <c r="F140" s="20" t="s">
+        <v>879</v>
+      </c>
+      <c r="G140" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H140" s="20" t="s">
+        <v>880</v>
+      </c>
+      <c r="I140" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J140" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K140" s="20" t="s">
+        <v>881</v>
+      </c>
+      <c r="L140" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M140" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N140" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K140" s="22"/>
-      <c r="L140" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M140" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N140" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="141" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A141" s="18"/>
       <c r="B141" s="19" t="s">
-        <v>872</v>
+        <v>882</v>
       </c>
       <c r="C141" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D141" s="22" t="s">
-        <v>873</v>
-      </c>
-      <c r="E141" s="22" t="s">
-        <v>874</v>
-      </c>
-      <c r="F141" s="22" t="s">
-        <v>875</v>
-      </c>
-      <c r="G141" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H141" s="22" t="s">
-        <v>876</v>
-      </c>
-      <c r="I141" s="22"/>
-      <c r="J141" s="22" t="s">
+      <c r="D141" s="20" t="s">
+        <v>883</v>
+      </c>
+      <c r="E141" s="20" t="s">
+        <v>884</v>
+      </c>
+      <c r="F141" s="20" t="s">
+        <v>885</v>
+      </c>
+      <c r="G141" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H141" s="20" t="s">
+        <v>886</v>
+      </c>
+      <c r="I141" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J141" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K141" s="20" t="s">
+        <v>887</v>
+      </c>
+      <c r="L141" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M141" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N141" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K141" s="22"/>
-      <c r="L141" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M141" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N141" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="142" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A142" s="18"/>
       <c r="B142" s="19" t="s">
-        <v>877</v>
+        <v>888</v>
       </c>
       <c r="C142" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D142" s="22" t="s">
-        <v>878</v>
-      </c>
-      <c r="E142" s="22" t="s">
-        <v>879</v>
-      </c>
-      <c r="F142" s="22" t="s">
-        <v>880</v>
-      </c>
-      <c r="G142" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H142" s="22" t="s">
-        <v>881</v>
-      </c>
-      <c r="I142" s="22"/>
-      <c r="J142" s="22" t="s">
+      <c r="D142" s="20" t="s">
+        <v>889</v>
+      </c>
+      <c r="E142" s="20" t="s">
+        <v>890</v>
+      </c>
+      <c r="F142" s="20" t="s">
+        <v>891</v>
+      </c>
+      <c r="G142" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H142" s="20" t="s">
+        <v>892</v>
+      </c>
+      <c r="I142" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J142" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K142" s="20" t="s">
+        <v>893</v>
+      </c>
+      <c r="L142" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M142" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N142" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K142" s="22"/>
-      <c r="L142" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M142" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N142" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="143" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A143" s="18"/>
       <c r="B143" s="19" t="s">
-        <v>882</v>
+        <v>894</v>
       </c>
       <c r="C143" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D143" s="22" t="s">
-        <v>883</v>
-      </c>
-      <c r="E143" s="22" t="s">
-        <v>884</v>
-      </c>
-      <c r="F143" s="22" t="s">
-        <v>885</v>
-      </c>
-      <c r="G143" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H143" s="22" t="s">
-        <v>886</v>
-      </c>
-      <c r="I143" s="22"/>
-      <c r="J143" s="22" t="s">
+      <c r="D143" s="20" t="s">
+        <v>895</v>
+      </c>
+      <c r="E143" s="20" t="s">
+        <v>896</v>
+      </c>
+      <c r="F143" s="20" t="s">
+        <v>897</v>
+      </c>
+      <c r="G143" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H143" s="20" t="s">
+        <v>898</v>
+      </c>
+      <c r="I143" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J143" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K143" s="20" t="s">
+        <v>899</v>
+      </c>
+      <c r="L143" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M143" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N143" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K143" s="22"/>
-      <c r="L143" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M143" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N143" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="144" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A144" s="18"/>
       <c r="B144" s="19" t="s">
-        <v>887</v>
+        <v>900</v>
       </c>
       <c r="C144" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D144" s="22" t="s">
-        <v>888</v>
-      </c>
-      <c r="E144" s="22" t="s">
-        <v>889</v>
-      </c>
-      <c r="F144" s="22" t="s">
-        <v>890</v>
-      </c>
-      <c r="G144" s="22" t="s">
+      <c r="D144" s="20" t="s">
+        <v>901</v>
+      </c>
+      <c r="E144" s="20" t="s">
+        <v>902</v>
+      </c>
+      <c r="F144" s="20" t="s">
+        <v>903</v>
+      </c>
+      <c r="G144" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H144" s="22" t="s">
-        <v>891</v>
-      </c>
-      <c r="I144" s="22"/>
-      <c r="J144" s="22" t="s">
+      <c r="H144" s="20" t="s">
+        <v>904</v>
+      </c>
+      <c r="I144" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J144" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K144" s="20" t="s">
+        <v>905</v>
+      </c>
+      <c r="L144" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M144" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N144" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K144" s="22"/>
-      <c r="L144" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M144" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N144" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="145" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A145" s="18"/>
       <c r="B145" s="19" t="s">
-        <v>892</v>
+        <v>906</v>
       </c>
       <c r="C145" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D145" s="22" t="s">
-        <v>893</v>
-      </c>
-      <c r="E145" s="22" t="s">
-        <v>894</v>
-      </c>
-      <c r="F145" s="22" t="s">
-        <v>895</v>
-      </c>
-      <c r="G145" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H145" s="22" t="s">
-        <v>896</v>
-      </c>
-      <c r="I145" s="22"/>
-      <c r="J145" s="22" t="s">
+      <c r="D145" s="20" t="s">
+        <v>907</v>
+      </c>
+      <c r="E145" s="20" t="s">
+        <v>908</v>
+      </c>
+      <c r="F145" s="20" t="s">
+        <v>909</v>
+      </c>
+      <c r="G145" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H145" s="20" t="s">
+        <v>910</v>
+      </c>
+      <c r="I145" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J145" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K145" s="20" t="s">
+        <v>911</v>
+      </c>
+      <c r="L145" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M145" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N145" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K145" s="22"/>
-      <c r="L145" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M145" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N145" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="146" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A146" s="18"/>
       <c r="B146" s="19" t="s">
-        <v>897</v>
+        <v>912</v>
       </c>
       <c r="C146" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D146" s="22" t="s">
-        <v>898</v>
-      </c>
-      <c r="E146" s="22" t="s">
-        <v>899</v>
-      </c>
-      <c r="F146" s="22" t="s">
-        <v>900</v>
-      </c>
-      <c r="G146" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H146" s="22" t="s">
-        <v>901</v>
-      </c>
-      <c r="I146" s="22"/>
-      <c r="J146" s="22" t="s">
+      <c r="D146" s="20" t="s">
+        <v>913</v>
+      </c>
+      <c r="E146" s="20" t="s">
+        <v>914</v>
+      </c>
+      <c r="F146" s="20" t="s">
+        <v>915</v>
+      </c>
+      <c r="G146" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H146" s="20" t="s">
+        <v>916</v>
+      </c>
+      <c r="I146" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J146" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K146" s="20" t="s">
+        <v>917</v>
+      </c>
+      <c r="L146" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M146" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N146" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K146" s="22"/>
-      <c r="L146" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M146" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N146" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="147" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A147" s="18"/>
       <c r="B147" s="19" t="s">
-        <v>902</v>
+        <v>918</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D147" s="22" t="s">
-        <v>903</v>
-      </c>
-      <c r="E147" s="22" t="s">
-        <v>904</v>
-      </c>
-      <c r="F147" s="22" t="s">
-        <v>905</v>
-      </c>
-      <c r="G147" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H147" s="22" t="s">
-        <v>906</v>
-      </c>
-      <c r="I147" s="22"/>
-      <c r="J147" s="22" t="s">
+      <c r="D147" s="20" t="s">
+        <v>919</v>
+      </c>
+      <c r="E147" s="20" t="s">
+        <v>920</v>
+      </c>
+      <c r="F147" s="20" t="s">
+        <v>921</v>
+      </c>
+      <c r="G147" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H147" s="20" t="s">
+        <v>922</v>
+      </c>
+      <c r="I147" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J147" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K147" s="20" t="s">
+        <v>923</v>
+      </c>
+      <c r="L147" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M147" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N147" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K147" s="22"/>
-      <c r="L147" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M147" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N147" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="148" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A148" s="18"/>
       <c r="B148" s="19" t="s">
-        <v>907</v>
+        <v>924</v>
       </c>
       <c r="C148" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D148" s="22" t="s">
-        <v>908</v>
-      </c>
-      <c r="E148" s="22" t="s">
-        <v>909</v>
-      </c>
-      <c r="F148" s="22" t="s">
-        <v>910</v>
-      </c>
-      <c r="G148" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H148" s="22" t="s">
-        <v>911</v>
-      </c>
-      <c r="I148" s="22"/>
-      <c r="J148" s="22" t="s">
+      <c r="D148" s="20" t="s">
+        <v>925</v>
+      </c>
+      <c r="E148" s="20" t="s">
+        <v>926</v>
+      </c>
+      <c r="F148" s="20" t="s">
+        <v>927</v>
+      </c>
+      <c r="G148" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H148" s="20" t="s">
+        <v>928</v>
+      </c>
+      <c r="I148" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J148" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K148" s="20" t="s">
+        <v>929</v>
+      </c>
+      <c r="L148" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M148" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N148" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K148" s="22"/>
-      <c r="L148" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M148" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N148" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="149" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A149" s="18"/>
       <c r="B149" s="19" t="s">
-        <v>912</v>
+        <v>930</v>
       </c>
       <c r="C149" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D149" s="22" t="s">
-        <v>913</v>
-      </c>
-      <c r="E149" s="22" t="s">
-        <v>914</v>
-      </c>
-      <c r="F149" s="22" t="s">
-        <v>915</v>
-      </c>
-      <c r="G149" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H149" s="22" t="s">
-        <v>916</v>
-      </c>
-      <c r="I149" s="22"/>
-      <c r="J149" s="22" t="s">
+      <c r="D149" s="20" t="s">
+        <v>931</v>
+      </c>
+      <c r="E149" s="20" t="s">
+        <v>932</v>
+      </c>
+      <c r="F149" s="20" t="s">
+        <v>933</v>
+      </c>
+      <c r="G149" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H149" s="20" t="s">
+        <v>934</v>
+      </c>
+      <c r="I149" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J149" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K149" s="20" t="s">
+        <v>935</v>
+      </c>
+      <c r="L149" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M149" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N149" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K149" s="22"/>
-      <c r="L149" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M149" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N149" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="150" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A150" s="18"/>
       <c r="B150" s="19" t="s">
-        <v>917</v>
+        <v>936</v>
       </c>
       <c r="C150" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D150" s="22" t="s">
-        <v>918</v>
-      </c>
-      <c r="E150" s="22" t="s">
-        <v>919</v>
-      </c>
-      <c r="F150" s="22" t="s">
-        <v>920</v>
-      </c>
-      <c r="G150" s="22" t="s">
+      <c r="D150" s="20" t="s">
+        <v>937</v>
+      </c>
+      <c r="E150" s="20" t="s">
+        <v>938</v>
+      </c>
+      <c r="F150" s="20" t="s">
+        <v>939</v>
+      </c>
+      <c r="G150" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H150" s="22" t="s">
-        <v>921</v>
-      </c>
-      <c r="I150" s="22"/>
-      <c r="J150" s="22" t="s">
-        <v>922</v>
-      </c>
-      <c r="K150" s="22"/>
-      <c r="L150" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M150" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N150" s="22" t="s">
-        <v>808</v>
+      <c r="H150" s="20" t="s">
+        <v>940</v>
+      </c>
+      <c r="I150" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J150" s="20" t="s">
+        <v>941</v>
+      </c>
+      <c r="K150" s="20" t="s">
+        <v>942</v>
+      </c>
+      <c r="L150" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M150" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N150" s="20" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="151" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A151" s="18"/>
       <c r="B151" s="19" t="s">
-        <v>923</v>
+        <v>943</v>
       </c>
       <c r="C151" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D151" s="22" t="s">
-        <v>924</v>
-      </c>
-      <c r="E151" s="22" t="s">
-        <v>925</v>
-      </c>
-      <c r="F151" s="22" t="s">
-        <v>926</v>
-      </c>
-      <c r="G151" s="22" t="s">
+      <c r="D151" s="20" t="s">
+        <v>944</v>
+      </c>
+      <c r="E151" s="20" t="s">
+        <v>945</v>
+      </c>
+      <c r="F151" s="20" t="s">
+        <v>946</v>
+      </c>
+      <c r="G151" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H151" s="22" t="s">
-        <v>927</v>
-      </c>
-      <c r="I151" s="22"/>
-      <c r="J151" s="22" t="s">
+      <c r="H151" s="20" t="s">
+        <v>947</v>
+      </c>
+      <c r="I151" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J151" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K151" s="20" t="s">
+        <v>850</v>
+      </c>
+      <c r="L151" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M151" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N151" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K151" s="22"/>
-      <c r="L151" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M151" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N151" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="152" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A152" s="18"/>
       <c r="B152" s="19" t="s">
-        <v>928</v>
+        <v>948</v>
       </c>
       <c r="C152" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D152" s="22" t="s">
-        <v>929</v>
-      </c>
-      <c r="E152" s="22" t="s">
-        <v>930</v>
-      </c>
-      <c r="F152" s="22" t="s">
-        <v>931</v>
-      </c>
-      <c r="G152" s="22" t="s">
+      <c r="D152" s="20" t="s">
+        <v>949</v>
+      </c>
+      <c r="E152" s="20" t="s">
+        <v>950</v>
+      </c>
+      <c r="F152" s="20" t="s">
+        <v>951</v>
+      </c>
+      <c r="G152" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H152" s="22" t="s">
-        <v>932</v>
-      </c>
-      <c r="I152" s="22"/>
-      <c r="J152" s="22" t="s">
+      <c r="H152" s="20" t="s">
+        <v>952</v>
+      </c>
+      <c r="I152" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J152" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K152" s="20" t="s">
+        <v>953</v>
+      </c>
+      <c r="L152" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M152" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N152" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K152" s="22"/>
-      <c r="L152" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M152" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N152" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="153" hidden="1" spans="1:14" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A153" s="18"/>
       <c r="B153" s="19" t="s">
-        <v>933</v>
+        <v>954</v>
       </c>
       <c r="C153" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="D153" s="22" t="s">
-        <v>934</v>
-      </c>
-      <c r="E153" s="22" t="s">
-        <v>935</v>
-      </c>
-      <c r="F153" s="22" t="s">
-        <v>936</v>
-      </c>
-      <c r="G153" s="22" t="s">
+      <c r="D153" s="20" t="s">
+        <v>955</v>
+      </c>
+      <c r="E153" s="20" t="s">
+        <v>956</v>
+      </c>
+      <c r="F153" s="20" t="s">
+        <v>957</v>
+      </c>
+      <c r="G153" s="20" t="s">
         <v>522</v>
       </c>
-      <c r="H153" s="22" t="s">
-        <v>937</v>
-      </c>
-      <c r="I153" s="22"/>
-      <c r="J153" s="22" t="s">
+      <c r="H153" s="20" t="s">
+        <v>958</v>
+      </c>
+      <c r="I153" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="J153" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="K153" s="20" t="s">
+        <v>959</v>
+      </c>
+      <c r="L153" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="M153" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="N153" s="20" t="s">
         <v>807</v>
-      </c>
-      <c r="K153" s="22"/>
-      <c r="L153" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M153" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="N153" s="22" t="s">
-        <v>808</v>
       </c>
     </row>
   </sheetData>
@@ -10006,914 +10164,914 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
-        <v>938</v>
-      </c>
-      <c r="B1" s="24" t="s">
-        <v>939</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>940</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>941</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>942</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>943</v>
-      </c>
-      <c r="G1" s="24" t="s">
+      <c r="A1" s="21" t="s">
+        <v>960</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>961</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>962</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>963</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>964</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>965</v>
+      </c>
+      <c r="G1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="24" t="s">
-        <v>944</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>945</v>
+      <c r="H1" s="22" t="s">
+        <v>966</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>967</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
-        <v>946</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>947</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>948</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>949</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>950</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>951</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="I2" s="28" t="s">
-        <v>952</v>
+      <c r="A2" s="24" t="s">
+        <v>968</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>969</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>970</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>971</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>972</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>973</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>974</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
-        <v>953</v>
-      </c>
-      <c r="B3" s="30" t="s">
-        <v>954</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>955</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E3" s="30" t="s">
-        <v>956</v>
-      </c>
-      <c r="F3" s="30" t="s">
-        <v>957</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I3" s="31" t="s">
-        <v>958</v>
+      <c r="A3" s="27" t="s">
+        <v>975</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>976</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>977</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>971</v>
+      </c>
+      <c r="E3" s="28" t="s">
+        <v>978</v>
+      </c>
+      <c r="F3" s="28" t="s">
+        <v>979</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="29" t="s">
+        <v>980</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
-        <v>959</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>960</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>961</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>962</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>963</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="31" t="s">
-        <v>964</v>
+      <c r="A4" s="27" t="s">
+        <v>981</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>982</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>983</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>971</v>
+      </c>
+      <c r="E4" s="28" t="s">
+        <v>984</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>985</v>
+      </c>
+      <c r="G4" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="29" t="s">
+        <v>986</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="29" t="s">
-        <v>965</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>966</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>967</v>
-      </c>
-      <c r="D5" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E5" s="30" t="s">
-        <v>968</v>
-      </c>
-      <c r="F5" s="30" t="s">
-        <v>969</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I5" s="31" t="s">
-        <v>970</v>
+      <c r="A5" s="27" t="s">
+        <v>987</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>988</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>989</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>971</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>990</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>991</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" s="29" t="s">
+        <v>992</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="27" t="s">
+        <v>993</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>487</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>994</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>971</v>
       </c>
-      <c r="B6" s="30" t="s">
-        <v>487</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>972</v>
-      </c>
-      <c r="D6" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E6" s="30" t="s">
-        <v>973</v>
-      </c>
-      <c r="F6" s="30" t="s">
-        <v>974</v>
-      </c>
-      <c r="G6" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I6" s="31" t="s">
-        <v>975</v>
+      <c r="E6" s="28" t="s">
+        <v>995</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>996</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="29" t="s">
+        <v>997</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
-        <v>976</v>
-      </c>
-      <c r="B7" s="30" t="s">
+      <c r="A7" s="27" t="s">
+        <v>998</v>
+      </c>
+      <c r="B7" s="28" t="s">
         <v>533</v>
       </c>
-      <c r="C7" s="30" t="s">
-        <v>977</v>
-      </c>
-      <c r="D7" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>978</v>
-      </c>
-      <c r="F7" s="30" t="s">
-        <v>979</v>
-      </c>
-      <c r="G7" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I7" s="31" t="s">
-        <v>980</v>
+      <c r="C7" s="28" t="s">
+        <v>999</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>971</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G7" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="29" t="s">
+        <v>1002</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
-        <v>981</v>
-      </c>
-      <c r="B8" s="30" t="s">
+      <c r="A8" s="27" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B8" s="28" t="s">
         <v>612</v>
       </c>
-      <c r="C8" s="30" t="s">
-        <v>982</v>
-      </c>
-      <c r="D8" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E8" s="30" t="s">
-        <v>983</v>
-      </c>
-      <c r="F8" s="30" t="s">
-        <v>984</v>
-      </c>
-      <c r="G8" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" s="31" t="s">
-        <v>985</v>
+      <c r="C8" s="28" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>971</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>1005</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>1006</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="29" t="s">
+        <v>1007</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
-        <v>986</v>
-      </c>
-      <c r="B9" s="30" t="s">
+      <c r="A9" s="27" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B9" s="28" t="s">
         <v>742</v>
       </c>
-      <c r="C9" s="30" t="s">
-        <v>987</v>
-      </c>
-      <c r="D9" s="30" t="s">
-        <v>949</v>
-      </c>
-      <c r="E9" s="30" t="s">
-        <v>988</v>
-      </c>
-      <c r="F9" s="30" t="s">
-        <v>989</v>
-      </c>
-      <c r="G9" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9" s="31" t="s">
-        <v>990</v>
+      <c r="C9" s="28" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>971</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>1010</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>1011</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="29" t="s">
+        <v>1012</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="32" t="s">
-        <v>991</v>
-      </c>
-      <c r="B10" s="33" t="s">
+      <c r="A10" s="30" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B10" s="31" t="s">
         <v>798</v>
       </c>
-      <c r="C10" s="33" t="s">
-        <v>992</v>
-      </c>
-      <c r="D10" s="33" t="s">
-        <v>949</v>
-      </c>
-      <c r="E10" s="33" t="s">
-        <v>993</v>
-      </c>
-      <c r="F10" s="33" t="s">
-        <v>994</v>
-      </c>
-      <c r="G10" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="I10" s="34" t="s">
-        <v>995</v>
+      <c r="C10" s="31" t="s">
+        <v>1014</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>971</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>1015</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>1016</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H10" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>1017</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
-        <v>996</v>
-      </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27" t="s">
-        <v>997</v>
-      </c>
-      <c r="D11" s="27" t="s">
-        <v>998</v>
-      </c>
-      <c r="E11" s="27" t="s">
-        <v>999</v>
-      </c>
-      <c r="F11" s="27" t="s">
-        <v>1000</v>
-      </c>
-      <c r="G11" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="I11" s="28" t="s">
-        <v>1001</v>
+      <c r="A11" s="24" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25" t="s">
+        <v>1019</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>1022</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" s="26" t="s">
+        <v>1023</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
-        <v>1002</v>
-      </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30" t="s">
-        <v>1003</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F12" s="30" t="s">
-        <v>1004</v>
-      </c>
-      <c r="G12" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H12" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I12" s="31" t="s">
-        <v>1005</v>
+      <c r="A12" s="27" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D12" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>1026</v>
+      </c>
+      <c r="G12" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="29" t="s">
+        <v>1027</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="29" t="s">
-        <v>1006</v>
-      </c>
-      <c r="B13" s="30"/>
-      <c r="C13" s="30" t="s">
-        <v>1007</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E13" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F13" s="30" t="s">
-        <v>1008</v>
-      </c>
-      <c r="G13" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H13" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I13" s="31" t="s">
+      <c r="A13" s="27" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28" t="s">
+        <v>1029</v>
+      </c>
+      <c r="D13" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E13" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>1030</v>
+      </c>
+      <c r="G13" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H13" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" s="29" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="27" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>1034</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="29" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="27" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E15" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>1038</v>
+      </c>
+      <c r="G15" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I15" s="29" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="27" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28" t="s">
+        <v>1041</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>1042</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="29" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="27" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>1046</v>
+      </c>
+      <c r="G17" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="29" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="27" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28" t="s">
+        <v>1049</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E18" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>1050</v>
+      </c>
+      <c r="G18" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" s="29" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="27" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E19" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>1054</v>
+      </c>
+      <c r="G19" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19" s="29" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28" t="s">
+        <v>1057</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>1058</v>
+      </c>
+      <c r="G20" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I20" s="29" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="27" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D21" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>1062</v>
+      </c>
+      <c r="G21" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="29" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="27" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28" t="s">
+        <v>1065</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>1066</v>
+      </c>
+      <c r="G22" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="29" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="27" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28" t="s">
         <v>1009</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="29" t="s">
-        <v>1010</v>
-      </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30" t="s">
-        <v>1011</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E14" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>1012</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H14" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="31" t="s">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="29" t="s">
-        <v>1014</v>
-      </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30" t="s">
-        <v>1015</v>
-      </c>
-      <c r="D15" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F15" s="30" t="s">
-        <v>1016</v>
-      </c>
-      <c r="G15" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I15" s="31" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="29" t="s">
-        <v>1018</v>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30" t="s">
-        <v>1019</v>
-      </c>
-      <c r="D16" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F16" s="30" t="s">
+      <c r="D23" s="28" t="s">
         <v>1020</v>
       </c>
-      <c r="G16" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I16" s="31" t="s">
+      <c r="E23" s="28" t="s">
         <v>1021</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="29" t="s">
-        <v>1022</v>
-      </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30" t="s">
-        <v>1023</v>
-      </c>
-      <c r="D17" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F17" s="30" t="s">
-        <v>1024</v>
-      </c>
-      <c r="G17" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H17" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I17" s="31" t="s">
-        <v>1025</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="29" t="s">
-        <v>1026</v>
-      </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30" t="s">
-        <v>1027</v>
-      </c>
-      <c r="D18" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F18" s="30" t="s">
-        <v>1028</v>
-      </c>
-      <c r="G18" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I18" s="31" t="s">
-        <v>1029</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
-        <v>1030</v>
-      </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30" t="s">
-        <v>1031</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F19" s="30" t="s">
-        <v>1032</v>
-      </c>
-      <c r="G19" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H19" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I19" s="31" t="s">
-        <v>1033</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
-        <v>1034</v>
-      </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30" t="s">
-        <v>1035</v>
-      </c>
-      <c r="D20" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F20" s="30" t="s">
-        <v>1036</v>
-      </c>
-      <c r="G20" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H20" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I20" s="31" t="s">
-        <v>1037</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="29" t="s">
-        <v>1038</v>
-      </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30" t="s">
-        <v>1039</v>
-      </c>
-      <c r="D21" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E21" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F21" s="30" t="s">
-        <v>1040</v>
-      </c>
-      <c r="G21" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H21" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I21" s="31" t="s">
-        <v>1041</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="29" t="s">
-        <v>1042</v>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30" t="s">
-        <v>1043</v>
-      </c>
-      <c r="D22" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F22" s="30" t="s">
-        <v>1044</v>
-      </c>
-      <c r="G22" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H22" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I22" s="31" t="s">
-        <v>1045</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="29" t="s">
-        <v>1046</v>
-      </c>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30" t="s">
-        <v>987</v>
-      </c>
-      <c r="D23" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E23" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F23" s="30" t="s">
-        <v>1047</v>
-      </c>
-      <c r="G23" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H23" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I23" s="31" t="s">
-        <v>1048</v>
+      <c r="F23" s="28" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G23" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H23" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="29" t="s">
+        <v>1070</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="29" t="s">
-        <v>1049</v>
-      </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30" t="s">
-        <v>1050</v>
-      </c>
-      <c r="D24" s="30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>999</v>
-      </c>
-      <c r="F24" s="30" t="s">
-        <v>1051</v>
-      </c>
-      <c r="G24" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="H24" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I24" s="31" t="s">
-        <v>1052</v>
+      <c r="A24" s="27" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D24" s="28" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E24" s="28" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>1073</v>
+      </c>
+      <c r="G24" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" s="29" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="35" t="s">
-        <v>1053</v>
-      </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="36" t="s">
-        <v>1054</v>
-      </c>
-      <c r="D25" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E25" s="36" t="s">
-        <v>999</v>
-      </c>
-      <c r="F25" s="36" t="s">
-        <v>1055</v>
-      </c>
-      <c r="G25" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="37" t="s">
-        <v>1056</v>
+      <c r="A25" s="33" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B25" s="34"/>
+      <c r="C25" s="34" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E25" s="34" t="s">
+        <v>1021</v>
+      </c>
+      <c r="F25" s="34" t="s">
+        <v>1077</v>
+      </c>
+      <c r="G25" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="35" t="s">
+        <v>1078</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="35" t="s">
-        <v>1057</v>
-      </c>
-      <c r="B26" s="36"/>
-      <c r="C26" s="36" t="s">
-        <v>1058</v>
-      </c>
-      <c r="D26" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E26" s="36" t="s">
-        <v>1059</v>
-      </c>
-      <c r="F26" s="36" t="s">
-        <v>1060</v>
-      </c>
-      <c r="G26" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I26" s="37" t="s">
-        <v>1061</v>
+      <c r="A26" s="33" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E26" s="34" t="s">
+        <v>1081</v>
+      </c>
+      <c r="F26" s="34" t="s">
+        <v>1082</v>
+      </c>
+      <c r="G26" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="35" t="s">
+        <v>1083</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="35" t="s">
-        <v>1062</v>
-      </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36" t="s">
-        <v>1063</v>
-      </c>
-      <c r="D27" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E27" s="36" t="s">
-        <v>1064</v>
-      </c>
-      <c r="F27" s="36" t="s">
-        <v>1065</v>
-      </c>
-      <c r="G27" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H27" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I27" s="37" t="s">
-        <v>1066</v>
+      <c r="A27" s="33" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34" t="s">
+        <v>1085</v>
+      </c>
+      <c r="D27" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E27" s="34" t="s">
+        <v>1086</v>
+      </c>
+      <c r="F27" s="34" t="s">
+        <v>1087</v>
+      </c>
+      <c r="G27" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H27" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="35" t="s">
+        <v>1088</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="35" t="s">
-        <v>1067</v>
-      </c>
-      <c r="B28" s="36"/>
-      <c r="C28" s="36" t="s">
-        <v>1068</v>
-      </c>
-      <c r="D28" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E28" s="36" t="s">
-        <v>1069</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>1070</v>
-      </c>
-      <c r="G28" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="37" t="s">
-        <v>1071</v>
+      <c r="A28" s="33" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E28" s="34" t="s">
+        <v>1091</v>
+      </c>
+      <c r="F28" s="34" t="s">
+        <v>1092</v>
+      </c>
+      <c r="G28" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="35" t="s">
+        <v>1093</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="35" t="s">
-        <v>1072</v>
-      </c>
-      <c r="B29" s="36"/>
-      <c r="C29" s="36" t="s">
-        <v>1073</v>
-      </c>
-      <c r="D29" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E29" s="36" t="s">
-        <v>1074</v>
-      </c>
-      <c r="F29" s="36" t="s">
-        <v>1075</v>
-      </c>
-      <c r="G29" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H29" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29" s="37" t="s">
-        <v>1076</v>
+      <c r="A29" s="33" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B29" s="34"/>
+      <c r="C29" s="34" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E29" s="34" t="s">
+        <v>1096</v>
+      </c>
+      <c r="F29" s="34" t="s">
+        <v>1097</v>
+      </c>
+      <c r="G29" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="35" t="s">
+        <v>1098</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="35" t="s">
-        <v>1077</v>
-      </c>
-      <c r="B30" s="36"/>
-      <c r="C30" s="36" t="s">
-        <v>1078</v>
-      </c>
-      <c r="D30" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E30" s="36" t="s">
-        <v>1079</v>
-      </c>
-      <c r="F30" s="36" t="s">
-        <v>1080</v>
-      </c>
-      <c r="G30" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="37" t="s">
-        <v>1081</v>
+      <c r="A30" s="33" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B30" s="34"/>
+      <c r="C30" s="34" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D30" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E30" s="34" t="s">
+        <v>1101</v>
+      </c>
+      <c r="F30" s="34" t="s">
+        <v>1102</v>
+      </c>
+      <c r="G30" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H30" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="35" t="s">
+        <v>1103</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="35" t="s">
-        <v>1082</v>
-      </c>
-      <c r="B31" s="36"/>
-      <c r="C31" s="36" t="s">
-        <v>987</v>
-      </c>
-      <c r="D31" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E31" s="36" t="s">
-        <v>1083</v>
-      </c>
-      <c r="F31" s="36" t="s">
-        <v>1084</v>
-      </c>
-      <c r="G31" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H31" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I31" s="37" t="s">
-        <v>1085</v>
+      <c r="A31" s="33" t="s">
+        <v>1104</v>
+      </c>
+      <c r="B31" s="34"/>
+      <c r="C31" s="34" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E31" s="34" t="s">
+        <v>1105</v>
+      </c>
+      <c r="F31" s="34" t="s">
+        <v>1106</v>
+      </c>
+      <c r="G31" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H31" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="35" t="s">
+        <v>1107</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="35" t="s">
-        <v>1086</v>
-      </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36" t="s">
-        <v>1087</v>
-      </c>
-      <c r="D32" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E32" s="36" t="s">
-        <v>1088</v>
-      </c>
-      <c r="F32" s="36" t="s">
-        <v>1089</v>
-      </c>
-      <c r="G32" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32" s="37" t="s">
-        <v>1090</v>
+      <c r="A32" s="33" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B32" s="34"/>
+      <c r="C32" s="34" t="s">
+        <v>1109</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E32" s="34" t="s">
+        <v>1110</v>
+      </c>
+      <c r="F32" s="34" t="s">
+        <v>1111</v>
+      </c>
+      <c r="G32" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" s="35" t="s">
+        <v>1112</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="35" t="s">
-        <v>1091</v>
-      </c>
-      <c r="B33" s="36"/>
-      <c r="C33" s="36" t="s">
-        <v>1092</v>
-      </c>
-      <c r="D33" s="36" t="s">
-        <v>998</v>
-      </c>
-      <c r="E33" s="36" t="s">
-        <v>1093</v>
-      </c>
-      <c r="F33" s="36" t="s">
-        <v>1094</v>
-      </c>
-      <c r="G33" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="H33" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="I33" s="37" t="s">
-        <v>1095</v>
+      <c r="A33" s="33" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34" t="s">
+        <v>1114</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E33" s="34" t="s">
+        <v>1115</v>
+      </c>
+      <c r="F33" s="34" t="s">
+        <v>1116</v>
+      </c>
+      <c r="G33" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H33" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="35" t="s">
+        <v>1117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: sync parity map with access administration
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="1118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2112" uniqueCount="1123">
   <si>
     <t>Bank of Z Legacy User Flows / Parity Map</t>
   </si>
@@ -3069,7 +3069,7 @@
     <t>Implement Feature 009 delivery operations and approved deviations.</t>
   </si>
   <si>
-    <t>Not checked: target implementation has not started. specs/009-delivery-operations/</t>
+    <t>Feature 009 delivered and independently accepted. specs/009-delivery-operations/; analysis/stage-08-feature-009-delivery.md; analysis/stage-09-feature-009-live-revision.md; analysis/reviews/stage-10-pass-014.md; deployed /z-bank-new/</t>
   </si>
   <si>
     <t>R1-D-001</t>
@@ -3370,13 +3370,28 @@
   </si>
   <si>
     <t>analysis/stage-04-requirements-revision.md#d-023</t>
+  </si>
+  <si>
+    <t>R1-D-024</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>The target Administrator route was exposed as a visible placeholder with no useful action. No equivalent identity-administration behavior exists in the legacy map.</t>
+  </si>
+  <si>
+    <t>Implement owner-approved Feature 010 Access Administration: user search and creation, governed role and lockout changes, and immutable security-audit review.</t>
+  </si>
+  <si>
+    <t>Owner-approved target-only correction. specs/010-access-administration/; analysis/stage-05-access-administration-report.md; analysis/stage-08-feature-010-delivery.md; analysis/stage-09-feature-010-live-acceptance.md; analysis/reviews/stage-10-pass-015.md; deployed /z-bank-new/administration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -3428,8 +3443,12 @@
       <sz val="10"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3499,11 +3518,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -3713,7 +3727,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3794,15 +3808,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3812,6 +3817,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10149,7 +10155,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -10447,7 +10453,7 @@
         <v>36</v>
       </c>
       <c r="H10" s="31" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I10" s="32" t="s">
         <v>1017</v>
@@ -10832,246 +10838,273 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="30" t="s">
         <v>1075</v>
       </c>
-      <c r="B25" s="34"/>
-      <c r="C25" s="34" t="s">
+      <c r="B25" s="31"/>
+      <c r="C25" s="31" t="s">
         <v>1076</v>
       </c>
-      <c r="D25" s="34" t="s">
+      <c r="D25" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E25" s="34" t="s">
+      <c r="E25" s="31" t="s">
         <v>1021</v>
       </c>
-      <c r="F25" s="34" t="s">
+      <c r="F25" s="31" t="s">
         <v>1077</v>
       </c>
-      <c r="G25" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="35" t="s">
+      <c r="G25" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="32" t="s">
         <v>1078</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="30" t="s">
         <v>1079</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34" t="s">
+      <c r="B26" s="31"/>
+      <c r="C26" s="31" t="s">
         <v>1080</v>
       </c>
-      <c r="D26" s="34" t="s">
+      <c r="D26" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E26" s="34" t="s">
+      <c r="E26" s="31" t="s">
         <v>1081</v>
       </c>
-      <c r="F26" s="34" t="s">
+      <c r="F26" s="31" t="s">
         <v>1082</v>
       </c>
-      <c r="G26" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I26" s="35" t="s">
+      <c r="G26" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H26" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="32" t="s">
         <v>1083</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="30" t="s">
         <v>1084</v>
       </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34" t="s">
+      <c r="B27" s="31"/>
+      <c r="C27" s="31" t="s">
         <v>1085</v>
       </c>
-      <c r="D27" s="34" t="s">
+      <c r="D27" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="31" t="s">
         <v>1086</v>
       </c>
-      <c r="F27" s="34" t="s">
+      <c r="F27" s="31" t="s">
         <v>1087</v>
       </c>
-      <c r="G27" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H27" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I27" s="35" t="s">
+      <c r="G27" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H27" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="32" t="s">
         <v>1088</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="33" t="s">
+      <c r="A28" s="30" t="s">
         <v>1089</v>
       </c>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="31" t="s">
         <v>1090</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="31" t="s">
         <v>1091</v>
       </c>
-      <c r="F28" s="34" t="s">
+      <c r="F28" s="31" t="s">
         <v>1092</v>
       </c>
-      <c r="G28" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="35" t="s">
+      <c r="G28" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="32" t="s">
         <v>1093</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="33" t="s">
+      <c r="A29" s="30" t="s">
         <v>1094</v>
       </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34" t="s">
+      <c r="B29" s="31"/>
+      <c r="C29" s="31" t="s">
         <v>1095</v>
       </c>
-      <c r="D29" s="34" t="s">
+      <c r="D29" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E29" s="34" t="s">
+      <c r="E29" s="31" t="s">
         <v>1096</v>
       </c>
-      <c r="F29" s="34" t="s">
+      <c r="F29" s="31" t="s">
         <v>1097</v>
       </c>
-      <c r="G29" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H29" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29" s="35" t="s">
+      <c r="G29" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H29" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="32" t="s">
         <v>1098</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="33" t="s">
+      <c r="A30" s="30" t="s">
         <v>1099</v>
       </c>
-      <c r="B30" s="34"/>
-      <c r="C30" s="34" t="s">
+      <c r="B30" s="31"/>
+      <c r="C30" s="31" t="s">
         <v>1100</v>
       </c>
-      <c r="D30" s="34" t="s">
+      <c r="D30" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E30" s="34" t="s">
+      <c r="E30" s="31" t="s">
         <v>1101</v>
       </c>
-      <c r="F30" s="34" t="s">
+      <c r="F30" s="31" t="s">
         <v>1102</v>
       </c>
-      <c r="G30" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="35" t="s">
+      <c r="G30" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H30" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="32" t="s">
         <v>1103</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="33" t="s">
+      <c r="A31" s="30" t="s">
         <v>1104</v>
       </c>
-      <c r="B31" s="34"/>
-      <c r="C31" s="34" t="s">
+      <c r="B31" s="31"/>
+      <c r="C31" s="31" t="s">
         <v>1009</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E31" s="34" t="s">
+      <c r="E31" s="31" t="s">
         <v>1105</v>
       </c>
-      <c r="F31" s="34" t="s">
+      <c r="F31" s="31" t="s">
         <v>1106</v>
       </c>
-      <c r="G31" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H31" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I31" s="35" t="s">
+      <c r="G31" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H31" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="32" t="s">
         <v>1107</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="33" t="s">
+      <c r="A32" s="30" t="s">
         <v>1108</v>
       </c>
-      <c r="B32" s="34"/>
-      <c r="C32" s="34" t="s">
+      <c r="B32" s="31"/>
+      <c r="C32" s="31" t="s">
         <v>1109</v>
       </c>
-      <c r="D32" s="34" t="s">
+      <c r="D32" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E32" s="34" t="s">
+      <c r="E32" s="31" t="s">
         <v>1110</v>
       </c>
-      <c r="F32" s="34" t="s">
+      <c r="F32" s="31" t="s">
         <v>1111</v>
       </c>
-      <c r="G32" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32" s="35" t="s">
+      <c r="G32" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" s="32" t="s">
         <v>1112</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="30" t="s">
         <v>1113</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34" t="s">
+      <c r="B33" s="31"/>
+      <c r="C33" s="31" t="s">
         <v>1114</v>
       </c>
-      <c r="D33" s="34" t="s">
+      <c r="D33" s="31" t="s">
         <v>1020</v>
       </c>
-      <c r="E33" s="34" t="s">
+      <c r="E33" s="31" t="s">
         <v>1115</v>
       </c>
-      <c r="F33" s="34" t="s">
+      <c r="F33" s="31" t="s">
         <v>1116</v>
       </c>
-      <c r="G33" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="H33" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="I33" s="35" t="s">
+      <c r="G33" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H33" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="32" t="s">
         <v>1117</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="33" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B34" s="33"/>
+      <c r="C34" s="33" t="s">
+        <v>1119</v>
+      </c>
+      <c r="D34" s="33" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>1120</v>
+      </c>
+      <c r="F34" s="33" t="s">
+        <v>1121</v>
+      </c>
+      <c r="G34" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="H34" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="I34" s="33" t="s">
+        <v>1122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: fix access administration map wrapping
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -3727,7 +3727,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3817,7 +3817,15 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11084,26 +11092,26 @@
       <c r="A34" s="33" t="s">
         <v>1118</v>
       </c>
-      <c r="B34" s="33"/>
-      <c r="C34" s="33" t="s">
+      <c r="B34" s="34"/>
+      <c r="C34" s="34" t="s">
         <v>1119</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="34" t="s">
         <v>1020</v>
       </c>
-      <c r="E34" s="33" t="s">
+      <c r="E34" s="34" t="s">
         <v>1120</v>
       </c>
-      <c r="F34" s="33" t="s">
+      <c r="F34" s="34" t="s">
         <v>1121</v>
       </c>
-      <c r="G34" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="H34" s="33" t="s">
-        <v>36</v>
-      </c>
-      <c r="I34" s="33" t="s">
+      <c r="G34" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="H34" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="I34" s="35" t="s">
         <v>1122</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: organize migration analysis artifacts
</commit_message>
<xml_diff>
--- a/analysis/legacy_user_flows.xlsx
+++ b/analysis/legacy_user_flows.xlsx
@@ -1905,7 +1905,7 @@
     <t>modern/backend/src/BankOfZ.Api/Contracts/GenerateStatementRequest.cs; modern/backend/src/BankOfZ.Application/Statements/StatementOptions.cs; StatementService.cs; StatementApiTests.cs</t>
   </si>
   <si>
-    <t>specs/007-monthly-statements/spec.md FR-001, FR-002; plan.md; analysis/stage-04-requirements-revision.md D-012</t>
+    <t>specs/007-monthly-statements/spec.md FR-001, FR-002; plan.md; analysis/stages/stage-04/stage-04-requirements-revision.md D-012</t>
   </si>
   <si>
     <t>Statement includes customer and account identity</t>
@@ -2025,7 +2025,7 @@
     <t>modern/frontend/bank-of-z-ui/src/app/statements/statement.component.html; modern/frontend/bank-of-z-ui/src/app/statements/statement.component.scss; statement.component.spec.ts</t>
   </si>
   <si>
-    <t>specs/007-monthly-statements/spec.md FR-010; plan.md; analysis/stage-04-requirements-revision.md D-012</t>
+    <t>specs/007-monthly-statements/spec.md FR-010; plan.md; analysis/stages/stage-04/stage-04-requirements-revision.md D-012</t>
   </si>
   <si>
     <t>Statement database operation fails</t>
@@ -2994,7 +2994,7 @@
     <t>Implement Feature 004 deposits and withdrawals.</t>
   </si>
   <si>
-    <t>Feature 004 delivered and browser-accepted. specs/004-cash-transactions/; analysis/reviews/feature-004-implementation-review.md; analysis/stage-08-feature-004-delivery.md; analysis/stage-09-feature-004-live-revision.md; deployed /z-bank-new/</t>
+    <t>Feature 004 delivered and browser-accepted. specs/004-cash-transactions/; analysis/reviews/feature-004-implementation-review.md; analysis/stages/stage-08/stage-08-feature-004-delivery.md; analysis/stages/stage-09/stage-09-feature-004-live-revision.md; deployed /z-bank-new/</t>
   </si>
   <si>
     <t>R1-G05</t>
@@ -3009,7 +3009,7 @@
     <t>Implement Feature 005 funds transfers.</t>
   </si>
   <si>
-    <t>Feature 005 delivered and browser-accepted. specs/005-funds-transfers/; analysis/reviews/feature-005-implementation-review.md; analysis/stage-08-feature-005-delivery.md; analysis/stage-09-feature-005-live-revision.md; deployed /z-bank-new/</t>
+    <t>Feature 005 delivered and browser-accepted. specs/005-funds-transfers/; analysis/reviews/feature-005-implementation-review.md; analysis/stages/stage-08/stage-08-feature-005-delivery.md; analysis/stages/stage-09/stage-09-feature-005-live-revision.md; deployed /z-bank-new/</t>
   </si>
   <si>
     <t>R1-G06</t>
@@ -3069,7 +3069,7 @@
     <t>Implement Feature 009 delivery operations and approved deviations.</t>
   </si>
   <si>
-    <t>Feature 009 delivered and independently accepted. specs/009-delivery-operations/; analysis/stage-08-feature-009-delivery.md; analysis/stage-09-feature-009-live-revision.md; analysis/reviews/stage-10-pass-014.md; deployed /z-bank-new/</t>
+    <t>Feature 009 delivered and independently accepted. specs/009-delivery-operations/; analysis/stages/stage-08/stage-08-feature-009-delivery.md; analysis/stages/stage-09/stage-09-feature-009-live-revision.md; analysis/reviews/stage-10-pass-014.md; deployed /z-bank-new/</t>
   </si>
   <si>
     <t>R1-D-001</t>
@@ -3087,7 +3087,7 @@
     <t>Owner-approved target decision D-001 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-001; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-001; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-002</t>
@@ -3099,7 +3099,7 @@
     <t>Owner-approved target decision D-002 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-002; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-002; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-003</t>
@@ -3111,7 +3111,7 @@
     <t>Owner-approved target decision D-003 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-003; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-003; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-004</t>
@@ -3123,7 +3123,7 @@
     <t>Owner-approved target decision D-004 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-004; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-004; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-005</t>
@@ -3135,7 +3135,7 @@
     <t>Owner-approved target decision D-005 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-005; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-005; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-006</t>
@@ -3147,7 +3147,7 @@
     <t>Owner-approved target decision D-006 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-006; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-006; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-007</t>
@@ -3159,7 +3159,7 @@
     <t>Owner-approved target decision D-007 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-007; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-007; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-008</t>
@@ -3171,7 +3171,7 @@
     <t>Owner-approved target decision D-008 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-008; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-008; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-009</t>
@@ -3183,7 +3183,7 @@
     <t>Owner-approved target decision D-009 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-009; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-009; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-010</t>
@@ -3195,7 +3195,7 @@
     <t>Owner-approved target decision D-010 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-010; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-010; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-011</t>
@@ -3207,7 +3207,7 @@
     <t>Owner-approved target decision D-011 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-011; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-011; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-012</t>
@@ -3219,7 +3219,7 @@
     <t>Owner-approved target decision D-012 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-012; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-012; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-013</t>
@@ -3228,7 +3228,7 @@
     <t>Owner-approved target decision D-013 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-013; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-013; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-014</t>
@@ -3240,7 +3240,7 @@
     <t>Owner-approved target decision D-014 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-014; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-014; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-015</t>
@@ -3252,7 +3252,7 @@
     <t>Owner-approved target decision D-015 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-015; approved by project owner on 2026-07-21.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-015; approved by project owner on 2026-07-21.</t>
   </si>
   <si>
     <t>R1-D-016</t>
@@ -3267,7 +3267,7 @@
     <t>Owner-approved target decision D-016 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-016; approved by project owner on 2026-07-22.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-016; approved by project owner on 2026-07-22.</t>
   </si>
   <si>
     <t>R1-D-017</t>
@@ -3282,7 +3282,7 @@
     <t>Owner-approved target decision D-017 recorded in Stage 4.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-017; approved by project owner on 2026-07-22.</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-017; approved by project owner on 2026-07-22.</t>
   </si>
   <si>
     <t>R1-D-018</t>
@@ -3297,7 +3297,7 @@
     <t>Target implements normalized search; failed lookup clears stale state and disables mutation.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-018</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-018</t>
   </si>
   <si>
     <t>R1-D-019</t>
@@ -3312,7 +3312,7 @@
     <t>Target returns the complete authorized portfolio through bounded pagination.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-019</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-019</t>
   </si>
   <si>
     <t>R1-D-020</t>
@@ -3327,7 +3327,7 @@
     <t>Target derives validated sort code from account/bank configuration.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-020</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-020</t>
   </si>
   <si>
     <t>R1-D-021</t>
@@ -3339,7 +3339,7 @@
     <t>Use guarded deterministic reset plus staged atomic import and resumable run ledger.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-021</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-021</t>
   </si>
   <si>
     <t>R1-D-022</t>
@@ -3354,7 +3354,7 @@
     <t>Move identity to configuration and do not port these utilities.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-022</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-022</t>
   </si>
   <si>
     <t>R1-D-023</t>
@@ -3369,7 +3369,7 @@
     <t>Target allocation/entity/audit persistence is atomic; identifier gaps are allowed.</t>
   </si>
   <si>
-    <t>analysis/stage-04-requirements-revision.md#d-023</t>
+    <t>analysis/stages/stage-04/stage-04-requirements-revision.md#d-023</t>
   </si>
   <si>
     <t>R1-D-024</t>
@@ -3384,7 +3384,7 @@
     <t>Implement owner-approved Feature 010 Access Administration: user search and creation, governed role and lockout changes, and immutable security-audit review.</t>
   </si>
   <si>
-    <t>Owner-approved target-only correction. specs/010-access-administration/; analysis/stage-05-access-administration-report.md; analysis/stage-08-feature-010-delivery.md; analysis/stage-09-feature-010-live-acceptance.md; analysis/reviews/stage-10-pass-015.md; deployed /z-bank-new/administration</t>
+    <t>Owner-approved target-only correction. specs/010-access-administration/; analysis/stages/stage-05/stage-05-access-administration-report.md; analysis/stages/stage-08/stage-08-feature-010-delivery.md; analysis/stages/stage-09/stage-09-feature-010-live-acceptance.md; analysis/reviews/stage-10-pass-015.md; deployed /z-bank-new/administration</t>
   </si>
 </sst>
 </file>

</xml_diff>